<commit_message>
improved loss function on mit-b3
</commit_message>
<xml_diff>
--- a/Scores.xlsx
+++ b/Scores.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="240">
   <si>
     <t xml:space="preserve">Description</t>
   </si>
@@ -2977,6 +2977,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">improved loss function
 </t>
@@ -2986,6 +2987,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">
 Segformer with mit_b1 encoder 
@@ -3045,6 +3047,606 @@
 360     | 310     | 0.142      | 0.826           | 0.654        | 0.059             | 0.238    0.079    0.148    0.009    0.431    0.344    0.337   | 0.725  0.549  0.714  | 0.081  0.055  0.041 
 276     | 276     | 0.244      | 0.837           | 0.707        | 0.076             | 0.458    0.100    0.176    0.024    0.703    0.558    0.394   | 0.774  0.608  0.709  | 0.105  0.093  0.030 </t>
   </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.25/0.75, 15 epoch, 
+final LR 3e-4
+(36m 8s)
+(Max GPU mem usage : 10716.875 MB) 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.650      | 0.396      | 0.424           | 0.135        | 0.382             | 0.394    0.735    0.992    0.478    0.427    0.353    0.361   | 0.243    0.447    0.511    0.382    0.416    0.367    0.388   | 0.269  0.096  0.000  | 0.076  0.072  1.000 
+2     | 0.000250  | 0.568      | 0.380      | 0.599           | 0.201        | 0.136             | 0.218    0.684    0.983    0.386    0.424    0.359    0.342   | 0.328    0.397    0.491    0.302    0.505    0.437    0.447   | 0.354  0.085  0.137  | 0.095  0.055  0.257 
+3     | 0.000500  | 0.552      | 0.349      | 0.653           | 0.322        | 0.127             | 0.287    0.640    0.975    0.305    0.463    0.401    0.384   | 0.405    0.331    0.452    0.209    0.601    0.422    0.490   | 0.477  0.258  0.230  | 0.168  0.132  0.080 
+4     | 0.000497  | 0.532      | 0.334      | 0.634           | 0.259        | 0.116             | 0.347    0.594    0.960    0.228    0.500    0.435    0.416   | 0.504    0.277    0.454    0.100    0.621    0.616    0.454   | 0.410  0.190  0.110  | 0.141  0.124  0.084 
+5     | 0.000487  | 0.431      | 0.294      | 0.712           | 0.399        | 0.079             | 0.508    0.406    0.753    0.058    0.660    0.575    0.533   | 0.651    0.175    0.326    0.025    0.653    0.641    0.734   | 0.540  0.292  0.377  | 0.090  0.072  0.075 
+6     | 0.000471  | 0.283      | 0.236      | 0.737           | 0.458        | 0.077             | 0.518    0.204    0.398    0.011    0.626    0.596    0.633   | 0.479    0.155    0.284    0.026    0.654    0.571    0.587   | 0.568  0.341  0.495  | 0.086  0.098  0.045 
+7     | 0.000450  | 0.224      | 0.219      | 0.754           | 0.479        | 0.063             | 0.431    0.154    0.300    0.008    0.591    0.555    0.581   | 0.413    0.154    0.281    0.027    0.548    0.520    0.557   | 0.576  0.364  0.564  | 0.050  0.072  0.066 
+8     | 0.000426  | 0.186      | 0.210      | 0.760           | 0.492        | 0.061             | 0.377    0.122    0.236    0.007    0.570    0.531    0.545   | 0.400    0.147    0.267    0.027    0.542    0.536    0.539   | 0.614  0.359  0.548  | 0.060  0.069  0.053 
+9     | 0.000400  | 0.166      | 0.230      | 0.736           | 0.448        | 0.073             | 0.343    0.107    0.207    0.006    0.556    0.512    0.526   | 0.455    0.155    0.276    0.033    0.617    0.530    0.532   | 0.513  0.331  0.566  | 0.055  0.083  0.080 
+10    | 0.000374  | 0.149      | 0.237      | 0.742           | 0.468        | 0.075             | 0.310    0.095    0.184    0.006    0.542    0.495    0.510   | 0.502    0.149    0.267    0.031    0.584    0.516    0.596   | 0.548  0.347  0.571  | 0.064  0.080  0.080 
+11    | 0.000350  | 0.138      | 0.217      | 0.751           | 0.475        | 0.066             | 0.284    0.090    0.173    0.006    0.530    0.480    0.484   | 0.429    0.146    0.261    0.030    0.591    0.530    0.542   | 0.556  0.359  0.573  | 0.067  0.075  0.055 
+12    | 0.000329  | 0.131      | 0.207      | 0.747           | 0.472        | 0.069             | 0.269    0.084    0.164    0.005    0.527    0.472    0.472   | 0.381    0.149    0.265    0.033    0.565    0.495    0.516   | 0.560  0.376  0.535  | 0.055  0.095  0.056 
+13    | 0.000313  | 0.121      | 0.191      | 0.765           | 0.511        | 0.065             | 0.249    0.079    0.152    0.005    0.516    0.461    0.463   | 0.340    0.141    0.250    0.032    0.553    0.471    0.489   | 0.588  0.389  0.582  | 0.063  0.072  0.060 
+14    | 0.000303  | 0.117      | 0.185      | 0.754           | 0.489        | 0.069             | 0.241    0.076    0.147    0.005    0.515    0.461    0.456   | 0.299    0.147    0.262    0.032    0.501    0.427    0.429   | 0.551  0.393  0.574  | 0.058  0.078  0.073 
+15    | 0.000300  | 0.115      | 0.188      | 0.763           | 0.506        | 0.065             | 0.236    0.074    0.143    0.005    0.510    0.459    0.448   | 0.302    0.150    0.268    0.031    0.485    0.388    0.416   | 0.586  0.371  0.581  | 0.067  0.064  0.064</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.25/0.75, 15 epoch, 
+final LR 2.5e-4
+(35m 32s)
+(Max GPU mem usage : 10716.875 MB) 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.651      | 0.400      | 0.427           | 0.144        | 0.385             | 0.389    0.738    0.992    0.483    0.428    0.349    0.358   | 0.264    0.445    0.510    0.380    0.424    0.359    0.418   | 0.287  0.111  0.000  | 0.077  0.077  1.000 
+2     | 0.000250  | 0.569      | 0.368      | 0.635           | 0.267        | 0.120             | 0.219    0.686    0.984    0.388    0.422    0.356    0.342   | 0.256    0.405    0.483    0.328    0.460    0.359    0.397   | 0.443  0.231  0.092  | 0.135  0.109  0.116 
+3     | 0.000500  | 0.550      | 0.373      | 0.640           | 0.331        | 0.154             | 0.295    0.635    0.974    0.297    0.475    0.413    0.392   | 0.342    0.384    0.482    0.285    0.540    0.505    0.379   | 0.502  0.178  0.249  | 0.174  0.162  0.124 
+4     | 0.000496  | 0.487      | 0.304      | 0.702           | 0.417        | 0.109             | 0.415    0.511    0.885    0.137    0.625    0.515    0.467   | 0.574    0.213    0.378    0.049    0.699    0.661    0.552   | 0.516  0.240  0.470  | 0.093  0.117  0.116 
+5     | 0.000483  | 0.329      | 0.267      | 0.709           | 0.401        | 0.085             | 0.537    0.259    0.501    0.017    0.657    0.622    0.619   | 0.530    0.180    0.329    0.031    0.590    0.594    0.663   | 0.520  0.333  0.378  | 0.081  0.074  0.098 
+6     | 0.000463  | 0.238      | 0.241      | 0.725           | 0.473        | 0.108             | 0.478    0.158    0.309    0.008    0.613    0.581    0.613   | 0.503    0.153    0.278    0.028    0.631    0.571    0.616   | 0.563  0.336  0.532  | 0.099  0.119  0.105 
+7     | 0.000438  | 0.200      | 0.227      | 0.750           | 0.464        | 0.060             | 0.407    0.131    0.255    0.007    0.583    0.549    0.571   | 0.447    0.153    0.279    0.027    0.577    0.530    0.558   | 0.544  0.342  0.550  | 0.058  0.073  0.048 
+8     | 0.000407  | 0.173      | 0.218      | 0.753           | 0.480        | 0.064             | 0.370    0.107    0.208    0.006    0.569    0.529    0.541   | 0.427    0.148    0.268    0.028    0.569    0.519    0.561   | 0.574  0.359  0.547  | 0.068  0.072  0.053 
+9     | 0.000375  | 0.156      | 0.230      | 0.742           | 0.467        | 0.074             | 0.333    0.097    0.187    0.006    0.558    0.513    0.516   | 0.479    0.148    0.264    0.031    0.597    0.553    0.528   | 0.541  0.337  0.575  | 0.065  0.099  0.059 
+10    | 0.000343  | 0.144      | 0.236      | 0.751           | 0.488        | 0.074             | 0.308    0.089    0.173    0.005    0.543    0.495    0.509   | 0.504    0.147    0.262    0.031    0.588    0.523    0.589   | 0.572  0.348  0.582  | 0.071  0.099  0.051 
+11    | 0.000313  | 0.135      | 0.224      | 0.752           | 0.480        | 0.067             | 0.281    0.086    0.166    0.005    0.533    0.480    0.487   | 0.463    0.144    0.258    0.029    0.584    0.561    0.551   | 0.556  0.361  0.549  | 0.057  0.077  0.068 
+12    | 0.000287  | 0.126      | 0.217      | 0.739           | 0.452        | 0.069             | 0.265    0.079    0.154    0.005    0.531    0.475    0.476   | 0.399    0.157    0.278    0.036    0.552    0.494    0.528   | 0.511  0.373  0.513  | 0.051  0.081  0.075 
+13    | 0.000267  | 0.118      | 0.199      | 0.751           | 0.477        | 0.066             | 0.247    0.075    0.145    0.005    0.519    0.467    0.465   | 0.352    0.148    0.262    0.035    0.552    0.470    0.507   | 0.556  0.368  0.554  | 0.054  0.097  0.047 
+14    | 0.000254  | 0.115      | 0.216      | 0.736           | 0.470        | 0.087             | 0.240    0.073    0.141    0.005    0.519    0.460    0.464   | 0.410    0.151    0.269    0.034    0.555    0.486    0.450   | 0.522  0.337  0.618  | 0.085  0.099  0.075 
+15    | 0.000250  | 0.112      | 0.180      | 0.770           | 0.522        | 0.065             | 0.232    0.072    0.139    0.005    0.514    0.455    0.452   | 0.295    0.141    0.252    0.030    0.506    0.449    0.445   | 0.598  0.385  0.616  | 0.062  0.091  0.042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.25/0.75, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+(35m 17s)
+(Max GPU mem usage : 10716.875 MB) 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.650      | 0.396      | 0.425           | 0.144        | 0.387             | 0.397    0.734    0.992    0.476    0.430    0.352    0.362   | 0.244    0.446    0.511    0.382    0.447    0.359    0.375   | 0.268  0.127  0.000  | 0.064  0.096  1.000 
+2     | 0.000250  | 0.569      | 0.364      | 0.646           | 0.288        | 0.115             | 0.224    0.684    0.983    0.384    0.426    0.360    0.343   | 0.312    0.381    0.483    0.279    0.526    0.419    0.451   | 0.455  0.254  0.122  | 0.115  0.092  0.139 
+3     | 0.000375  | 0.534      | 0.352      | 0.671           | 0.386        | 0.140             | 0.222    0.637    0.972    0.303    0.465    0.400    0.378   | 0.316    0.365    0.474    0.255    0.523    0.464    0.377   | 0.512  0.226  0.369  | 0.151  0.146  0.122 
+4     | 0.000500  | 0.514      | 0.297      | 0.688           | 0.388        | 0.111             | 0.429    0.542    0.908    0.176    0.606    0.496    0.462   | 0.483    0.236    0.400    0.071    0.678    0.548    0.529   | 0.529  0.216  0.410  | 0.093  0.095  0.146 
+5     | 0.000495  | 0.337      | 0.270      | 0.708           | 0.405        | 0.090             | 0.536    0.270    0.519    0.021    0.663    0.626    0.607   | 0.558    0.174    0.320    0.028    0.629    0.625    0.656   | 0.529  0.297  0.428  | 0.078  0.127  0.066 
+6     | 0.000480  | 0.238      | 0.232      | 0.734           | 0.461        | 0.085             | 0.485    0.155    0.302    0.008    0.610    0.584    0.616   | 0.448    0.160    0.292    0.029    0.595    0.578    0.565   | 0.568  0.325  0.515  | 0.055  0.099  0.100 
+7     | 0.000457  | 0.201      | 0.222      | 0.743           | 0.449        | 0.061             | 0.420    0.128    0.249    0.007    0.588    0.552    0.572   | 0.420    0.156    0.286    0.027    0.561    0.537    0.550   | 0.558  0.342  0.475  | 0.060  0.072  0.051 
+8     | 0.000427  | 0.171      | 0.251      | 0.726           | 0.410        | 0.064             | 0.367    0.106    0.205    0.006    0.567    0.525    0.542   | 0.520    0.162    0.290    0.033    0.595    0.532    0.588   | 0.516  0.306  0.458  | 0.058  0.077  0.056 
+9     | 0.000393  | 0.158      | 0.220      | 0.750           | 0.464        | 0.059             | 0.334    0.099    0.191    0.006    0.557    0.515    0.514   | 0.439    0.147    0.264    0.029    0.599    0.550    0.513   | 0.535  0.327  0.609  | 0.055  0.081  0.042 
+10    | 0.000357  | 0.140      | 0.218      | 0.752           | 0.494        | 0.075             | 0.298    0.088    0.171    0.005    0.540    0.493    0.503   | 0.437    0.145    0.259    0.030    0.576    0.508    0.552   | 0.582  0.346  0.611  | 0.068  0.112  0.046 
+11    | 0.000323  | 0.133      | 0.224      | 0.748           | 0.465        | 0.064             | 0.280    0.084    0.162    0.005    0.530    0.480    0.483   | 0.449    0.149    0.266    0.031    0.579    0.520    0.557   | 0.559  0.345  0.507  | 0.062  0.075  0.055 
+12    | 0.000293  | 0.120      | 0.228      | 0.738           | 0.441        | 0.064             | 0.254    0.075    0.146    0.005    0.529    0.471    0.472   | 0.440    0.157    0.279    0.035    0.533    0.505    0.563   | 0.541  0.353  0.459  | 0.059  0.074  0.060 
+13    | 0.000270  | 0.116      | 0.204      | 0.765           | 0.519        | 0.071             | 0.243    0.074    0.143    0.005    0.518    0.463    0.465   | 0.405    0.136    0.242    0.030    0.557    0.484    0.536   | 0.601  0.369  0.610  | 0.068  0.088  0.056 
+14    | 0.000255  | 0.113      | 0.183      | 0.761           | 0.524        | 0.080             | 0.237    0.072    0.139    0.005    0.515    0.460    0.459   | 0.306    0.143    0.253    0.032    0.528    0.467    0.465   | 0.599  0.394  0.621  | 0.056  0.092  0.093 
+15    | 0.000250  | 0.111      | 0.183      | 0.772           | 0.516        | 0.058             | 0.233    0.070    0.135    0.005    0.513    0.455    0.455   | 0.295    0.146    0.256    0.035    0.506    0.432    0.419   | 0.585  0.388  0.606  | 0.056  0.077  0.042 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.25/0.75, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.25 i.e. 0.25D + 0.75B
+(35m 12s)
+(Max GPU mem usage : 10716.875 MB) 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.552      | 0.364      | 0.397           | 0.036        | 0.363             | 0.452    0.585    0.994    0.448    0.460    0.377    0.392   | 0.364    0.364    0.524    0.311    0.485    0.470    0.491   | 0.082  0.013  0.000  | 0.037  0.051  1.000 
+2     | 0.000250  | 0.446      | 0.345      | 0.425           | 0.126        | 0.376             | 0.352    0.477    0.988    0.306    0.491    0.435    0.426   | 0.366    0.338    0.510    0.281    0.420    0.398    0.512   | 0.321  0.004  0.000  | 0.092  0.037  1.000 
+3     | 0.000375  | 0.437      | 0.344      | 0.471           | 0.187        | 0.341             | 0.462    0.428    0.980    0.244    0.537    0.483    0.471   | 0.287    0.363    0.503    0.317    0.497    0.375    0.368   | 0.375  0.134  0.000  | 0.116  0.106  0.800 
+4     | 0.000500  | 0.343      | 0.232      | 0.683           | 0.398        | 0.128             | 0.435    0.312    0.924    0.109    0.597    0.530    0.509   | 0.486    0.148    0.424    0.055    0.636    0.558    0.547   | 0.505  0.250  0.399  | 0.123  0.112  0.148 
+5     | 0.000495  | 0.261      | 0.227      | 0.682           | 0.385        | 0.120             | 0.401    0.214    0.752    0.035    0.630    0.540    0.512   | 0.566    0.113    0.367    0.029    0.641    0.626    0.607   | 0.518  0.283  0.365  | 0.117  0.120  0.125 
+6     | 0.000480  | 0.217      | 0.205      | 0.721           | 0.447        | 0.096             | 0.409    0.153    0.564    0.016    0.608    0.546    0.558   | 0.537    0.094    0.310    0.023    0.626    0.568    0.636   | 0.579  0.303  0.483  | 0.107  0.103  0.077 
+7     | 0.000457  | 0.181      | 0.180      | 0.742           | 0.492        | 0.092             | 0.394    0.110    0.413    0.010    0.587    0.542    0.561   | 0.454    0.089    0.291    0.022    0.593    0.549    0.564   | 0.598  0.330  0.562  | 0.078  0.099  0.099 
+8     | 0.000427  | 0.156      | 0.184      | 0.730           | 0.448        | 0.082             | 0.359    0.088    0.330    0.008    0.569    0.521    0.543   | 0.462    0.092    0.293    0.025    0.588    0.542    0.557   | 0.585  0.347  0.445  | 0.073  0.105  0.067 
+9     | 0.000393  | 0.139      | 0.179      | 0.733           | 0.434        | 0.067             | 0.327    0.076    0.285    0.007    0.558    0.508    0.520   | 0.425    0.098    0.302    0.030    0.551    0.541    0.532   | 0.517  0.326  0.502  | 0.048  0.101  0.052 
+10    | 0.000357  | 0.127      | 0.165      | 0.746           | 0.477        | 0.075             | 0.302    0.068    0.255    0.006    0.546    0.494    0.505   | 0.388    0.090    0.285    0.025    0.542    0.509    0.534   | 0.565  0.354  0.556  | 0.059  0.090  0.075 
+11    | 0.000323  | 0.115      | 0.176      | 0.724           | 0.425        | 0.076             | 0.277    0.062    0.230    0.006    0.534    0.482    0.489   | 0.419    0.095    0.295    0.029    0.559    0.539    0.539   | 0.507  0.345  0.458  | 0.059  0.095  0.074 
+12    | 0.000293  | 0.111      | 0.169      | 0.731           | 0.438        | 0.074             | 0.267    0.060    0.222    0.006    0.530    0.475    0.477   | 0.395    0.094    0.285    0.030    0.572    0.505    0.535   | 0.555  0.358  0.449  | 0.055  0.098  0.069 
+13    | 0.000270  | 0.102      | 0.150      | 0.749           | 0.484        | 0.074             | 0.247    0.054    0.200    0.005    0.522    0.467    0.469   | 0.335    0.088    0.270    0.027    0.552    0.471    0.475   | 0.595  0.356  0.534  | 0.051  0.100  0.071 
+14    | 0.000255  | 0.099      | 0.147      | 0.738           | 0.474        | 0.086             | 0.239    0.052    0.194    0.005    0.520    0.463    0.463   | 0.313    0.092    0.280    0.029    0.529    0.459    0.426   | 0.579  0.373  0.521  | 0.058  0.097  0.101 
+15    | 0.000250  | 0.096      | 0.140      | 0.762           | 0.519        | 0.075             | 0.232    0.051    0.190    0.005    0.515    0.456    0.455   | 0.302    0.085    0.264    0.026    0.496    0.450    0.444   | 0.621  0.373  0.572  | 0.065  0.091  0.070 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.3/0.7, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.5
+(35m 24s)
+(Max GPU mem usage : 10716.875 MB) 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.641      | 0.395      | 0.413           | 0.143        | 0.407             | 0.406    0.741    0.992    0.489    0.422    0.349    0.361   | 0.238    0.463    0.511    0.414    0.430    0.321    0.398   | 0.331  0.046  0.000  | 0.112  0.110  1.000 
+2     | 0.000250  | 0.544      | 0.388      | 0.643           | 0.246        | 0.093             | 0.178    0.700    0.985    0.416    0.404    0.331    0.316   | 0.266    0.440    0.489    0.392    0.390    0.298    0.389   | 0.387  0.220  0.112  | 0.082  0.074  0.122 
+3     | 0.000375  | 0.530      | 0.341      | 0.675           | 0.353        | 0.110             | 0.195    0.674    0.979    0.370    0.424    0.356    0.336   | 0.258    0.377    0.464    0.289    0.470    0.395    0.379   | 0.533  0.270  0.249  | 0.125  0.089  0.117 
+4     | 0.000500  | 0.505      | 0.459      | 0.625           | 0.259        | 0.132             | 0.217    0.628    0.967    0.288    0.453    0.385    0.363   | 0.832    0.300    0.458    0.141    0.793    0.763    0.268   | 0.410  0.142  0.274  | 0.139  0.185  0.072 
+5     | 0.000495  | 0.462      | 0.302      | 0.704           | 0.419        | 0.106             | 0.409    0.485    0.849    0.120    0.619    0.504    0.452   | 0.551    0.196    0.357    0.034    0.639    0.610    0.630   | 0.572  0.272  0.403  | 0.083  0.097  0.138 
+6     | 0.000480  | 0.311      | 0.243      | 0.728           | 0.492        | 0.115             | 0.448    0.253    0.489    0.017    0.615    0.583    0.572   | 0.453    0.153    0.282    0.023    0.621    0.590    0.571   | 0.581  0.342  0.559  | 0.125  0.116  0.105 
+7     | 0.000457  | 0.235      | 0.243      | 0.740           | 0.459        | 0.074             | 0.409    0.161    0.314    0.008    0.579    0.546    0.571   | 0.444    0.156    0.285    0.027    0.588    0.562    0.557   | 0.566  0.352  0.516  | 0.084  0.070  0.068 
+8     | 0.000427  | 0.193      | 0.227      | 0.753           | 0.466        | 0.055             | 0.350    0.125    0.244    0.007    0.556    0.515    0.535   | 0.405    0.151    0.275    0.027    0.576    0.543    0.508   | 0.604  0.338  0.501  | 0.064  0.068  0.033 
+9     | 0.000393  | 0.171      | 0.233      | 0.746           | 0.475        | 0.074             | 0.313    0.110    0.214    0.006    0.542    0.497    0.509   | 0.436    0.146    0.263    0.029    0.580    0.532    0.502   | 0.564  0.336  0.594  | 0.057  0.079  0.084 
+10    | 0.000357  | 0.153      | 0.210      | 0.770           | 0.516        | 0.061             | 0.283    0.098    0.190    0.006    0.533    0.481    0.491   | 0.369    0.141    0.255    0.028    0.569    0.480    0.530   | 0.573  0.364  0.636  | 0.061  0.079  0.044 
+11    | 0.000323  | 0.139      | 0.221      | 0.761           | 0.528        | 0.084             | 0.252    0.090    0.175    0.005    0.519    0.466    0.468   | 0.424    0.134    0.241    0.026    0.570    0.519    0.533   | 0.603  0.373  0.625  | 0.061  0.094  0.097 
+12    | 0.000293  | 0.131      | 0.218      | 0.764           | 0.496        | 0.057             | 0.239    0.084    0.163    0.005    0.514    0.458    0.457   | 0.379    0.150    0.267    0.033    0.523    0.463    0.530   | 0.578  0.356  0.568  | 0.055  0.067  0.049 
+13    | 0.000270  | 0.125      | 0.203      | 0.774           | 0.526        | 0.062             | 0.227    0.081    0.157    0.005    0.507    0.453    0.451   | 0.358    0.137    0.242    0.031    0.556    0.475    0.483   | 0.620  0.364  0.618  | 0.061  0.077  0.047 
+14    | 0.000255  | 0.119      | 0.189      | 0.766           | 0.523        | 0.073             | 0.219    0.077    0.148    0.005    0.505    0.446    0.447   | 0.310    0.137    0.245    0.029    0.511    0.454    0.426   | 0.602  0.377  0.625  | 0.059  0.074  0.084 
+15    | 0.000250  | 0.113      | 0.187      | 0.772           | 0.520        | 0.060             | 0.206    0.073    0.141    0.005    0.500    0.440    0.438   | 0.295    0.142    0.254    0.029    0.481    0.410    0.423   | 0.594  0.348  0.641  | 0.064  0.067  0.049 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.3/0.7, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.5
+Dropout = 0.3
+(35m 35s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.637      | 0.386      | 0.414           | 0.112        | 0.385             | 0.390    0.744    0.993    0.495    0.422    0.344    0.357   | 0.204    0.463    0.515    0.411    0.425    0.333    0.366   | 0.273  0.026  0.000  | 0.081  0.074  1.000 
+2     | 0.000250  | 0.546      | 0.362      | 0.610           | 0.292        | 0.179             | 0.183    0.701    0.985    0.417    0.402    0.331    0.314   | 0.249    0.410    0.476    0.344    0.484    0.380    0.364   | 0.478  0.233  0.115  | 0.156  0.091  0.289 
+3     | 0.000375  | 0.529      | 0.348      | 0.653           | 0.342        | 0.140             | 0.203    0.669    0.978    0.360    0.436    0.364    0.341   | 0.324    0.358    0.465    0.252    0.545    0.447    0.432   | 0.476  0.213  0.270  | 0.161  0.145  0.113 
+4     | 0.000500  | 0.505      | 0.340      | 0.655           | 0.347        | 0.139             | 0.225    0.625    0.968    0.282    0.468    0.394    0.375   | 0.298    0.359    0.456    0.261    0.523    0.447    0.332   | 0.485  0.179  0.297  | 0.152  0.145  0.120 
+5     | 0.000495  | 0.430      | 0.330      | 0.686           | 0.413        | 0.133             | 0.331    0.472    0.833    0.111    0.608    0.494    0.435   | 0.634    0.199    0.356    0.043    0.669    0.667    0.575   | 0.519  0.273  0.455  | 0.084  0.121  0.194 
+6     | 0.000480  | 0.303      | 0.248      | 0.738           | 0.460        | 0.076             | 0.453    0.239    0.463    0.014    0.613    0.580    0.589   | 0.450    0.162    0.298    0.026    0.594    0.556    0.563   | 0.583  0.329  0.506  | 0.071  0.077  0.081 
+7     | 0.000457  | 0.227      | 0.260      | 0.751           | 0.474        | 0.064             | 0.396    0.154    0.300    0.008    0.573    0.543    0.567   | 0.520    0.148    0.271    0.025    0.583    0.558    0.597   | 0.613  0.342  0.488  | 0.054  0.070  0.068 
+8     | 0.000427  | 0.190      | 0.222      | 0.761           | 0.506        | 0.069             | 0.344    0.124    0.240    0.007    0.557    0.512    0.532   | 0.410    0.141    0.255    0.027    0.577    0.523    0.508   | 0.612  0.375  0.578  | 0.077  0.079  0.049 
+9     | 0.000393  | 0.168      | 0.213      | 0.759           | 0.480        | 0.056             | 0.310    0.108    0.209    0.006    0.541    0.495    0.507   | 0.364    0.148    0.266    0.030    0.555    0.470    0.513   | 0.565  0.347  0.589  | 0.049  0.082  0.036 
+10    | 0.000357  | 0.154      | 0.226      | 0.755           | 0.504        | 0.077             | 0.283    0.099    0.192    0.006    0.528    0.478    0.489   | 0.429    0.140    0.251    0.029    0.572    0.522    0.535   | 0.581  0.357  0.616  | 0.058  0.085  0.089 
+11    | 0.000323  | 0.137      | 0.219      | 0.771           | 0.514        | 0.057             | 0.251    0.088    0.172    0.005    0.516    0.463    0.467   | 0.413    0.136    0.244    0.027    0.581    0.512    0.548   | 0.605  0.362  0.618  | 0.059  0.072  0.041 
+12    | 0.000293  | 0.128      | 0.206      | 0.768           | 0.508        | 0.058             | 0.236    0.081    0.158    0.005    0.512    0.455    0.457   | 0.360    0.139    0.248    0.031    0.520    0.480    0.524   | 0.600  0.384  0.557  | 0.057  0.068  0.050 
+13    | 0.000270  | 0.121      | 0.192      | 0.777           | 0.527        | 0.056             | 0.221    0.078    0.150    0.005    0.504    0.448    0.452   | 0.324    0.136    0.244    0.029    0.533    0.449    0.484   | 0.606  0.389  0.627  | 0.056  0.069  0.042 
+14    | 0.000255  | 0.119      | 0.192      | 0.755           | 0.500        | 0.075             | 0.219    0.076    0.148    0.005    0.504    0.446    0.446   | 0.299    0.146    0.261    0.031    0.503    0.431    0.456   | 0.561  0.383  0.584  | 0.052  0.073  0.098 
+15    | 0.000250  | 0.114      | 0.177      | 0.775           | 0.524        | 0.057             | 0.210    0.073    0.142    0.005    0.497    0.442    0.440   | 0.258    0.142    0.255    0.028    0.480    0.416    0.424   | 0.614  0.389  0.601  | 0.063  0.069  0.040 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.3/0.7, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.3 (0.3D+0.7B)
+Dropout = 0.3
+(35m 12s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.565      | 0.383      | 0.353           | 0.017        | 0.423             | 0.402    0.634    0.995    0.480    0.428    0.350    0.362   | 0.370    0.389    0.521    0.333    0.524    0.453    0.420   | 0.050  0.000  0.000  | 0.036  0.233  1.000 
+2     | 0.000250  | 0.459      | 0.380      | 0.588           | 0.193        | 0.148             | 0.217    0.562    0.988    0.380    0.425    0.361    0.349   | 0.404    0.369    0.499    0.314    0.495    0.439    0.477   | 0.398  0.086  0.043  | 0.138  0.049  0.258 
+3     | 0.000375  | 0.464      | 0.323      | 0.584           | 0.272        | 0.209             | 0.359    0.509    0.983    0.306    0.481    0.425    0.405   | 0.363    0.305    0.490    0.226    0.621    0.468    0.428   | 0.486  0.248  0.002  | 0.146  0.076  0.405 
+4     | 0.000500  | 0.398      | 0.279      | 0.646           | 0.345        | 0.153             | 0.344    0.422    0.960    0.191    0.525    0.460    0.441   | 0.423    0.217    0.460    0.112    0.633    0.545    0.479   | 0.526  0.234  0.223  | 0.138  0.150  0.171 
+5     | 0.000495  | 0.306      | 0.250      | 0.690           | 0.383        | 0.106             | 0.340    0.291    0.825    0.062    0.606    0.503    0.469   | 0.503    0.142    0.382    0.039    0.629    0.601    0.561   | 0.527  0.247  0.421  | 0.071  0.129  0.118 
+6     | 0.000480  | 0.247      | 0.201      | 0.738           | 0.482        | 0.092             | 0.366    0.196    0.607    0.020    0.597    0.531    0.519   | 0.413    0.110    0.312    0.024    0.572    0.557    0.544   | 0.580  0.317  0.582  | 0.101  0.081  0.094 
+7     | 0.000457  | 0.203      | 0.195      | 0.742           | 0.464        | 0.073             | 0.363    0.134    0.424    0.010    0.572    0.524    0.544   | 0.411    0.103    0.292    0.022    0.580    0.552    0.542   | 0.579  0.342  0.518  | 0.063  0.087  0.070 
+8     | 0.000427  | 0.167      | 0.200      | 0.758           | 0.486        | 0.060             | 0.324    0.100    0.315    0.007    0.553    0.507    0.523   | 0.435    0.099    0.276    0.023    0.567    0.528    0.543   | 0.573  0.348  0.595  | 0.063  0.077  0.040 
+9     | 0.000393  | 0.151      | 0.186      | 0.762           | 0.489        | 0.055             | 0.297    0.088    0.279    0.007    0.542    0.489    0.499   | 0.384    0.101    0.274    0.026    0.555    0.508    0.512   | 0.558  0.350  0.614  | 0.044  0.079  0.042 
+10    | 0.000357  | 0.134      | 0.177      | 0.763           | 0.499        | 0.061             | 0.268    0.077    0.243    0.006    0.527    0.476    0.481   | 0.357    0.100    0.274    0.025    0.541    0.489    0.503   | 0.590  0.370  0.593  | 0.056  0.081  0.046 
+11    | 0.000323  | 0.122      | 0.178      | 0.756           | 0.503        | 0.075             | 0.248    0.069    0.216    0.005    0.516    0.464    0.465   | 0.369    0.095    0.262    0.024    0.558    0.494    0.533   | 0.560  0.364  0.633  | 0.062  0.072  0.093 
+12    | 0.000293  | 0.114      | 0.189      | 0.754           | 0.480        | 0.064             | 0.231    0.065    0.204    0.005    0.513    0.456    0.455   | 0.392    0.101    0.274    0.027    0.534    0.468    0.522   | 0.575  0.362  0.532  | 0.058  0.077  0.056 
+13    | 0.000270  | 0.110      | 0.169      | 0.761           | 0.508        | 0.071             | 0.222    0.062    0.194    0.005    0.505    0.448    0.449   | 0.339    0.096    0.257    0.027    0.546    0.467    0.480   | 0.582  0.356  0.628  | 0.066  0.083  0.063 
+14    | 0.000255  | 0.105      | 0.170      | 0.749           | 0.487        | 0.076             | 0.212    0.060    0.188    0.005    0.504    0.443    0.442   | 0.332    0.100    0.266    0.029    0.525    0.456    0.435   | 0.549  0.367  0.607  | 0.059  0.078  0.092 
+15    | 0.000250  | 0.103      | 0.148      | 0.764           | 0.542        | 0.088             | 0.207    0.058    0.184    0.005    0.499    0.439    0.435   | 0.275    0.093    0.248    0.026    0.510    0.427    0.437   | 0.633  0.370  0.667  | 0.086  0.091  0.089 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">current issue : final valid presence loss &gt; initial valid presence loss. Either increase number of epochs or increase BCE weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.3/0.7, 
+20 epoch, 5 warmup epoch – linear warmup,
+Start LR 1e-4
+final LR 2e-4
+Loss wt : 0.5 (0.5D+0.5B)
+Dropout = 0.3
+(45m 56s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000100  | 0.633      | 0.402      | 0.406           | 0.120        | 0.403             | 0.370    0.746    0.993    0.499    0.417    0.341    0.351   | 0.295    0.447    0.510    0.384    0.491    0.395    0.388   | 0.272  0.040  0.000  | 0.136  0.073  1.000 
+2     | 0.000200  | 0.544      | 0.412      | 0.639           | 0.196        | 0.065             | 0.171    0.704    0.986    0.423    0.400    0.329    0.311   | 0.336    0.445    0.494    0.396    0.355    0.261    0.432   | 0.350  0.130  0.090  | 0.093  0.059  0.044 
+3     | 0.000300  | 0.525      | 0.363      | 0.667           | 0.356        | 0.125             | 0.165    0.679    0.978    0.380    0.416    0.347    0.329   | 0.275    0.401    0.468    0.334    0.479    0.366    0.309   | 0.480  0.243  0.322  | 0.167  0.089  0.120 
+4     | 0.000400  | 0.514      | 0.338      | 0.645           | 0.341        | 0.153             | 0.215    0.643    0.971    0.314    0.450    0.379    0.355   | 0.436    0.296    0.462    0.130    0.554    0.461    0.607   | 0.456  0.253  0.320  | 0.164  0.167  0.127 
+5     | 0.000500  | 0.487      | 0.389      | 0.639           | 0.249        | 0.102             | 0.297    0.568    0.935    0.201    0.534    0.438    0.406   | 0.706    0.254    0.449    0.059    0.694    0.667    0.631   | 0.255  0.244  0.294  | 0.071  0.134  0.100 
+6     | 0.000497  | 0.353      | 0.265      | 0.719           | 0.429        | 0.088             | 0.446    0.313    0.594    0.032    0.635    0.570    0.553   | 0.488    0.170    0.316    0.024    0.624    0.601    0.573   | 0.568  0.314  0.436  | 0.081  0.089  0.094 
+7     | 0.000487  | 0.247      | 0.240      | 0.748           | 0.458        | 0.058             | 0.422    0.172    0.336    0.009    0.586    0.553    0.579   | 0.433    0.158    0.289    0.027    0.584    0.559    0.560   | 0.549  0.335  0.527  | 0.050  0.075  0.049 
+8     | 0.000471  | 0.190      | 0.237      | 0.743           | 0.453        | 0.063             | 0.345    0.123    0.239    0.007    0.558    0.517    0.534   | 0.435    0.152    0.276    0.028    0.568    0.542    0.512   | 0.569  0.352  0.510  | 0.070  0.073  0.047 
+9     | 0.000450  | 0.174      | 0.242      | 0.740           | 0.447        | 0.065             | 0.316    0.113    0.219    0.007    0.544    0.496    0.504   | 0.442    0.157    0.281    0.033    0.569    0.544    0.531   | 0.522  0.337  0.552  | 0.050  0.078  0.067 
+10    | 0.000425  | 0.157      | 0.231      | 0.756           | 0.499        | 0.072             | 0.285    0.102    0.198    0.006    0.530    0.477    0.487   | 0.433    0.144    0.260    0.028    0.567    0.487    0.535   | 0.571  0.356  0.610  | 0.084  0.089  0.044 
+11    | 0.000396  | 0.136      | 0.226      | 0.745           | 0.479        | 0.078             | 0.244    0.090    0.175    0.006    0.513    0.458    0.461   | 0.414    0.145    0.260    0.030    0.570    0.504    0.539   | 0.571  0.379  0.526  | 0.064  0.070  0.101 
+12    | 0.000366  | 0.127      | 0.216      | 0.752           | 0.487        | 0.072             | 0.230    0.083    0.161    0.005    0.512    0.452    0.449   | 0.369    0.150    0.269    0.031    0.486    0.428    0.503   | 0.580  0.360  0.534  | 0.056  0.065  0.094 
+13    | 0.000334  | 0.120      | 0.212      | 0.760           | 0.490        | 0.060             | 0.218    0.078    0.151    0.005    0.499    0.444    0.443   | 0.364    0.147    0.261    0.032    0.521    0.446    0.492   | 0.549  0.359  0.576  | 0.053  0.076  0.053 
+14    | 0.000304  | 0.116      | 0.196      | 0.755           | 0.502        | 0.077             | 0.208    0.077    0.149    0.005    0.498    0.437    0.434   | 0.319    0.143    0.258    0.028    0.509    0.450    0.421   | 0.583  0.372  0.587  | 0.058  0.076  0.098 
+15    | 0.000275  | 0.111      | 0.190      | 0.760           | 0.516        | 0.077             | 0.199    0.073    0.140    0.005    0.492    0.436    0.428   | 0.299    0.143    0.257    0.029    0.488    0.410    0.415   | 0.612  0.356  0.575  | 0.058  0.076  0.098 
+16    | 0.000250  | 0.104      | 0.215      | 0.759           | 0.486        | 0.059             | 0.184    0.069    0.134    0.004    0.487    0.425    0.421   | 0.372    0.147    0.260    0.034    0.536    0.476    0.445   | 0.564  0.376  0.573  | 0.059  0.078  0.039 
+17    | 0.000229  | 0.100      | 0.187      | 0.769           | 0.530        | 0.072             | 0.179    0.067    0.130    0.004    0.485    0.421    0.414   | 0.302    0.138    0.245    0.031    0.506    0.447    0.439   | 0.614  0.396  0.612  | 0.073  0.078  0.063 
+18    | 0.000213  | 0.098      | 0.185      | 0.762           | 0.522        | 0.078             | 0.176    0.065    0.126    0.004    0.481    0.418    0.411   | 0.293    0.138    0.245    0.032    0.510    0.456    0.449   | 0.614  0.403  0.595  | 0.061  0.076  0.096 
+19    | 0.000203  | 0.099      | 0.207      | 0.744           | 0.488        | 0.085             | 0.176    0.066    0.127    0.004    0.483    0.417    0.406   | 0.346    0.148    0.257    0.038    0.526    0.463    0.424   | 0.553  0.357  0.604  | 0.073  0.081  0.102 
+20    | 0.000200  | 0.094      | 0.213      | 0.737           | 0.458        | 0.077             | 0.164    0.064    0.124    0.004    0.477    0.410    0.399   | 0.355    0.153    0.267    0.038    0.487    0.446    0.440   | 0.545  0.364  0.524  | 0.061  0.076  0.096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.3/0.7, 
+20 epoch, 5 warmup epoch – linear warmup,
+Start LR 1e-4
+final LR 2e-4
+Loss wt : 0.3 (0.3D+0.7B)
+Dropout = 0.3
+(45m 55s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000100  | 0.563      | 0.383      | 0.155           | 0.001        | 0.743             | 0.388    0.638    0.995    0.485    0.428    0.353    0.351   | 0.265    0.433    0.534    0.390    0.400    0.345    0.399   | 0.002  0.000  0.000  | 0.229  1.000  1.000 
+2     | 0.000200  | 0.460      | 0.370      | 0.541           | 0.108        | 0.170             | 0.203    0.571    0.989    0.391    0.420    0.356    0.340   | 0.405    0.355    0.505    0.291    0.495    0.435    0.521   | 0.261  0.006  0.016  | 0.056  0.034  0.420 
+3     | 0.000300  | 0.430      | 0.320      | 0.610           | 0.231        | 0.136             | 0.239    0.512    0.981    0.312    0.463    0.400    0.384   | 0.403    0.284    0.478    0.202    0.606    0.486    0.400   | 0.418  0.166  0.064  | 0.116  0.074  0.219 
+4     | 0.000400  | 0.428      | 0.267      | 0.656           | 0.306        | 0.111             | 0.350    0.461    0.974    0.242    0.505    0.439    0.426   | 0.358    0.227    0.480    0.119    0.546    0.516    0.465   | 0.504  0.261  0.099  | 0.117  0.133  0.083 
+5     | 0.000500  | 0.336      | 0.245      | 0.687           | 0.397        | 0.120             | 0.348    0.331    0.884    0.094    0.588    0.499    0.470   | 0.482    0.143    0.392    0.037    0.635    0.613    0.568   | 0.510  0.267  0.449  | 0.102  0.122  0.136 
+6     | 0.000497  | 0.261      | 0.217      | 0.723           | 0.457        | 0.100             | 0.359    0.218    0.664    0.028    0.600    0.521    0.503   | 0.456    0.115    0.322    0.026    0.608    0.552    0.572   | 0.571  0.284  0.565  | 0.118  0.101  0.080 
+7     | 0.000487  | 0.207      | 0.194      | 0.746           | 0.512        | 0.098             | 0.363    0.140    0.442    0.011    0.572    0.522    0.543   | 0.412    0.100    0.280    0.023    0.604    0.535    0.541   | 0.584  0.338  0.617  | 0.100  0.099  0.095 
+8     | 0.000471  | 0.173      | 0.196      | 0.744           | 0.463        | 0.068             | 0.329    0.106    0.334    0.008    0.551    0.504    0.521   | 0.410    0.104    0.288    0.025    0.549    0.509    0.548   | 0.579  0.337  0.556  | 0.066  0.096  0.042 
+9     | 0.000450  | 0.154      | 0.205      | 0.731           | 0.459        | 0.088             | 0.302    0.091    0.287    0.007    0.537    0.489    0.496   | 0.443    0.103    0.279    0.028    0.563    0.547    0.486   | 0.516  0.330  0.602  | 0.049  0.112  0.103 
+10    | 0.000425  | 0.133      | 0.193      | 0.731           | 0.465        | 0.091             | 0.264    0.077    0.242    0.006    0.523    0.470    0.476   | 0.409    0.101    0.275    0.026    0.560    0.501    0.481   | 0.553  0.327  0.582  | 0.065  0.111  0.097 
+11    | 0.000396  | 0.122      | 0.191      | 0.753           | 0.507        | 0.084             | 0.241    0.071    0.223    0.006    0.510    0.457    0.457   | 0.419    0.094    0.257    0.023    0.553    0.499    0.558   | 0.591  0.360  0.584  | 0.073  0.083  0.095 
+12    | 0.000366  | 0.114      | 0.182      | 0.744           | 0.480        | 0.080             | 0.229    0.065    0.204    0.005    0.508    0.450    0.446   | 0.379    0.098    0.261    0.028    0.535    0.477    0.513   | 0.578  0.364  0.552  | 0.060  0.086  0.096 
+13    | 0.000334  | 0.106      | 0.165      | 0.755           | 0.487        | 0.067             | 0.210    0.061    0.191    0.005    0.499    0.440    0.439   | 0.317    0.100    0.267    0.029    0.505    0.435    0.448   | 0.570  0.381  0.570  | 0.050  0.084  0.066 
+14    | 0.000304  | 0.102      | 0.159      | 0.758           | 0.495        | 0.066             | 0.203    0.059    0.184    0.005    0.496    0.435    0.431   | 0.301    0.099    0.265    0.027    0.501    0.428    0.384   | 0.561  0.386  0.616  | 0.055  0.098  0.043 
+15    | 0.000275  | 0.096      | 0.147      | 0.774           | 0.537        | 0.068             | 0.191    0.055    0.172    0.005    0.490    0.430    0.425   | 0.280    0.089    0.243    0.024    0.478    0.414    0.400   | 0.632  0.399  0.646  | 0.081  0.088  0.037 
+16    | 0.000250  | 0.091      | 0.166      | 0.758           | 0.489        | 0.064             | 0.180    0.053    0.165    0.005    0.487    0.424    0.416   | 0.311    0.104    0.270    0.032    0.502    0.440    0.429   | 0.593  0.369  0.557  | 0.060  0.084  0.047 
+17    | 0.000229  | 0.090      | 0.154      | 0.770           | 0.537        | 0.074             | 0.180    0.052    0.161    0.005    0.484    0.420    0.411   | 0.297    0.092    0.245    0.027    0.503    0.456    0.410   | 0.603  0.399  0.664  | 0.064  0.112  0.047 
+18    | 0.000213  | 0.086      | 0.157      | 0.759           | 0.528        | 0.088             | 0.172    0.049    0.155    0.004    0.480    0.415    0.408   | 0.308    0.093    0.247    0.027    0.516    0.470    0.434   | 0.595  0.391  0.660  | 0.074  0.096  0.093 
+19    | 0.000203  | 0.085      | 0.161      | 0.766           | 0.517        | 0.068             | 0.168    0.050    0.155    0.004    0.481    0.414    0.404   | 0.300    0.101    0.256    0.034    0.496    0.450    0.431   | 0.571  0.385  0.611  | 0.059  0.098  0.049 
+20    | 0.000200  | 0.081      | 0.158      | 0.756           | 0.532        | 0.094             | 0.160    0.047    0.148    0.004    0.475    0.410    0.398   | 0.308    0.093    0.243    0.029    0.486    0.452    0.430   | 0.628  0.409  0.612  | 0.089  0.097  0.095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.3/0.7, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.4 (0.4D+0.6B)
+Dropout = 0.3
+(34m 40s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.595      | 0.379      | 0.403           | 0.084        | 0.384             | 0.378    0.688    0.994    0.485    0.423    0.346    0.357   | 0.247    0.436    0.518    0.381    0.423    0.379    0.388   | 0.202  0.027  0.000  | 0.059  0.094  1.000 
+2     | 0.000250  | 0.504      | 0.378      | 0.595           | 0.179        | 0.128             | 0.201    0.635    0.987    0.400    0.412    0.346    0.328   | 0.392    0.372    0.493    0.291    0.460    0.347    0.530   | 0.390  0.031  0.069  | 0.096  0.044  0.243 
+3     | 0.000375  | 0.505      | 0.331      | 0.652           | 0.298        | 0.111             | 0.280    0.601    0.981    0.348    0.458    0.389    0.366   | 0.298    0.345    0.473    0.260    0.549    0.386    0.372   | 0.485  0.274  0.089  | 0.128  0.090  0.116 
+4     | 0.000500  | 0.444      | 0.274      | 0.666           | 0.329        | 0.110             | 0.267    0.520    0.963    0.225    0.497    0.429    0.407   | 0.323    0.252    0.457    0.116    0.546    0.516    0.407   | 0.462  0.278  0.260  | 0.107  0.087  0.137 
+5     | 0.000495  | 0.378      | 0.290      | 0.693           | 0.382        | 0.100             | 0.350    0.389    0.840    0.088    0.601    0.498    0.456   | 0.563    0.172    0.372    0.039    0.659    0.630    0.588   | 0.496  0.252  0.431  | 0.064  0.093  0.142 
+6     | 0.000480  | 0.281      | 0.241      | 0.715           | 0.433        | 0.097             | 0.417    0.222    0.531    0.017    0.608    0.560    0.559   | 0.482    0.138    0.305    0.027    0.605    0.559    0.604   | 0.562  0.313  0.471  | 0.087  0.105  0.098 
+7     | 0.000457  | 0.213      | 0.208      | 0.735           | 0.437        | 0.067             | 0.377    0.143    0.346    0.008    0.574    0.534    0.559   | 0.370    0.138    0.306    0.026    0.545    0.535    0.545   | 0.589  0.321  0.446  | 0.075  0.089  0.038 
+8     | 0.000427  | 0.187      | 0.238      | 0.747           | 0.477        | 0.073             | 0.338    0.123    0.295    0.008    0.555    0.508    0.528   | 0.512    0.121    0.263    0.026    0.622    0.570    0.565   | 0.596  0.332  0.543  | 0.096  0.076  0.047 
+9     | 0.000393  | 0.162      | 0.205      | 0.751           | 0.464        | 0.057             | 0.307    0.100    0.241    0.007    0.542    0.493    0.503   | 0.384    0.128    0.277    0.028    0.571    0.481    0.513   | 0.548  0.342  0.558  | 0.053  0.069  0.049 
+10    | 0.000357  | 0.148      | 0.207      | 0.743           | 0.473        | 0.078             | 0.282    0.091    0.218    0.006    0.531    0.478    0.489   | 0.408    0.121    0.260    0.029    0.574    0.499    0.536   | 0.553  0.356  0.554  | 0.064  0.114  0.055 
+11    | 0.000323  | 0.132      | 0.189      | 0.764           | 0.517        | 0.072             | 0.249    0.083    0.198    0.006    0.519    0.462    0.467   | 0.366    0.113    0.241    0.027    0.573    0.504    0.529   | 0.593  0.378  0.612  | 0.059  0.113  0.043 
+12    | 0.000293  | 0.122      | 0.177      | 0.752           | 0.483        | 0.070             | 0.233    0.075    0.180    0.005    0.514    0.456    0.458   | 0.303    0.123    0.262    0.031    0.509    0.485    0.477   | 0.557  0.381  0.580  | 0.062  0.095  0.052 
+13    | 0.000270  | 0.118      | 0.176      | 0.760           | 0.489        | 0.060             | 0.224    0.072    0.173    0.005    0.504    0.447    0.451   | 0.299    0.124    0.261    0.032    0.510    0.437    0.482   | 0.575  0.380  0.567  | 0.054  0.081  0.046 
+14    | 0.000255  | 0.112      | 0.160      | 0.772           | 0.531        | 0.067             | 0.215    0.068    0.163    0.005    0.503    0.444    0.443   | 0.257    0.118    0.252    0.029    0.509    0.443    0.411   | 0.599  0.380  0.640  | 0.057  0.095  0.050 
+15    | 0.000250  | 0.108      | 0.186      | 0.755           | 0.473        | 0.058             | 0.207    0.066    0.158    0.005    0.498    0.441    0.438   | 0.307    0.134    0.284    0.034    0.450    0.376    0.440   | 0.556  0.345  0.560  | 0.054  0.067  0.052 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.3/0.7, 
+20 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.3 (0.3D+0.7B)
+Dropout = 0.3
+(45m 12s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.568      | 0.377      | 0.358           | 0.044        | 0.433             | 0.412    0.634    0.994    0.480    0.436    0.351    0.372   | 0.291    0.414    0.523    0.367    0.474    0.378    0.436   | 0.118  0.001  0.000  | 0.055  0.245  1.000 
+2     | 0.000250  | 0.458      | 0.353      | 0.493           | 0.116        | 0.255             | 0.231    0.556    0.989    0.370    0.434    0.369    0.356   | 0.409    0.329    0.508    0.252    0.474    0.493    0.485   | 0.260  0.021  0.028  | 0.086  0.064  0.614 
+3     | 0.000375  | 0.442      | 0.335      | 0.670           | 0.318        | 0.096             | 0.292    0.506    0.982    0.303    0.470    0.408    0.390   | 0.282    0.357    0.492    0.299    0.508    0.382    0.331   | 0.497  0.246  0.165  | 0.130  0.101  0.055 
+4     | 0.000500  | 0.436      | 0.272      | 0.629           | 0.297        | 0.149             | 0.479    0.417    0.963    0.184    0.549    0.487    0.479   | 0.422    0.208    0.470    0.096    0.621    0.551    0.471   | 0.431  0.252  0.177  | 0.159  0.133  0.155 
+5     | 0.000498  | 0.313      | 0.266      | 0.692           | 0.400        | 0.113             | 0.363    0.291    0.834    0.058    0.599    0.504    0.468   | 0.570    0.136    0.376    0.033    0.640    0.584    0.591   | 0.556  0.248  0.350  | 0.111  0.108  0.122 
+6     | 0.000490  | 0.257      | 0.216      | 0.706           | 0.448        | 0.123             | 0.371    0.208    0.640    0.023    0.594    0.527    0.508   | 0.444    0.119    0.328    0.029    0.598    0.566    0.528   | 0.586  0.262  0.514  | 0.116  0.134  0.118 
+7     | 0.000479  | 0.211      | 0.209      | 0.738           | 0.470        | 0.084             | 0.367    0.144    0.454    0.011    0.574    0.524    0.539   | 0.450    0.105    0.290    0.026    0.605    0.544    0.551   | 0.588  0.300  0.538  | 0.070  0.113  0.069 
+8     | 0.000463  | 0.175      | 0.190      | 0.731           | 0.453        | 0.084             | 0.332    0.107    0.339    0.008    0.555    0.506    0.525   | 0.379    0.109    0.300    0.027    0.553    0.514    0.504   | 0.580  0.327  0.501  | 0.060  0.106  0.086 
+9     | 0.000444  | 0.156      | 0.218      | 0.714           | 0.411        | 0.084             | 0.301    0.094    0.294    0.008    0.541    0.488    0.498   | 0.464    0.113    0.308    0.029    0.539    0.532    0.528   | 0.481  0.299  0.494  | 0.064  0.074  0.112 
+10    | 0.000423  | 0.139      | 0.173      | 0.748           | 0.483        | 0.076             | 0.274    0.081    0.254    0.007    0.527    0.475    0.482   | 0.332    0.105    0.287    0.028    0.523    0.486    0.491   | 0.632  0.355  0.483  | 0.074  0.106  0.049 
+11    | 0.000399  | 0.127      | 0.201      | 0.723           | 0.422        | 0.077             | 0.252    0.074    0.231    0.006    0.515    0.462    0.466   | 0.415    0.109    0.296    0.029    0.548    0.484    0.542   | 0.543  0.322  0.429  | 0.060  0.075  0.096 
+12    | 0.000375  | 0.120      | 0.199      | 0.731           | 0.454        | 0.085             | 0.239    0.070    0.218    0.006    0.512    0.454    0.454   | 0.419    0.104    0.271    0.033    0.559    0.507    0.535   | 0.573  0.361  0.457  | 0.056  0.096  0.103 
+13    | 0.000351  | 0.110      | 0.175      | 0.751           | 0.478        | 0.067             | 0.221    0.063    0.197    0.005    0.503    0.446    0.444   | 0.345    0.102    0.270    0.030    0.542    0.456    0.463   | 0.590  0.352  0.539  | 0.065  0.079  0.057 
+14    | 0.000327  | 0.108      | 0.154      | 0.750           | 0.504        | 0.086             | 0.214    0.062    0.195    0.005    0.502    0.438    0.437   | 0.278    0.100    0.268    0.029    0.508    0.431    0.425   | 0.577  0.364  0.613  | 0.052  0.102  0.104 
+15    | 0.000306  | 0.102      | 0.157      | 0.748           | 0.482        | 0.075             | 0.202    0.059    0.185    0.005    0.496    0.433    0.430   | 0.285    0.102    0.274    0.029    0.480    0.413    0.416   | 0.614  0.367  0.519  | 0.062  0.089  0.072 
+16    | 0.000287  | 0.098      | 0.180      | 0.741           | 0.461        | 0.073             | 0.195    0.057    0.176    0.005    0.491    0.428    0.422   | 0.346    0.109    0.276    0.037    0.525    0.447    0.453   | 0.553  0.353  0.550  | 0.066  0.098  0.054 
+17    | 0.000271  | 0.094      | 0.183      | 0.731           | 0.446        | 0.079             | 0.187    0.055    0.170    0.005    0.487    0.422    0.418   | 0.350    0.112    0.289    0.036    0.492    0.422    0.467   | 0.545  0.345  0.486  | 0.062  0.077  0.097 
+18    | 0.000260  | 0.090      | 0.183      | 0.745           | 0.491        | 0.086             | 0.179    0.052    0.164    0.005    0.484    0.419    0.411   | 0.375    0.100    0.259    0.032    0.547    0.461    0.445   | 0.591  0.361  0.553  | 0.064  0.096  0.098 
+19    | 0.000252  | 0.088      | 0.164      | 0.734           | 0.459        | 0.083             | 0.173    0.052    0.162    0.005    0.482    0.414    0.407   | 0.293    0.108    0.277    0.036    0.497    0.431    0.437   | 0.545  0.356  0.515  | 0.056  0.096  0.096 
+20    | 0.000250  | 0.085      | 0.163      | 0.736           | 0.465        | 0.083             | 0.168    0.049    0.154    0.005    0.477    0.413    0.401   | 0.292    0.108    0.277    0.036    0.476    0.415    0.435   | 0.542  0.356  0.551  | 0.062  0.098  0.090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on data subset
+presence/seg loss weight = 0.3/0.7, 
+20 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.5
+Dropout = 0.3
+(45m 35s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.638      | 0.384      | 0.425           | 0.138        | 0.384             | 0.388    0.745    0.993    0.497    0.418    0.343    0.355   | 0.199    0.464    0.513    0.414    0.425    0.350    0.358   | 0.279  0.095  0.000  | 0.072  0.079  1.000 
+2     | 0.000250  | 0.546      | 0.392      | 0.648           | 0.306        | 0.125             | 0.183    0.701    0.985    0.417    0.400    0.331    0.315   | 0.303    0.430    0.479    0.381    0.443    0.327    0.418   | 0.490  0.203  0.172  | 0.171  0.077  0.126 
+3     | 0.000375  | 0.532      | 0.363      | 0.670           | 0.336        | 0.107             | 0.186    0.680    0.979    0.381    0.416    0.344    0.326   | 0.248    0.412    0.469    0.354    0.475    0.348    0.315   | 0.499  0.252  0.243  | 0.113  0.109  0.099 
+4     | 0.000500  | 0.513      | 0.340      | 0.680           | 0.376        | 0.117             | 0.217    0.640    0.971    0.308    0.448    0.379    0.360   | 0.374    0.326    0.451    0.200    0.499    0.482    0.465   | 0.468  0.274  0.390  | 0.121  0.117  0.114 
+5     | 0.000498  | 0.474      | 0.325      | 0.668           | 0.384        | 0.143             | 0.266    0.563    0.937    0.189    0.524    0.430    0.408   | 0.533    0.235    0.403    0.068    0.698    0.625    0.493   | 0.522  0.202  0.410  | 0.133  0.166  0.128 
+6     | 0.000490  | 0.350      | 0.252      | 0.737           | 0.484        | 0.095             | 0.436    0.313    0.595    0.031    0.631    0.565    0.549   | 0.480    0.154    0.287    0.022    0.611    0.548    0.606   | 0.596  0.330  0.578  | 0.107  0.086  0.091 
+7     | 0.000479  | 0.245      | 0.233      | 0.753           | 0.477        | 0.062             | 0.412    0.174    0.338    0.009    0.583    0.547    0.575   | 0.422    0.152    0.281    0.023    0.563    0.529    0.549   | 0.573  0.332  0.562  | 0.073  0.073  0.041 
+8     | 0.000463  | 0.199      | 0.224      | 0.755           | 0.482        | 0.063             | 0.354    0.133    0.258    0.007    0.560    0.518    0.532   | 0.402    0.147    0.267    0.027    0.593    0.519    0.509   | 0.568  0.358  0.564  | 0.074  0.078  0.038 
+9     | 0.000444  | 0.168      | 0.231      | 0.746           | 0.470        | 0.070             | 0.303    0.110    0.213    0.006    0.541    0.492    0.504   | 0.422    0.149    0.268    0.030    0.575    0.564    0.506   | 0.539  0.364  0.570  | 0.052  0.102  0.056 
+10    | 0.000423  | 0.153      | 0.215      | 0.747           | 0.461        | 0.063             | 0.278    0.099    0.193    0.006    0.527    0.474    0.486   | 0.351    0.157    0.283    0.031    0.529    0.442    0.501   | 0.529  0.386  0.496  | 0.067  0.076  0.046 
+11    | 0.000399  | 0.136      | 0.239      | 0.748           | 0.477        | 0.071             | 0.246    0.089    0.173    0.005    0.512    0.458    0.463   | 0.460    0.144    0.260    0.029    0.558    0.491    0.584   | 0.555  0.403  0.497  | 0.058  0.074  0.081 
+12    | 0.000375  | 0.128      | 0.225      | 0.749           | 0.458        | 0.058             | 0.232    0.083    0.160    0.005    0.514    0.451    0.452   | 0.385    0.156    0.278    0.035    0.473    0.436    0.504   | 0.518  0.385  0.473  | 0.042  0.077  0.055 
+13    | 0.000351  | 0.119      | 0.207      | 0.761           | 0.493        | 0.061             | 0.212    0.079    0.152    0.005    0.499    0.440    0.441   | 0.356    0.143    0.254    0.032    0.528    0.470    0.476   | 0.570  0.387  0.582  | 0.060  0.077  0.046 
+14    | 0.000327  | 0.114      | 0.190      | 0.760           | 0.509        | 0.072             | 0.206    0.074    0.143    0.005    0.498    0.437    0.433   | 0.300    0.142    0.255    0.030    0.486    0.419    0.393   | 0.588  0.399  0.568  | 0.078  0.071  0.067 
+15    | 0.000306  | 0.112      | 0.195      | 0.765           | 0.508        | 0.063             | 0.203    0.073    0.141    0.005    0.494    0.434    0.430   | 0.312    0.145    0.256    0.034    0.517    0.442    0.405   | 0.599  0.377  0.576  | 0.075  0.075  0.040 
+16    | 0.000287  | 0.107      | 0.205      | 0.755           | 0.473        | 0.057             | 0.190    0.071    0.138    0.005    0.486    0.426    0.420   | 0.335    0.149    0.262    0.035    0.499    0.460    0.426   | 0.574  0.392  0.515  | 0.054  0.077  0.040 
+17    | 0.000271  | 0.102      | 0.197      | 0.766           | 0.510        | 0.063             | 0.180    0.069    0.133    0.005    0.483    0.420    0.415   | 0.324    0.142    0.250    0.034    0.492    0.431    0.445   | 0.570  0.383  0.599  | 0.059  0.081  0.050 
+18    | 0.000260  | 0.100      | 0.201      | 0.764           | 0.516        | 0.070             | 0.176    0.067    0.130    0.005    0.478    0.414    0.409   | 0.352    0.137    0.241    0.033    0.519    0.483    0.465   | 0.581  0.372  0.616  | 0.070  0.092  0.047 
+19    | 0.000252  | 0.100      | 0.204      | 0.758           | 0.482        | 0.059             | 0.172    0.069    0.133    0.005    0.478    0.414    0.405   | 0.324    0.153    0.264    0.041    0.484    0.443    0.454   | 0.550  0.396  0.537  | 0.051  0.073  0.052 
+20    | 0.000250  | 0.095      | 0.197      | 0.749           | 0.483        | 0.074             | 0.163    0.066    0.127    0.005    0.474    0.410    0.397   | 0.307    0.150    0.260    0.039    0.500    0.458    0.440   | 0.571  0.382  0.553  | 0.065  0.086  0.069 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function
+presence/seg loss weight = 0.3/0.7, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.5
+Dropout = 0.3
+(3h 42m 52s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.552      | 0.324      | 0.749           | 0.506        | 0.088             | 0.259    0.677    0.976    0.379    0.436    0.379    0.334   | 0.230    0.365    0.424    0.305    0.427    0.370    0.297   | 0.577  0.427  0.466  | 0.099  0.091  0.075 
+2     | 0.000250  | 0.362      | 0.208      | 0.809           | 0.635        | 0.075             | 0.409    0.343    0.603    0.082    0.581    0.532    0.507   | 0.466    0.098    0.181    0.014    0.598    0.549    0.556   | 0.653  0.559  0.704  | 0.064  0.104  0.059 
+3     | 0.000375  | 0.189      | 0.152      | 0.836           | 0.685        | 0.064             | 0.322    0.131    0.253    0.010    0.535    0.498    0.472   | 0.305    0.086    0.158    0.015    0.537    0.467    0.377   | 0.713  0.605  0.733  | 0.072  0.068  0.050 
+4     | 0.000500  | 0.155      | 0.131      | 0.840           | 0.703        | 0.068             | 0.249    0.114    0.218    0.011    0.492    0.447    0.408   | 0.253    0.079    0.145    0.014    0.464    0.424    0.386   | 0.725  0.625  0.755  | 0.069  0.082  0.052 
+5     | 0.000495  | 0.130      | 0.131      | 0.838           | 0.689        | 0.064             | 0.197    0.101    0.192    0.010    0.468    0.417    0.371   | 0.238    0.084    0.152    0.016    0.434    0.415    0.334   | 0.714  0.603  0.747  | 0.071  0.071  0.049 
+6     | 0.000480  | 0.117      | 0.126      | 0.843           | 0.694        | 0.058             | 0.170    0.094    0.178    0.010    0.452    0.398    0.348   | 0.229    0.082    0.147    0.017    0.428    0.370    0.342   | 0.713  0.630  0.749  | 0.066  0.067  0.042 
+7     | 0.000457  | 0.105      | 0.125      | 0.839           | 0.693        | 0.063             | 0.147    0.087    0.165    0.010    0.442    0.385    0.333   | 0.233    0.078    0.141    0.016    0.459    0.382    0.296   | 0.713  0.622  0.763  | 0.078  0.073  0.038 
+8     | 0.000427  | 0.098      | 0.121      | 0.849           | 0.703        | 0.054             | 0.130    0.084    0.159    0.009    0.434    0.376    0.321   | 0.216    0.080    0.142    0.018    0.422    0.371    0.300   | 0.722  0.628  0.760  | 0.058  0.060  0.043 
+9     | 0.000393  | 0.091      | 0.115      | 0.846           | 0.707        | 0.061             | 0.116    0.080    0.151    0.009    0.427    0.366    0.310   | 0.202    0.077    0.138    0.017    0.417    0.367    0.279   | 0.733  0.631  0.760  | 0.067  0.081  0.036 
+10    | 0.000357  | 0.085      | 0.122      | 0.837           | 0.689        | 0.064             | 0.104    0.077    0.145    0.009    0.422    0.360    0.302   | 0.215    0.082    0.145    0.019    0.420    0.360    0.287   | 0.720  0.609  0.743  | 0.067  0.072  0.052 
+11    | 0.000323  | 0.077      | 0.115      | 0.849           | 0.713        | 0.061             | 0.091    0.072    0.135    0.008    0.418    0.353    0.297   | 0.201    0.078    0.137    0.018    0.411    0.355    0.275   | 0.736  0.635  0.772  | 0.073  0.082  0.028 
+12    | 0.000293  | 0.075      | 0.112      | 0.856           | 0.719        | 0.052             | 0.085    0.070    0.132    0.008    0.414    0.349    0.291   | 0.198    0.076    0.134    0.018    0.395    0.346    0.269   | 0.741  0.643  0.783  | 0.060  0.072  0.025 
+13    | 0.000270  | 0.069      | 0.107      | 0.855           | 0.720        | 0.055             | 0.075    0.066    0.125    0.008    0.411    0.345    0.286   | 0.178    0.076    0.135    0.018    0.389    0.329    0.269   | 0.738  0.648  0.769  | 0.059  0.060  0.045 
+14    | 0.000255  | 0.067      | 0.117      | 0.856           | 0.715        | 0.050             | 0.072    0.065    0.123    0.008    0.409    0.341    0.282   | 0.207    0.078    0.137    0.020    0.388    0.330    0.255   | 0.729  0.633  0.787  | 0.062  0.054  0.033 
+15    | 0.000250  | 0.064      | 0.116      | 0.857           | 0.718        | 0.050             | 0.066    0.063    0.120    0.007    0.406    0.340    0.279   | 0.202    0.080    0.140    0.020    0.376    0.325    0.246   | 0.735  0.635  0.782  | 0.059  0.066  0.025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2366  1859  1424
+FP   117   134    49
+FN   211   210   102
+TN  4602  5093  5721
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.324  0.255  0.195
+FP  0.016  0.018  0.007
+FN  0.029  0.029  0.014
+TN  0.631  0.698  0.784
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.116      | 0.857           | 0.718        | 0.050             | 0.202    0.080    0.140    0.020    0.376    0.325    0.246   | 0.735  0.635  0.782  | 0.059  0.066  0.025 
+266     | 266     | 0.114      | 0.856           | 0.718        | 0.052             | 0.199    0.077    0.133    0.021    0.368    0.321    0.236   | 0.733  0.636  0.789  | 0.061  0.070  0.025 
+360     | 310     | 0.117      | 0.845           | 0.671        | 0.039             | 0.205    0.079    0.150    0.009    0.349    0.286    0.301   | 0.682  0.569  0.763  | 0.050  0.040  0.026 
+276     | 276     | 0.129      | 0.886           | 0.774        | 0.039             | 0.250    0.078    0.137    0.019    0.619    0.496    0.344   | 0.847  0.691  0.704  | 0.043  0.043  0.032 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function
+presence/seg loss weight = 0.3/0.7, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.3 (0.3D+0.7B)
+Dropout = 0.3
+(3h 45m 6s)
+(Max GPU mem usage : 10716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.463      | 0.280      | 0.738           | 0.466        | 0.080             | 0.331    0.519    0.979    0.322    0.477    0.425    0.386   | 0.310    0.267    0.430    0.196    0.481    0.448    0.358   | 0.557  0.382  0.409  | 0.123  0.061  0.056 
+2     | 0.000250  | 0.298      | 0.175      | 0.813           | 0.641        | 0.071             | 0.414    0.248    0.691    0.058    0.586    0.532    0.501   | 0.412    0.073    0.213    0.013    0.562    0.508    0.533   | 0.685  0.548  0.678  | 0.089  0.088  0.038 
+3     | 0.000375  | 0.166      | 0.146      | 0.797           | 0.646        | 0.102             | 0.314    0.103    0.320    0.010    0.532    0.494    0.470   | 0.339    0.063    0.176    0.015    0.538    0.480    0.410   | 0.697  0.558  0.672  | 0.111  0.124  0.071 
+4     | 0.000500  | 0.133      | 0.113      | 0.839           | 0.683        | 0.057             | 0.245    0.085    0.260    0.010    0.488    0.445    0.406   | 0.244    0.056    0.161    0.012    0.449    0.422    0.366   | 0.710  0.604  0.733  | 0.058  0.074  0.039 
+5     | 0.000495  | 0.108      | 0.110      | 0.844           | 0.699        | 0.060             | 0.194    0.072    0.218    0.009    0.466    0.415    0.369   | 0.237    0.055    0.153    0.013    0.445    0.402    0.341   | 0.730  0.611  0.744  | 0.086  0.064  0.029 
+6     | 0.000480  | 0.095      | 0.109      | 0.841           | 0.699        | 0.064             | 0.164    0.066    0.200    0.009    0.452    0.396    0.346   | 0.239    0.053    0.144    0.014    0.448    0.398    0.334   | 0.726  0.624  0.753  | 0.074  0.080  0.038 
+7     | 0.000457  | 0.086      | 0.111      | 0.822           | 0.680        | 0.083             | 0.144    0.061    0.185    0.008    0.441    0.383    0.333   | 0.240    0.055    0.151    0.014    0.463    0.396    0.297   | 0.704  0.609  0.750  | 0.092  0.111  0.046 
+8     | 0.000427  | 0.079      | 0.095      | 0.848           | 0.709        | 0.060             | 0.128    0.058    0.176    0.008    0.433    0.374    0.318   | 0.194    0.052    0.142    0.014    0.419    0.344    0.298   | 0.731  0.626  0.781  | 0.063  0.068  0.048 
+9     | 0.000393  | 0.073      | 0.102      | 0.842           | 0.696        | 0.060             | 0.114    0.055    0.166    0.008    0.426    0.365    0.308   | 0.209    0.057    0.152    0.016    0.405    0.347    0.268   | 0.716  0.617  0.741  | 0.079  0.064  0.038 
+10    | 0.000357  | 0.068      | 0.091      | 0.850           | 0.710        | 0.057             | 0.103    0.052    0.158    0.007    0.421    0.358    0.302   | 0.181    0.052    0.142    0.014    0.401    0.334    0.287   | 0.738  0.631  0.761  | 0.057  0.069  0.044 
+11    | 0.000323  | 0.062      | 0.098      | 0.847           | 0.708        | 0.061             | 0.089    0.050    0.150    0.007    0.417    0.352    0.295   | 0.207    0.052    0.139    0.015    0.427    0.365    0.270   | 0.732  0.632  0.762  | 0.064  0.087  0.031 
+12    | 0.000293  | 0.058      | 0.088      | 0.850           | 0.713        | 0.059             | 0.083    0.048    0.143    0.007    0.414    0.348    0.289   | 0.177    0.050    0.135    0.014    0.408    0.360    0.265   | 0.736  0.641  0.774  | 0.074  0.076  0.028 
+13    | 0.000270  | 0.054      | 0.097      | 0.845           | 0.711        | 0.065             | 0.074    0.046    0.137    0.006    0.410    0.344    0.285   | 0.201    0.052    0.137    0.016    0.412    0.347    0.263   | 0.732  0.629  0.772  | 0.069  0.076  0.050 
+14    | 0.000255  | 0.053      | 0.094      | 0.846           | 0.710        | 0.063             | 0.071    0.046    0.136    0.007    0.408    0.341    0.281   | 0.191    0.052    0.138    0.015    0.404    0.345    0.255   | 0.741  0.615  0.769  | 0.072  0.074  0.043 
+15    | 0.000250  | 0.050      | 0.098      | 0.859           | 0.716        | 0.046             | 0.065    0.044    0.132    0.006    0.406    0.337    0.278   | 0.201    0.054    0.141    0.016    0.390    0.317    0.247   | 0.742  0.630  0.777  | 0.060  0.052  0.025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2449  1875  1416
+FP   168   165    42
+FN   128   194   110
+TN  4551  5062  5728
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.336  0.257  0.194
+FP  0.023  0.023  0.006
+FN  0.018  0.027  0.015
+TN  0.624  0.694  0.785
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.098      | 0.859           | 0.716        | 0.046             | 0.201    0.054    0.141    0.016    0.390    0.317    0.247   | 0.742  0.630  0.777  | 0.060  0.052  0.025 
+266     | 266     | 0.094      | 0.860           | 0.719        | 0.046             | 0.194    0.052    0.133    0.017    0.382    0.315    0.237   | 0.740  0.636  0.786  | 0.062  0.053  0.025 
+360     | 310     | 0.106      | 0.838           | 0.656        | 0.040             | 0.236    0.051    0.151    0.007    0.360    0.267    0.297   | 0.700  0.526  0.736  | 0.050  0.047  0.024 
+276     | 276     | 0.137      | 0.878           | 0.754        | 0.040             | 0.326    0.057    0.150    0.017    0.648    0.479    0.350   | 0.824  0.664  0.707  | 0.044  0.045  0.032 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on mit-b2
+presence/seg loss weight = 0.3/0.7, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.5
+Dropout = 0.3
+(5h 1m 18s)
+(Max GPU mem usage : 14394.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.546      | 0.308      | 0.754           | 0.547        | 0.109             | 0.249    0.674    0.975    0.373    0.430    0.380    0.339   | 0.239    0.338    0.407    0.269    0.454    0.405    0.341   | 0.617  0.452  0.538  | 0.137  0.103  0.088 
+2     | 0.000250  | 0.349      | 0.182      | 0.823           | 0.666        | 0.072             | 0.429    0.314    0.558    0.070    0.590    0.541    0.515   | 0.384    0.095    0.178    0.013    0.554    0.517    0.494   | 0.698  0.571  0.740  | 0.086  0.084  0.047 
+3     | 0.000375  | 0.177      | 0.150      | 0.837           | 0.679        | 0.058             | 0.308    0.120    0.231    0.009    0.534    0.487    0.461   | 0.310    0.082    0.149    0.014    0.504    0.491    0.396   | 0.712  0.588  0.752  | 0.065  0.071  0.039 
+4     | 0.000500  | 0.145      | 0.135      | 0.839           | 0.700        | 0.068             | 0.236    0.106    0.203    0.010    0.492    0.437    0.400   | 0.266    0.079    0.142    0.016    0.476    0.441    0.370   | 0.728  0.609  0.773  | 0.072  0.083  0.049 
+5     | 0.000495  | 0.123      | 0.125      | 0.840           | 0.708        | 0.072             | 0.191    0.093    0.177    0.009    0.469    0.409    0.368   | 0.231    0.080    0.144    0.016    0.449    0.387    0.359   | 0.733  0.625  0.756  | 0.098  0.064  0.053 
+6     | 0.000480  | 0.111      | 0.133      | 0.831           | 0.691        | 0.075             | 0.164    0.089    0.168    0.010    0.453    0.391    0.344   | 0.258    0.079    0.141    0.017    0.462    0.415    0.325   | 0.716  0.606  0.761  | 0.073  0.104  0.049 
+7     | 0.000457  | 0.099      | 0.121      | 0.847           | 0.703        | 0.057             | 0.140    0.081    0.153    0.009    0.441    0.378    0.331   | 0.222    0.077    0.136    0.018    0.441    0.379    0.308   | 0.730  0.626  0.756  | 0.068  0.070  0.034 
+8     | 0.000427  | 0.092      | 0.113      | 0.851           | 0.720        | 0.062             | 0.127    0.077    0.145    0.009    0.434    0.369    0.318   | 0.200    0.076    0.135    0.017    0.421    0.356    0.301   | 0.748  0.642  0.771  | 0.063  0.065  0.059 
+9     | 0.000393  | 0.084      | 0.127      | 0.831           | 0.689        | 0.074             | 0.109    0.073    0.137    0.008    0.427    0.361    0.309   | 0.229    0.083    0.148    0.019    0.424    0.365    0.294   | 0.720  0.622  0.722  | 0.070  0.080  0.070 
+10    | 0.000357  | 0.081      | 0.125      | 0.845           | 0.711        | 0.065             | 0.102    0.072    0.136    0.008    0.423    0.354    0.302   | 0.238    0.076    0.133    0.020    0.437    0.388    0.290   | 0.735  0.635  0.772  | 0.067  0.078  0.050 
+11    | 0.000323  | 0.073      | 0.108      | 0.855           | 0.717        | 0.053             | 0.089    0.067    0.126    0.008    0.418    0.349    0.295   | 0.183    0.076    0.134    0.018    0.400    0.343    0.276   | 0.749  0.642  0.766  | 0.061  0.057  0.042 
+12    | 0.000293  | 0.070      | 0.116      | 0.852           | 0.714        | 0.057             | 0.081    0.065    0.123    0.008    0.414    0.345    0.289   | 0.201    0.079    0.140    0.018    0.382    0.323    0.275   | 0.725  0.641  0.776  | 0.057  0.078  0.035 
+13    | 0.000270  | 0.065      | 0.122      | 0.853           | 0.722        | 0.060             | 0.072    0.062    0.117    0.007    0.411    0.341    0.285   | 0.232    0.074    0.128    0.020    0.410    0.344    0.287   | 0.748  0.637  0.780  | 0.071  0.066  0.044 
+14    | 0.000255  | 0.063      | 0.113      | 0.854           | 0.721        | 0.058             | 0.069    0.060    0.114    0.007    0.409    0.339    0.281   | 0.204    0.073    0.128    0.018    0.414    0.350    0.276   | 0.745  0.638  0.787  | 0.070  0.059  0.046 
+15    | 0.000250  | 0.060      | 0.111      | 0.855           | 0.727        | 0.061             | 0.064    0.059    0.111    0.007    0.406    0.335    0.279   | 0.199    0.074    0.127    0.020    0.410    0.349    0.260   | 0.754  0.651  0.784  | 0.068  0.079  0.035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2522  1999  1449
+FP   234   265    74
+FN    55    70    77
+TN  4485  4962  5696
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.346  0.274  0.199
+FP  0.032  0.036  0.010
+FN  0.008  0.010  0.011
+TN  0.615  0.680  0.781
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.111      | 0.855           | 0.727        | 0.061             | 0.199    0.074    0.127    0.020    0.410    0.349    0.260   | 0.754  0.651  0.784  | 0.068  0.079  0.035 
+266     | 266     | 0.107      | 0.854           | 0.728        | 0.062             | 0.192    0.071    0.121    0.021    0.402    0.347    0.250   | 0.750  0.654  0.792  | 0.071  0.083  0.033 
+360     | 310     | 0.114      | 0.846           | 0.696        | 0.055             | 0.223    0.067    0.124    0.009    0.388    0.312    0.311   | 0.749  0.583  0.766  | 0.058  0.050  0.057 
+276     | 276     | 0.180      | 0.876           | 0.756        | 0.043             | 0.389    0.090    0.155    0.025    0.654    0.493    0.377   | 0.821  0.674  0.697  | 0.045  0.052  0.031 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved loss function on mit-b3
+Batch size = 16   grad_accu_steps = 4
+presence/seg loss weight = 0.3/0.7, 
+15 epoch, 4 warmup epoch – linear warmup,
+final LR 2.5e-4
+Loss wt : 0.5
+Dropout = 0.3
+(6h 55m 27s)
+(Max GPU mem usage : 9900.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.527      | 0.251      | 0.755           | 0.531        | 0.096             | 0.313    0.618    0.946    0.290    0.474    0.441    0.380   | 0.480    0.152    0.252    0.053    0.679    0.595    0.460   | 0.584  0.463  0.556  | 0.113  0.099  0.075 
+2     | 0.000250  | 0.258      | 0.155      | 0.844           | 0.700        | 0.060             | 0.434    0.183    0.353    0.013    0.625    0.556    0.552   | 0.358    0.069    0.124    0.013    0.550    0.479    0.456   | 0.740  0.593  0.748  | 0.075  0.055  0.051 
+3     | 0.000375  | 0.175      | 0.138      | 0.846           | 0.703        | 0.059             | 0.302    0.120    0.230    0.010    0.544    0.478    0.460   | 0.316    0.061    0.109    0.014    0.527    0.456    0.438   | 0.726  0.621  0.773  | 0.069  0.061  0.046 
+4     | 0.000500  | 0.143      | 0.136      | 0.840           | 0.676        | 0.051             | 0.231    0.105    0.199    0.010    0.503    0.434    0.403   | 0.279    0.074    0.131    0.017    0.476    0.380    0.364   | 0.702  0.595  0.697  | 0.050  0.066  0.037 
+5     | 0.000495  | 0.126      | 0.109      | 0.861           | 0.723        | 0.047             | 0.194    0.096    0.183    0.010    0.477    0.408    0.370   | 0.224    0.060    0.104    0.015    0.455    0.384    0.343   | 0.747  0.644  0.777  | 0.058  0.062  0.022 
+6     | 0.000480  | 0.109      | 0.114      | 0.848           | 0.703        | 0.055             | 0.160    0.087    0.164    0.009    0.459    0.391    0.347   | 0.237    0.062    0.106    0.018    0.452    0.378    0.340   | 0.734  0.624  0.747  | 0.062  0.060  0.044 
+7     | 0.000457  | 0.108      | 0.121      | 0.838           | 0.682        | 0.058             | 0.152    0.089    0.168    0.010    0.451    0.379    0.334   | 0.254    0.063    0.108    0.018    0.477    0.400    0.322   | 0.712  0.604  0.748  | 0.072  0.058  0.043 
+8     | 0.000427  | 0.092      | 0.107      | 0.846           | 0.704        | 0.059             | 0.124    0.078    0.148    0.009    0.439    0.369    0.320   | 0.218    0.060    0.103    0.017    0.441    0.369    0.319   | 0.735  0.637  0.756  | 0.065  0.066  0.045 
+9     | 0.000393  | 0.082      | 0.111      | 0.857           | 0.712        | 0.047             | 0.105    0.072    0.136    0.008    0.432    0.361    0.309   | 0.229    0.060    0.102    0.018    0.437    0.383    0.295   | 0.741  0.638  0.763  | 0.057  0.061  0.024 
+10    | 0.000357  | 0.082      | 0.108      | 0.851           | 0.712        | 0.056             | 0.101    0.074    0.139    0.008    0.427    0.356    0.304   | 0.219    0.061    0.104    0.019    0.428    0.364    0.296   | 0.728  0.642  0.774  | 0.059  0.065  0.043 
+11    | 0.000323  | 0.074      | 0.099      | 0.856           | 0.721        | 0.053             | 0.089    0.067    0.127    0.008    0.423    0.351    0.296   | 0.191    0.059    0.100    0.018    0.429    0.358    0.269   | 0.743  0.644  0.783  | 0.061  0.065  0.035 
+12    | 0.000293  | 0.067      | 0.103      | 0.861           | 0.726        | 0.050             | 0.078    0.063    0.118    0.007    0.419    0.345    0.291   | 0.203    0.060    0.099    0.020    0.416    0.354    0.283   | 0.749  0.656  0.785  | 0.060  0.051  0.038 
+13    | 0.000270  | 0.064      | 0.119      | 0.854           | 0.711        | 0.051             | 0.072    0.061    0.115    0.007    0.415    0.342    0.286   | 0.255    0.060    0.101    0.020    0.429    0.365    0.258   | 0.730  0.640  0.766  | 0.065  0.063  0.024 
+14    | 0.000255  | 0.063      | 0.109      | 0.856           | 0.719        | 0.054             | 0.068    0.060    0.114    0.007    0.413    0.338    0.282   | 0.220    0.062    0.103    0.020    0.406    0.336    0.267   | 0.740  0.640  0.787  | 0.070  0.055  0.036 
+15    | 0.000250  | 0.059      | 0.112      | 0.858           | 0.722        | 0.052             | 0.061    0.058    0.109    0.007    0.409    0.336    0.278   | 0.231    0.061    0.101    0.022    0.420    0.355    0.262   | 0.739  0.645  0.794  | 0.066  0.062  0.028 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2514  2004  1445
+FP   263   287    58
+FN    63    65    81
+TN  4456  4940  5712
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.345  0.275  0.198
+FP  0.036  0.039  0.008
+FN  0.009  0.009  0.011
+TN  0.611  0.677  0.783
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.112      | 0.858           | 0.722        | 0.052             | 0.231    0.061    0.101    0.022    0.420    0.355    0.262   | 0.739  0.645  0.794  | 0.066  0.062  0.028 
+266     | 266     | 0.109      | 0.859           | 0.724        | 0.052             | 0.218    0.062    0.102    0.023    0.411    0.353    0.254   | 0.737  0.650  0.801  | 0.066  0.060  0.029 
+360     | 310     | 0.120      | 0.845           | 0.685        | 0.049             | 0.291    0.046    0.082    0.011    0.406    0.320    0.315   | 0.718  0.582  0.771  | 0.053  0.071  0.022 
+276     | 276     | 0.175      | 0.856           | 0.738        | 0.064             | 0.417    0.071    0.117    0.026    0.675    0.504    0.367   | 0.808  0.644  0.720  | 0.076  0.085  0.032 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA cutoff (47m 18s)
+best cutoff found : (0.75,0.75,0.75)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cutoffs(LB,SB,S) | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.104      | 0.862169        | 0.732        | 0.051             | 0.216    0.056    0.093    0.019    0.424    0.358    0.273   | 0.751  0.661  0.802  | 0.061  0.056  0.036 
+(0.25,0.25,0.25) | 0.104      | 0.862168        | 0.732        | 0.051             | 0.216    0.056    0.093    0.019    0.424    0.358    0.273   | 0.751  0.661  0.802  | 0.061  0.056  0.036 
+(0.50,0.50,0.50) | 0.104      | 0.862847        | 0.734        | 0.051             | 0.216    0.056    0.093    0.019    0.424    0.358    0.273   | 0.752  0.664  0.802  | 0.061  0.056  0.036 
+(0.75,0.75,0.75) | 0.104      | 0.866112        | 0.739        | 0.049             | 0.216    0.056    0.093    0.019    0.424    0.358    0.273   | 0.757  0.668  0.807  | 0.059  0.056  0.032 
+(0.60,0.70,0.70) | 0.104      | 0.865608        | 0.738        | 0.049             | 0.216    0.056    0.093    0.019    0.424    0.358    0.273   | 0.754  0.667  0.806  | 0.060  0.056  0.032 
+(0.60,0.70,0.80) | 0.104      | 0.865711        | 0.738        | 0.049             | 0.216    0.056    0.093    0.019    0.424    0.358    0.273   | 0.754  0.667  0.807  | 0.060  0.056  0.032 
+(0.50,0.75,0.75) | 0.104      | 0.865132        | 0.737        | 0.049             | 0.216    0.056    0.093    0.019    0.424    0.358    0.273   | 0.752  0.668  0.807  | 0.061  0.056  0.032 
+(0.75, 0.75, 0.75) tensor(0.8661)
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2512  1987  1474
+FP   239   259    82
+FN    65    82    52
+TN  4480  4968  5688
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.344  0.272  0.202
+FP  0.033  0.035  0.011
+FN  0.009  0.011  0.007
+TN  0.614  0.681  0.780
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.104      | 0.866           | 0.739        | 0.049             | 0.216    0.056    0.093    0.019    0.424    0.358    0.273   | 0.757  0.668  0.807  | 0.059  0.056  0.032 
+266     | 266     | 0.101      | 0.867           | 0.742        | 0.050             | 0.204    0.057    0.094    0.020    0.415    0.355    0.264   | 0.756  0.674  0.814  | 0.062  0.055  0.033 
+360     | 310     | 0.104      | 0.856           | 0.700        | 0.039             | 0.251    0.041    0.072    0.010    0.409    0.324    0.326   | 0.739  0.610  0.795  | 0.043  0.058  0.017 
+276     | 276     | 0.179      | 0.865           | 0.738        | 0.050             | 0.435    0.069    0.113    0.024    0.684    0.514    0.386   | 0.799  0.651  0.726  | 0.043  0.073  0.034 </t>
+  </si>
 </sst>
 </file>
 
@@ -3053,7 +3655,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -3087,17 +3689,6 @@
       <name val="Courier New"/>
       <family val="3"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -3153,7 +3744,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3198,12 +3789,12 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -3246,16 +3837,28 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3441,15 +4044,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K224"/>
+  <dimension ref="A1:K270"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="12.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="12.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="12.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="207.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="13.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="11.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="252.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="65.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="12.23"/>
   </cols>
   <sheetData>
@@ -3486,7 +4089,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="n">
@@ -3498,13 +4101,15 @@
       <c r="D4" s="2" t="n">
         <v>0.82138</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11"/>
+    </row>
     <row r="6" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="2" t="n">
@@ -3516,12 +4121,15 @@
       <c r="D6" s="2" t="n">
         <v>0.8158</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="12" t="s">
         <v>9</v>
       </c>
     </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11"/>
+    </row>
     <row r="8" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="2" t="n">
@@ -3533,12 +4141,15 @@
       <c r="D8" s="2" t="n">
         <v>0.81291</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="12" t="s">
         <v>11</v>
       </c>
     </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11"/>
+    </row>
     <row r="10" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="2" t="n">
@@ -3550,12 +4161,15 @@
       <c r="D10" s="13" t="n">
         <v>0.821</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="12" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11"/>
+    </row>
     <row r="12" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="11" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="2" t="n">
@@ -3567,9 +4181,12 @@
       <c r="D12" s="13" t="n">
         <v>0.82377</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="12" t="s">
         <v>15</v>
       </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
@@ -3584,9 +4201,12 @@
       <c r="D14" s="13" t="n">
         <v>0.81809</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="12" t="s">
         <v>17</v>
       </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
@@ -3601,66 +4221,87 @@
       <c r="D16" s="13" t="n">
         <v>0.81975</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="12" t="s">
         <v>19</v>
       </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="12" t="s">
         <v>21</v>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11"/>
+    </row>
     <row r="20" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="11" t="s">
         <v>22</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>0.83</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="12" t="s">
         <v>23</v>
       </c>
     </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11"/>
+    </row>
     <row r="22" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="12" t="s">
         <v>25</v>
       </c>
     </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11"/>
+    </row>
     <row r="24" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="12" t="s">
         <v>27</v>
       </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="12" t="s">
         <v>29</v>
       </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="E28" s="12" t="s">
         <v>31</v>
       </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="11" t="s">
+      <c r="E30" s="12" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3671,33 +4312,45 @@
       <c r="A32" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E32" s="11" t="s">
+      <c r="E32" s="12" t="s">
         <v>35</v>
       </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E34" s="11" t="s">
+      <c r="E34" s="12" t="s">
         <v>37</v>
       </c>
     </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11"/>
+    </row>
     <row r="36" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1" t="s">
+      <c r="A36" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="E36" s="11" t="s">
+      <c r="E36" s="12" t="s">
         <v>39</v>
       </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E38" s="11" t="s">
+      <c r="E38" s="12" t="s">
         <v>41</v>
       </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
@@ -3712,12 +4365,15 @@
       <c r="D40" s="16" t="n">
         <v>0.82371</v>
       </c>
-      <c r="E40" s="11" t="s">
+      <c r="E40" s="12" t="s">
         <v>43</v>
       </c>
     </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="11"/>
+    </row>
     <row r="42" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="11" t="s">
         <v>44</v>
       </c>
       <c r="B42" s="2" t="n">
@@ -3729,11 +4385,12 @@
       <c r="D42" s="13" t="n">
         <v>0.82784</v>
       </c>
-      <c r="E42" s="11" t="s">
+      <c r="E42" s="12" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="11"/>
       <c r="E43" s="9"/>
     </row>
     <row r="44" s="3" customFormat="true" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3749,11 +4406,12 @@
       <c r="D44" s="13" t="n">
         <v>0.83243</v>
       </c>
-      <c r="E44" s="11" t="s">
+      <c r="E44" s="12" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="11"/>
       <c r="E45" s="9"/>
     </row>
     <row r="46" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3769,9 +4427,12 @@
       <c r="D46" s="13" t="n">
         <v>0.83364</v>
       </c>
-      <c r="E46" s="11" t="s">
+      <c r="E46" s="12" t="s">
         <v>49</v>
       </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
@@ -3786,9 +4447,12 @@
       <c r="D48" s="13" t="n">
         <v>0.83249</v>
       </c>
-      <c r="E48" s="11" t="s">
+      <c r="E48" s="12" t="s">
         <v>51</v>
       </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="11"/>
     </row>
     <row r="50" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="s">
@@ -3803,11 +4467,13 @@
       <c r="D50" s="13" t="n">
         <v>0.83234</v>
       </c>
-      <c r="E50" s="11" t="s">
+      <c r="E50" s="12" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="11"/>
+    </row>
     <row r="52" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="s">
         <v>54</v>
@@ -3821,9 +4487,12 @@
       <c r="D52" s="13" t="n">
         <v>0.83193</v>
       </c>
-      <c r="E52" s="11" t="s">
+      <c r="E52" s="12" t="s">
         <v>55</v>
       </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="11"/>
     </row>
     <row r="54" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="8" t="s">
@@ -3832,9 +4501,12 @@
       <c r="B54" s="2" t="n">
         <v>0.839</v>
       </c>
-      <c r="E54" s="11" t="s">
+      <c r="E54" s="12" t="s">
         <v>57</v>
       </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="11"/>
     </row>
     <row r="56" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="s">
@@ -3843,9 +4515,12 @@
       <c r="B56" s="2" t="n">
         <v>0.828</v>
       </c>
-      <c r="E56" s="11" t="s">
+      <c r="E56" s="12" t="s">
         <v>59</v>
       </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="11"/>
     </row>
     <row r="58" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="8" t="s">
@@ -3854,9 +4529,12 @@
       <c r="B58" s="2" t="n">
         <v>0.664</v>
       </c>
-      <c r="E58" s="11" t="s">
+      <c r="E58" s="12" t="s">
         <v>61</v>
       </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="11"/>
     </row>
     <row r="60" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="s">
@@ -3865,9 +4543,12 @@
       <c r="B60" s="2" t="n">
         <v>0.822</v>
       </c>
-      <c r="E60" s="11" t="s">
+      <c r="E60" s="12" t="s">
         <v>63</v>
       </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="11"/>
     </row>
     <row r="62" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="s">
@@ -3876,9 +4557,12 @@
       <c r="B62" s="2" t="n">
         <v>0.684</v>
       </c>
-      <c r="E62" s="11" t="s">
+      <c r="E62" s="12" t="s">
         <v>65</v>
       </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="11"/>
     </row>
     <row r="64" customFormat="false" ht="138.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="s">
@@ -3893,11 +4577,13 @@
       <c r="D64" s="13" t="n">
         <v>0.82728</v>
       </c>
-      <c r="E64" s="11" t="s">
+      <c r="E64" s="12" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="65" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="11"/>
+    </row>
     <row r="66" customFormat="false" ht="199.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="8" t="s">
         <v>68</v>
@@ -3911,11 +4597,13 @@
       <c r="D66" s="13" t="n">
         <v>0.8276</v>
       </c>
-      <c r="E66" s="11" t="s">
+      <c r="E66" s="12" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="67" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="11"/>
+    </row>
     <row r="68" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="8" t="s">
         <v>70</v>
@@ -3923,9 +4611,12 @@
       <c r="B68" s="2" t="n">
         <v>0.834</v>
       </c>
-      <c r="E68" s="11" t="s">
+      <c r="E68" s="12" t="s">
         <v>71</v>
       </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="11"/>
     </row>
     <row r="70" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="8" t="s">
@@ -3940,9 +4631,12 @@
       <c r="D70" s="13" t="n">
         <v>0.83245</v>
       </c>
-      <c r="E70" s="11" t="s">
+      <c r="E70" s="12" t="s">
         <v>73</v>
       </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="11"/>
     </row>
     <row r="72" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="8" t="s">
@@ -3951,9 +4645,12 @@
       <c r="B72" s="14" t="n">
         <v>0.827</v>
       </c>
-      <c r="E72" s="11" t="s">
+      <c r="E72" s="12" t="s">
         <v>75</v>
       </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="11"/>
     </row>
     <row r="74" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="8" t="s">
@@ -3968,9 +4665,12 @@
       <c r="D74" s="13" t="n">
         <v>0.83245</v>
       </c>
-      <c r="E74" s="11" t="s">
+      <c r="E74" s="12" t="s">
         <v>77</v>
       </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="11"/>
     </row>
     <row r="76" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="8" t="s">
@@ -3985,9 +4685,12 @@
       <c r="D76" s="13" t="n">
         <v>0.8311</v>
       </c>
-      <c r="E76" s="11" t="s">
+      <c r="E76" s="12" t="s">
         <v>79</v>
       </c>
+    </row>
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="11"/>
     </row>
     <row r="78" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="8" t="s">
@@ -3996,9 +4699,12 @@
       <c r="B78" s="2" t="n">
         <v>0.829</v>
       </c>
-      <c r="E78" s="11" t="s">
+      <c r="E78" s="12" t="s">
         <v>81</v>
       </c>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="11"/>
     </row>
     <row r="80" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="8" t="s">
@@ -4013,9 +4719,12 @@
       <c r="D80" s="2" t="n">
         <v>0.83537</v>
       </c>
-      <c r="E80" s="11" t="s">
+      <c r="E80" s="12" t="s">
         <v>83</v>
       </c>
+    </row>
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="11"/>
     </row>
     <row r="82" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="8" t="s">
@@ -4030,9 +4739,12 @@
       <c r="D82" s="2" t="n">
         <v>0.8408</v>
       </c>
-      <c r="E82" s="11" t="s">
+      <c r="E82" s="12" t="s">
         <v>85</v>
       </c>
+    </row>
+    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="11"/>
     </row>
     <row r="84" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="8" t="s">
@@ -4047,9 +4759,12 @@
       <c r="D84" s="13" t="n">
         <v>0.82848</v>
       </c>
-      <c r="E84" s="11" t="s">
+      <c r="E84" s="12" t="s">
         <v>87</v>
       </c>
+    </row>
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="11"/>
     </row>
     <row r="86" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="8" t="s">
@@ -4064,9 +4779,12 @@
       <c r="D86" s="2" t="n">
         <v>0.83301</v>
       </c>
-      <c r="E86" s="11" t="s">
+      <c r="E86" s="12" t="s">
         <v>89</v>
       </c>
+    </row>
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="11"/>
     </row>
     <row r="88" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="8" t="s">
@@ -4081,9 +4799,12 @@
       <c r="D88" s="2" t="n">
         <v>0.83529</v>
       </c>
-      <c r="E88" s="11" t="s">
+      <c r="E88" s="12" t="s">
         <v>91</v>
       </c>
+    </row>
+    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="11"/>
     </row>
     <row r="90" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="8" t="s">
@@ -4098,9 +4819,12 @@
       <c r="D90" s="2" t="n">
         <v>0.84112</v>
       </c>
-      <c r="E90" s="11" t="s">
+      <c r="E90" s="12" t="s">
         <v>93</v>
       </c>
+    </row>
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="11"/>
     </row>
     <row r="92" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="8" t="s">
@@ -4115,9 +4839,12 @@
       <c r="D92" s="2" t="n">
         <v>0.84107</v>
       </c>
-      <c r="E92" s="11" t="s">
+      <c r="E92" s="12" t="s">
         <v>95</v>
       </c>
+    </row>
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="11"/>
     </row>
     <row r="94" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="8" t="s">
@@ -4132,9 +4859,12 @@
       <c r="D94" s="2" t="n">
         <v>0.84292</v>
       </c>
-      <c r="E94" s="11" t="s">
+      <c r="E94" s="12" t="s">
         <v>97</v>
       </c>
+    </row>
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="11"/>
     </row>
     <row r="96" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="8" t="s">
@@ -4143,9 +4873,12 @@
       <c r="B96" s="2" t="n">
         <v>0.824</v>
       </c>
-      <c r="E96" s="11" t="s">
+      <c r="E96" s="12" t="s">
         <v>99</v>
       </c>
+    </row>
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="11"/>
     </row>
     <row r="98" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="8" t="s">
@@ -4160,9 +4893,12 @@
       <c r="D98" s="2" t="n">
         <v>0.83613</v>
       </c>
-      <c r="E98" s="11" t="s">
+      <c r="E98" s="12" t="s">
         <v>101</v>
       </c>
+    </row>
+    <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="11"/>
     </row>
     <row r="100" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="8" t="s">
@@ -4177,7 +4913,7 @@
       <c r="D100" s="13" t="n">
         <v>0.84072</v>
       </c>
-      <c r="E100" s="11" t="s">
+      <c r="E100" s="12" t="s">
         <v>103</v>
       </c>
     </row>
@@ -4209,6 +4945,9 @@
         <v>0.84371</v>
       </c>
     </row>
+    <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="11"/>
+    </row>
     <row r="104" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="8" t="s">
         <v>106</v>
@@ -4222,12 +4961,12 @@
       <c r="D104" s="14" t="n">
         <v>0.8418</v>
       </c>
-      <c r="E104" s="11" t="s">
+      <c r="E104" s="12" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="1" t="s">
+      <c r="A105" s="11" t="s">
         <v>108</v>
       </c>
       <c r="B105" s="2" t="n">
@@ -4239,6 +4978,9 @@
       <c r="D105" s="14" t="n">
         <v>0.83303</v>
       </c>
+    </row>
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="11"/>
     </row>
     <row r="107" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="8" t="s">
@@ -4253,12 +4995,12 @@
       <c r="D107" s="14" t="n">
         <v>0.84214</v>
       </c>
-      <c r="E107" s="11" t="s">
+      <c r="E107" s="12" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="1" t="s">
+      <c r="A108" s="11" t="s">
         <v>111</v>
       </c>
       <c r="B108" s="2" t="n">
@@ -4270,6 +5012,9 @@
       <c r="D108" s="14" t="n">
         <v>0.83613</v>
       </c>
+    </row>
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="11"/>
     </row>
     <row r="110" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="8" t="s">
@@ -4284,12 +5029,12 @@
       <c r="D110" s="14" t="n">
         <v>0.84085</v>
       </c>
-      <c r="E110" s="11" t="s">
+      <c r="E110" s="12" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="1" t="s">
+      <c r="A111" s="11" t="s">
         <v>104</v>
       </c>
       <c r="B111" s="2" t="n">
@@ -4301,6 +5046,9 @@
       <c r="D111" s="14" t="n">
         <v>0.841</v>
       </c>
+    </row>
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="11"/>
     </row>
     <row r="113" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="8" t="s">
@@ -4315,12 +5063,12 @@
       <c r="D113" s="14" t="n">
         <v>0.84427</v>
       </c>
-      <c r="E113" s="11" t="s">
+      <c r="E113" s="12" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="1" t="s">
+      <c r="A114" s="11" t="s">
         <v>105</v>
       </c>
       <c r="B114" s="2" t="n">
@@ -4332,6 +5080,9 @@
       <c r="D114" s="14" t="n">
         <v>0.84507</v>
       </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="11"/>
     </row>
     <row r="116" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="8" t="s">
@@ -4346,9 +5097,12 @@
       <c r="D116" s="14" t="n">
         <v>0.84438</v>
       </c>
-      <c r="E116" s="11" t="s">
+      <c r="E116" s="12" t="s">
         <v>117</v>
       </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="11"/>
     </row>
     <row r="118" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="8" t="s">
@@ -4363,12 +5117,12 @@
       <c r="D118" s="14" t="n">
         <v>0.844</v>
       </c>
-      <c r="E118" s="11" t="s">
+      <c r="E118" s="12" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="1" t="s">
+      <c r="A119" s="11" t="s">
         <v>105</v>
       </c>
       <c r="B119" s="2" t="n">
@@ -4380,6 +5134,9 @@
       <c r="D119" s="14" t="n">
         <v>0.8404</v>
       </c>
+    </row>
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="11"/>
     </row>
     <row r="121" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="8" t="s">
@@ -4394,12 +5151,12 @@
       <c r="D121" s="14" t="n">
         <v>0.83443</v>
       </c>
-      <c r="E121" s="11" t="s">
+      <c r="E121" s="12" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="1" t="s">
+      <c r="A122" s="11" t="s">
         <v>104</v>
       </c>
       <c r="B122" s="2" t="n">
@@ -4411,6 +5168,9 @@
       <c r="D122" s="14" t="n">
         <v>0.83667</v>
       </c>
+    </row>
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="11"/>
     </row>
     <row r="124" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="8" t="s">
@@ -4425,12 +5185,12 @@
       <c r="D124" s="13" t="n">
         <v>0.84691</v>
       </c>
-      <c r="E124" s="11" t="s">
+      <c r="E124" s="12" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="1" t="s">
+      <c r="A125" s="11" t="s">
         <v>104</v>
       </c>
       <c r="B125" s="2" t="n">
@@ -4444,7 +5204,7 @@
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="1" t="s">
+      <c r="A126" s="11" t="s">
         <v>105</v>
       </c>
       <c r="B126" s="2" t="n">
@@ -4457,7 +5217,10 @@
         <v>0.83256</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="471.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="11"/>
+    </row>
+    <row r="128" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="8" t="s">
         <v>124</v>
       </c>
@@ -4475,7 +5238,7 @@
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="1" t="s">
+      <c r="A129" s="11" t="s">
         <v>104</v>
       </c>
       <c r="B129" s="2" t="n">
@@ -4488,7 +5251,10 @@
         <v>0.84537</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="829.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="11"/>
+    </row>
+    <row r="131" customFormat="false" ht="661.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="8" t="s">
         <v>126</v>
       </c>
@@ -4501,12 +5267,12 @@
       <c r="D131" s="2" t="n">
         <v>0.82678</v>
       </c>
-      <c r="E131" s="11" t="s">
+      <c r="E131" s="12" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="1" t="s">
+      <c r="A132" s="11" t="s">
         <v>104</v>
       </c>
       <c r="B132" s="2" t="n">
@@ -4519,7 +5285,10 @@
         <v>0.8331</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="807.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="11"/>
+    </row>
+    <row r="134" customFormat="false" ht="639.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="8" t="s">
         <v>128</v>
       </c>
@@ -4532,11 +5301,11 @@
       <c r="D134" s="2" t="n">
         <v>0.83507</v>
       </c>
-      <c r="E134" s="11" t="s">
+      <c r="E134" s="12" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="17" t="s">
         <v>130</v>
       </c>
@@ -4549,11 +5318,11 @@
       <c r="D135" s="2" t="n">
         <v>0.84632</v>
       </c>
-      <c r="E135" s="11" t="s">
+      <c r="E135" s="12" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="314.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="247.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="17" t="s">
         <v>132</v>
       </c>
@@ -4566,11 +5335,14 @@
       <c r="D136" s="2" t="n">
         <v>0.84591</v>
       </c>
-      <c r="E136" s="11" t="s">
+      <c r="E136" s="12" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="605.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="11"/>
+    </row>
+    <row r="138" customFormat="false" ht="538.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="8" t="s">
         <v>134</v>
       </c>
@@ -4583,7 +5355,7 @@
       <c r="D138" s="2" t="n">
         <v>0.83892</v>
       </c>
-      <c r="E138" s="11" t="s">
+      <c r="E138" s="12" t="s">
         <v>135</v>
       </c>
     </row>
@@ -4598,7 +5370,10 @@
         <v>0.84523</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="617.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="11"/>
+    </row>
+    <row r="141" customFormat="false" ht="550" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="8" t="s">
         <v>137</v>
       </c>
@@ -4611,7 +5386,7 @@
       <c r="D141" s="2" t="n">
         <v>0.83337</v>
       </c>
-      <c r="E141" s="11" t="s">
+      <c r="E141" s="12" t="s">
         <v>138</v>
       </c>
     </row>
@@ -4626,7 +5401,10 @@
         <v>0.83464</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="583.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="11"/>
+    </row>
+    <row r="144" customFormat="false" ht="516.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="8" t="s">
         <v>139</v>
       </c>
@@ -4639,7 +5417,7 @@
       <c r="D144" s="2" t="n">
         <v>0.84165</v>
       </c>
-      <c r="E144" s="11" t="s">
+      <c r="E144" s="12" t="s">
         <v>140</v>
       </c>
     </row>
@@ -4680,7 +5458,10 @@
         <v>0.84618</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="561.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="11"/>
+    </row>
+    <row r="149" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="8" t="s">
         <v>143</v>
       </c>
@@ -4693,7 +5474,7 @@
       <c r="D149" s="2" t="n">
         <v>0.82896</v>
       </c>
-      <c r="E149" s="11" t="s">
+      <c r="E149" s="12" t="s">
         <v>144</v>
       </c>
     </row>
@@ -4733,7 +5514,10 @@
         <v>0.83038</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="941.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="11"/>
+    </row>
+    <row r="154" customFormat="false" ht="706.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="8" t="s">
         <v>145</v>
       </c>
@@ -4746,7 +5530,7 @@
       <c r="D154" s="2" t="n">
         <v>0.83194</v>
       </c>
-      <c r="E154" s="11" t="s">
+      <c r="E154" s="12" t="s">
         <v>146</v>
       </c>
     </row>
@@ -4806,7 +5590,7 @@
       <c r="C159" s="20"/>
       <c r="D159" s="20"/>
     </row>
-    <row r="160" customFormat="false" ht="572.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="505.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="9" t="s">
         <v>148</v>
       </c>
@@ -4815,18 +5599,24 @@
       </c>
       <c r="C160" s="20"/>
       <c r="D160" s="20"/>
-      <c r="E160" s="11" t="s">
+      <c r="E160" s="12" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="561.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="11"/>
+    </row>
+    <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="11"/>
+    </row>
+    <row r="163" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="8" t="s">
         <v>150</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>0.85</v>
       </c>
-      <c r="E163" s="11" t="s">
+      <c r="E163" s="12" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4838,7 +5628,16 @@
         <v>0.851</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="572.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="11"/>
+    </row>
+    <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="11"/>
+    </row>
+    <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="11"/>
+    </row>
+    <row r="168" customFormat="false" ht="505.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="10" t="s">
         <v>152</v>
       </c>
@@ -4851,7 +5650,7 @@
       <c r="D168" s="2" t="n">
         <v>0.8448</v>
       </c>
-      <c r="E168" s="11" t="s">
+      <c r="E168" s="12" t="s">
         <v>153</v>
       </c>
     </row>
@@ -4869,7 +5668,7 @@
         <v>0.83892</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="505.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="337.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="17" t="s">
         <v>136</v>
       </c>
@@ -4882,7 +5681,7 @@
       <c r="D170" s="2" t="n">
         <v>0.8503</v>
       </c>
-      <c r="E170" s="11" t="s">
+      <c r="E170" s="12" t="s">
         <v>154</v>
       </c>
     </row>
@@ -4911,7 +5710,10 @@
         <v>0.8539</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="572.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="11"/>
+    </row>
+    <row r="174" customFormat="false" ht="505.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="10" t="s">
         <v>156</v>
       </c>
@@ -4924,7 +5726,7 @@
       <c r="D174" s="2" t="n">
         <v>0.84376</v>
       </c>
-      <c r="E174" s="11" t="s">
+      <c r="E174" s="12" t="s">
         <v>157</v>
       </c>
     </row>
@@ -4939,7 +5741,10 @@
         <v>0.85129</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="572.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="11"/>
+    </row>
+    <row r="177" customFormat="false" ht="505.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="10" t="s">
         <v>158</v>
       </c>
@@ -4952,7 +5757,7 @@
       <c r="D177" s="2" t="n">
         <v>0.84458</v>
       </c>
-      <c r="E177" s="11" t="s">
+      <c r="E177" s="12" t="s">
         <v>159</v>
       </c>
     </row>
@@ -4992,7 +5797,10 @@
         <v>0.84798</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="561.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="11"/>
+    </row>
+    <row r="182" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="10" t="s">
         <v>160</v>
       </c>
@@ -5005,7 +5813,7 @@
       <c r="D182" s="2" t="n">
         <v>0.83935</v>
       </c>
-      <c r="E182" s="11" t="s">
+      <c r="E182" s="12" t="s">
         <v>161</v>
       </c>
     </row>
@@ -5023,7 +5831,7 @@
         <v>0.83951</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="505.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="337.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="17" t="s">
         <v>136</v>
       </c>
@@ -5036,7 +5844,7 @@
       <c r="D184" s="2" t="n">
         <v>0.85075</v>
       </c>
-      <c r="E184" s="11" t="s">
+      <c r="E184" s="12" t="s">
         <v>162</v>
       </c>
     </row>
@@ -5065,7 +5873,10 @@
         <v>0.85173</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="561.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="11"/>
+    </row>
+    <row r="188" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="10" t="s">
         <v>164</v>
       </c>
@@ -5078,7 +5889,7 @@
       <c r="D188" s="2" t="n">
         <v>0.83834</v>
       </c>
-      <c r="E188" s="11" t="s">
+      <c r="E188" s="12" t="s">
         <v>165</v>
       </c>
     </row>
@@ -5118,18 +5929,27 @@
         <v>0.83963</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="561.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="11"/>
+    </row>
+    <row r="193" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="10" t="s">
         <v>168</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>0.835</v>
       </c>
-      <c r="E193" s="11" t="s">
+      <c r="E193" s="12" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="673.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="11"/>
+    </row>
+    <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="11"/>
+    </row>
+    <row r="196" customFormat="false" ht="605.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="10" t="s">
         <v>170</v>
       </c>
@@ -5142,7 +5962,7 @@
       <c r="D196" s="2" t="n">
         <v>0.84335</v>
       </c>
-      <c r="E196" s="11" t="s">
+      <c r="E196" s="12" t="s">
         <v>171</v>
       </c>
     </row>
@@ -5182,7 +6002,13 @@
         <v>0.85397</v>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="673.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="11"/>
+    </row>
+    <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="11"/>
+    </row>
+    <row r="202" customFormat="false" ht="605.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="10" t="s">
         <v>174</v>
       </c>
@@ -5195,7 +6021,7 @@
       <c r="D202" s="2" t="n">
         <v>0.84582</v>
       </c>
-      <c r="E202" s="11" t="s">
+      <c r="E202" s="12" t="s">
         <v>175</v>
       </c>
     </row>
@@ -5210,7 +6036,10 @@
         <v>0.85247</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="673.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="11"/>
+    </row>
+    <row r="205" customFormat="false" ht="605.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="10" t="s">
         <v>176</v>
       </c>
@@ -5223,7 +6052,7 @@
       <c r="D205" s="2" t="n">
         <v>0.84595</v>
       </c>
-      <c r="E205" s="11" t="s">
+      <c r="E205" s="12" t="s">
         <v>177</v>
       </c>
     </row>
@@ -5263,6 +6092,9 @@
         <v>0.85492</v>
       </c>
     </row>
+    <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="11"/>
+    </row>
     <row r="210" customFormat="false" ht="370.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="8" t="s">
         <v>180</v>
@@ -5274,7 +6106,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="8" t="s">
         <v>182</v>
       </c>
@@ -5282,7 +6114,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="212" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="8" t="s">
         <v>184</v>
       </c>
@@ -5290,7 +6122,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="8" t="s">
         <v>186</v>
       </c>
@@ -5298,7 +6130,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="8" t="s">
         <v>188</v>
       </c>
@@ -5306,7 +6138,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="8" t="s">
         <v>190</v>
       </c>
@@ -5314,7 +6146,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="8" t="s">
         <v>192</v>
       </c>
@@ -5322,7 +6154,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="8" t="s">
         <v>194</v>
       </c>
@@ -5330,7 +6162,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="8" t="s">
         <v>196</v>
       </c>
@@ -5343,14 +6175,17 @@
         <v>198</v>
       </c>
     </row>
+    <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="11"/>
+    </row>
     <row r="221" customFormat="false" ht="379.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A221" s="24" t="s">
+      <c r="A221" s="10" t="s">
         <v>199</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>0.829</v>
       </c>
-      <c r="E221" s="25" t="s">
+      <c r="E221" s="12" t="s">
         <v>200</v>
       </c>
     </row>
@@ -5384,7 +6219,338 @@
         <v>0.84748</v>
       </c>
     </row>
+    <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="11"/>
+    </row>
+    <row r="226" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="E226" s="12" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="11"/>
+    </row>
+    <row r="228" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="E228" s="12" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="11"/>
+    </row>
+    <row r="230" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="E230" s="12" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="11"/>
+    </row>
+    <row r="232" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="E232" s="12" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="11"/>
+    </row>
+    <row r="234" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="E234" s="12" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="11"/>
+    </row>
+    <row r="236" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="E236" s="12" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="11"/>
+    </row>
+    <row r="238" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="E238" s="12" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="11"/>
+    </row>
+    <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="3" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="11"/>
+    </row>
+    <row r="242" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="E242" s="12" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="11"/>
+    </row>
+    <row r="244" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="E244" s="12" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="11"/>
+    </row>
+    <row r="246" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="E246" s="12" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="11"/>
+    </row>
+    <row r="248" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="E248" s="12" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="11"/>
+    </row>
+    <row r="250" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A250" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="E250" s="12" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A251" s="11"/>
+    </row>
+    <row r="252" customFormat="false" ht="191.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A252" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="B252" s="2" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="C252" s="2" t="n">
+        <v>0.83974</v>
+      </c>
+      <c r="D252" s="2" t="n">
+        <v>0.8266</v>
+      </c>
+      <c r="E252" s="12" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="253" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A253" s="24"/>
+      <c r="E253" s="12" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A254" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B254" s="3"/>
+      <c r="C254" s="2" t="n">
+        <v>0.86345</v>
+      </c>
+      <c r="D254" s="2" t="n">
+        <v>0.85124</v>
+      </c>
+    </row>
+    <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A255" s="11"/>
+    </row>
+    <row r="256" customFormat="false" ht="191.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A256" s="24" t="s">
+        <v>229</v>
+      </c>
+      <c r="B256" s="2" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="C256" s="2" t="n">
+        <v>0.84048</v>
+      </c>
+      <c r="D256" s="2" t="n">
+        <v>0.83625</v>
+      </c>
+      <c r="E256" s="12" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="257" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A257" s="24"/>
+      <c r="E257" s="12" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C258" s="2" t="n">
+        <v>0.85897</v>
+      </c>
+      <c r="D258" s="2" t="n">
+        <v>0.85112</v>
+      </c>
+    </row>
+    <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="11"/>
+    </row>
+    <row r="260" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="B260" s="2" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="C260" s="2" t="n">
+        <v>0.85414</v>
+      </c>
+      <c r="D260" s="2" t="n">
+        <v>0.84257</v>
+      </c>
+      <c r="E260" s="25" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="261" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="0"/>
+      <c r="E261" s="25" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C262" s="2" t="n">
+        <v>0.86397</v>
+      </c>
+      <c r="D262" s="2" t="n">
+        <v>0.85458</v>
+      </c>
+    </row>
+    <row r="264" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="B264" s="2" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="C264" s="2" t="n">
+        <v>0.8591</v>
+      </c>
+      <c r="D264" s="2" t="n">
+        <v>0.85003</v>
+      </c>
+      <c r="E264" s="25" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="265" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E265" s="25" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B266" s="26" t="n">
+        <v>0.862847</v>
+      </c>
+      <c r="C266" s="23" t="n">
+        <v>0.86487</v>
+      </c>
+      <c r="D266" s="2" t="n">
+        <v>0.86004</v>
+      </c>
+    </row>
+    <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A267" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="C267" s="2" t="n">
+        <v>0.85518</v>
+      </c>
+      <c r="D267" s="2" t="n">
+        <v>0.84837</v>
+      </c>
+    </row>
+    <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A268" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="C268" s="2" t="n">
+        <v>0.86308</v>
+      </c>
+      <c r="D268" s="2" t="n">
+        <v>0.85689</v>
+      </c>
+    </row>
+    <row r="270" customFormat="false" ht="337.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A270" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="B270" s="2" t="n">
+        <v>0.866112</v>
+      </c>
+      <c r="C270" s="28" t="n">
+        <v>0.86495</v>
+      </c>
+      <c r="D270" s="2" t="n">
+        <v>0.8611</v>
+      </c>
+      <c r="E270" s="25" t="s">
+        <v>239</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A252:A253"/>
+    <mergeCell ref="A256:A257"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
mitb4 full data train, mitb5, other config for mitb1
</commit_message>
<xml_diff>
--- a/Scores.xlsx
+++ b/Scores.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="343">
   <si>
     <t xml:space="preserve">Description</t>
   </si>
@@ -2529,25 +2529,7 @@
 276     | 276     | 0.102      | 0.865           | 0.737        | 0.050             | 0.278    0.043    0.194    0.008    0.220    0.015    0.136    0.004   | 0.817  0.666  0.640  | 0.042  0.057  0.050 </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15 epoch from stable best model config
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t xml:space="preserve">15 epoch from stable best model config
 (15 epoch &amp; final_lr to 2.5e-4 changed from
 warmup&amp;cosdec,0.1LR pres,DL Lo(.5),.25PLo+.75SLo)
 Segformer with mit_b1 encoder 
@@ -2572,8 +2554,8 @@
 with grad_accu = 2, BS = 32    
 BS = 32 (train/valid/test)
 (3h 44m 18s)  
-(Max GPU mem usage : 10716.875 MB)   </t>
-    </r>
+(Max GPU mem usage : 10716.875 MB)   
+https://www.kaggle.com/code/abhivij/gi-tract-image-segmentation?scriptVersionId=278667321 </t>
   </si>
   <si>
     <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-LB-D TLo-LB-B TLo-SB-D TLo-SB-B TLo-S-D  TLo-S-B | VLo-Pres VLo-Seg  VLo-LB-D VLo-LB-B VLo-SB-D VLo-SB-B VLo-S-D  VLo-S-B | D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
@@ -4334,6 +4316,16 @@
 (Max GPU mem usage : 5708.875 MB)  </t>
   </si>
   <si>
+    <t xml:space="preserve">0.862
+(This config
+ used for 
+ Larger 
+ Models.
+ Taken as
+ Mit-b1 best.
+)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
 ------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
 1     | 0.000125  | 0.589      | 0.299      | 0.736           | 0.482        | 0.095             | 0.564    0.600    0.935    0.264    0.550    0.490    0.461   | 0.616    0.164    0.265    0.062    0.682    0.584    0.504   | 0.580  0.399  0.451  | 0.113  0.083  0.087 
@@ -4743,6 +4735,309 @@
   <si>
     <t xml:space="preserve">EMA with cutoff (0.6, 0.7, 0.8)</t>
   </si>
+  <si>
+    <t xml:space="preserve">Same config mitb4 with full data for training
+(9h 5m 34s)
+(Max GPU mem usage : 12716.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3
+-----------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.534      | 0.579    0.515    0.843    0.187    0.589    0.570    0.481   
+2     | 0.000250  | 0.268      | 0.554    0.145    0.282    0.009    0.602    0.569    0.574   
+3     | 0.000375  | 0.204      | 0.448    0.100    0.191    0.008    0.529    0.492    0.473   
+4     | 0.000500  | 0.187      | 0.410    0.091    0.173    0.009    0.490    0.454    0.424   
+5     | 0.000495  | 0.170      | 0.382    0.080    0.151    0.008    0.468    0.426    0.390   
+6     | 0.000480  | 0.164      | 0.371    0.076    0.143    0.008    0.453    0.410    0.374   
+7     | 0.000457  | 0.156      | 0.359    0.069    0.130    0.007    0.443    0.399    0.362   
+8     | 0.000427  | 0.152      | 0.355    0.066    0.124    0.007    0.436    0.392    0.351   
+9     | 0.000393  | 0.150      | 0.351    0.063    0.120    0.007    0.431    0.385    0.346   
+10    | 0.000357  | 0.144      | 0.345    0.059    0.110    0.007    0.425    0.381    0.341   
+11    | 0.000323  | 0.142      | 0.341    0.056    0.106    0.006    0.420    0.377    0.337   
+12    | 0.000293  | 0.139      | 0.339    0.054    0.102    0.006    0.418    0.374    0.335   
+13    | 0.000270  | 0.137      | 0.336    0.051    0.096    0.006    0.415    0.372    0.333   
+14    | 0.000255  | 0.137      | 0.337    0.051    0.096    0.006    0.414    0.370    0.332   
+15    | 0.000250  | 0.135      | 0.335    0.050    0.094    0.006    0.412    0.369    0.331  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">With cutoff (0.75, 0.75, 0.75)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 14 with cutoff (0.5, 0.5, 0.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 14 with cutoff (0.6, 0.7, 0.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 14 with cutoff (0.6, 0.7, 0.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 15 with cutoff (0.5, 0.5, 0.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 15 with cutoff (0.6, 0.7, 0.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 15 with cutoff (0.6, 0.7, 0.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit-b5 with LLRD and aux weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(10h 22m 53s)
+(Max GPU mem usage : 15024.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.571      | 0.287      | 0.763           | 0.524        | 0.077             | 0.550    0.580    0.921    0.239    0.555    0.509    0.488   | 0.616    0.146    0.245    0.046    0.672    0.576    0.538   | 0.593  0.478  0.493  | 0.087  0.069  0.074 
+2     | 0.000250  | 0.306      | 0.212      | 0.837           | 0.681        | 0.059             | 0.592    0.183    0.353    0.012    0.636    0.599    0.593   | 0.549    0.067    0.120    0.014    0.614    0.559    0.497   | 0.706  0.586  0.755  | 0.076  0.070  0.032 
+3     | 0.000375  | 0.217      | 0.187      | 0.852           | 0.703        | 0.049             | 0.471    0.108    0.207    0.008    0.553    0.516    0.498   | 0.480    0.061    0.109    0.013    0.527    0.512    0.449   | 0.733  0.617  0.782  | 0.061  0.064  0.021 
+4     | 0.000500  | 0.191      | 0.175      | 0.851           | 0.712        | 0.057             | 0.421    0.092    0.176    0.008    0.511    0.472    0.444   | 0.442    0.060    0.105    0.015    0.501    0.448    0.389   | 0.744  0.624  0.779  | 0.074  0.067  0.029 
+5     | 0.000495  | 0.174      | 0.181      | 0.855           | 0.705        | 0.045             | 0.392    0.081    0.153    0.008    0.486    0.442    0.411   | 0.446    0.067    0.118    0.016    0.440    0.411    0.385   | 0.728  0.619  0.764  | 0.051  0.050  0.034 
+6     | 0.000480  | 0.165      | 0.173      | 0.861           | 0.727        | 0.050             | 0.377    0.075    0.142    0.008    0.471    0.426    0.391   | 0.432    0.062    0.107    0.017    0.486    0.387    0.356   | 0.752  0.633  0.796  | 0.062  0.052  0.036 
+7     | 0.000457  | 0.160      | 0.182      | 0.842           | 0.689        | 0.056             | 0.367    0.071    0.134    0.008    0.460    0.414    0.377   | 0.445    0.069    0.120    0.019    0.417    0.373    0.394   | 0.733  0.595  0.723  | 0.051  0.051  0.068 
+8     | 0.000427  | 0.152      | 0.169      | 0.856           | 0.722        | 0.054             | 0.356    0.064    0.122    0.007    0.450    0.404    0.365   | 0.419    0.062    0.104    0.019    0.437    0.392    0.352   | 0.744  0.642  0.782  | 0.056  0.062  0.045 
+9     | 0.000393  | 0.149      | 0.175      | 0.851           | 0.712        | 0.056             | 0.352    0.061    0.116    0.007    0.445    0.396    0.359   | 0.441    0.061    0.103    0.020    0.453    0.404    0.341   | 0.739  0.623  0.779  | 0.060  0.062  0.046 
+10    | 0.000357  | 0.145      | 0.164      | 0.867           | 0.739        | 0.048             | 0.347    0.059    0.111    0.007    0.438    0.392    0.353   | 0.412    0.058    0.096    0.019    0.442    0.398    0.324   | 0.763  0.660  0.804  | 0.062  0.053  0.029 
+11    | 0.000323  | 0.142      | 0.166      | 0.864           | 0.737        | 0.051             | 0.343    0.056    0.106    0.006    0.434    0.388    0.348   | 0.418    0.059    0.098    0.019    0.425    0.376    0.339   | 0.758  0.658  0.794  | 0.054  0.054  0.045 
+12    | 0.000293  | 0.140      | 0.167      | 0.862           | 0.735        | 0.053             | 0.341    0.055    0.103    0.006    0.430    0.383    0.345   | 0.421    0.058    0.096    0.020    0.425    0.389    0.333   | 0.757  0.659  0.793  | 0.058  0.058  0.045 
+13    | 0.000270  | 0.138      | 0.164      | 0.862           | 0.737        | 0.054             | 0.338    0.052    0.098    0.006    0.428    0.381    0.342   | 0.416    0.057    0.093    0.020    0.417    0.377    0.335   | 0.759  0.666  0.792  | 0.055  0.058  0.049 
+14    | 0.000255  | 0.137      | 0.166      | 0.866           | 0.738        | 0.048             | 0.337    0.051    0.097    0.006    0.425    0.378    0.339   | 0.420    0.058    0.094    0.022    0.426    0.384    0.325   | 0.762  0.661  0.806  | 0.053  0.060  0.031 
+15    | 0.000250  | 0.136      | 0.166      | 0.863           | 0.734        | 0.051             | 0.337    0.050    0.094    0.006    0.424    0.375    0.338   | 0.416    0.059    0.097    0.022    0.422    0.390    0.320   | 0.759  0.652  0.800  | 0.058  0.055  0.039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2518  1990  1469
+FP   210   238    82
+FN    59    79    57
+TN  4509  4989  5688
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.345  0.273  0.201
+FP  0.029  0.033  0.011
+FN  0.008  0.011  0.008
+TN  0.618  0.684  0.780
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.166      | 0.863048        | 0.733518     | 0.050600          | 0.416    0.059    0.097    0.022    0.422    0.390    0.320   | 0.759  0.652  0.800  | 0.058  0.055  0.039 
+266     | 266     | 0.165      | 0.863382        | 0.736840     | 0.052258          | 0.413    0.060    0.096    0.023    0.415    0.388    0.313   | 0.757  0.659  0.808  | 0.059  0.056  0.041 
+360     | 310     | 0.167      | 0.849617        | 0.684172     | 0.040086          | 0.438    0.051    0.092    0.010    0.406    0.359    0.366   | 0.735  0.561  0.774  | 0.049  0.049  0.023 
+276     | 276     | 0.190      | 0.876007        | 0.749633     | 0.039744          | 0.465    0.072    0.118    0.026    0.645    0.520    0.406   | 0.825  0.662  0.714  | 0.044  0.047  0.029 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit-b1 
+loss_wt = 0   i.e. only BCE
+with LLRD and aux weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(3h 45m 9s)
+(Max GPU mem usage : 5708.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.342      | 0.229      | 0.684           | 0.286        | 0.051             | 0.628    0.219    0.968    0.219    0.569    0.537    0.517   | 0.549    0.092    0.339    0.092    0.561    0.570    0.459   | 0.429  0.204  0.181  | 0.056  0.054  0.041 
+2     | 0.000250  | 0.185      | 0.177      | 0.764           | 0.531        | 0.081             | 0.501    0.050    0.884    0.050    0.548    0.526    0.494   | 0.517    0.031    0.261    0.031    0.545    0.498    0.477   | 0.617  0.387  0.556  | 0.124  0.067  0.053 
+3     | 0.000375  | 0.149      | 0.159      | 0.783           | 0.560        | 0.069             | 0.436    0.026    0.769    0.026    0.503    0.474    0.437   | 0.485    0.020    0.227    0.020    0.495    0.468    0.420   | 0.619  0.427  0.626  | 0.086  0.065  0.056 
+4     | 0.000500  | 0.134      | 0.141      | 0.810           | 0.622        | 0.065             | 0.407    0.017    0.671    0.017    0.476    0.443    0.403   | 0.433    0.016    0.205    0.016    0.460    0.430    0.352   | 0.666  0.522  0.666  | 0.080  0.071  0.044 
+5     | 0.000495  | 0.124      | 0.142      | 0.816           | 0.630        | 0.061             | 0.384    0.013    0.592    0.013    0.458    0.422    0.381   | 0.446    0.011    0.195    0.011    0.423    0.383    0.361   | 0.656  0.541  0.679  | 0.068  0.063  0.051 
+6     | 0.000480  | 0.119      | 0.136      | 0.829           | 0.651        | 0.052             | 0.373    0.011    0.530    0.011    0.447    0.409    0.369   | 0.430    0.010    0.183    0.010    0.398    0.390    0.352   | 0.679  0.570  0.702  | 0.065  0.054  0.036 
+7     | 0.000457  | 0.115      | 0.135      | 0.824           | 0.666        | 0.071             | 0.364    0.009    0.480    0.009    0.439    0.399    0.360   | 0.428    0.009    0.170    0.009    0.440    0.412    0.314   | 0.703  0.587  0.702  | 0.100  0.075  0.038 
+8     | 0.000427  | 0.113      | 0.135      | 0.830           | 0.662        | 0.058             | 0.359    0.008    0.444    0.008    0.433    0.393    0.354   | 0.429    0.008    0.166    0.008    0.411    0.372    0.337   | 0.705  0.550  0.715  | 0.061  0.055  0.058 
+9     | 0.000393  | 0.111      | 0.135      | 0.834           | 0.666        | 0.054             | 0.354    0.007    0.405    0.007    0.428    0.387    0.349   | 0.431    0.008    0.164    0.008    0.404    0.370    0.322   | 0.703  0.562  0.713  | 0.064  0.050  0.047 
+10    | 0.000357  | 0.109      | 0.132      | 0.837           | 0.676        | 0.056             | 0.348    0.006    0.378    0.006    0.425    0.383    0.344   | 0.424    0.008    0.163    0.008    0.409    0.358    0.323   | 0.717  0.591  0.698  | 0.068  0.056  0.045 
+11    | 0.000323  | 0.108      | 0.135      | 0.835           | 0.682        | 0.064             | 0.346    0.006    0.358    0.006    0.422    0.380    0.342   | 0.433    0.007    0.147    0.007    0.423    0.388    0.347   | 0.715  0.607  0.711  | 0.070  0.067  0.055 
+12    | 0.000293  | 0.107      | 0.131      | 0.842           | 0.693        | 0.059             | 0.343    0.006    0.330    0.006    0.420    0.377    0.340   | 0.421    0.007    0.143    0.007    0.413    0.390    0.324   | 0.727  0.612  0.734  | 0.069  0.064  0.045 
+13    | 0.000270  | 0.106      | 0.136      | 0.838           | 0.687        | 0.061             | 0.341    0.005    0.313    0.005    0.417    0.375    0.338   | 0.435    0.007    0.149    0.007    0.397    0.362    0.338   | 0.725  0.603  0.707  | 0.067  0.058  0.059 
+14    | 0.000255  | 0.105      | 0.131      | 0.844           | 0.695        | 0.056             | 0.340    0.005    0.299    0.005    0.416    0.374    0.336   | 0.420    0.007    0.144    0.007    0.404    0.367    0.319   | 0.734  0.598  0.739  | 0.066  0.059  0.044 
+15    | 0.000250  | 0.105      | 0.133      | 0.848           | 0.703        | 0.055             | 0.338    0.005    0.285    0.005    0.414    0.372    0.335   | 0.427    0.007    0.139    0.007    0.400    0.361    0.314   | 0.731  0.623  0.741  | 0.063  0.064  0.037 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2461  1933  1412
+FP   157   175    70
+FN   116   136   114
+TN  4562  5052  5700
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.337  0.265  0.194
+FP  0.022  0.024  0.010
+FN  0.016  0.019  0.016
+TN  0.625  0.692  0.781
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.133      | 0.848333        | 0.703095     | 0.054842          | 0.427    0.007    0.139    0.007    0.400    0.361    0.314   | 0.731  0.623  0.741  | 0.063  0.064  0.037 
+266     | 266     | 0.133      | 0.848978        | 0.706371     | 0.055951          | 0.425    0.007    0.137    0.007    0.394    0.360    0.304   | 0.728  0.625  0.753  | 0.066  0.065  0.037 
+360     | 310     | 0.132      | 0.829728        | 0.646231     | 0.047941          | 0.431    0.004    0.139    0.004    0.372    0.316    0.371   | 0.717  0.561  0.681  | 0.048  0.061  0.035 
+276     | 276     | 0.144      | 0.863225        | 0.729182     | 0.047413          | 0.463    0.008    0.177    0.008    0.629    0.502    0.434   | 0.795  0.665  0.662  | 0.050  0.057  0.035 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit-b1 
+loss_wt = 1   i.e. only Dice
+with LLRD and aux weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(3h 43m 20s)
+(Max GPU mem usage : 5708.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.760      | 0.356      | 0.771           | 0.541        | 0.075             | 0.557    0.846    0.846    0.515    0.556    0.488    0.412   | 0.770    0.179    0.179    0.022    0.692    0.676    0.707   | 0.613  0.472  0.543  | 0.090  0.068  0.067 
+2     | 0.000250  | 0.385      | 0.255      | 0.836           | 0.667        | 0.052             | 0.616    0.286    0.286    0.012    0.632    0.598    0.603   | 0.558    0.126    0.126    0.016    0.619    0.506    0.535   | 0.700  0.580  0.710  | 0.057  0.055  0.043 
+3     | 0.000375  | 0.299      | 0.223      | 0.849           | 0.695        | 0.049             | 0.495    0.214    0.214    0.012    0.561    0.518    0.507   | 0.470    0.118    0.118    0.018    0.507    0.463    0.437   | 0.716  0.614  0.761  | 0.060  0.052  0.034 
+4     | 0.000500  | 0.268      | 0.210      | 0.840           | 0.704        | 0.070             | 0.446    0.191    0.191    0.013    0.520    0.481    0.454   | 0.449    0.108    0.108    0.022    0.490    0.459    0.427   | 0.734  0.629  0.752  | 0.089  0.074  0.048 
+5     | 0.000495  | 0.243      | 0.211      | 0.841           | 0.699        | 0.064             | 0.414    0.170    0.170    0.013    0.494    0.451    0.418   | 0.440    0.113    0.113    0.023    0.473    0.401    0.390   | 0.734  0.615  0.753  | 0.070  0.057  0.067 
+6     | 0.000480  | 0.231      | 0.204      | 0.853           | 0.708        | 0.050             | 0.398    0.160    0.160    0.013    0.480    0.434    0.399   | 0.431    0.108    0.108    0.025    0.444    0.427    0.386   | 0.729  0.633  0.777  | 0.060  0.061  0.029 
+7     | 0.000457  | 0.220      | 0.208      | 0.839           | 0.693        | 0.063             | 0.384    0.149    0.149    0.013    0.469    0.420    0.386   | 0.440    0.108    0.108    0.030    0.470    0.443    0.341   | 0.716  0.613  0.766  | 0.073  0.095  0.022 
+8     | 0.000427  | 0.220      | 0.200      | 0.855           | 0.717        | 0.053             | 0.380    0.151    0.151    0.015    0.459    0.412    0.377   | 0.423    0.105    0.105    0.027    0.433    0.407    0.354   | 0.741  0.645  0.758  | 0.054  0.066  0.040 
+9     | 0.000393  | 0.207      | 0.202      | 0.859           | 0.716        | 0.046             | 0.369    0.138    0.138    0.014    0.452    0.404    0.363   | 0.425    0.107    0.107    0.028    0.430    0.386    0.328   | 0.736  0.638  0.781  | 0.055  0.055  0.027 
+10    | 0.000357  | 0.200      | 0.197      | 0.856           | 0.718        | 0.052             | 0.362    0.131    0.131    0.013    0.444    0.400    0.358   | 0.420    0.101    0.101    0.030    0.456    0.392    0.351   | 0.747  0.638  0.769  | 0.071  0.056  0.030 
+11    | 0.000323  | 0.197      | 0.199      | 0.853           | 0.718        | 0.057             | 0.358    0.128    0.128    0.013    0.440    0.392    0.354   | 0.426    0.102    0.102    0.032    0.441    0.405    0.347   | 0.748  0.638  0.770  | 0.068  0.070  0.032 
+12    | 0.000293  | 0.191      | 0.196      | 0.864           | 0.726        | 0.044             | 0.353    0.122    0.122    0.013    0.435    0.388    0.349   | 0.419    0.101    0.101    0.033    0.418    0.385    0.340   | 0.745  0.651  0.791  | 0.052  0.054  0.026 
+13    | 0.000270  | 0.188      | 0.198      | 0.862           | 0.727        | 0.048             | 0.351    0.118    0.118    0.013    0.432    0.387    0.347   | 0.418    0.103    0.103    0.033    0.409    0.373    0.328   | 0.752  0.644  0.784  | 0.058  0.052  0.035 
+14    | 0.000255  | 0.189      | 0.200      | 0.857           | 0.722        | 0.054             | 0.354    0.119    0.119    0.013    0.431    0.385    0.348   | 0.424    0.104    0.104    0.035    0.431    0.409    0.344   | 0.744  0.645  0.779  | 0.060  0.065  0.036 
+15    | 0.000250  | 0.186      | 0.192      | 0.861           | 0.729        | 0.051             | 0.350    0.116    0.116    0.013    0.429    0.383    0.344   | 0.415    0.097    0.097    0.035    0.415    0.385    0.340   | 0.748  0.657  0.788  | 0.057  0.063  0.034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2508  1985  1473
+FP   230   243    86
+FN    69    84    53
+TN  4489  4984  5684
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.344  0.272  0.202
+FP  0.032  0.033  0.012
+FN  0.009  0.012  0.007
+TN  0.615  0.683  0.779
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.192      | 0.860836        | 0.729033     | 0.051296          | 0.415    0.097    0.097    0.035    0.415    0.385    0.340   | 0.748  0.657  0.788  | 0.057  0.063  0.034 
+266     | 266     | 0.192      | 0.861713        | 0.731204     | 0.051281          | 0.412    0.097    0.097    0.036    0.410    0.385    0.333   | 0.745  0.660  0.798  | 0.058  0.063  0.033 
+360     | 310     | 0.188      | 0.845783        | 0.689742     | 0.050189          | 0.435    0.082    0.082    0.015    0.388    0.336    0.377   | 0.728  0.596  0.766  | 0.058  0.067  0.026 
+276     | 276     | 0.215      | 0.867904        | 0.749246     | 0.052990          | 0.457    0.111    0.111    0.037    0.625    0.500    0.462   | 0.825  0.685  0.676  | 0.042  0.067  0.050 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit-b1 
+loss_wt = 0.133   i.e.  0.133*Dice + 0.867*BCE
+with LLRD and aux weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(3h 48m 1s)
+(Max GPU mem usage : 5708.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.405      | 0.247      | 0.727           | 0.458        | 0.093             | 0.608    0.319    0.957    0.221    0.567    0.532    0.510   | 0.538    0.123    0.316    0.093    0.566    0.547    0.448   | 0.540  0.365  0.425  | 0.135  0.056  0.089 
+2     | 0.000250  | 0.249      | 0.193      | 0.797           | 0.606        | 0.076             | 0.513    0.136    0.772    0.039    0.572    0.536    0.507   | 0.546    0.042    0.192    0.019    0.565    0.511    0.541   | 0.666  0.502  0.625  | 0.080  0.083  0.065 
+3     | 0.000375  | 0.191      | 0.164      | 0.822           | 0.656        | 0.067             | 0.464    0.075    0.482    0.012    0.535    0.503    0.481   | 0.475    0.031    0.154    0.012    0.492    0.492    0.454   | 0.702  0.554  0.684  | 0.072  0.068  0.062 
+4     | 0.000500  | 0.164      | 0.151      | 0.841           | 0.692        | 0.060             | 0.426    0.052    0.330    0.009    0.499    0.467    0.440   | 0.446    0.025    0.126    0.010    0.495    0.456    0.401   | 0.723  0.608  0.744  | 0.071  0.060  0.048 
+5     | 0.000495  | 0.147      | 0.149      | 0.843           | 0.687        | 0.053             | 0.395    0.041    0.260    0.007    0.476    0.441    0.408   | 0.431    0.027    0.131    0.012    0.446    0.399    0.368   | 0.716  0.586  0.748  | 0.065  0.054  0.039 
+6     | 0.000480  | 0.139      | 0.143      | 0.845           | 0.700        | 0.059             | 0.380    0.036    0.227    0.007    0.461    0.424    0.389   | 0.419    0.025    0.117    0.011    0.421    0.416    0.374   | 0.730  0.621  0.759  | 0.065  0.065  0.046 
+7     | 0.000457  | 0.133      | 0.147      | 0.845           | 0.699        | 0.057             | 0.369    0.032    0.201    0.006    0.452    0.412    0.374   | 0.432    0.025    0.118    0.011    0.449    0.418    0.316   | 0.730  0.625  0.730  | 0.073  0.062  0.037 
+8     | 0.000427  | 0.130      | 0.143      | 0.855           | 0.711        | 0.049             | 0.363    0.031    0.191    0.006    0.444    0.403    0.366   | 0.417    0.025    0.115    0.011    0.422    0.383    0.347   | 0.735  0.629  0.766  | 0.057  0.058  0.031 
+9     | 0.000393  | 0.126      | 0.141      | 0.857           | 0.717        | 0.050             | 0.355    0.028    0.173    0.006    0.437    0.396    0.357   | 0.413    0.024    0.111    0.010    0.424    0.387    0.336   | 0.748  0.631  0.771  | 0.058  0.058  0.033 
+10    | 0.000357  | 0.124      | 0.143      | 0.856           | 0.713        | 0.049             | 0.351    0.026    0.162    0.005    0.433    0.391    0.352   | 0.419    0.024    0.110    0.011    0.435    0.377    0.331   | 0.736  0.637  0.765  | 0.062  0.059  0.025 
+11    | 0.000323  | 0.122      | 0.144      | 0.851           | 0.714        | 0.058             | 0.347    0.025    0.155    0.005    0.429    0.386    0.349   | 0.424    0.024    0.108    0.011    0.426    0.392    0.334   | 0.739  0.639  0.767  | 0.065  0.065  0.045 
+12    | 0.000293  | 0.120      | 0.143      | 0.859           | 0.719        | 0.047             | 0.344    0.024    0.147    0.005    0.426    0.383    0.344   | 0.419    0.025    0.112    0.012    0.397    0.368    0.329   | 0.737  0.643  0.776  | 0.059  0.055  0.027 
+13    | 0.000270  | 0.119      | 0.141      | 0.859           | 0.724        | 0.051             | 0.342    0.023    0.143    0.005    0.424    0.381    0.342   | 0.413    0.024    0.108    0.011    0.406    0.367    0.330   | 0.751  0.646  0.771  | 0.065  0.055  0.031 
+14    | 0.000255  | 0.118      | 0.140      | 0.861           | 0.728        | 0.051             | 0.340    0.022    0.138    0.005    0.421    0.379    0.339   | 0.413    0.024    0.105    0.011    0.408    0.373    0.312   | 0.752  0.645  0.780  | 0.060  0.060  0.033 
+15    | 0.000250  | 0.117      | 0.140      | 0.853           | 0.716        | 0.056             | 0.339    0.022    0.134    0.005    0.419    0.375    0.338   | 0.412    0.024    0.104    0.012    0.415    0.380    0.329   | 0.740  0.642  0.765  | 0.062  0.057  0.048 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2508  1976  1472
+FP   247   241   110
+FN    69    93    54
+TN  4472  4986  5660
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.344  0.271  0.202
+FP  0.034  0.033  0.015
+FN  0.009  0.013  0.007
+TN  0.613  0.683  0.776
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.140      | 0.852966        | 0.715970     | 0.055703          | 0.412    0.024    0.104    0.012    0.415    0.380    0.329   | 0.740  0.642  0.765  | 0.062  0.057  0.048 
+266     | 266     | 0.139      | 0.853521        | 0.720544     | 0.057827          | 0.407    0.024    0.104    0.012    0.410    0.380    0.320   | 0.741  0.649  0.774  | 0.065  0.059  0.049 
+360     | 310     | 0.150      | 0.835849        | 0.646248     | 0.037751          | 0.455    0.019    0.102    0.006    0.376    0.332    0.373   | 0.661  0.528  0.749  | 0.044  0.043  0.026 
+276     | 276     | 0.155      | 0.867184        | 0.739632     | 0.047780          | 0.453    0.028    0.125    0.013    0.631    0.497    0.448   | 0.823  0.669  0.648  | 0.041  0.052  0.051 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit-b1 
+loss_wt = 0.05   i.e.  0.05*Dice + 0.95*BCE
+with LLRD and aux weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(3h 43m 52s)
+(Max GPU mem usage : 5708.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.363      | 0.233      | 0.709           | 0.370        | 0.065             | 0.621    0.252    0.963    0.215    0.572    0.540    0.519   | 0.544    0.100    0.328    0.088    0.561    0.552    0.466   | 0.494  0.293  0.282  | 0.083  0.063  0.049 
+2     | 0.000250  | 0.210      | 0.176      | 0.783           | 0.588        | 0.087             | 0.501    0.086    0.841    0.046    0.553    0.528    0.496   | 0.504    0.036    0.230    0.026    0.545    0.499    0.487   | 0.648  0.480  0.617  | 0.118  0.084  0.060 
+3     | 0.000375  | 0.169      | 0.157      | 0.801           | 0.617        | 0.076             | 0.442    0.052    0.659    0.020    0.515    0.482    0.449   | 0.465    0.024    0.191    0.015    0.489    0.449    0.441   | 0.657  0.509  0.665  | 0.093  0.066  0.067 
+4     | 0.000500  | 0.149      | 0.146      | 0.824           | 0.661        | 0.068             | 0.413    0.036    0.501    0.012    0.487    0.453    0.421   | 0.448    0.017    0.159    0.010    0.474    0.446    0.367   | 0.697  0.577  0.688  | 0.096  0.073  0.034 
+5     | 0.000495  | 0.136      | 0.143      | 0.834           | 0.673        | 0.059             | 0.389    0.027    0.387    0.009    0.468    0.432    0.399   | 0.439    0.017    0.149    0.010    0.447    0.397    0.368   | 0.705  0.581  0.720  | 0.072  0.059  0.044 
+6     | 0.000480  | 0.130      | 0.139      | 0.842           | 0.688        | 0.055             | 0.378    0.023    0.325    0.007    0.456    0.418    0.383   | 0.426    0.016    0.139    0.009    0.420    0.393    0.365   | 0.714  0.608  0.739  | 0.061  0.064  0.040 
+7     | 0.000457  | 0.124      | 0.136      | 0.840           | 0.693        | 0.063             | 0.367    0.020    0.280    0.006    0.447    0.407    0.372   | 0.418    0.015    0.127    0.009    0.429    0.412    0.339   | 0.725  0.613  0.746  | 0.078  0.073  0.038 
+8     | 0.000427  | 0.121      | 0.136      | 0.847           | 0.699        | 0.055             | 0.360    0.018    0.254    0.006    0.440    0.399    0.363   | 0.418    0.014    0.126    0.009    0.411    0.381    0.349   | 0.724  0.621  0.757  | 0.066  0.061  0.039 
+9     | 0.000393  | 0.118      | 0.138      | 0.845           | 0.695        | 0.056             | 0.353    0.017    0.228    0.006    0.434    0.393    0.356   | 0.425    0.015    0.125    0.009    0.408    0.377    0.343   | 0.721  0.614  0.751  | 0.068  0.058  0.041 
+10    | 0.000357  | 0.116      | 0.133      | 0.848           | 0.707        | 0.057             | 0.350    0.016    0.213    0.005    0.430    0.389    0.351   | 0.411    0.014    0.125    0.008    0.404    0.353    0.333   | 0.734  0.632  0.751  | 0.071  0.060  0.042 
+11    | 0.000323  | 0.114      | 0.138      | 0.845           | 0.703        | 0.060             | 0.346    0.015    0.198    0.005    0.427    0.384    0.347   | 0.425    0.015    0.119    0.009    0.424    0.385    0.328   | 0.730  0.627  0.749  | 0.065  0.064  0.050 
+12    | 0.000293  | 0.112      | 0.135      | 0.854           | 0.713        | 0.053             | 0.343    0.014    0.185    0.005    0.424    0.381    0.343   | 0.415    0.015    0.119    0.009    0.393    0.369    0.330   | 0.739  0.633  0.756  | 0.058  0.057  0.043 
+13    | 0.000270  | 0.112      | 0.140      | 0.851           | 0.705        | 0.053             | 0.342    0.013    0.179    0.005    0.421    0.379    0.341   | 0.432    0.015    0.119    0.010    0.407    0.357    0.331   | 0.736  0.616  0.748  | 0.062  0.055  0.041 
+14    | 0.000255  | 0.111      | 0.137      | 0.851           | 0.708        | 0.053             | 0.341    0.013    0.172    0.004    0.419    0.377    0.339   | 0.423    0.015    0.120    0.009    0.395    0.367    0.303   | 0.734  0.621  0.765  | 0.060  0.061  0.039 
+15    | 0.000250  | 0.110      | 0.137      | 0.854           | 0.711        | 0.050             | 0.337    0.012    0.164    0.004    0.417    0.374    0.337   | 0.422    0.015    0.113    0.009    0.407    0.363    0.323   | 0.735  0.633  0.770  | 0.063  0.052  0.034 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2448  1916  1450
+FP   161   173    80
+FN   129   153    76
+TN  4558  5054  5690
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.336  0.263  0.199
+FP  0.022  0.024  0.011
+FN  0.018  0.021  0.010
+TN  0.625  0.693  0.780
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.137      | 0.854365        | 0.710977     | 0.050043          | 0.422    0.015    0.113    0.009    0.407    0.363    0.323   | 0.735  0.633  0.770  | 0.063  0.052  0.034 
+266     | 266     | 0.137      | 0.854203        | 0.713052     | 0.051696          | 0.421    0.015    0.113    0.010    0.401    0.360    0.314   | 0.732  0.636  0.777  | 0.066  0.053  0.036 
+360     | 310     | 0.137      | 0.840701        | 0.662977     | 0.040815          | 0.436    0.010    0.102    0.005    0.392    0.331    0.380   | 0.710  0.552  0.752  | 0.054  0.047  0.022 
+276     | 276     | 0.138      | 0.876183        | 0.746781     | 0.037549          | 0.421    0.016    0.131    0.010    0.625    0.512    0.422   | 0.806  0.684  0.697  | 0.037  0.050  0.025 </t>
+  </si>
 </sst>
 </file>
 
@@ -4751,7 +5046,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -4787,22 +5082,26 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Courier New"/>
-      <family val="3"/>
+      <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFA6"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -4845,7 +5144,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4938,7 +5237,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4950,48 +5249,16 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -5040,7 +5307,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFFFA6"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -5177,7 +5444,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K384"/>
+  <dimension ref="A1:K429"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50.36"/>
@@ -7083,7 +7350,7 @@
       <c r="A195" s="11"/>
     </row>
     <row r="196" customFormat="false" ht="605.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A196" s="10" t="s">
+      <c r="A196" s="23" t="s">
         <v>170</v>
       </c>
       <c r="B196" s="2" t="n">
@@ -7496,7 +7763,7 @@
       <c r="A251" s="11"/>
     </row>
     <row r="252" customFormat="false" ht="191.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A252" s="23" t="s">
+      <c r="A252" s="24" t="s">
         <v>226</v>
       </c>
       <c r="B252" s="2" t="n">
@@ -7513,7 +7780,7 @@
       </c>
     </row>
     <row r="253" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A253" s="23"/>
+      <c r="A253" s="24"/>
       <c r="E253" s="12" t="s">
         <v>228</v>
       </c>
@@ -7672,7 +7939,7 @@
       <c r="C270" s="2" t="n">
         <v>0.86495</v>
       </c>
-      <c r="D270" s="26" t="n">
+      <c r="D270" s="2" t="n">
         <v>0.8611</v>
       </c>
       <c r="E270" s="12" t="s">
@@ -7962,7 +8229,7 @@
       <c r="A299" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="C299" s="26" t="n">
+      <c r="C299" s="2" t="n">
         <v>0.86615</v>
       </c>
       <c r="D299" s="2" t="n">
@@ -8183,8 +8450,8 @@
       <c r="A338" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="B338" s="2" t="n">
-        <v>0.862</v>
+      <c r="B338" s="26" t="s">
+        <v>285</v>
       </c>
       <c r="C338" s="2" t="n">
         <v>0.8538</v>
@@ -8193,12 +8460,12 @@
         <v>0.84127</v>
       </c>
       <c r="E338" s="12" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="339" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E339" s="12" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8216,8 +8483,8 @@
       <c r="A341" s="17"/>
     </row>
     <row r="343" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A343" s="27" t="s">
-        <v>287</v>
+      <c r="A343" s="8" t="s">
+        <v>288</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>0.861</v>
@@ -8229,12 +8496,12 @@
         <v>0.84327</v>
       </c>
       <c r="E343" s="12" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="344" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E344" s="12" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8252,10 +8519,10 @@
       </c>
     </row>
     <row r="346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A346" s="28" t="s">
+      <c r="A346" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="C346" s="26" t="n">
+      <c r="C346" s="2" t="n">
         <v>0.86199</v>
       </c>
       <c r="D346" s="2" t="n">
@@ -8275,7 +8542,7 @@
     </row>
     <row r="349" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A349" s="8" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>0.863</v>
@@ -8287,12 +8554,12 @@
         <v>0.84315</v>
       </c>
       <c r="E349" s="12" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="350" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E350" s="12" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8308,7 +8575,7 @@
     </row>
     <row r="353" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A353" s="8" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>0.861</v>
@@ -8320,12 +8587,12 @@
         <v>0.85141</v>
       </c>
       <c r="E353" s="12" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="354" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E354" s="12" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8366,7 +8633,7 @@
     </row>
     <row r="361" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="8" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>0.861</v>
@@ -8378,12 +8645,12 @@
         <v>0.83826</v>
       </c>
       <c r="E361" s="12" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="362" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E362" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8424,7 +8691,7 @@
     </row>
     <row r="367" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="8" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>0.863</v>
@@ -8436,12 +8703,12 @@
         <v>0.84412</v>
       </c>
       <c r="E367" s="12" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="368" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E368" s="12" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8471,7 +8738,7 @@
     </row>
     <row r="371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="17" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C371" s="2" t="n">
         <v>0.85918</v>
@@ -8482,7 +8749,7 @@
     </row>
     <row r="373" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="8" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>0.864</v>
@@ -8494,12 +8761,12 @@
         <v>0.83975</v>
       </c>
       <c r="E373" s="12" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="374" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E374" s="12" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8513,9 +8780,9 @@
         <v>0.84867</v>
       </c>
     </row>
-    <row r="377" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A377" s="29" t="s">
-        <v>306</v>
+    <row r="377" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A377" s="8" t="s">
+        <v>307</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>0.865</v>
@@ -8526,13 +8793,13 @@
       <c r="D377" s="2" t="n">
         <v>0.8534</v>
       </c>
-      <c r="E377" s="30" t="s">
-        <v>307</v>
+      <c r="E377" s="12" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="378" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E378" s="30" t="s">
-        <v>308</v>
+      <c r="E378" s="12" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8549,24 +8816,22 @@
         <v>0.85661</v>
       </c>
     </row>
-    <row r="380" s="34" customFormat="true" ht="337.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A380" s="28" t="s">
+    <row r="380" s="3" customFormat="true" ht="337.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A380" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="B380" s="31" t="n">
+      <c r="B380" s="14" t="n">
         <v>0.870575</v>
       </c>
-      <c r="C380" s="26" t="n">
+      <c r="C380" s="2" t="n">
         <v>0.86571</v>
       </c>
-      <c r="D380" s="26" t="n">
+      <c r="D380" s="2" t="n">
         <v>0.86091</v>
       </c>
-      <c r="E380" s="32" t="s">
-        <v>309</v>
-      </c>
-      <c r="F380" s="33"/>
-      <c r="G380" s="33"/>
+      <c r="E380" s="12" t="s">
+        <v>310</v>
+      </c>
     </row>
     <row r="381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="17" t="s">
@@ -8581,9 +8846,9 @@
     </row>
     <row r="382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A382" s="17" t="s">
-        <v>310</v>
-      </c>
-      <c r="B382" s="35" t="n">
+        <v>311</v>
+      </c>
+      <c r="B382" s="14" t="n">
         <v>0.872343</v>
       </c>
       <c r="C382" s="2" t="n">
@@ -8595,12 +8860,12 @@
     </row>
     <row r="383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A383" s="17" t="s">
-        <v>311</v>
-      </c>
-      <c r="B383" s="35" t="n">
+        <v>312</v>
+      </c>
+      <c r="B383" s="14" t="n">
         <v>0.871923</v>
       </c>
-      <c r="C383" s="36" t="n">
+      <c r="C383" s="2" t="n">
         <v>0.86619</v>
       </c>
       <c r="D383" s="2" t="n">
@@ -8609,23 +8874,419 @@
     </row>
     <row r="384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A384" s="17" t="s">
-        <v>312</v>
-      </c>
-      <c r="B384" s="35" t="n">
+        <v>313</v>
+      </c>
+      <c r="B384" s="14" t="n">
         <v>0.871967</v>
       </c>
       <c r="C384" s="2" t="n">
         <v>0.86606</v>
       </c>
-      <c r="D384" s="36" t="n">
+      <c r="D384" s="2" t="n">
         <v>0.86181</v>
       </c>
+    </row>
+    <row r="386" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A386" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="E386" s="12" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="387" customFormat="false" ht="15.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A387" s="17" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A388" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="C388" s="2" t="n">
+        <v>0.84964</v>
+      </c>
+      <c r="D388" s="2" t="n">
+        <v>0.8447</v>
+      </c>
+    </row>
+    <row r="389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A389" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="C389" s="2" t="n">
+        <v>0.86978</v>
+      </c>
+      <c r="D389" s="2" t="n">
+        <v>0.8628</v>
+      </c>
+    </row>
+    <row r="390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A390" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="C390" s="2" t="n">
+        <v>0.85554</v>
+      </c>
+      <c r="D390" s="2" t="n">
+        <v>0.84827</v>
+      </c>
+    </row>
+    <row r="391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A391" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="C391" s="2" t="n">
+        <v>0.87148</v>
+      </c>
+      <c r="D391" s="2" t="n">
+        <v>0.86193</v>
+      </c>
+    </row>
+    <row r="392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A392" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="C392" s="2" t="n">
+        <v>0.85869</v>
+      </c>
+      <c r="D392" s="2" t="n">
+        <v>0.84887</v>
+      </c>
+    </row>
+    <row r="393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A393" s="18" t="s">
+        <v>319</v>
+      </c>
+      <c r="C393" s="2" t="n">
+        <v>0.87088</v>
+      </c>
+      <c r="D393" s="2" t="n">
+        <v>0.8613</v>
+      </c>
+    </row>
+    <row r="394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A394" s="17" t="s">
+        <v>320</v>
+      </c>
+      <c r="C394" s="2" t="n">
+        <v>0.8716</v>
+      </c>
+      <c r="D394" s="2" t="n">
+        <v>0.86209</v>
+      </c>
+    </row>
+    <row r="395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A395" s="17" t="s">
+        <v>321</v>
+      </c>
+      <c r="C395" s="27" t="n">
+        <v>0.87178</v>
+      </c>
+      <c r="D395" s="2" t="n">
+        <v>0.86248</v>
+      </c>
+    </row>
+    <row r="396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A396" s="17" t="s">
+        <v>322</v>
+      </c>
+      <c r="C396" s="2" t="n">
+        <v>0.8716</v>
+      </c>
+      <c r="D396" s="2" t="n">
+        <v>0.86241</v>
+      </c>
+    </row>
+    <row r="397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A397" s="17" t="s">
+        <v>323</v>
+      </c>
+      <c r="C397" s="2" t="n">
+        <v>0.8712</v>
+      </c>
+      <c r="D397" s="2" t="n">
+        <v>0.8622</v>
+      </c>
+    </row>
+    <row r="398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A398" s="17" t="s">
+        <v>324</v>
+      </c>
+      <c r="C398" s="2" t="n">
+        <v>0.8709</v>
+      </c>
+      <c r="D398" s="2" t="n">
+        <v>0.86205</v>
+      </c>
+    </row>
+    <row r="399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A399" s="17" t="s">
+        <v>325</v>
+      </c>
+      <c r="C399" s="2" t="n">
+        <v>0.87077</v>
+      </c>
+      <c r="D399" s="2" t="n">
+        <v>0.86195</v>
+      </c>
+    </row>
+    <row r="401" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A401" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="B401" s="2" t="n">
+        <v>0.863</v>
+      </c>
+      <c r="C401" s="2" t="n">
+        <v>0.8567</v>
+      </c>
+      <c r="D401" s="2" t="n">
+        <v>0.84883</v>
+      </c>
+      <c r="E401" s="12" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="402" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E402" s="12" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A403" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="B403" s="2" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="C403" s="2" t="n">
+        <v>0.85851</v>
+      </c>
+      <c r="D403" s="2" t="n">
+        <v>0.84615</v>
+      </c>
+    </row>
+    <row r="404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A404" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C404" s="2" t="n">
+        <v>0.86671</v>
+      </c>
+      <c r="D404" s="2" t="n">
+        <v>0.85281</v>
+      </c>
+    </row>
+    <row r="405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A405" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="C405" s="2" t="n">
+        <v>0.86519</v>
+      </c>
+      <c r="D405" s="2" t="n">
+        <v>0.85489</v>
+      </c>
+    </row>
+    <row r="407" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A407" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="B407" s="2" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="C407" s="2" t="n">
+        <v>0.83415</v>
+      </c>
+      <c r="D407" s="2" t="n">
+        <v>0.82301</v>
+      </c>
+      <c r="E407" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="408" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A408" s="28"/>
+      <c r="E408" s="12" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A409" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C409" s="2" t="n">
+        <v>0.84304</v>
+      </c>
+      <c r="D409" s="2" t="n">
+        <v>0.83211</v>
+      </c>
+    </row>
+    <row r="412" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A412" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="B412" s="2" t="n">
+        <v>0.861</v>
+      </c>
+      <c r="C412" s="2" t="n">
+        <v>0.85819</v>
+      </c>
+      <c r="D412" s="2" t="n">
+        <v>0.84705</v>
+      </c>
+      <c r="E412" s="12" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="413" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A413" s="3"/>
+      <c r="B413" s="3"/>
+      <c r="E413" s="12" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A414" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="B414" s="2" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="C414" s="2" t="n">
+        <v>0.84966</v>
+      </c>
+      <c r="D414" s="2" t="n">
+        <v>0.83805</v>
+      </c>
+    </row>
+    <row r="415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A415" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C415" s="2" t="n">
+        <v>0.8597</v>
+      </c>
+      <c r="D415" s="2" t="n">
+        <v>0.85049</v>
+      </c>
+    </row>
+    <row r="416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A416" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="C416" s="2" t="n">
+        <v>0.85944</v>
+      </c>
+      <c r="D416" s="2" t="n">
+        <v>0.84941</v>
+      </c>
+    </row>
+    <row r="418" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A418" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="B418" s="2" t="n">
+        <v>0.853</v>
+      </c>
+      <c r="C418" s="2" t="n">
+        <v>0.85212</v>
+      </c>
+      <c r="D418" s="2" t="n">
+        <v>0.84279</v>
+      </c>
+      <c r="E418" s="12" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="419" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A419" s="3"/>
+      <c r="B419" s="3"/>
+      <c r="E419" s="12" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A420" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B420" s="2" t="n">
+        <v>0.861</v>
+      </c>
+      <c r="C420" s="2" t="n">
+        <v>0.84972</v>
+      </c>
+      <c r="D420" s="2" t="n">
+        <v>0.84318</v>
+      </c>
+    </row>
+    <row r="421" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A421" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C421" s="2" t="n">
+        <v>0.85681</v>
+      </c>
+      <c r="D421" s="2" t="n">
+        <v>0.84815</v>
+      </c>
+    </row>
+    <row r="422" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A422" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C422" s="2" t="n">
+        <v>0.85625</v>
+      </c>
+      <c r="D422" s="2" t="n">
+        <v>0.84815</v>
+      </c>
+    </row>
+    <row r="424" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A424" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="B424" s="2" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="C424" s="2" t="n">
+        <v>0.84565</v>
+      </c>
+      <c r="D424" s="2" t="n">
+        <v>0.83331</v>
+      </c>
+      <c r="E424" s="12" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="425" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E425" s="12" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A426" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C426" s="2" t="n">
+        <v>0.85576</v>
+      </c>
+      <c r="D426" s="2" t="n">
+        <v>0.84338</v>
+      </c>
+    </row>
+    <row r="429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A429" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A252:A253"/>
     <mergeCell ref="A256:A257"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A196" r:id="rId1" display="15 epoch from stable best model config&#10;&#10;(15 epoch &amp; final_lr to 2.5e-4 changed from&#10;warmup&amp;cosdec,0.1LR pres,DL Lo(.5),.25PLo+.75SLo)&#10;&#10;Segformer with mit_b1 encoder &#10;with presence head with dropout 0.4&#10;&#10;per class seg loss : &#10;dice * 0.5 +  bce * 0.5&#10;&#10;total_loss = 0.25 * presence_loss + 0.75 * seg_loss&#10;(seg_loss is presence gated avg of &#10;per class seg loss)&#10;presence_gate = &#10;       Presence_true.mean(dim=0) + 1e-3&#10;&#10;Presence loss pos_weight = [60/40, 70/30, 75/25]&#10;&#10;On padded images&#10;With AdamW optim &#10;1e-6 weight decay for presence head&#10;1e-4 weight_decay for other params except &#10;                               bias &amp; norm&#10;&#10;On 384x384 images with &#10;LR 1.25e-4, 2.5e-4, 5e-4, cos decay to 2.5e-4 for 15 epochs&#10;LR*0.1 for presence head&#10;(used LOAD_RESIZED = False)&#10;with grad_accu = 2, BS = 32    &#10;BS = 32 (train/valid/test)&#10;&#10;(3h 44m 18s)  &#10;(Max GPU mem usage : 10716.875 MB)   &#10;&#10;https://www.kaggle.com/code/abhivij/gi-tract-image-segmentation?scriptVersionId=278667321 "/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
exploring UNet, hausdorff surrogate loss
</commit_message>
<xml_diff>
--- a/Scores.xlsx
+++ b/Scores.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="426">
   <si>
     <t xml:space="preserve">Description</t>
   </si>
@@ -5038,6 +5038,1524 @@
 360     | 310     | 0.137      | 0.840701        | 0.662977     | 0.040815          | 0.436    0.010    0.102    0.005    0.392    0.331    0.380   | 0.710  0.552  0.752  | 0.054  0.047  0.022 
 276     | 276     | 0.138      | 0.876183        | 0.746781     | 0.037549          | 0.421    0.016    0.131    0.010    0.625    0.512    0.422   | 0.806  0.684  0.697  | 0.037  0.050  0.025 </t>
   </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 9m 24s)
+(Max GPU mem usage : 6602.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.659      | 0.358      | 0.698           | 0.424        | 0.120             | 0.547    0.707    0.977    0.437    0.474    0.456    0.410   | 0.515    0.290    0.331    0.249    0.538    0.497    0.403   | 0.469  0.343  0.491  | 0.111  0.109  0.138 
+2     | 0.000250  | 0.442      | 0.267      | 0.797           | 0.619        | 0.085             | 0.639    0.357    0.648    0.067    0.651    0.604    0.557   | 0.718    0.074    0.134    0.015    0.636    0.630    0.686   | 0.661  0.526  0.716  | 0.086  0.109  0.059 
+3     | 0.000375  | 0.257      | 0.202      | 0.841           | 0.700        | 0.065             | 0.565    0.125    0.240    0.011    0.573    0.555    0.570   | 0.519    0.066    0.116    0.015    0.526    0.479    0.546   | 0.728  0.622  0.751  | 0.066  0.083  0.044 
+4     | 0.000500  | 0.213      | 0.202      | 0.827           | 0.667        | 0.066             | 0.479    0.099    0.187    0.011    0.521    0.493    0.488   | 0.526    0.064    0.109    0.018    0.534    0.530    0.493   | 0.707  0.577  0.755  | 0.072  0.075  0.052 
+5     | 0.000495  | 0.192      | 0.183      | 0.842           | 0.702        | 0.065             | 0.440    0.086    0.162    0.010    0.493    0.460    0.447   | 0.461    0.064    0.108    0.019    0.518    0.452    0.414   | 0.724  0.631  0.767  | 0.068  0.092  0.035 
+6     | 0.000480  | 0.180      | 0.179      | 0.854           | 0.719        | 0.055             | 0.416    0.078    0.147    0.010    0.475    0.441    0.422   | 0.457    0.060    0.102    0.017    0.489    0.431    0.426   | 0.746  0.644  0.771  | 0.063  0.064  0.040 
+7     | 0.000457  | 0.169      | 0.178      | 0.851           | 0.714        | 0.058             | 0.399    0.071    0.133    0.009    0.462    0.425    0.402   | 0.452    0.060    0.101    0.018    0.468    0.433    0.377   | 0.741  0.641  0.770  | 0.076  0.070  0.028 
+8     | 0.000427  | 0.164      | 0.174      | 0.853           | 0.710        | 0.051             | 0.391    0.067    0.126    0.008    0.454    0.415    0.391   | 0.442    0.059    0.100    0.019    0.472    0.460    0.368   | 0.738  0.633  0.780  | 0.065  0.067  0.022 
+9     | 0.000393  | 0.159      | 0.174      | 0.854           | 0.711        | 0.051             | 0.381    0.064    0.121    0.008    0.446    0.407    0.380   | 0.430    0.064    0.109    0.019    0.410    0.391    0.362   | 0.733  0.634  0.774  | 0.065  0.063  0.026 
+10    | 0.000357  | 0.156      | 0.175      | 0.849           | 0.706        | 0.056             | 0.377    0.061    0.115    0.008    0.442    0.402    0.373   | 0.431    0.066    0.110    0.021    0.416    0.392    0.370   | 0.722  0.641  0.767  | 0.048  0.091  0.030 
+11    | 0.000323  | 0.154      | 0.171      | 0.855           | 0.721        | 0.056             | 0.374    0.059    0.111    0.007    0.437    0.397    0.369   | 0.430    0.060    0.101    0.020    0.425    0.392    0.350   | 0.739  0.642  0.788  | 0.063  0.072  0.033 
+12    | 0.000293  | 0.149      | 0.171      | 0.853           | 0.720        | 0.059             | 0.366    0.056    0.106    0.007    0.433    0.392    0.362   | 0.432    0.059    0.099    0.020    0.436    0.393    0.359   | 0.738  0.645  0.789  | 0.070  0.081  0.025 
+13    | 0.000270  | 0.147      | 0.172      | 0.861           | 0.727        | 0.050             | 0.364    0.054    0.102    0.007    0.430    0.389    0.359   | 0.435    0.060    0.099    0.021    0.435    0.378    0.346   | 0.745  0.644  0.797  | 0.060  0.064  0.026 
+14    | 0.000255  | 0.146      | 0.175      | 0.845           | 0.702        | 0.060             | 0.363    0.054    0.101    0.006    0.428    0.388    0.356   | 0.444    0.060    0.100    0.021    0.449    0.412    0.335   | 0.725  0.624  0.786  | 0.067  0.075  0.038 
+15    | 0.000250  | 0.144      | 0.172      | 0.858           | 0.728        | 0.056             | 0.360    0.051    0.096    0.006    0.425    0.383    0.354   | 0.433    0.060    0.100    0.021    0.430    0.392    0.328   | 0.746  0.646  0.796  | 0.071  0.064  0.033 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2485  1940  1456
+FP   217   214    65
+FN    92   129    70
+TN  4502  5013  5705
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.341  0.266  0.200
+FP  0.030  0.029  0.009
+FN  0.013  0.018  0.010
+TN  0.617  0.687  0.782
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.172      | 0.857503        | 0.727909     | 0.056101          | 0.433    0.060    0.100    0.021    0.430    0.392    0.328   | 0.746  0.646  0.796  | 0.071  0.064  0.033 
+266     | 266     | 0.171      | 0.858513        | 0.732037     | 0.057170          | 0.430    0.061    0.100    0.021    0.424    0.390    0.320   | 0.746  0.653  0.805  | 0.073  0.064  0.034 
+360     | 310     | 0.179      | 0.832435        | 0.663612     | 0.055016          | 0.470    0.055    0.098    0.011    0.416    0.369    0.372   | 0.697  0.532  0.762  | 0.069  0.073  0.023 
+276     | 276     | 0.185      | 0.876763        | 0.754168     | 0.041507          | 0.450    0.071    0.114    0.027    0.639    0.518    0.430   | 0.815  0.671  0.730  | 0.046  0.050  0.028 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,5e-5
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 8m 12s)
+(Max GPU mem usage : 6602.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.659      | 0.357      | 0.693           | 0.412        | 0.120             | 0.548    0.707    0.977    0.437    0.475    0.456    0.410   | 0.523    0.286    0.330    0.242    0.525    0.519    0.419   | 0.437  0.337  0.494  | 0.114  0.113  0.133 
+2     | 0.000250  | 0.442      | 0.256      | 0.801           | 0.623        | 0.080             | 0.641    0.357    0.646    0.067    0.651    0.604    0.558   | 0.671    0.078    0.139    0.016    0.609    0.586    0.675   | 0.668  0.545  0.675  | 0.104  0.073  0.063 
+3     | 0.000375  | 0.256      | 0.205      | 0.837           | 0.689        | 0.064             | 0.564    0.124    0.237    0.011    0.572    0.555    0.570   | 0.526    0.068    0.119    0.016    0.528    0.507    0.538   | 0.721  0.600  0.733  | 0.067  0.078  0.048 
+4     | 0.000500  | 0.215      | 0.190      | 0.847           | 0.693        | 0.051             | 0.481    0.101    0.190    0.011    0.521    0.493    0.488   | 0.483    0.064    0.110    0.017    0.527    0.491    0.434   | 0.722  0.617  0.760  | 0.058  0.068  0.028 
+5     | 0.000491  | 0.191      | 0.180      | 0.848           | 0.711        | 0.061             | 0.437    0.086    0.162    0.010    0.491    0.458    0.446   | 0.458    0.061    0.104    0.018    0.483    0.468    0.416   | 0.740  0.635  0.774  | 0.068  0.068  0.048 
+6     | 0.000464  | 0.181      | 0.181      | 0.850           | 0.715        | 0.060             | 0.419    0.079    0.148    0.010    0.475    0.440    0.422   | 0.459    0.062    0.107    0.017    0.471    0.419    0.428   | 0.742  0.634  0.782  | 0.082  0.069  0.029 
+7     | 0.000422  | 0.170      | 0.175      | 0.854           | 0.715        | 0.054             | 0.400    0.072    0.134    0.009    0.462    0.425    0.403   | 0.447    0.059    0.100    0.018    0.466    0.423    0.362   | 0.737  0.636  0.786  | 0.075  0.055  0.031 
+8     | 0.000368  | 0.162      | 0.179      | 0.852           | 0.708        | 0.052             | 0.387    0.066    0.124    0.008    0.454    0.415    0.392   | 0.445    0.065    0.110    0.019    0.450    0.422    0.360   | 0.724  0.633  0.772  | 0.064  0.068  0.023 
+9     | 0.000307  | 0.157      | 0.170      | 0.857           | 0.724        | 0.055             | 0.379    0.062    0.116    0.008    0.447    0.407    0.382   | 0.426    0.061    0.103    0.018    0.428    0.395    0.367   | 0.742  0.652  0.789  | 0.064  0.070  0.030 
+10    | 0.000243  | 0.152      | 0.176      | 0.845           | 0.699        | 0.058             | 0.372    0.058    0.109    0.007    0.443    0.403    0.375   | 0.446    0.061    0.102    0.019    0.456    0.413    0.366   | 0.718  0.624  0.775  | 0.071  0.072  0.030 
+11    | 0.000182  | 0.149      | 0.169      | 0.856           | 0.723        | 0.056             | 0.368    0.055    0.104    0.007    0.439    0.398    0.369   | 0.425    0.059    0.099    0.020    0.432    0.386    0.355   | 0.744  0.648  0.785  | 0.079  0.058  0.030 
+12    | 0.000128  | 0.145      | 0.173      | 0.861           | 0.725        | 0.048             | 0.362    0.052    0.099    0.006    0.436    0.393    0.366   | 0.432    0.062    0.104    0.020    0.419    0.367    0.350   | 0.743  0.649  0.785  | 0.063  0.057  0.024 
+13    | 0.000086  | 0.144      | 0.171      | 0.862           | 0.725        | 0.047             | 0.360    0.051    0.096    0.006    0.434    0.391    0.362   | 0.427    0.062    0.104    0.020    0.411    0.367    0.339   | 0.738  0.645  0.794  | 0.062  0.051  0.028 
+14    | 0.000059  | 0.142      | 0.173      | 0.855           | 0.723        | 0.057             | 0.357    0.050    0.094    0.006    0.433    0.390    0.360   | 0.437    0.059    0.098    0.020    0.434    0.399    0.335   | 0.740  0.643  0.796  | 0.074  0.067  0.029 
+15    | 0.000050  | 0.141      | 0.172      | 0.861           | 0.731        | 0.052             | 0.355    0.049    0.092    0.006    0.431    0.388    0.359   | 0.437    0.058    0.097    0.020    0.439    0.393    0.333   | 0.750  0.651  0.797  | 0.072  0.060  0.023 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2503  1941  1436
+FP   208   208    61
+FN    74   128    90
+TN  4511  5019  5709
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.343  0.266  0.197
+FP  0.029  0.029  0.008
+FN  0.010  0.018  0.012
+TN  0.618  0.688  0.782
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.172      | 0.861489        | 0.731293     | 0.051713          | 0.437    0.058    0.097    0.020    0.439    0.393    0.333   | 0.750  0.651  0.797  | 0.072  0.060  0.023 
+266     | 266     | 0.170      | 0.862821        | 0.736271     | 0.052812          | 0.431    0.058    0.097    0.020    0.434    0.392    0.326   | 0.751  0.657  0.808  | 0.075  0.061  0.022 
+360     | 310     | 0.181      | 0.837030        | 0.669130     | 0.051037          | 0.478    0.053    0.097    0.010    0.405    0.356    0.366   | 0.703  0.552  0.751  | 0.064  0.063  0.026 
+276     | 276     | 0.201      | 0.873463        | 0.737848     | 0.036127          | 0.501    0.072    0.119    0.025    0.652    0.526    0.445   | 0.798  0.666  0.699  | 0.039  0.040  0.030 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 9m 33s)
+(Max GPU mem usage : 6602.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.571      | 0.276      | 0.698           | 0.459        | 0.143             | 0.522    0.592    0.940    0.243    0.420    0.396    0.369   | 0.483    0.187    0.310    0.065    0.391    0.371    0.268   | 0.508  0.392  0.469  | 0.111  0.118  0.199 
+2     | 0.000250  | 0.283      | 0.185      | 0.830           | 0.667        | 0.060             | 0.432    0.219    0.421    0.018    0.414    0.383    0.349   | 0.456    0.069    0.124    0.014    0.383    0.347    0.287   | 0.695  0.593  0.721  | 0.082  0.073  0.026 
+3     | 0.000375  | 0.194      | 0.175      | 0.847           | 0.701        | 0.056             | 0.415    0.099    0.189    0.010    0.413    0.381    0.345   | 0.439    0.062    0.109    0.014    0.385    0.392    0.300   | 0.727  0.622  0.765  | 0.071  0.062  0.035 
+4     | 0.000500  | 0.181      | 0.172      | 0.849           | 0.705        | 0.054             | 0.403    0.085    0.162    0.009    0.412    0.379    0.343   | 0.437    0.059    0.103    0.015    0.412    0.360    0.320   | 0.734  0.627  0.769  | 0.066  0.062  0.036 
+5     | 0.000495  | 0.171      | 0.174      | 0.850           | 0.698        | 0.048             | 0.392    0.077    0.145    0.009    0.411    0.377    0.340   | 0.431    0.064    0.112    0.016    0.395    0.344    0.305   | 0.717  0.632  0.748  | 0.060  0.056  0.028 
+6     | 0.000480  | 0.165      | 0.172      | 0.853           | 0.713        | 0.053             | 0.385    0.071    0.133    0.008    0.410    0.376    0.339   | 0.432    0.060    0.104    0.015    0.385    0.343    0.332   | 0.739  0.642  0.767  | 0.060  0.064  0.036 
+7     | 0.000457  | 0.162      | 0.173      | 0.856           | 0.716        | 0.051             | 0.381    0.068    0.128    0.008    0.410    0.376    0.338   | 0.437    0.059    0.102    0.016    0.407    0.376    0.308   | 0.741  0.650  0.758  | 0.063  0.060  0.028 
+8     | 0.000427  | 0.155      | 0.169      | 0.853           | 0.709        | 0.051             | 0.372    0.063    0.118    0.007    0.409    0.373    0.338   | 0.424    0.060    0.104    0.017    0.401    0.398    0.309   | 0.738  0.646  0.755  | 0.069  0.054  0.031 
+9     | 0.000393  | 0.153      | 0.169      | 0.855           | 0.716        | 0.053             | 0.369    0.060    0.113    0.007    0.409    0.372    0.337   | 0.426    0.059    0.101    0.017    0.383    0.359    0.300   | 0.742  0.644  0.773  | 0.064  0.058  0.035 
+10    | 0.000357  | 0.151      | 0.173      | 0.853           | 0.711        | 0.052             | 0.368    0.058    0.109    0.006    0.409    0.373    0.337   | 0.439    0.059    0.101    0.016    0.396    0.385    0.306   | 0.732  0.638  0.781  | 0.060  0.064  0.034 
+11    | 0.000323  | 0.148      | 0.170      | 0.854           | 0.720        | 0.057             | 0.365    0.055    0.104    0.006    0.408    0.371    0.337   | 0.434    0.057    0.098    0.016    0.386    0.367    0.307   | 0.739  0.656  0.785  | 0.064  0.067  0.039 
+12    | 0.000293  | 0.145      | 0.169      | 0.857           | 0.717        | 0.049             | 0.360    0.052    0.099    0.006    0.408    0.370    0.336   | 0.428    0.058    0.100    0.016    0.404    0.366    0.327   | 0.736  0.656  0.766  | 0.056  0.061  0.031 
+13    | 0.000270  | 0.146      | 0.167      | 0.848           | 0.712        | 0.061             | 0.360    0.054    0.102    0.006    0.408    0.370    0.336   | 0.424    0.057    0.097    0.016    0.404    0.375    0.306   | 0.731  0.640  0.789  | 0.078  0.062  0.042 
+14    | 0.000255  | 0.142      | 0.170      | 0.852           | 0.708        | 0.052             | 0.356    0.050    0.094    0.005    0.407    0.369    0.335   | 0.431    0.058    0.098    0.017    0.399    0.393    0.303   | 0.731  0.647  0.758  | 0.060  0.060  0.037 
+15    | 0.000250  | 0.141      | 0.169      | 0.857           | 0.727        | 0.056             | 0.356    0.049    0.093    0.005    0.408    0.369    0.335   | 0.430    0.057    0.096    0.017    0.417    0.397    0.315   | 0.747  0.654  0.793  | 0.061  0.066  0.043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(This config
+ taken as
+ Unet best.
+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2514  1961  1471
+FP   233   240    93
+FN    63   108    55
+TN  4486  4987  5677
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.345  0.269  0.202
+FP  0.032  0.033  0.013
+FN  0.009  0.015  0.008
+TN  0.615  0.684  0.778
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.169      | 0.857086        | 0.727457     | 0.056494          | 0.430    0.057    0.096    0.017    0.417    0.397    0.315   | 0.747  0.654  0.793  | 0.061  0.066  0.043 
+266     | 266     | 0.168      | 0.857393        | 0.729146     | 0.057109          | 0.428    0.057    0.097    0.017    0.413    0.397    0.306   | 0.746  0.656  0.798  | 0.063  0.067  0.042 
+360     | 310     | 0.163      | 0.847944        | 0.692762     | 0.048601          | 0.439    0.044    0.080    0.008    0.376    0.346    0.362   | 0.721  0.596  0.800  | 0.053  0.066  0.027 
+276     | 276     | 0.188      | 0.864908        | 0.748963     | 0.057795          | 0.472    0.066    0.114    0.019    0.623    0.513    0.422   | 0.811  0.682  0.702  | 0.031  0.055  0.087 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-3
+pres_smooth_eps = 0
+Aux head LR : 1/8   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 9m 55s)
+(Max GPU mem usage : 6602.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.482      | 0.203      | 0.701           | 0.471        | 0.145             | 0.229    0.591    0.939    0.243    0.397    0.345    0.295   | 0.242    0.186    0.308    0.065    0.379    0.329    0.223   | 0.518  0.387  0.500  | 0.102  0.113  0.220 
+2     | 0.000250  | 0.186      | 0.108      | 0.827           | 0.670        | 0.068             | 0.112    0.217    0.418    0.017    0.382    0.315    0.250   | 0.205    0.067    0.121    0.013    0.368    0.322    0.238   | 0.709  0.595  0.708  | 0.072  0.073  0.061 
+3     | 0.000375  | 0.098      | 0.117      | 0.828           | 0.682        | 0.074             | 0.092    0.101    0.192    0.010    0.378    0.309    0.243   | 0.245    0.062    0.110    0.015    0.382    0.327    0.237   | 0.712  0.616  0.733  | 0.069  0.079  0.073 
+4     | 0.000500  | 0.084      | 0.125      | 0.832           | 0.674        | 0.063             | 0.077    0.086    0.164    0.009    0.377    0.305    0.239   | 0.264    0.065    0.114    0.016    0.396    0.327    0.257   | 0.711  0.596  0.712  | 0.063  0.061  0.064 
+5     | 0.000495  | 0.073      | 0.107      | 0.848           | 0.702        | 0.054             | 0.059    0.078    0.148    0.009    0.375    0.302    0.237   | 0.219    0.060    0.103    0.017    0.382    0.302    0.233   | 0.732  0.626  0.769  | 0.067  0.060  0.037 
+6     | 0.000480  | 0.066      | 0.105      | 0.843           | 0.698        | 0.061             | 0.051    0.072    0.136    0.008    0.375    0.301    0.234   | 0.208    0.061    0.107    0.016    0.364    0.300    0.235   | 0.722  0.638  0.738  | 0.065  0.069  0.049 
+7     | 0.000457  | 0.058      | 0.106      | 0.856           | 0.716        | 0.050             | 0.040    0.066    0.124    0.007    0.374    0.300    0.233   | 0.220    0.057    0.099    0.016    0.371    0.302    0.206   | 0.748  0.652  0.756  | 0.060  0.058  0.033 
+8     | 0.000427  | 0.052      | 0.101      | 0.851           | 0.711        | 0.056             | 0.029    0.062    0.117    0.007    0.373    0.298    0.232   | 0.198    0.059    0.102    0.016    0.370    0.306    0.211   | 0.725  0.646  0.775  | 0.054  0.072  0.042 
+9     | 0.000393  | 0.051      | 0.101      | 0.849           | 0.714        | 0.060             | 0.027    0.061    0.114    0.007    0.373    0.297    0.231   | 0.200    0.059    0.100    0.017    0.374    0.332    0.225   | 0.748  0.642  0.764  | 0.065  0.074  0.042 
+10    | 0.000357  | 0.047      | 0.103      | 0.854           | 0.716        | 0.054             | 0.020    0.059    0.112    0.006    0.373    0.297    0.230   | 0.204    0.060    0.104    0.016    0.357    0.295    0.228   | 0.730  0.654  0.778  | 0.057  0.066  0.040 
+11    | 0.000323  | 0.045      | 0.105      | 0.859           | 0.724        | 0.052             | 0.020    0.056    0.106    0.006    0.373    0.296    0.230   | 0.215    0.057    0.099    0.016    0.369    0.309    0.219   | 0.748  0.652  0.784  | 0.065  0.059  0.031 
+12    | 0.000293  | 0.042      | 0.109      | 0.862           | 0.731        | 0.051             | 0.015    0.054    0.103    0.006    0.372    0.295    0.229   | 0.229    0.057    0.097    0.016    0.371    0.310    0.224   | 0.755  0.657  0.785  | 0.057  0.061  0.034 
+13    | 0.000270  | 0.040      | 0.123      | 0.855           | 0.722        | 0.056             | 0.010    0.052    0.099    0.006    0.372    0.295    0.229   | 0.280    0.056    0.097    0.016    0.377    0.311    0.232   | 0.741  0.655  0.776  | 0.060  0.066  0.042 
+14    | 0.000255  | 0.037      | 0.118      | 0.860           | 0.723        | 0.048             | 0.008    0.050    0.095    0.005    0.372    0.294    0.228   | 0.255    0.059    0.102    0.016    0.362    0.293    0.240   | 0.750  0.660  0.760  | 0.059  0.060  0.026 
+15    | 0.000250  | 0.037      | 0.130      | 0.857           | 0.721        | 0.053             | 0.009    0.049    0.092    0.005    0.372    0.294    0.229   | 0.300    0.058    0.098    0.017    0.379    0.304    0.203   | 0.748  0.652  0.771  | 0.064  0.066  0.028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2521  1952  1399
+FP   237   237    52
+FN    56   117   127
+TN  4482  4990  5718
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.346  0.268  0.192
+FP  0.032  0.032  0.007
+FN  0.008  0.016  0.017
+TN  0.614  0.684  0.784
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.130      | 0.856804        | 0.720786     | 0.052518          | 0.300    0.058    0.098    0.017    0.379    0.304    0.203   | 0.748  0.652  0.771  | 0.064  0.066  0.028 
+266     | 266     | 0.126      | 0.856961        | 0.723385     | 0.053988          | 0.286    0.058    0.099    0.017    0.372    0.302    0.196   | 0.743  0.655  0.792  | 0.066  0.067  0.029 
+360     | 310     | 0.152      | 0.843757        | 0.676951     | 0.045039          | 0.395    0.048    0.088    0.009    0.353    0.263    0.226   | 0.767  0.612  0.626  | 0.051  0.059  0.025 
+276     | 276     | 0.185      | 0.871588        | 0.739639     | 0.040447          | 0.457    0.069    0.117    0.021    0.616    0.448    0.328   | 0.803  0.662  0.708  | 0.037  0.054  0.031 </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">unet-effnetv2s improved hyperparams
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,1.25e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+Aux head dropout = 0.3, pooling=max
+Aux head LR : 1/8   
+weight decay 1e-2
+pres_smooth_eps = 0.01
+seg_loss = 0.7dice + 0.3bce
+grad_accu=4, effBS = 16*4 = 64
+(4h 16m 5s)
+(Max GPU mem usage : 6602.875 MB)  </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.810      | 0.307      | 0.733           | 0.497        | 0.109             | 1.045    0.709    0.909    0.243    0.402    0.343    0.309   | 0.558    0.199    0.264    0.047    0.369    0.339    0.238   | 0.613  0.449  0.387  | 0.080  0.122  0.126 
+2     | 0.000250  | 0.323      | 0.199      | 0.825           | 0.657        | 0.064             | 0.485    0.253    0.355    0.015    0.391    0.329    0.276   | 0.450    0.092    0.125    0.015    0.369    0.319    0.236   | 0.696  0.588  0.685  | 0.074  0.076  0.041 
+3     | 0.000375  | 0.217      | 0.174      | 0.830           | 0.682        | 0.071             | 0.377    0.148    0.207    0.012    0.387    0.326    0.269   | 0.381    0.085    0.115    0.018    0.373    0.300    0.238   | 0.716  0.612  0.713  | 0.072  0.078  0.064 
+4     | 0.000500  | 0.190      | 0.176      | 0.834           | 0.683        | 0.066             | 0.333    0.129    0.179    0.012    0.385    0.323    0.265   | 0.392    0.084    0.112    0.018    0.380    0.326    0.264   | 0.717  0.605  0.743  | 0.065  0.084  0.047 
+5     | 0.000492  | 0.160      | 0.158      | 0.831           | 0.679        | 0.068             | 0.262    0.116    0.161    0.011    0.384    0.321    0.261   | 0.334    0.083    0.110    0.020    0.374    0.331    0.248   | 0.715  0.599  0.733  | 0.078  0.072  0.056 
+6     | 0.000470  | 0.147      | 0.182      | 0.816           | 0.679        | 0.093             | 0.233    0.110    0.152    0.010    0.383    0.319    0.260   | 0.409    0.085    0.114    0.018    0.389    0.336    0.248   | 0.715  0.608  0.722  | 0.111  0.115  0.054 
+7     | 0.000435  | 0.143      | 0.136      | 0.854           | 0.711        | 0.050             | 0.228    0.107    0.148    0.010    0.384    0.320    0.260   | 0.272    0.078    0.104    0.017    0.369    0.322    0.227   | 0.725  0.646  0.772  | 0.050  0.067  0.034 
+8     | 0.000390  | 0.122      | 0.134      | 0.854           | 0.711        | 0.050             | 0.181    0.098    0.135    0.009    0.382    0.317    0.257   | 0.261    0.080    0.106    0.018    0.372    0.311    0.253   | 0.741  0.646  0.754  | 0.060  0.058  0.032 
+9     | 0.000339  | 0.110      | 0.135      | 0.853           | 0.713        | 0.054             | 0.157    0.090    0.125    0.009    0.382    0.315    0.256   | 0.266    0.079    0.105    0.019    0.371    0.320    0.235   | 0.744  0.635  0.761  | 0.075  0.056  0.032 
+10    | 0.000286  | 0.099      | 0.136      | 0.850           | 0.701        | 0.050             | 0.136    0.083    0.116    0.008    0.381    0.314    0.254   | 0.254    0.085    0.113    0.019    0.358    0.322    0.237   | 0.724  0.625  0.761  | 0.056  0.067  0.028 
+11    | 0.000235  | 0.093      | 0.129      | 0.856           | 0.718        | 0.052             | 0.125    0.080    0.110    0.008    0.380    0.313    0.253   | 0.251    0.076    0.101    0.019    0.368    0.313    0.242   | 0.741  0.650  0.765  | 0.059  0.069  0.027 
+12    | 0.000190  | 0.089      | 0.129      | 0.859           | 0.728        | 0.054             | 0.118    0.077    0.106    0.007    0.380    0.312    0.252   | 0.253    0.075    0.100    0.018    0.376    0.318    0.236   | 0.748  0.651  0.784  | 0.067  0.060  0.035 
+13    | 0.000155  | 0.086      | 0.133      | 0.848           | 0.713        | 0.062             | 0.113    0.075    0.103    0.007    0.380    0.311    0.251   | 0.257    0.079    0.105    0.020    0.369    0.302    0.241   | 0.740  0.629  0.770  | 0.068  0.076  0.041 
+14    | 0.000133  | 0.085      | 0.139      | 0.856           | 0.712        | 0.048             | 0.112    0.073    0.101    0.007    0.379    0.310    0.251   | 0.283    0.078    0.103    0.019    0.372    0.314    0.226   | 0.733  0.639  0.757  | 0.060  0.054  0.029 
+15    | 0.000125  | 0.082      | 0.127      | 0.859           | 0.728        | 0.054             | 0.110    0.070    0.097    0.007    0.379    0.310    0.251   | 0.247    0.076    0.100    0.019    0.364    0.306    0.245   | 0.750  0.653  0.781  | 0.067  0.061  0.035 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2462  1912  1453
+FP   167   173    81
+FN   115   157    73
+TN  4552  5054  5689
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.337  0.262  0.199
+FP  0.023  0.024  0.011
+FN  0.016  0.022  0.010
+TN  0.624  0.693  0.780
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.127      | 0.858655        | 0.727957     | 0.054214          | 0.247    0.076    0.100    0.019    0.364    0.306    0.245   | 0.750  0.653  0.781  | 0.067  0.061  0.035 
+266     | 266     | 0.125      | 0.860457        | 0.732024     | 0.053920          | 0.240    0.076    0.100    0.020    0.359    0.304    0.235   | 0.753  0.658  0.786  | 0.068  0.063  0.031 
+360     | 310     | 0.137      | 0.823039        | 0.664953     | 0.071570          | 0.288    0.073    0.099    0.011    0.317    0.266    0.299   | 0.676  0.553  0.784  | 0.083  0.049  0.083 
+276     | 276     | 0.157      | 0.878688        | 0.749933     | 0.035476          | 0.336    0.080    0.106    0.021    0.604    0.453    0.379   | 0.815  0.689  0.705  | 0.034  0.046  0.026 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,1.25e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+Aux head dropout = 0.3, pooling=max
+Aux head LR : 1/8   
+weight decay 1e-3
+pres_smooth_eps = 0.01
+seg_loss = 0.5dice + 0.5bce
+grad_accu=4, effBS = 16*4 = 64
+(4h 8m 5s)
+(Max GPU mem usage : 6602.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.729      | 0.319      | 0.691           | 0.444        | 0.145             | 1.049    0.592    0.941    0.243    0.401    0.342    0.310   | 0.622    0.189    0.311    0.066    0.382    0.340    0.235   | 0.501  0.373  0.455  | 0.104  0.111  0.220 
+2     | 0.000250  | 0.308      | 0.195      | 0.816           | 0.654        | 0.076             | 0.490    0.230    0.441    0.018    0.391    0.329    0.277   | 0.484    0.070    0.128    0.013    0.382    0.334    0.229   | 0.692  0.586  0.681  | 0.089  0.087  0.052 
+3     | 0.000375  | 0.191      | 0.161      | 0.831           | 0.679        | 0.068             | 0.375    0.112    0.213    0.010    0.387    0.326    0.270   | 0.382    0.066    0.117    0.014    0.357    0.286    0.251   | 0.717  0.603  0.710  | 0.076  0.075  0.053 
+4     | 0.000500  | 0.162      | 0.173      | 0.818           | 0.641        | 0.063             | 0.319    0.095    0.180    0.010    0.385    0.323    0.265   | 0.405    0.073    0.128    0.018    0.365    0.319    0.224   | 0.671  0.601  0.662  | 0.073  0.082  0.034 
+5     | 0.000492  | 0.142      | 0.142      | 0.828           | 0.671        | 0.068             | 0.274    0.086    0.163    0.009    0.384    0.321    0.262   | 0.317    0.068    0.117    0.018    0.368    0.334    0.219   | 0.687  0.603  0.735  | 0.074  0.097  0.032 
+6     | 0.000470  | 0.126      | 0.144      | 0.844           | 0.701        | 0.061             | 0.237    0.079    0.149    0.009    0.383    0.319    0.260   | 0.339    0.061    0.106    0.016    0.366    0.305    0.254   | 0.728  0.630  0.753  | 0.073  0.067  0.043 
+7     | 0.000435  | 0.113      | 0.133      | 0.846           | 0.707        | 0.061             | 0.206    0.073    0.138    0.008    0.382    0.318    0.258   | 0.303    0.060    0.105    0.015    0.373    0.308    0.220   | 0.730  0.634  0.759  | 0.074  0.066  0.041 
+8     | 0.000390  | 0.104      | 0.123      | 0.850           | 0.705        | 0.053             | 0.182    0.070    0.132    0.008    0.382    0.317    0.257   | 0.266    0.061    0.107    0.016    0.351    0.304    0.238   | 0.717  0.641  0.752  | 0.058  0.066  0.035 
+9     | 0.000339  | 0.093      | 0.121      | 0.850           | 0.715        | 0.059             | 0.155    0.066    0.125    0.007    0.381    0.315    0.256   | 0.268    0.058    0.101    0.015    0.352    0.322    0.246   | 0.735  0.651  0.766  | 0.058  0.080  0.040 
+10    | 0.000286  | 0.083      | 0.129      | 0.843           | 0.705        | 0.066             | 0.135    0.061    0.115    0.007    0.380    0.313    0.254   | 0.293    0.058    0.100    0.016    0.379    0.343    0.250   | 0.723  0.634  0.766  | 0.085  0.076  0.036 
+11    | 0.000235  | 0.077      | 0.119      | 0.853           | 0.716        | 0.055             | 0.121    0.058    0.109    0.006    0.380    0.312    0.252   | 0.260    0.059    0.101    0.016    0.367    0.314    0.235   | 0.734  0.647  0.766  | 0.067  0.065  0.034 
+12    | 0.000190  | 0.073      | 0.120      | 0.856           | 0.718        | 0.053             | 0.115    0.055    0.105    0.006    0.379    0.311    0.252   | 0.264    0.059    0.102    0.016    0.377    0.316    0.227   | 0.741  0.649  0.767  | 0.065  0.066  0.028 
+13    | 0.000155  | 0.071      | 0.117      | 0.859           | 0.722        | 0.050             | 0.112    0.054    0.102    0.006    0.379    0.311    0.251   | 0.256    0.058    0.101    0.016    0.370    0.306    0.232   | 0.743  0.651  0.779  | 0.060  0.065  0.026 
+14    | 0.000133  | 0.070      | 0.119      | 0.852           | 0.715        | 0.056             | 0.109    0.054    0.102    0.006    0.379    0.310    0.251   | 0.258    0.059    0.103    0.016    0.375    0.317    0.233   | 0.734  0.642  0.773  | 0.062  0.073  0.033 
+15    | 0.000125  | 0.069      | 0.119      | 0.855           | 0.726        | 0.059             | 0.109    0.051    0.097    0.006    0.379    0.310    0.251   | 0.259    0.060    0.103    0.017    0.366    0.305    0.250   | 0.745  0.648  0.785  | 0.067  0.070  0.040 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2462  1920  1478
+FP   149   158   104
+FN   115   149    48
+TN  4570  5069  5666
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.337  0.263  0.203
+FP  0.020  0.022  0.014
+FN  0.016  0.020  0.007
+TN  0.626  0.695  0.777
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.119      | 0.855126        | 0.726449     | 0.059090          | 0.259    0.060    0.103    0.017    0.366    0.305    0.250   | 0.745  0.648  0.785  | 0.067  0.070  0.040 
+266     | 266     | 0.119      | 0.855356        | 0.728540     | 0.060099          | 0.255    0.060    0.103    0.017    0.360    0.302    0.240   | 0.744  0.650  0.789  | 0.071  0.067  0.042 
+360     | 310     | 0.119      | 0.846614        | 0.684478     | 0.045295          | 0.272    0.053    0.097    0.009    0.335    0.277    0.310   | 0.706  0.588  0.788  | 0.042  0.067  0.027 
+276     | 276     | 0.142      | 0.863582        | 0.752480     | 0.062350          | 0.321    0.065    0.111    0.019    0.602    0.450    0.376   | 0.818  0.690  0.699  | 0.039  0.118  0.030 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+Aux head dropout = 0.3, pooling=max
+Aux head LR : 1/8   
+weight decay 1e-2 for aux head, 1e-3 for others
+pres_smooth_eps = 0.01
+seg_loss = 0.5dice + 0.5bce
+grad_accu=4, effBS = 16*4 = 64
+(4h 10m 43s)
+(Max GPU mem usage : 6602.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.726      | 0.306      | 0.694           | 0.459        | 0.149             | 1.038    0.592    0.940    0.243    0.401    0.342    0.309   | 0.581    0.188    0.310    0.066    0.352    0.320    0.226   | 0.487  0.386  0.503  | 0.109  0.122  0.216 
+2     | 0.000250  | 0.310      | 0.204      | 0.812           | 0.636        | 0.071             | 0.495    0.231    0.444    0.018    0.391    0.329    0.277   | 0.509    0.073    0.132    0.015    0.366    0.331    0.233   | 0.686  0.556  0.682  | 0.082  0.096  0.037 
+3     | 0.000375  | 0.193      | 0.158      | 0.823           | 0.674        | 0.078             | 0.383    0.112    0.214    0.011    0.387    0.326    0.270   | 0.371    0.067    0.119    0.015    0.351    0.290    0.241   | 0.706  0.594  0.718  | 0.088  0.084  0.063 
+4     | 0.000500  | 0.167      | 0.164      | 0.830           | 0.655        | 0.053             | 0.332    0.096    0.181    0.010    0.385    0.323    0.266   | 0.381    0.070    0.124    0.017    0.358    0.319    0.247   | 0.708  0.616  0.650  | 0.063  0.066  0.031 
+5     | 0.000495  | 0.141      | 0.149      | 0.809           | 0.645        | 0.082             | 0.268    0.086    0.163    0.009    0.384    0.321    0.261   | 0.324    0.074    0.129    0.019    0.357    0.307    0.256   | 0.697  0.594  0.645  | 0.091  0.089  0.067 
+6     | 0.000480  | 0.124      | 0.136      | 0.836           | 0.694        | 0.070             | 0.224    0.081    0.153    0.009    0.383    0.319    0.260   | 0.308    0.063    0.109    0.016    0.372    0.332    0.230   | 0.729  0.626  0.748  | 0.082  0.084  0.044 
+7     | 0.000457  | 0.112      | 0.151      | 0.835           | 0.706        | 0.079             | 0.202    0.074    0.140    0.008    0.383    0.318    0.258   | 0.354    0.065    0.104    0.026    0.387    0.320    0.229   | 0.725  0.643  0.770  | 0.140  0.057  0.040 
+8     | 0.000427  | 0.101      | 0.126      | 0.850           | 0.711        | 0.058             | 0.174    0.069    0.131    0.008    0.381    0.317    0.256   | 0.273    0.063    0.110    0.016    0.366    0.334    0.248   | 0.728  0.644  0.766  | 0.061  0.076  0.037 
+9     | 0.000393  | 0.093      | 0.124      | 0.838           | 0.704        | 0.072             | 0.157    0.066    0.125    0.007    0.381    0.315    0.256   | 0.274    0.060    0.105    0.015    0.355    0.307    0.252   | 0.729  0.640  0.749  | 0.063  0.064  0.089 
+10    | 0.000357  | 0.084      | 0.128      | 0.847           | 0.706        | 0.059             | 0.138    0.061    0.116    0.007    0.380    0.313    0.254   | 0.284    0.061    0.106    0.017    0.358    0.324    0.230   | 0.737  0.637  0.757  | 0.073  0.075  0.030 
+11    | 0.000323  | 0.081      | 0.116      | 0.850           | 0.708        | 0.056             | 0.128    0.061    0.114    0.007    0.380    0.313    0.253   | 0.250    0.059    0.102    0.016    0.360    0.316    0.240   | 0.716  0.647  0.775  | 0.063  0.074  0.031 
+12    | 0.000293  | 0.080      | 0.125      | 0.851           | 0.703        | 0.049             | 0.127    0.059    0.112    0.006    0.380    0.313    0.253   | 0.268    0.063    0.109    0.017    0.358    0.304    0.224   | 0.719  0.636  0.758  | 0.057  0.062  0.029 
+13    | 0.000270  | 0.078      | 0.142      | 0.824           | 0.681        | 0.080             | 0.125    0.058    0.109    0.006    0.380    0.313    0.253   | 0.326    0.063    0.107    0.018    0.415    0.351    0.257   | 0.698  0.608  0.762  | 0.110  0.100  0.030 
+14    | 0.000255  | 0.076      | 0.129      | 0.853           | 0.708        | 0.050             | 0.120    0.057    0.108    0.006    0.380    0.312    0.252   | 0.284    0.063    0.108    0.017    0.374    0.313    0.242   | 0.724  0.635  0.771  | 0.066  0.057  0.028 
+15    | 0.000250  | 0.074      | 0.116      | 0.853           | 0.720        | 0.059             | 0.118    0.055    0.103    0.006    0.380    0.312    0.252   | 0.251    0.058    0.101    0.016    0.385    0.317    0.242   | 0.745  0.648  0.772  | 0.063  0.067  0.045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2517  1966  1439
+FP   240   246    90
+FN    60   103    87
+TN  4479  4981  5680
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.345  0.269  0.197
+FP  0.033  0.034  0.012
+FN  0.008  0.014  0.012
+TN  0.614  0.683  0.779
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.116      | 0.852969        | 0.720217     | 0.058530          | 0.251    0.058    0.101    0.016    0.385    0.317    0.242   | 0.745  0.648  0.772  | 0.063  0.067  0.045 
+266     | 266     | 0.116      | 0.853119        | 0.723010     | 0.060142          | 0.249    0.059    0.101    0.017    0.379    0.315    0.232   | 0.746  0.653  0.772  | 0.064  0.068  0.048 
+360     | 310     | 0.113      | 0.841776        | 0.679179     | 0.049826          | 0.268    0.047    0.085    0.009    0.358    0.285    0.309   | 0.698  0.571  0.799  | 0.067  0.058  0.025 
+276     | 276     | 0.132      | 0.865816        | 0.733478     | 0.045958          | 0.285    0.067    0.115    0.019    0.628    0.464    0.362   | 0.790  0.653  0.713  | 0.039  0.070  0.028 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+decoder_attention_type=scse
+Aux head dropout = 0.3, pooling=avg
+Aux head LR : 1/16
+weight decay 1e-5
+pres_smooth_eps = 0.05
+seg_loss = 0.5dice + 0.5bce
+grad_accu=4, effBS = 16*4 = 64
+(4h 37m 24s)
+(Max GPU mem usage : 7424.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.598      | 0.296      | 0.595           | 0.262        | 0.183             | 0.523    0.630    0.957    0.303    0.423    0.395    0.369   | 0.481    0.217    0.337    0.096    0.392    0.367    0.362   | 0.338  0.407  0.000  | 0.120  0.121  0.308 
+2     | 0.000250  | 0.336      | 0.187      | 0.828           | 0.664        | 0.063             | 0.438    0.292    0.553    0.030    0.414    0.383    0.348   | 0.458    0.071    0.127    0.015    0.401    0.377    0.305   | 0.693  0.581  0.717  | 0.077  0.068  0.046 
+3     | 0.000375  | 0.201      | 0.188      | 0.833           | 0.672        | 0.059             | 0.423    0.106    0.201    0.011    0.413    0.382    0.345   | 0.461    0.071    0.122    0.020    0.381    0.328    0.312   | 0.703  0.595  0.711  | 0.073  0.074  0.029 
+4     | 0.000500  | 0.185      | 0.180      | 0.838           | 0.701        | 0.072             | 0.409    0.089    0.168    0.010    0.412    0.380    0.343   | 0.460    0.060    0.104    0.015    0.412    0.418    0.400   | 0.740  0.640  0.707  | 0.092  0.058  0.064 
+5     | 0.000495  | 0.174      | 0.171      | 0.849           | 0.702        | 0.054             | 0.395    0.079    0.149    0.009    0.411    0.378    0.341   | 0.428    0.061    0.106    0.016    0.388    0.367    0.321   | 0.731  0.635  0.741  | 0.065  0.059  0.037 
+6     | 0.000480  | 0.167      | 0.170      | 0.853           | 0.713        | 0.054             | 0.387    0.072    0.136    0.008    0.411    0.376    0.339   | 0.432    0.058    0.100    0.016    0.395    0.381    0.297   | 0.737  0.644  0.769  | 0.072  0.060  0.031 
+7     | 0.000457  | 0.161      | 0.169      | 0.855           | 0.716        | 0.053             | 0.381    0.067    0.126    0.007    0.410    0.375    0.339   | 0.428    0.059    0.101    0.016    0.398    0.363    0.322   | 0.743  0.646  0.765  | 0.067  0.060  0.033 
+8     | 0.000427  | 0.156      | 0.168      | 0.854           | 0.709        | 0.049             | 0.375    0.062    0.117    0.007    0.409    0.374    0.337   | 0.423    0.059    0.103    0.016    0.412    0.378    0.293   | 0.742  0.636  0.747  | 0.067  0.054  0.027 
+9     | 0.000393  | 0.155      | 0.168      | 0.855           | 0.721        | 0.055             | 0.373    0.062    0.117    0.007    0.410    0.373    0.338   | 0.422    0.059    0.103    0.016    0.397    0.353    0.310   | 0.745  0.652  0.767  | 0.069  0.054  0.041 
+10    | 0.000357  | 0.155      | 0.172      | 0.850           | 0.710        | 0.058             | 0.375    0.062    0.116    0.007    0.409    0.373    0.338   | 0.436    0.060    0.103    0.016    0.368    0.346    0.304   | 0.741  0.651  0.748  | 0.071  0.067  0.034 
+11    | 0.000323  | 0.149      | 0.174      | 0.846           | 0.706        | 0.061             | 0.367    0.056    0.106    0.006    0.409    0.372    0.337   | 0.446    0.057    0.098    0.016    0.411    0.366    0.340   | 0.723  0.634  0.783  | 0.074  0.069  0.039 
+12    | 0.000293  | 0.148      | 0.170      | 0.860           | 0.727        | 0.052             | 0.364    0.055    0.103    0.006    0.409    0.372    0.336   | 0.424    0.061    0.106    0.016    0.396    0.362    0.320   | 0.752  0.661  0.771  | 0.070  0.058  0.028 
+13    | 0.000270  | 0.144      | 0.173      | 0.845           | 0.708        | 0.064             | 0.358    0.052    0.098    0.006    0.408    0.369    0.335   | 0.435    0.060    0.103    0.017    0.385    0.370    0.321   | 0.736  0.626  0.779  | 0.084  0.074  0.032 
+14    | 0.000255  | 0.143      | 0.173      | 0.855           | 0.716        | 0.052             | 0.357    0.051    0.096    0.006    0.408    0.370    0.335   | 0.435    0.061    0.105    0.017    0.389    0.374    0.298   | 0.741  0.643  0.771  | 0.059  0.062  0.036 
+15    | 0.000250  | 0.141      | 0.171      | 0.858           | 0.722        | 0.052             | 0.356    0.049    0.093    0.005    0.408    0.369    0.334   | 0.435    0.058    0.100    0.017    0.414    0.376    0.296   | 0.744  0.648  0.776  | 0.067  0.056  0.032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2490  1939  1456
+FP   221   225   100
+FN    87   130    70
+TN  4498  5002  5670
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.341  0.266  0.200
+FP  0.030  0.031  0.014
+FN  0.012  0.018  0.010
+TN  0.617  0.686  0.777
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.171      | 0.857598        | 0.721667     | 0.051780          | 0.435    0.058    0.100    0.017    0.414    0.376    0.296   | 0.744  0.648  0.776  | 0.067  0.056  0.032 
+266     | 266     | 0.170      | 0.859229        | 0.726834     | 0.052507          | 0.430    0.059    0.100    0.018    0.408    0.374    0.288   | 0.747  0.654  0.783  | 0.070  0.055  0.033 
+360     | 310     | 0.170      | 0.836324        | 0.667493     | 0.051121          | 0.453    0.049    0.090    0.009    0.383    0.341    0.337   | 0.684  0.579  0.769  | 0.065  0.066  0.022 
+276     | 276     | 0.201      | 0.860062        | 0.712799     | 0.041763          | 0.504    0.071    0.120    0.022    0.636    0.521    0.407   | 0.778  0.644  0.679  | 0.039  0.053  0.034 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segformer mit-b1
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+Aux head dropout = 0.3, pooling=avg
+Aux head LR : 1/16
+weight decay 1e-5
+pres_smooth_eps = 0.05
+seg_loss = 0.5dice + 0.5bce
+grad_accu=4, effBS = 16*4 = 64
+(3h 43m 57s)
+(Max GPU mem usage : 5708.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres TLo-Seg  TLo-D    TLo-B    TLo-PmC1 TLo-PmC2 TLo-PmC3| VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.459      | 0.208      | 0.790           | 0.574        | 0.065             | 0.467    0.456    0.790    0.122    0.420    0.394    0.365   | 0.444    0.107    0.196    0.019    0.440    0.393    0.341   | 0.651  0.464  0.574  | 0.076  0.068  0.051 
+2     | 0.000250  | 0.233      | 0.175      | 0.838           | 0.672        | 0.051             | 0.404    0.160    0.310    0.010    0.412    0.381    0.345   | 0.425    0.069    0.124    0.013    0.401    0.421    0.333   | 0.708  0.582  0.728  | 0.062  0.051  0.040 
+3     | 0.000375  | 0.194      | 0.170      | 0.840           | 0.682        | 0.055             | 0.389    0.111    0.213    0.009    0.411    0.378    0.342   | 0.419    0.064    0.115    0.013    0.391    0.382    0.326   | 0.717  0.593  0.740  | 0.064  0.055  0.046 
+4     | 0.000500  | 0.183      | 0.170      | 0.844           | 0.694        | 0.056             | 0.379    0.099    0.189    0.009    0.410    0.377    0.338   | 0.417    0.064    0.113    0.015    0.396    0.357    0.321   | 0.728  0.611  0.742  | 0.061  0.059  0.046 
+5     | 0.000495  | 0.173      | 0.173      | 0.841           | 0.692        | 0.060             | 0.371    0.088    0.169    0.008    0.409    0.374    0.337   | 0.422    0.066    0.116    0.016    0.387    0.358    0.299   | 0.717  0.604  0.762  | 0.067  0.052  0.061 
+6     | 0.000480  | 0.167      | 0.168      | 0.852           | 0.705        | 0.049             | 0.365    0.083    0.157    0.008    0.409    0.373    0.335   | 0.413    0.063    0.110    0.015    0.372    0.365    0.314   | 0.731  0.630  0.769  | 0.064  0.057  0.027 
+7     | 0.000457  | 0.161      | 0.177      | 0.846           | 0.696        | 0.054             | 0.359    0.076    0.144    0.007    0.408    0.371    0.335   | 0.442    0.063    0.110    0.016    0.424    0.434    0.282   | 0.724  0.613  0.760  | 0.062  0.075  0.025 
+8     | 0.000427  | 0.160      | 0.169      | 0.856           | 0.715        | 0.049             | 0.357    0.076    0.144    0.007    0.408    0.371    0.334   | 0.419    0.062    0.107    0.017    0.393    0.369    0.316   | 0.739  0.627  0.777  | 0.061  0.054  0.031 
+9     | 0.000393  | 0.156      | 0.169      | 0.857           | 0.716        | 0.049             | 0.351    0.072    0.136    0.007    0.408    0.370    0.334   | 0.420    0.061    0.106    0.016    0.372    0.357    0.316   | 0.739  0.642  0.771  | 0.048  0.058  0.041 
+10    | 0.000357  | 0.153      | 0.167      | 0.855           | 0.720        | 0.055             | 0.349    0.068    0.130    0.007    0.407    0.370    0.333   | 0.420    0.058    0.101    0.016    0.427    0.396    0.331   | 0.749  0.637  0.779  | 0.067  0.055  0.044 
+11    | 0.000323  | 0.151      | 0.170      | 0.856           | 0.720        | 0.053             | 0.348    0.066    0.126    0.006    0.407    0.369    0.333   | 0.425    0.060    0.104    0.017    0.402    0.358    0.314   | 0.744  0.640  0.770  | 0.061  0.059  0.040 
+12    | 0.000293  | 0.147      | 0.169      | 0.853           | 0.717        | 0.056             | 0.343    0.063    0.119    0.006    0.406    0.368    0.332   | 0.430    0.058    0.098    0.017    0.423    0.407    0.316   | 0.741  0.640  0.781  | 0.071  0.061  0.036 
+13    | 0.000270  | 0.146      | 0.169      | 0.859           | 0.723        | 0.051             | 0.342    0.061    0.117    0.006    0.407    0.368    0.332   | 0.425    0.060    0.103    0.017    0.402    0.353    0.311   | 0.745  0.640  0.785  | 0.059  0.052  0.041 
+14    | 0.000255  | 0.143      | 0.168      | 0.857           | 0.721        | 0.053             | 0.339    0.058    0.111    0.006    0.406    0.367    0.331   | 0.425    0.058    0.099    0.017    0.402    0.367    0.311   | 0.742  0.638  0.789  | 0.060  0.062  0.037 
+15    | 0.000250  | 0.143      | 0.178      | 0.857           | 0.711        | 0.046             | 0.340    0.058    0.110    0.006    0.406    0.367    0.331   | 0.441    0.065    0.112    0.019    0.374    0.342    0.304   | 0.732  0.633  0.771  | 0.050  0.050  0.038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2366  1851  1432
+FP   121   126    64
+FN   211   218    94
+TN  4598  5101  5706
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.324  0.254  0.196
+FP  0.017  0.017  0.009
+FN  0.029  0.030  0.013
+TN  0.630  0.699  0.782
+Slice_W | Slice_H | Valid Loss | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres VLo-Seg  VLo-D    VLo-B    VLo-PmC1 VLo-PmC2 VLo-PmC3| D-LB   D-SB   D-S    | H-LB   H-SB   H-S   
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.178      | 0.856843        | 0.711456     | 0.046232          | 0.441    0.065    0.112    0.019    0.374    0.342    0.304   | 0.732  0.633  0.771  | 0.050  0.050  0.038 
+266     | 266     | 0.178      | 0.857119        | 0.713135     | 0.046892          | 0.438    0.066    0.113    0.020    0.366    0.338    0.296   | 0.730  0.635  0.781  | 0.051  0.051  0.039 
+360     | 310     | 0.170      | 0.844831        | 0.675229     | 0.042102          | 0.449    0.051    0.094    0.008    0.366    0.315    0.352   | 0.709  0.573  0.739  | 0.054  0.048  0.024 
+276     | 276     | 0.190      | 0.869422        | 0.736318     | 0.041843          | 0.479    0.067    0.116    0.018    0.614    0.501    0.429   | 0.792  0.689  0.670  | 0.043  0.050  0.032 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).mean(dim=(2,3))
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.95D + 0.05H 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 60s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.683033     | 0.386122     | 0.471540        | 0.166396     | 0.325030          | 0.581763     0.726434     0.473821     0.979049     0.031001    | 0.478697     0.346447     0.265696     0.427198     0.019609    | 0.324445  0.141283  0.014869  | 0.264160  0.395112  0.315818 
+2     | 0.000500  | 0.509415     | 0.297542     | 0.642098        | 0.304912     | 0.133112          | 0.455396     0.532567     0.134789     0.930344     0.009825    | 0.475274     0.221372     0.065964     0.376780     0.004283    | 0.451965  0.206001  0.191198  | 0.092349  0.099107  0.207880 
+3     | 0.000438  | 0.398468     | 0.256801     | 0.720326        | 0.422179     | 0.080909          | 0.417003     0.390524     0.039699     0.741349     0.002212    | 0.464984     0.167579     0.037043     0.298115     0.001124    | 0.483599  0.248122  0.585649  | 0.093034  0.093364  0.056328 
+4     | 0.000313  | 0.312432     | 0.243414     | 0.719411        | 0.410000     | 0.074315          | 0.395927     0.276649     0.019193     0.534105     0.000567    | 0.458752     0.151126     0.028875     0.273376     0.000439    | 0.524483  0.281736  0.466514  | 0.082403  0.107685  0.032857 
+5     | 0.000250  | 0.225111     | 0.227393     | 0.732582        | 0.452030     | 0.080383          | 0.382609     0.157612     0.007153     0.308071     0.000128    | 0.448624     0.132580     0.027841     0.237318     0.000175    | 0.514476  0.354874  0.555176  | 0.074634  0.108831  0.057685 
+6     | 0.000125  | 0.252062     | 0.295624     | 0.744955        | 0.456910     | 0.063015          | 0.380075     0.197199     0.005585     0.207575     0.000049    | 0.470116     0.220842     0.030472     0.232458     0.000129    | 0.522096  0.343033  0.565943  | 0.063227  0.078959  0.046860 
+7     | 0.000250  | 0.236463     | 0.286211     | 0.744217        | 0.458888     | 0.065563          | 0.384452     0.173040     0.006191     0.182146     0.000029    | 0.457498     0.212802     0.032811     0.223997     0.000103    | 0.563776  0.358708  0.535627  | 0.074415  0.073429  0.048845 
+8     | 0.000375  | 0.223233     | 0.298139     | 0.731909        | 0.425442     | 0.063780          | 0.394914     0.149655     0.006342     0.157530     0.000018    | 0.463803     0.227139     0.043634     0.239089     0.000100    | 0.487465  0.365145  0.491546  | 0.069047  0.078326  0.043968 
+9     | 0.000500  | 0.216301     | 0.290431     | 0.738440        | 0.454727     | 0.072418          | 0.396348     0.139139     0.006758     0.146461     0.000013    | 0.440767     0.226001     0.045550     0.237891     0.000103    | 0.564945  0.367414  0.485086  | 0.081937  0.081678  0.053640 
+10    | 0.000483  | 0.205693     | 0.289178     | 0.734580        | 0.439593     | 0.068763          | 0.386729     0.128106     0.006655     0.134848     0.000011    | 0.449679     0.220392     0.047908     0.231987     0.000092    | 0.501041  0.353094  0.551478  | 0.069876  0.082491  0.053922 
+11    | 0.000438  | 0.191456     | 0.294479     | 0.731380        | 0.422393     | 0.062628          | 0.383646     0.109088     0.005930     0.114830     0.000007    | 0.465015     0.221392     0.048101     0.233041     0.000069    | 0.465800  0.334339  0.548045  | 0.067942  0.072351  0.047591 
+12    | 0.000375  | 0.180875     | 0.288081     | 0.754246        | 0.481953     | 0.064225          | 0.374158     0.098039     0.005446     0.103199     0.000006    | 0.455402     0.216372     0.050547     0.227757     0.000076    | 0.537331  0.370956  0.583158  | 0.067083  0.071697  0.053894 
+13    | 0.000313  | 0.173785     | 0.302076     | 0.746083        | 0.456815     | 0.061072          | 0.365987     0.091413     0.005084     0.096224     0.000005    | 0.465100     0.232209     0.051788     0.244428     0.000052    | 0.536163  0.302886  0.589378  | 0.061823  0.074843  0.046551 
+14    | 0.000267  | 0.173565     | 0.283811     | 0.741000        | 0.466160     | 0.075773          | 0.368710     0.089932     0.005225     0.094665     0.000004    | 0.451480     0.211954     0.049437     0.223104     0.000090    | 0.554962  0.357216  0.558540  | 0.098548  0.088143  0.040629 
+15    | 0.000250  | 0.168937     | 0.284910     | 0.750973        | 0.468202     | 0.060513          | 0.364837     0.084980     0.004820     0.089453     0.000004    | 0.438965     0.218886     0.054514     0.230402     0.000083    | 0.543903  0.356079  0.560024  | 0.065901  0.074747  0.040892 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.97D + 0.03H 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 19s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.685472     | 0.390900     | 0.480409        | 0.181521     | 0.320333          | 0.589670     0.726530     0.473873     0.979187     4570.950684 | 0.493634     0.346872     0.266848     0.426895     2907.763428 | 0.329325  0.148591  0.011352  | 0.257638  0.394789  0.308572 
+2     | 0.000500  | 0.507721     | 0.292515     | 0.663191        | 0.349123     | 0.127430          | 0.449102     0.532844     0.134859     0.930829     1450.327026 | 0.465557     0.218355     0.071529     0.365181     670.949158  | 0.481206  0.241143  0.310829  | 0.109183  0.132592  0.140516 
+3     | 0.000438  | 0.396924     | 0.258055     | 0.710522        | 0.407682     | 0.087584          | 0.415816     0.388828     0.039528     0.738129     326.503082  | 0.470098     0.167180     0.038806     0.295553     170.592026  | 0.480648  0.247653  0.566184  | 0.096645  0.093262  0.072847 
+4     | 0.000313  | 0.308418     | 0.231011     | 0.730957        | 0.472301     | 0.096605          | 0.396713     0.270577     0.017048     0.524104     77.818817   | 0.459102     0.133258     0.023353     0.243162     49.358307   | 0.573270  0.341098  0.565740  | 0.077291  0.118980  0.093545 
+5     | 0.000250  | 0.220137     | 0.229768     | 0.720432        | 0.434416     | 0.088891          | 0.383977     0.149920     0.006843     0.292997     16.041384   | 0.452852     0.134161     0.028715     0.239607     24.566214   | 0.496569  0.353203  0.519627  | 0.077737  0.095647  0.093290 
+6     | 0.000125  | 0.332618     | 0.640896     | 0.720683        | 0.380752     | 0.052697          | 0.381976     0.311464     0.006157     0.210117     3.588352    | 0.490343     0.705419     0.035881     0.258834     15.145002   | 0.390936  0.338269  0.505766  | 0.046357  0.071861  0.039872 
+7     | 0.000250  | 0.273916     | 0.533382     | 0.739125        | 0.432604     | 0.056528          | 0.390597     0.223909     0.006973     0.186580     1.430893    | 0.458449     0.565496     0.037000     0.234135     11.279524   | 0.497145  0.351286  0.537130  | 0.053691  0.072389  0.043503 
+8     | 0.000375  | 0.244528     | 0.477037     | 0.736169        | 0.428847     | 0.058949          | 0.394469     0.180267     0.006846     0.158992     0.868161    | 0.472879     0.478819     0.039112     0.234113     8.390992    | 0.504320  0.357469  0.514734  | 0.065099  0.061821  0.049927 
+9     | 0.000500  | 0.250519     | 0.447797     | 0.719332        | 0.385731     | 0.058268          | 0.399195     0.186800     0.008444     0.162347     0.977470    | 0.483122     0.432657     0.049202     0.260950     5.984532    | 0.430726  0.293698  0.522443  | 0.054271  0.063415  0.057117 
+10    | 0.000483  | 0.230044     | 0.603679     | 0.735796        | 0.435558     | 0.064045          | 0.397281     0.158371     0.007652     0.144446     0.608628    | 0.452746     0.668364     0.049352     0.237455     14.601106   | 0.472021  0.361230  0.552693  | 0.068437  0.078937  0.044762 
+11    | 0.000438  | 0.208794     | 0.560933     | 0.740009        | 0.441683     | 0.061108          | 0.385522     0.133053     0.006665     0.122205     0.483821    | 0.468358     0.600609     0.046801     0.226978     12.681323   | 0.493317  0.334626  0.577478  | 0.061418  0.072007  0.049898 
+12    | 0.000375  | 0.201548     | 0.514144     | 0.741889        | 0.454376     | 0.066436          | 0.376632     0.126511     0.006450     0.116259     0.457999    | 0.459019     0.537769     0.047782     0.223681     10.693254   | 0.537517  0.355815  0.553645  | 0.068570  0.079414  0.051324 
+13    | 0.000313  | 0.189602     | 0.527050     | 0.740036        | 0.456997     | 0.071272          | 0.370627     0.112020     0.005828     0.104464     0.356320    | 0.461703     0.555056     0.048623     0.225442     11.212595   | 0.521670  0.362130  0.579857  | 0.060818  0.086083  0.066914 
+14    | 0.000267  | 0.184098     | 0.506990     | 0.746831        | 0.462894     | 0.063879          | 0.369157     0.104787     0.005495     0.098181     0.318379    | 0.470371     0.522684     0.046233     0.221478     10.261664   | 0.537179  0.370609  0.558162  | 0.064650  0.079008  0.047978 
+15    | 0.000250  | 0.182501     | 0.476101     | 0.746605        | 0.453386     | 0.057916          | 0.366898     0.103474     0.005463     0.096973     0.313666    | 0.474507     0.476784     0.050257     0.228641     8.500095    | 0.515623  0.346671  0.585649  | 0.061456  0.065159  0.047133 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 13s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">taken as best run 
+With Haus surro
+In data subset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.684073     | 0.384596     | 0.473457        | 0.164027     | 0.320256          | 0.585437     0.726345     0.473389     0.979301     4563.643555 | 0.475736     0.345536     0.263806     0.427265     2877.298096 | 0.328415  0.122756  0.011226  | 0.257572  0.394785  0.308413 
+2     | 0.000500  | 0.507900     | 0.297128     | 0.666376        | 0.279430     | 0.075661          | 0.450877     0.532338     0.133966     0.930711     1441.775269 | 0.470099     0.222997     0.066101     0.379893     614.620117  | 0.427992  0.221084  0.175657  | 0.096375  0.090408  0.040199 
+3     | 0.000438  | 0.396723     | 0.253453     | 0.710585        | 0.408757     | 0.088196          | 0.414396     0.389150     0.039362     0.738938     321.716492  | 0.448049     0.170054     0.040477     0.299632     179.628464  | 0.502995  0.262112  0.510790  | 0.108455  0.102800  0.053332 
+4     | 0.000313  | 0.312850     | 0.245485     | 0.703400        | 0.410287     | 0.101192          | 0.393352     0.278349     0.020056     0.536642     84.602547   | 0.470819     0.148912     0.033056     0.264769     84.431114   | 0.507991  0.262509  0.488381  | 0.093295  0.098193  0.112087 
+5     | 0.000250  | 0.234344     | 0.229170     | 0.743392        | 0.464191     | 0.070475          | 0.382881     0.170686     0.008671     0.332700     24.492037   | 0.459265     0.130559     0.026524     0.234594     25.186287   | 0.524465  0.361464  0.569052  | 0.079925  0.090837  0.040662 
+6     | 0.000125  | 0.261862     | 0.352992     | 0.739717        | 0.426361     | 0.051378          | 0.380518     0.211009     0.006663     0.241634     4.467174    | 0.475837     0.300345     0.029173     0.244491     8.312460    | 0.485626  0.341168  0.535471  | 0.058399  0.063285  0.032452 
+7     | 0.000250  | 0.203938     | 0.352644     | 0.737367        | 0.419680     | 0.050843          | 0.381017     0.128047     0.006213     0.189643     1.603890    | 0.448616     0.311514     0.034740     0.249253     8.617852    | 0.488569  0.342395  0.502794  | 0.059214  0.061850  0.031464 
+8     | 0.000375  | 0.196027     | 0.353498     | 0.731492        | 0.405472     | 0.051162          | 0.390020     0.112887     0.007057     0.180840     1.040896    | 0.491102     0.294524     0.040291     0.255100     7.489142    | 0.441629  0.333066  0.515285  | 0.059451  0.059874  0.034161 
+9     | 0.000500  | 0.185622     | 0.378514     | 0.729536        | 0.419110     | 0.063513          | 0.390789     0.097693     0.006922     0.158089     0.841910    | 0.456226     0.345210     0.044988     0.250705     10.016015   | 0.505215  0.340511  0.458135  | 0.074279  0.075133  0.041126 
+10    | 0.000483  | 0.176654     | 0.335122     | 0.753505        | 0.462844     | 0.052720          | 0.389435     0.085463     0.006457     0.143392     0.601844    | 0.448095     0.286706     0.042357     0.231054     7.636719    | 0.541301  0.363656  0.539447  | 0.057667  0.059821  0.040673 
+11    | 0.000438  | 0.163164     | 0.366331     | 0.752784        | 0.470389     | 0.058953          | 0.379442     0.070474     0.005508     0.119121     0.470268    | 0.464213     0.324382     0.040101     0.216907     9.922383    | 0.514171  0.369729  0.598559  | 0.066919  0.070492  0.039447 
+12    | 0.000375  | 0.157555     | 0.363265     | 0.756125        | 0.473124     | 0.055208          | 0.372088     0.065612     0.005057     0.112329     0.404628    | 0.454339     0.324234     0.043774     0.226016     9.601841    | 0.551039  0.375394  0.547094  | 0.067169  0.063478  0.034976 
+13    | 0.000313  | 0.152824     | 0.371411     | 0.753969        | 0.477299     | 0.061585          | 0.366932     0.061064     0.004858     0.105017     0.361244    | 0.443206     0.340642     0.043174     0.217289     10.650764   | 0.559533  0.379277  0.558533  | 0.062900  0.077677  0.044179 
+14    | 0.000267  | 0.149788     | 0.332335     | 0.748773        | 0.466627     | 0.063131          | 0.364742     0.057665     0.004608     0.099929     0.322092    | 0.442851     0.284972     0.043283     0.223455     7.713509    | 0.560228  0.368712  0.550655  | 0.069501  0.072957  0.046934 
+15    | 0.000250  | 0.148081     | 0.350561     | 0.756330        | 0.481592     | 0.060512          | 0.364310     0.055412     0.004520     0.096070     0.306140    | 0.436695     0.313646     0.043963     0.216074     9.311402    | 0.587398  0.378724  0.546118  | 0.070417  0.063758  0.047362 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+10 epochs : 0.5D + 0.5B
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+5 epochs :  0.02H + 0.49D + 0.49B 
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 54s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.738284     | 0.467502     | 0.387112        | 0.112082     | 0.429534          | 0.618518     0.789613     0.597698     0.981528     5558.331055 | 0.512886     0.448052     0.463011     0.433093     4611.374512 | 0.193815  0.068694  0.057513  | 0.375900  0.413433  0.499268 
+2     | 0.000250  | 0.576388     | 0.362080     | 0.585903        | 0.246670     | 0.187942          | 0.465261     0.624014     0.274355     0.973673     2897.793701 | 0.507637     0.299699     0.181369     0.418029     2007.698486 | 0.436792  0.227676  0.011670  | 0.116561  0.145037  0.302229 
+3     | 0.000375  | 0.491551     | 0.300349     | 0.625419        | 0.260447     | 0.131267          | 0.433596     0.516389     0.113132     0.919647     1211.708740 | 0.476418     0.224891     0.079925     0.369857     732.798157  | 0.475542  0.243711  0.010086  | 0.114605  0.110211  0.168985 
+4     | 0.000500  | 0.401090     | 0.265552     | 0.680881        | 0.383974     | 0.121181          | 0.409490     0.397490     0.042258     0.752723     370.931580  | 0.484890     0.171550     0.038665     0.304435     189.755859  | 0.475132  0.258593  0.446768  | 0.074003  0.132220  0.157319 
+5     | 0.000483  | 0.275722     | 0.259029     | 0.714518        | 0.384709     | 0.065609          | 0.397816     0.223396     0.011064     0.435728     52.852238   | 0.509632     0.151628     0.032341     0.270915     21.948494   | 0.380278  0.332503  0.506531  | 0.065283  0.083936  0.047608 
+6     | 0.000438  | 0.201646     | 0.235624     | 0.717652        | 0.405061     | 0.073953          | 0.396391     0.118184     0.006682     0.229687     7.500936    | 0.467912     0.136073     0.035866     0.236279     26.628571   | 0.452592  0.325327  0.547751  | 0.065625  0.108542  0.047692 
+7     | 0.000375  | 0.176981     | 0.229273     | 0.738581        | 0.453503     | 0.071367          | 0.388430     0.086360     0.005622     0.167098     3.472807    | 0.469672     0.126245     0.033709     0.218781     14.888218   | 0.505146  0.356504  0.586378  | 0.076427  0.074398  0.063277 
+8     | 0.000313  | 0.169129     | 0.233044     | 0.745283        | 0.460227     | 0.064679          | 0.383953     0.077062     0.005395     0.148730     2.344778    | 0.467590     0.132524     0.037927     0.227121     18.340193   | 0.543563  0.355344  0.530823  | 0.072688  0.085587  0.035762 
+9     | 0.000267  | 0.160309     | 0.232792     | 0.743355        | 0.459179     | 0.067195          | 0.377579     0.067193     0.004958     0.129428     1.830697    | 0.464006     0.133700     0.039820     0.227580     15.027086   | 0.560527  0.345333  0.527540  | 0.069049  0.073685  0.058852 
+10    | 0.000250  | 0.154870     | 0.235043     | 0.732649        | 0.425618     | 0.062664          | 0.370920     0.062278     0.004631     0.119924     1.535878    | 0.462532     0.137548     0.042339     0.232757     15.713588   | 0.479420  0.354373  0.518668  | 0.063348  0.083712  0.040930 
+11    | 0.000250  | 0.170186     | 0.452805     | 0.709296        | 0.356276     | 0.055358          | 0.371289     0.084000     0.005411     0.124835     1.008937    | 0.498443     0.433245     0.049882     0.258867     14.097895   | 0.340411  0.333602  0.487626  | 0.052981  0.075275  0.037818 
+12    | 0.000500  | 0.175733     | 0.364311     | 0.727503        | 0.411043     | 0.061524          | 0.380932     0.087791     0.006756     0.139764     0.799837    | 0.491100     0.309973     0.047369     0.250058     8.211725    | 0.504917  0.215053  0.538485  | 0.086890  0.053959  0.043723 
+13    | 0.000438  | 0.170412     | 0.423637     | 0.733087        | 0.432269     | 0.066368          | 0.382327     0.079591     0.006741     0.130589     0.614975    | 0.470525     0.403543     0.050383     0.230484     13.295895   | 0.515696  0.344673  0.505888  | 0.054411  0.101049  0.043643 
+14    | 0.000313  | 0.157197     | 0.378824     | 0.739991        | 0.439662     | 0.059789          | 0.375100     0.063810     0.005409     0.109009     0.387271    | 0.525417     0.315998     0.045342     0.231072     9.027761    | 0.507151  0.333771  0.554489  | 0.054064  0.075948  0.049356 
+15    | 0.000250  | 0.150277     | 0.370522     | 0.743701        | 0.474644     | 0.076928          | 0.366608     0.057564     0.004908     0.098642     0.341258    | 0.455500     0.334103     0.047347     0.217252     10.222479   | 0.558613  0.339670  0.589663  | 0.054984  0.078942  0.096857 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+10 epochs : 0.5D + 0.5B
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+5 epochs :  0.01H + 0.1D + 0.89B 
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 34s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.739592     | 0.460257     | 0.387636        | 0.111442     | 0.428234          | 0.623461     0.789363     0.597034     0.981692     5543.206543 | 0.494657     0.445514     0.457753     0.433275     4574.350098 | 0.194666  0.068026  0.059339  | 0.374801  0.410776  0.499125 
+2     | 0.000250  | 0.574095     | 0.355320     | 0.572420        | 0.250013     | 0.212643          | 0.457685     0.623985     0.273710     0.974260     2893.181152 | 0.482402     0.300856     0.185613     0.416099     2040.184326 | 0.443953  0.228686  0.010102  | 0.112695  0.224859  0.300373 
+3     | 0.000375  | 0.492164     | 0.300273     | 0.616348        | 0.251219     | 0.140233          | 0.432895     0.517565     0.113648     0.921481     1216.240234 | 0.477344     0.224385     0.075139     0.373631     701.582275  | 0.483474  0.231996  0.003584  | 0.136243  0.107938  0.176517 
+4     | 0.000500  | 0.403851     | 0.264727     | 0.693415        | 0.408199     | 0.116442          | 0.415383     0.398909     0.043012     0.754806     373.935516  | 0.487226     0.169370     0.038932     0.299808     190.076218  | 0.530800  0.255170  0.474940  | 0.104849  0.120756  0.123719 
+5     | 0.000483  | 0.276463     | 0.238018     | 0.722805        | 0.433396     | 0.084255          | 0.394745     0.225770     0.011763     0.439776     54.231125   | 0.463502     0.141382     0.028992     0.253771     27.907379   | 0.505278  0.319259  0.519739  | 0.074415  0.084938  0.093414 
+6     | 0.000438  | 0.198995     | 0.240981     | 0.736138        | 0.444335     | 0.069327          | 0.392570     0.116034     0.006543     0.225524     7.401748    | 0.486898     0.135587     0.031931     0.239243     15.712357   | 0.501687  0.340413  0.569020  | 0.073444  0.091714  0.042823 
+7     | 0.000375  | 0.174017     | 0.223012     | 0.758783        | 0.506579     | 0.073082          | 0.386016     0.083160     0.005311     0.161009     3.334690    | 0.454070     0.123987     0.032877     0.215097     14.603605   | 0.583674  0.368877  0.613096  | 0.068454  0.077332  0.073460 
+8     | 0.000313  | 0.164880     | 0.235085     | 0.732757        | 0.448736     | 0.077895          | 0.380289     0.072561     0.004987     0.140136     2.219630    | 0.477418     0.131228     0.035560     0.226895     12.458936   | 0.532435  0.348762  0.551082  | 0.066622  0.076429  0.090633 
+9     | 0.000267  | 0.159112     | 0.227273     | 0.757540        | 0.488053     | 0.062802          | 0.375793     0.066248     0.004823     0.127674     1.810220    | 0.458960     0.127979     0.036497     0.219461     11.963871   | 0.565118  0.342086  0.605758  | 0.070905  0.074179  0.043321 
+10    | 0.000250  | 0.152626     | 0.222283     | 0.748490        | 0.484615     | 0.075593          | 0.370739     0.059149     0.004391     0.113906     1.499743    | 0.450576     0.124442     0.036887     0.211998     18.024797   | 0.555953  0.331522  0.622231  | 0.068156  0.088595  0.070028 
+11    | 0.000250  | 0.129088     | 0.248503     | 0.744891        | 0.445989     | 0.055842          | 0.369986     0.025846     0.004771     0.122003     0.939934    | 0.464326     0.156007     0.036986     0.226386     10.045136   | 0.521623  0.351759  0.563861  | 0.063575  0.071315  0.032635 
+12    | 0.000500  | 0.129144     | 0.258908     | 0.724136        | 0.392623     | 0.054856          | 0.370937     0.025519     0.005161     0.132050     0.772053    | 0.463621     0.171173     0.046243     0.250666     10.495039   | 0.405887  0.319396  0.531086  | 0.054070  0.068241  0.042256 
+13    | 0.000438  | 0.125394     | 0.253502     | 0.743776        | 0.447940     | 0.059000          | 0.368410     0.021244     0.004615     0.121156     0.502088    | 0.454752     0.167253     0.038172     0.227405     11.053905   | 0.508907  0.344700  0.567609  | 0.056632  0.078025  0.042342 
+14    | 0.000313  | 0.122878     | 0.244082     | 0.753218        | 0.469365     | 0.057546          | 0.366848     0.018319     0.004003     0.108943     0.386221    | 0.450295     0.155705     0.035661     0.221840     10.178316   | 0.538583  0.378576  0.571820  | 0.058004  0.076090  0.038545 
+15    | 0.000250  | 0.120730     | 0.254127     | 0.744455        | 0.450269     | 0.059422          | 0.362591     0.017076     0.003669     0.103953     0.341522    | 0.444317     0.172617     0.038831     0.226263     11.543139   | 0.537976  0.344734  0.555165  | 0.058057  0.082131  0.038076 </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+10 epochs : 0.5D + 0.5B
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+5 epochs :  0.01H + 0.495D + 0.495B 
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF3465A4"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">weight decay 1e-3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 29s)
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.741949     | 0.466389     | 0.386245        | 0.110362     | 0.429833          | 0.630926     0.789531     0.597441     0.981621     5558.728516 | 0.511804     0.446925     0.460582     0.433267     4590.976074 | 0.195185  0.066746  0.057757  | 0.375676  0.414734  0.499089 
+2     | 0.000250  | 0.576423     | 0.359871     | 0.580197        | 0.245515     | 0.196682          | 0.465353     0.624025     0.274327     0.973723     2900.488525 | 0.497914     0.300710     0.186741     0.414680     2050.245605 | 0.430264  0.224227  0.012211  | 0.115812  0.172520  0.301715 
+3     | 0.000375  | 0.492849     | 0.302933     | 0.616778        | 0.261848     | 0.146602          | 0.436331     0.517070     0.113624     0.920517     1214.763062 | 0.482256     0.226080     0.080138     0.372022     740.208435  | 0.456992  0.242040  0.006338  | 0.116219  0.116918  0.206669 
+4     | 0.000500  | 0.405818     | 0.270811     | 0.682318        | 0.362785     | 0.104660          | 0.414673     0.402022     0.043417     0.760627     379.975830  | 0.482567     0.180058     0.038198     0.321919     190.140060  | 0.432209  0.259102  0.453139  | 0.091286  0.094286  0.128407 
+5     | 0.000483  | 0.278293     | 0.232456     | 0.731749        | 0.450538     | 0.080776          | 0.396638     0.227573     0.011783     0.443363     57.473202   | 0.449710     0.139347     0.027851     0.250842     20.436995   | 0.528865  0.326150  0.517442  | 0.076150  0.101664  0.064515 
+6     | 0.000438  | 0.201146     | 0.234689     | 0.734046        | 0.427178     | 0.061376          | 0.394785     0.118157     0.006779     0.229535     7.756716    | 0.459623     0.138289     0.033983     0.242596     17.634104   | 0.502815  0.351210  0.512020  | 0.065005  0.080777  0.038345 
+7     | 0.000375  | 0.178433     | 0.225379     | 0.758063        | 0.501010     | 0.070569          | 0.387485     0.088839     0.005728     0.171949     3.643147    | 0.459402     0.125084     0.033144     0.217025     13.697089   | 0.580658  0.350809  0.573669  | 0.077860  0.070224  0.063622 
+8     | 0.000313  | 0.165530     | 0.224868     | 0.753668        | 0.479545     | 0.063584          | 0.380244     0.073509     0.004988     0.142030     2.276982    | 0.450453     0.128189     0.034140     0.222237     12.516740   | 0.575804  0.364877  0.541543  | 0.067011  0.076683  0.047058 
+9     | 0.000267  | 0.157692     | 0.215701     | 0.760795        | 0.498372     | 0.064256          | 0.375279     0.064440     0.004682     0.124198     1.749302    | 0.434507     0.121927     0.035489     0.208365     15.635253   | 0.600246  0.349882  0.619524  | 0.075881  0.074971  0.041914 
+10    | 0.000250  | 0.153884     | 0.221742     | 0.748923        | 0.467832     | 0.063683          | 0.371269     0.060719     0.004419     0.117019     1.506790    | 0.434070     0.130743     0.038185     0.223302     14.687926   | 0.566790  0.354515  0.552122  | 0.071816  0.073918  0.045315 
+11    | 0.000250  | 0.157442     | 0.335919     | 0.739355        | 0.438376     | 0.059993          | 0.369201     0.066688     0.004419     0.110045     1.002835    | 0.459715     0.282864     0.041287     0.231711     14.772966   | 0.505808  0.342633  0.558486  | 0.065398  0.072597  0.041983 
+12    | 0.000500  | 0.167467     | 0.306602     | 0.727685        | 0.415524     | 0.064208          | 0.376363     0.077940     0.006141     0.129689     1.070466    | 0.508330     0.220148     0.043436     0.230597     8.450132    | 0.460519  0.310486  0.542453  | 0.053642  0.067742  0.071239 
+13    | 0.000438  | 0.160118     | 0.315148     | 0.749589        | 0.457981     | 0.056005          | 0.377731     0.066855     0.005557     0.115952     0.670835    | 0.448903     0.257825     0.045967     0.225953     12.322474   | 0.601255  0.333743  0.469267  | 0.068131  0.067295  0.032589 
+14    | 0.000313  | 0.154637     | 0.302202     | 0.765887        | 0.503222     | 0.059003          | 0.373271     0.060938     0.005176     0.107390     0.521767    | 0.462753     0.233395     0.039738     0.206487     11.151383   | 0.605460  0.369090  0.610828  | 0.066376  0.067162  0.043470 
+15    | 0.000250  | 0.146709     | 0.321047     | 0.751216        | 0.482994     | 0.069969          | 0.365419     0.052977     0.004322     0.094032     0.429098    | 0.436884     0.271403     0.047433     0.216716     14.064903   | 0.552918  0.371405  0.593197  | 0.068210  0.069943  0.071753</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+10 epochs : 0.5D + 0.5B
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+5 epochs :  0.01H + 0.495D + 0.495B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, …, 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-3
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(43m 53s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.739932     | 0.469884     | 0.386533        | 0.110816     | 0.429655          | 0.624698     0.789318     0.597018     0.981619     5537.404785 | 0.525314     0.446129     0.458970     0.433288     4577.714355 | 0.187437  0.067067  0.059816  | 0.375856  0.414228  0.498880 
+2     | 0.000250  | 0.576730     | 0.365744     | 0.565265        | 0.243160     | 0.219999          | 0.466777     0.623853     0.273882     0.973824     2902.868652 | 0.517833     0.300563     0.184722     0.416404     2029.493408 | 0.414560  0.219582  0.012931  | 0.138436  0.221672  0.299890 
+3     | 0.000375  | 0.491748     | 0.305112     | 0.619711        | 0.246605     | 0.131551          | 0.433043     0.516908     0.113539     0.920277     1215.650146 | 0.495551     0.223495     0.074956     0.372034     708.052917  | 0.466946  0.233796  0.005673  | 0.104605  0.104925  0.185124 
+4     | 0.000500  | 0.401309     | 0.261416     | 0.681327        | 0.399230     | 0.130609          | 0.411446     0.396965     0.042476     0.751453     372.290558  | 0.485848     0.165231     0.034433     0.296029     171.467972  | 0.501514  0.259557  0.458340  | 0.094796  0.140586  0.156446 
+5     | 0.000483  | 0.274714     | 0.245119     | 0.713871        | 0.397956     | 0.075519          | 0.399798     0.221107     0.010939     0.431276     51.106899   | 0.471585     0.148062     0.032054     0.264070     23.396763   | 0.380822  0.320325  0.549985  | 0.065955  0.080890  0.079713 
+6     | 0.000438  | 0.199671     | 0.237025     | 0.724242        | 0.425749     | 0.076763          | 0.396942     0.115126     0.006561     0.223691     7.102225    | 0.479624     0.133054     0.032504     0.233603     16.365000   | 0.482854  0.350266  0.529138  | 0.075805  0.112110  0.042373 
+7     | 0.000375  | 0.177424     | 0.228225     | 0.743945        | 0.487012     | 0.084767          | 0.390086     0.086283     0.005646     0.166921     3.470822    | 0.473759     0.122995     0.032233     0.213758     13.236599   | 0.518919  0.381805  0.592564  | 0.076584  0.073765  0.103952 
+8     | 0.000313  | 0.168149     | 0.231332     | 0.736960        | 0.466571     | 0.082781          | 0.383119     0.076020     0.005268     0.146771     2.252439    | 0.475919     0.126510     0.034841     0.218178     13.452687   | 0.541184  0.367127  0.562180  | 0.077642  0.079771  0.090930 
+9     | 0.000267  | 0.158601     | 0.225918     | 0.741639        | 0.453875     | 0.066519          | 0.375318     0.065722     0.004843     0.126601     1.744922    | 0.452339     0.128880     0.037608     0.220151     12.119533   | 0.543562  0.359773  0.535543  | 0.077170  0.069927  0.052460 
+10    | 0.000250  | 0.153245     | 0.225872     | 0.750691        | 0.479365     | 0.068424          | 0.370253     0.060242     0.004335     0.116150     1.489801    | 0.463379     0.124083     0.035995     0.212172     12.389678   | 0.577160  0.377533  0.567914  | 0.075996  0.078189  0.051086 
+11    | 0.000125  | 0.155850     | 0.300875     | 0.747705        | 0.455523     | 0.057508          | 0.366371     0.065627     0.004285     0.107544     1.027083    | 0.486334     0.221392     0.036803     0.222645     9.296569    | 0.523162  0.365378  0.568016  | 0.066647  0.064741  0.041136 
+12    | 0.000250  | 0.152971     | 0.283909     | 0.743094        | 0.434441     | 0.051138          | 0.365499     0.061888     0.004220     0.105073     0.778774    | 0.457100     0.209684     0.044450     0.237754     6.999365    | 0.521714  0.320559  0.539684  | 0.059675  0.055043  0.038695 
+13    | 0.000375  | 0.161753     | 0.312800     | 0.744486        | 0.460122     | 0.065938          | 0.370415     0.072326     0.005753     0.121039     0.956403    | 0.461981     0.248865     0.041850     0.219324     11.958438   | 0.527470  0.348599  0.580169  | 0.077550  0.071126  0.049137 
+14    | 0.000313  | 0.158379     | 0.315793     | 0.742725        | 0.453112     | 0.064200          | 0.377187     0.064604     0.005302     0.112998     0.604531    | 0.481217     0.244897     0.043048     0.217710     11.582143   | 0.492642  0.353029  0.586452  | 0.071720  0.065708  0.055172 
+15    | 0.000250  | 0.148606     | 0.290743     | 0.731232        | 0.413015     | 0.056623          | 0.367909     0.054619     0.004478     0.096461     0.465405    | 0.452849     0.221269     0.049497     0.245870     7.506310    | 0.475650  0.333340  0.508502  | 0.060352  0.059269  0.050249 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.01H + 0.495D + 0.495B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-3
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 18s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.685645     | 0.387409     | 0.473377        | 0.165906     | 0.321642          | 0.590916     0.726243     0.473105     0.979380     4571.039551 | 0.484221     0.345918     0.264333     0.427503     2884.082520 | 0.317444  0.118945  0.008758  | 0.260601  0.394780  0.309545 
+2     | 0.000500  | 0.507741     | 0.294440     | 0.670836        | 0.364987     | 0.125265          | 0.449079     0.532882     0.134215     0.931550     1444.178101 | 0.475142     0.216996     0.067979     0.366013     640.161133  | 0.503327  0.244704  0.351434  | 0.100633  0.103818  0.171345 
+3     | 0.000438  | 0.396773     | 0.255285     | 0.717825        | 0.416301     | 0.081159          | 0.413612     0.389557     0.039452     0.739662     323.866913  | 0.464245     0.165730     0.035045     0.296416     152.328690  | 0.494310  0.250540  0.570371  | 0.094775  0.093521  0.055180 
+4     | 0.000313  | 0.310800     | 0.244962     | 0.703317        | 0.405346     | 0.098036          | 0.391951     0.276021     0.019373     0.532669     82.199730   | 0.467318     0.149666     0.033526     0.265807     81.703041   | 0.510272  0.263373  0.511189  | 0.089146  0.095207  0.109754 
+5     | 0.000250  | 0.232960     | 0.236516     | 0.715537        | 0.400442     | 0.074399          | 0.381207     0.169425     0.008809     0.330041     24.606632   | 0.454569     0.143064     0.033005     0.253123     35.655914   | 0.440659  0.330671  0.526618  | 0.074666  0.104061  0.044470 
+6     | 0.000125  | 0.228107     | 0.370264     | 0.722045        | 0.390315     | 0.056801          | 0.378171     0.163794     0.005843     0.222532     5.074768    | 0.478150     0.324027     0.033661     0.254720     18.127777   | 0.429551  0.320403  0.510489  | 0.063053  0.075534  0.031816 
+7     | 0.000250  | 0.197558     | 0.318694     | 0.741499        | 0.450656     | 0.064606          | 0.383009     0.118079     0.006017     0.189079     2.150640    | 0.448258     0.263167     0.032667     0.226510     13.487482   | 0.554608  0.335680  0.550688  | 0.082591  0.069926  0.041301 
+8     | 0.000375  | 0.190517     | 0.289933     | 0.723878        | 0.395002     | 0.056872          | 0.389210     0.105363     0.006737     0.175879     1.496758    | 0.470128     0.212707     0.040728     0.249581     6.900355    | 0.416545  0.354699  0.501315  | 0.066698  0.060891  0.043028 
+9     | 0.000500  | 0.176044     | 0.332545     | 0.735252        | 0.438277     | 0.066765          | 0.388632     0.084935     0.006185     0.145568     0.981750    | 0.448761     0.282738     0.044584     0.240960     14.139382   | 0.546980  0.338773  0.488933  | 0.069275  0.086590  0.044430 
+10    | 0.000483  | 0.167861     | 0.312962     | 0.722469        | 0.400831     | 0.063106          | 0.381940     0.076113     0.005789     0.131982     0.791643    | 0.478308     0.242099     0.043875     0.239644     10.175707   | 0.426186  0.343133  0.537713  | 0.061105  0.070436  0.057779 
+11    | 0.000438  | 0.160760     | 0.319274     | 0.734719        | 0.419047     | 0.054834          | 0.379444     0.067038     0.005313     0.117979     0.600877    | 0.471882     0.253871     0.045118     0.232450     11.647522   | 0.454390  0.335970  0.565295  | 0.055049  0.074318  0.035134 
+12    | 0.000375  | 0.154658     | 0.314465     | 0.728687        | 0.404232     | 0.055009          | 0.372601     0.061254     0.004959     0.108570     0.505683    | 0.469509     0.248017     0.049099     0.242564     10.364390   | 0.455070  0.344095  0.495688  | 0.060809  0.067039  0.037180 
+13    | 0.000313  | 0.148488     | 0.305984     | 0.733258        | 0.434610     | 0.067643          | 0.365901     0.055310     0.004443     0.098833     0.418854    | 0.460149     0.239913     0.046682     0.229536     10.318450   | 0.508674  0.340237  0.541367  | 0.063125  0.080793  0.059011 
+14    | 0.000267  | 0.145808     | 0.295723     | 0.739492        | 0.444466     | 0.063823          | 0.363744     0.052407     0.004269     0.093934     0.379683    | 0.461741     0.224572     0.043802     0.225900     9.106997    | 0.516357  0.349304  0.562364  | 0.064741  0.078764  0.047966 
+15    | 0.000250  | 0.145473     | 0.301557     | 0.739205        | 0.436445     | 0.058955          | 0.363752     0.051924     0.004344     0.093062     0.370848    | 0.457477     0.234734     0.048113     0.232491     9.583490    | 0.489978  0.325297  0.572156  | 0.059788  0.073572  0.043506 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on full train-valid data
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 16m 9s)
+(Max GPU mem usage : 6632.875 MB)  
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.463445     | 0.195456     | 0.815970        | 0.631233     | 0.060873          | 0.495718     0.449613     0.134842     0.764386     1318.503662 | 0.454313     0.084517     0.012331     0.156703     19.978571   | 0.671350  0.538137  0.671386  | 0.056267  0.062034  0.064317 
+2     | 0.000500  | 0.210667     | 0.177933     | 0.839838        | 0.685344     | 0.057167          | 0.429021     0.117087     0.010453     0.223721     6.388138    | 0.445972     0.063059     0.014192     0.111926     6.113956    | 0.700582  0.616175  0.749939  | 0.064566  0.061275  0.045659 
+3     | 0.000438  | 0.181372     | 0.176996     | 0.837809        | 0.688310     | 0.062525          | 0.401104     0.087200     0.009155     0.165246     2.720654    | 0.447006     0.061277     0.015206     0.107349     6.861999    | 0.714058  0.620597  0.744451  | 0.079555  0.070505  0.037516 
+4     | 0.000313  | 0.166898     | 0.175204     | 0.849460        | 0.702569     | 0.052612          | 0.383960     0.073871     0.007952     0.139789     1.854562    | 0.435694     0.063566     0.016081     0.111050     5.640822    | 0.717189  0.628290  0.762603  | 0.051293  0.071053  0.035491 
+5     | 0.000250  | 0.159371     | 0.173484     | 0.850093        | 0.697004     | 0.047847          | 0.374196     0.067303     0.007231     0.127376     1.403342    | 0.426928     0.064865     0.017236     0.112494     6.298545    | 0.714597  0.616786  0.773478  | 0.062645  0.053251  0.027646 
+6     | 0.000125  | 0.164320     | 0.221254     | 0.859016        | 0.710684     | 0.042096          | 0.366608     0.077625     0.007497     0.124480     0.647772    | 0.426216     0.133413     0.016812     0.106084     3.659695    | 0.732362  0.641976  0.762352  | 0.049663  0.050917  0.025708 
+7     | 0.000250  | 0.166527     | 0.223539     | 0.850564        | 0.691673     | 0.043509          | 0.370247     0.079218     0.008300     0.128871     0.600201    | 0.440171     0.130696     0.017731     0.109993     3.405572    | 0.712950  0.618470  0.750548  | 0.056874  0.050351  0.023304 
+8     | 0.000375  | 0.171262     | 0.222871     | 0.853117        | 0.697751     | 0.043306          | 0.376991     0.083093     0.009120     0.135800     0.604093    | 0.429962     0.134117     0.018952     0.112629     3.482126    | 0.704174  0.629621  0.777163  | 0.038003  0.061534  0.030382 
+9     | 0.000500  | 0.175396     | 0.221959     | 0.851903        | 0.689514     | 0.039838          | 0.381263     0.087167     0.009560     0.142513     0.632526    | 0.437945     0.129394     0.017753     0.113748     3.247951    | 0.710469  0.605422  0.757743  | 0.048630  0.047440  0.023443 
+10    | 0.000483  | 0.163890     | 0.212613     | 0.853875        | 0.700669     | 0.043988          | 0.374967     0.073428     0.008023     0.122341     0.477490    | 0.430642     0.119172     0.017565     0.108016     2.881872    | 0.716335  0.621675  0.787307  | 0.053564  0.046914  0.031485 
+11    | 0.000438  | 0.161228     | 0.222626     | 0.854880        | 0.702665     | 0.043643          | 0.370474     0.071551     0.007770     0.119284     0.464713    | 0.441519     0.128814     0.016998     0.105658     3.435635    | 0.718089  0.628847  0.772014  | 0.052458  0.048205  0.030267 
+12    | 0.000375  | 0.157936     | 0.211722     | 0.855635        | 0.701081     | 0.041329          | 0.366689     0.068471     0.007366     0.114798     0.430551    | 0.430676     0.117884     0.018203     0.109879     2.756193    | 0.713983  0.623212  0.784325  | 0.048273  0.053412  0.022303 
+13    | 0.000313  | 0.152110     | 0.218535     | 0.861845        | 0.718181     | 0.042378          | 0.361308     0.062453     0.006677     0.105995     0.362189    | 0.436520     0.125113     0.017004     0.101009     3.364369    | 0.736297  0.637635  0.786831  | 0.052647  0.050694  0.023794 
+14    | 0.000267  | 0.148685     | 0.218303     | 0.863022        | 0.718275     | 0.040479          | 0.357553     0.059170     0.006189     0.101023     0.331834    | 0.427092     0.128821     0.017773     0.103436     3.471454    | 0.737546  0.636630  0.785716  | 0.049228  0.048473  0.023738 
+15    | 0.000250  | 0.147484     | 0.218030     | 0.863845        | 0.722265     | 0.041768          | 0.355461     0.058351     0.006206     0.099710     0.322595    | 0.431362     0.126601     0.017503     0.101444     3.415887    | 0.736793  0.642503  0.791408  | 0.049166  0.050731  0.025406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2444  1907  1468
+FP   187   201    87
+FN   133   162    58
+TN  4532  5026  5683
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.335  0.261  0.201
+FP  0.026  0.028  0.012
+FN  0.018  0.022  0.008
+TN  0.621  0.689  0.779
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+-----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.218030     | 0.863845        | 0.722265     | 0.041768          | 0.431362     0.126601     0.017503     0.101444     3.415887    | 0.736793  0.642503  0.791408  | 0.049166  0.050731  0.025406 
+266     | 266     | 0.220494     | 0.866130        | 0.729936     | 0.043074          | 0.427199     0.131906     0.018093     0.101275     3.670799    | 0.747083  0.647900  0.795873  | 0.050888  0.052360  0.025973 
+360     | 310     | 0.185561     | 0.833194        | 0.635865     | 0.035253          | 0.464911     0.065840     0.009581     0.096236     0.699464    | 0.594724  0.565700  0.794233  | 0.041705  0.046301  0.017754 
+276     | 276     | 0.229412     | 0.869902        | 0.721056     | 0.030867          | 0.463235     0.129202     0.020567     0.118512     3.052676    | 0.772302  0.655716  0.712317  | 0.033286  0.032209  0.027104 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(29m 25s)
+Cutoffs(LB,SB,S) | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.213134     | 0.866542        | 0.729533     | 0.042118          | 0.428545     0.120815     0.016800     0.097486     3.240755    | 0.748539  0.654691  0.799641  | 0.049029  0.051855  0.025470 
+(0.25,0.25,0.25) | 0.213134     | 0.867552        | 0.728947     | 0.040044          | 0.428545     0.120815     0.016800     0.097486     3.240755    | 0.742073  0.656042  0.803113  | 0.049029  0.047637  0.023466 
+(0.50,0.50,0.50) | 0.213134     | 0.868263        | 0.730091     | 0.039622          | 0.428545     0.120815     0.016800     0.097486     3.240755    | 0.742243  0.656388  0.804964  | 0.048267  0.047637  0.022961 
+(0.75,0.75,0.75) | 0.213134     | 0.868686        | 0.730723     | 0.039338          | 0.428545     0.120815     0.016800     0.097486     3.240755    | 0.741791  0.657679  0.808338  | 0.048225  0.047411  0.022377 
+(0.60,0.70,0.70) | 0.213134     | 0.868889        | 0.731474     | 0.039500          | 0.428545     0.120815     0.016800     0.097486     3.240755    | 0.741600  0.656983  0.806681  | 0.048267  0.047411  0.022823 
+(0.60,0.70,0.80) | 0.213134     | 0.869013        | 0.731429     | 0.039265          | 0.428545     0.120815     0.016800     0.097486     3.240755    | 0.741600  0.656983  0.807679  | 0.048267  0.047411  0.022115 
+(0.50,0.75,0.75) | 0.213134     | 0.869063        | 0.731687     | 0.039352          | 0.428545     0.120815     0.016800     0.097486     3.240755    | 0.742243  0.657679  0.808338  | 0.048267  0.047411  0.022377 
+(0.5, 0.75, 0.75) tensor(0.8691)
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2458  1916  1470
+FP   192   187    68
+FN   119   153    56
+TN  4527  5040  5702
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.337  0.263  0.201
+FP  0.026  0.026  0.009
+FN  0.016  0.021  0.008
+TN  0.620  0.691  0.782
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+-----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.213134     | 0.869063        | 0.731687     | 0.039352          | 0.428545     0.120815     0.016800     0.097486     3.240755    | 0.742243  0.657679  0.808338  | 0.048267  0.047411  0.022377 
+266     | 266     | 0.215747     | 0.870533        | 0.737492     | 0.040773          | 0.423950     0.126517     0.017413     0.097852     3.501848    | 0.749164  0.661982  0.812966  | 0.050381  0.049164  0.022774 
+360     | 310     | 0.179114     | 0.844630        | 0.657749     | 0.030783          | 0.462525     0.057653     0.008753     0.086517     0.548519    | 0.622300  0.589946  0.819412  | 0.038910  0.039192  0.014246 
+276     | 276     | 0.224236     | 0.879358        | 0.742588     | 0.029463          | 0.471050     0.118458     0.019553     0.113930     2.652566    | 0.799847  0.677048  0.712939  | 0.029043  0.032083  0.027262 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA cutoff (0.5, 0.75, 0.75)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA cutoff (0.6, 0.7, 0.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA cutoff (0.6, 0.7, 0.7)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF3465A4"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">weight decay 1e-3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 14s)
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.684441     | 0.393364     | 0.475949        | 0.172964     | 0.322060          | 0.587050     0.726180     0.473006     0.979354     4573.292969 | 0.498674     0.348231     0.269412     0.427049     2916.253906 | 0.314610  0.138898  0.014244  | 0.262167  0.395372  0.308641 
+2     | 0.000500  | 0.508583     | 0.306754     | 0.633235        | 0.270603     | 0.125010          | 0.452632     0.532562     0.134662     0.930464     1447.625244 | 0.503673     0.222360     0.068051     0.376668     642.453064  | 0.419760  0.229764  0.148509  | 0.094905  0.098546  0.181579 
+3     | 0.000438  | 0.398776     | 0.259291     | 0.693273        | 0.391844     | 0.105774          | 0.417420     0.390786     0.039579     0.741993     324.469849  | 0.474726     0.166962     0.034985     0.298939     148.462540  | 0.493761  0.217704  0.564374  | 0.090120  0.093852  0.133350 
+4     | 0.000313  | 0.313163     | 0.241488     | 0.715015        | 0.427234     | 0.093131          | 0.395809     0.277743     0.019804     0.535681     84.251701   | 0.462011     0.146978     0.034489     0.259466     87.926559   | 0.556491  0.270175  0.499811  | 0.092416  0.118725  0.068252 
+5     | 0.000250  | 0.232591     | 0.225876     | 0.738599        | 0.470848     | 0.082900          | 0.382544     0.168325     0.008260     0.328390     23.495085   | 0.457409     0.126647     0.025288     0.228006     24.919209   | 0.565792  0.343712  0.571926  | 0.092662  0.085488  0.070550 
+6     | 0.000125  | 0.254107     | 0.383410     | 0.732373        | 0.409724     | 0.052528          | 0.379821     0.200230     0.006148     0.227359     4.290578    | 0.470676     0.346010     0.031326     0.251055     10.382164   | 0.444974  0.339823  0.532205  | 0.043783  0.073377  0.040425 
+7     | 0.000250  | 0.202861     | 0.352521     | 0.755223        | 0.463214     | 0.050105          | 0.384274     0.125113     0.006266     0.187475     1.509026    | 0.452788     0.309550     0.032860     0.229886     9.040180    | 0.579178  0.308927  0.567106  | 0.067695  0.059531  0.023089 
+8     | 0.000375  | 0.209603     | 0.404422     | 0.709544        | 0.371738     | 0.065252          | 0.391309     0.131729     0.008470     0.199195     1.498634    | 0.482419     0.370994     0.042891     0.263797     11.035830   | 0.436768  0.302646  0.447401  | 0.074757  0.085166  0.035832 
+9     | 0.000500  | 0.187187     | 0.360403     | 0.749770        | 0.461986     | 0.058374          | 0.398548     0.096603     0.007081     0.160432     0.726086    | 0.457304     0.318874     0.040224     0.234959     9.201733    | 0.540595  0.329836  0.599880  | 0.072041  0.062363  0.040719 
+10    | 0.000483  | 0.173162     | 0.356587     | 0.740703        | 0.434138     | 0.054921          | 0.384070     0.082774     0.006156     0.139040     0.581360    | 0.453563     0.315027     0.042665     0.237482     8.887741    | 0.496378  0.355181  0.533928  | 0.048430  0.066799  0.049534 
+11    | 0.000438  | 0.164829     | 0.377473     | 0.734242        | 0.419666     | 0.056040          | 0.381219     0.072091     0.005809     0.122796     0.453729    | 0.472390     0.336794     0.042834     0.232652     10.090305   | 0.468580  0.340804  0.574367  | 0.060953  0.067829  0.039337 
+12    | 0.000375  | 0.157901     | 0.379008     | 0.746416        | 0.453573     | 0.058355          | 0.372639     0.065870     0.005164     0.112813     0.403055    | 0.459326     0.344586     0.043676     0.223663     10.679494   | 0.536600  0.355106  0.564007  | 0.071370  0.069174  0.034521 
+13    | 0.000313  | 0.152134     | 0.390545     | 0.750561        | 0.466999     | 0.060397          | 0.366819     0.060126     0.004878     0.103821     0.343172    | 0.452219     0.364114     0.044867     0.221179     11.687554   | 0.546481  0.359579  0.600931  | 0.071137  0.069648  0.040406 
+14    | 0.000267  | 0.150236     | 0.353292     | 0.739981        | 0.441100     | 0.060764          | 0.365912     0.057804     0.004714     0.100605     0.309868    | 0.463336     0.306131     0.044474     0.229804     8.586725    | 0.517656  0.364801  0.542566  | 0.070416  0.068638  0.043238 
+15    | 0.000250  | 0.146735     | 0.363541     | 0.745322        | 0.461005     | 0.065133          | 0.363191     0.053967     0.004377     0.094021     0.287614    | 0.444383     0.328895     0.044495     0.222488     9.903646    | 0.531308  0.363243  0.587618  | 0.077566  0.074109  0.043723 </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF3465A4"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">weight decay 1e-2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 26s)
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.683531     | 0.386288     | 0.469428        | 0.160230     | 0.324439          | 0.583681     0.726325     0.473364     0.979285     4574.341797 | 0.478897     0.346598     0.265529     0.427667     2887.679443 | 0.322999  0.124619  0.006621  | 0.261549  0.402056  0.309713 
+2     | 0.000500  | 0.509254     | 0.314846     | 0.656654        | 0.289459     | 0.098549          | 0.454161     0.532865     0.134441     0.931290     1442.688599 | 0.524293     0.225083     0.066454     0.383713     615.967834  | 0.418812  0.219374  0.204174  | 0.092451  0.090460  0.112736 
+3     | 0.000438  | 0.397108     | 0.256648     | 0.701089        | 0.415159     | 0.108291          | 0.416008     0.389008     0.039390     0.738627     324.805573  | 0.461477     0.168865     0.044043     0.293686     203.975586  | 0.492872  0.252632  0.528715  | 0.113932  0.128992  0.081948 
+4     | 0.000313  | 0.311101     | 0.235234     | 0.719293        | 0.448429     | 0.100132          | 0.395736     0.274829     0.018697     0.530962     80.984711   | 0.450630     0.142922     0.025115     0.260728     64.080864   | 0.602394  0.285189  0.496859  | 0.091668  0.100889  0.107837 
+5     | 0.000250  | 0.225260     | 0.226596     | 0.734996        | 0.461840     | 0.082900          | 0.385485     0.156593     0.007187     0.305998     18.358646   | 0.453463     0.129366     0.027304     0.231429     28.490110   | 0.531654  0.372427  0.547367  | 0.076412  0.108711  0.063578 
+6     | 0.000125  | 0.248928     | 0.361931     | 0.728876        | 0.413918     | 0.061152          | 0.380037     0.192738     0.006053     0.222868     4.028348    | 0.461578     0.319225     0.031298     0.246587     9.153091    | 0.476196  0.345515  0.498696  | 0.059320  0.079623  0.044513 
+7     | 0.000250  | 0.205781     | 0.348577     | 0.740523        | 0.451222     | 0.066609          | 0.385003     0.128972     0.006420     0.192681     1.570625    | 0.442689     0.308243     0.034084     0.232074     8.891302    | 0.455387  0.369918  0.589729  | 0.056114  0.076277  0.067435 
+8     | 0.000375  | 0.186790     | 0.349566     | 0.735343        | 0.424130     | 0.057183          | 0.388211     0.100466     0.006336     0.162721     0.881409    | 0.472961     0.296682     0.038455     0.235028     8.133771    | 0.492412  0.361831  0.506481  | 0.063167  0.076900  0.031480 
+9     | 0.000500  | 0.183627     | 0.353542     | 0.744579        | 0.447301     | 0.057235          | 0.388043     0.096019     0.006978     0.157018     0.783082    | 0.522292     0.281220     0.043817     0.242055     7.057135    | 0.541474  0.295623  0.572851  | 0.062263  0.061227  0.048215 
+10    | 0.000483  | 0.176824     | 0.370644     | 0.705943        | 0.354719     | 0.059908          | 0.384794     0.087694     0.006673     0.145978     0.644760    | 0.455395     0.334322     0.052705     0.273901     8.714285    | 0.384219  0.335237  0.409359  | 0.059051  0.068427  0.052246 
+11    | 0.000438  | 0.169096     | 0.396048     | 0.728978        | 0.413999     | 0.061035          | 0.384497     0.076780     0.006166     0.129777     0.508422    | 0.470104     0.364309     0.045437     0.238395     11.261598   | 0.476224  0.308183  0.551490  | 0.059755  0.083158  0.040192 
+12    | 0.000375  | 0.158016     | 0.383101     | 0.733454        | 0.421205     | 0.058379          | 0.372806     0.065963     0.005254     0.113316     0.393181    | 0.474249     0.344038     0.047370     0.238292     10.203147   | 0.476124  0.313694  0.573201  | 0.062119  0.074472  0.038548 
+13    | 0.000313  | 0.150236     | 0.381620     | 0.744017        | 0.452313     | 0.061513          | 0.365516     0.057974     0.004671     0.099980     0.334741    | 0.453521     0.350804     0.044569     0.224840     10.939691   | 0.540340  0.332102  0.564895  | 0.069046  0.067997  0.047497 
+14    | 0.000267  | 0.149273     | 0.351099     | 0.741706        | 0.444181     | 0.059944          | 0.364456     0.057052     0.004621     0.098854     0.317464    | 0.470094     0.300101     0.044365     0.229503     8.295287    | 0.534408  0.343194  0.540208  | 0.069214  0.073080  0.037538 
+15    | 0.000250  | 0.146851     | 0.358286     | 0.740685        | 0.446464     | 0.063167          | 0.362679     0.054353     0.004445     0.094436     0.295059    | 0.454078     0.317232     0.044900     0.223739     9.279951    | 0.513410  0.355200  0.578745  | 0.068650  0.082061  0.038791 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+diff = torch.abs(seg_pred - seg_true)
+hd_loss = (dist_map * diff).sum(dim=(2,3)) / seg_true.sum(dim=(2,3)).clamp(min=1)
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 41s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">taken as new best run 
+With Haus surro
+In data subset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.684028     | 0.385609     | 0.469708        | 0.163152     | 0.325922          | 0.585853     0.726103     0.472937     0.979269     4.565955    | 0.476089     0.346833     0.265944     0.427721     2.643569    | 0.312823  0.116371  0.014525  | 0.268096  0.394803  0.314866 
+2     | 0.000500  | 0.508741     | 0.289804     | 0.654754        | 0.340967     | 0.136054          | 0.452858     0.532691     0.134423     0.930960     1.428040    | 0.452641     0.220016     0.068273     0.371759     0.510672    | 0.479823  0.244437  0.276509  | 0.108641  0.116256  0.183266 
+3     | 0.000438  | 0.397270     | 0.257831     | 0.703898        | 0.424163     | 0.109612          | 0.416035     0.389228     0.039304     0.739151     0.344429    | 0.465527     0.168818     0.038771     0.298865     0.147855    | 0.535909  0.239186  0.528756  | 0.110982  0.136398  0.081455 
+4     | 0.000313  | 0.313928     | 0.237934     | 0.719544        | 0.447246     | 0.098925          | 0.395781     0.278848     0.020076     0.537621     0.088989    | 0.448270     0.147790     0.035720     0.259860     0.105944    | 0.566784  0.273302  0.541503  | 0.103702  0.124986  0.068086 
+5     | 0.000250  | 0.239204     | 0.224939     | 0.744688        | 0.477978     | 0.077505          | 0.384214     0.177057     0.009491     0.344622     0.028992    | 0.452444     0.127436     0.025928     0.228944     0.022338    | 0.570098  0.337570  0.575524  | 0.072650  0.081559  0.078305 
+6     | 0.000125  | 0.188711     | 0.223618     | 0.751433        | 0.484335     | 0.070501          | 0.376937     0.108043     0.005320     0.214858     0.007811    | 0.457354     0.123446     0.026424     0.224904     0.014748    | 0.595045  0.341937  0.571466  | 0.073381  0.076489  0.061634 
+7     | 0.000250  | 0.179333     | 0.214025     | 0.750647        | 0.501079     | 0.082975          | 0.379837     0.093403     0.005225     0.185187     0.005052    | 0.438399     0.117865     0.027138     0.212847     0.013605    | 0.602627  0.368713  0.573697  | 0.074558  0.084760  0.089607 
+8     | 0.000375  | 0.173643     | 0.224868     | 0.756491        | 0.482860     | 0.061088          | 0.385766     0.082733     0.005423     0.163298     0.003005    | 0.457206     0.125295     0.032235     0.223099     0.009047    | 0.603096  0.314759  0.588220  | 0.067831  0.069638  0.045795 
+9     | 0.000500  | 0.170634     | 0.240628     | 0.735718        | 0.431651     | 0.061570          | 0.389124     0.076996     0.005924     0.151116     0.002310    | 0.465541     0.144237     0.043628     0.250381     0.008608    | 0.517026  0.327014  0.499743  | 0.064596  0.068172  0.051942 
+10    | 0.000483  | 0.168843     | 0.232582     | 0.743270        | 0.454832     | 0.064438          | 0.388781     0.074584     0.005948     0.146188     0.001834    | 0.456597     0.136576     0.040955     0.237381     0.009565    | 0.469634  0.367432  0.573249  | 0.065824  0.076507  0.050984 
+11    | 0.000438  | 0.157988     | 0.231943     | 0.745574        | 0.460599     | 0.064443          | 0.382458     0.061787     0.005091     0.120961     0.001059    | 0.464653     0.132211     0.039951     0.229442     0.010390    | 0.548598  0.343315  0.573779  | 0.067446  0.081866  0.044017 
+12    | 0.000375  | 0.148415     | 0.220292     | 0.745757        | 0.478959     | 0.076378          | 0.370098     0.053409     0.004455     0.104511     0.000759    | 0.446125     0.123507     0.039902     0.211720     0.010597    | 0.594563  0.373259  0.542096  | 0.070295  0.077028  0.081810 
+13    | 0.000313  | 0.144481     | 0.219918     | 0.757882        | 0.496430     | 0.067817          | 0.364496     0.050189     0.004204     0.098197     0.000625    | 0.445898     0.123069     0.040285     0.210411     0.011415    | 0.620751  0.362705  0.577413  | 0.064606  0.080310  0.058534 
+14    | 0.000267  | 0.142912     | 0.217328     | 0.759043        | 0.504497     | 0.071261          | 0.364421     0.047980     0.004057     0.093839     0.000549    | 0.441003     0.121467     0.038559     0.208949     0.009409    | 0.619428  0.371385  0.580317  | 0.075916  0.080758  0.057108 
+15    | 0.000250  | 0.139732     | 0.216311     | 0.762237        | 0.502708     | 0.064744          | 0.360623     0.045065     0.003750     0.088202     0.000447    | 0.429667     0.124872     0.041365     0.213012     0.011357    | 0.616720  0.360522  0.583792  | 0.069476  0.079108  0.045648 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+diff = torch.abs(seg_pred - seg_true)
+hd_loss = (dist_map * diff).sum(dim=(2,3)) / seg_true.sum(dim=(2,3)).clamp(min=1)
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.1H + 0.45D + 0.45B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 31s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.683341     | 0.389554     | 0.466142        | 0.149854     | 0.322999          | 0.583030     0.726332     0.473145     0.979518     4.702015    | 0.487408     0.347616     0.267297     0.427935     2.643010    | 0.292383  0.123730  0.009248  | 0.264482  0.394655  0.309859 
+2     | 0.000500  | 0.508864     | 0.298956     | 0.659794        | 0.371146     | 0.147773          | 0.454099     0.532336     0.134270     0.930400     1.427420    | 0.484912     0.219261     0.067906     0.370616     0.510424    | 0.475083  0.248827  0.405105  | 0.101668  0.097314  0.244338 
+3     | 0.000438  | 0.395156     | 0.253795     | 0.708504        | 0.413515     | 0.094836          | 0.410466     0.388595     0.038708     0.738482     0.346338    | 0.456294     0.167010     0.036772     0.297247     0.129417    | 0.508081  0.242138  0.541036  | 0.090184  0.112171  0.082153 
+4     | 0.000313  | 0.308648     | 0.247075     | 0.713950        | 0.410876     | 0.084001          | 0.392476     0.272721     0.019008     0.526434     0.085037    | 0.469838     0.151605     0.030713     0.272498     0.069871    | 0.537650  0.264565  0.490866  | 0.079734  0.112299  0.059969 
+5     | 0.000250  | 0.227454     | 0.225395     | 0.750612        | 0.485176     | 0.072430          | 0.380552     0.161841     0.007890     0.315791     0.021589    | 0.455395     0.126823     0.027243     0.226404     0.019455    | 0.557020  0.348930  0.607715  | 0.082556  0.071834  0.062899 
+6     | 0.000125  | 0.181966     | 0.225140     | 0.741899        | 0.450603     | 0.063904          | 0.378420     0.097771     0.005276     0.210366     0.007320    | 0.467597     0.121230     0.029775     0.234856     0.021456    | 0.497383  0.337604  0.581620  | 0.062985  0.085730  0.042997 
+7     | 0.000250  | 0.173539     | 0.216920     | 0.750021        | 0.472874     | 0.065214          | 0.379261     0.085372     0.005128     0.183474     0.005014    | 0.458488     0.113391     0.029198     0.219773     0.013539    | 0.525361  0.351448  0.594651  | 0.075812  0.072664  0.047166 
+8     | 0.000375  | 0.169455     | 0.225680     | 0.748852        | 0.466761     | 0.063087          | 0.386415     0.076471     0.005352     0.163945     0.002880    | 0.463872     0.123598     0.038383     0.233913     0.010644    | 0.547892  0.344670  0.536689  | 0.071008  0.081204  0.037048 
+9     | 0.000500  | 0.165687     | 0.227964     | 0.746719        | 0.457475     | 0.060452          | 0.386476     0.071063     0.005719     0.151715     0.002178    | 0.472282     0.123256     0.038845     0.233736     0.005948    | 0.550651  0.345850  0.540368  | 0.067444  0.066300  0.047611 
+10    | 0.000483  | 0.159652     | 0.226648     | 0.725499        | 0.436590     | 0.081895          | 0.381351     0.064638     0.005570     0.137730     0.001525    | 0.477742     0.119036     0.038152     0.223053     0.014937    | 0.498337  0.371221  0.519042  | 0.094743  0.097195  0.053746 
+11    | 0.000438  | 0.154126     | 0.223075     | 0.739318        | 0.448404     | 0.066739          | 0.379711     0.057447     0.005128     0.122291     0.001085    | 0.466095     0.118923     0.039974     0.221157     0.014143    | 0.530059  0.347603  0.553287  | 0.080990  0.072059  0.047169 
+12    | 0.000375  | 0.146516     | 0.214681     | 0.755908        | 0.480743     | 0.060649          | 0.370574     0.050491     0.004506     0.107527     0.000762    | 0.440238     0.118013     0.040974     0.218816     0.011077    | 0.576587  0.353983  0.561214  | 0.068079  0.075897  0.037971 
+13    | 0.000313  | 0.141091     | 0.218822     | 0.754244        | 0.487054     | 0.067628          | 0.363098     0.045946     0.004072     0.097876     0.000697    | 0.465817     0.112967     0.040883     0.207852     0.010367    | 0.572989  0.344767  0.582088  | 0.067773  0.075259  0.059853 
+14    | 0.000267  | 0.139334     | 0.215886     | 0.755069        | 0.482484     | 0.063208          | 0.362350     0.043756     0.003857     0.093252     0.000569    | 0.448254     0.116300     0.040915     0.215306     0.010003    | 0.577161  0.351981  0.565737  | 0.066936  0.077551  0.045137 
+15    | 0.000250  | 0.138306     | 0.213992     | 0.750347        | 0.484623     | 0.072503          | 0.362106     0.042391     0.003850     0.090243     0.000494    | 0.443683     0.115553     0.042733     0.211613     0.010978    | 0.580339  0.361688  0.583372  | 0.084780  0.084108  0.048621 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+diff = torch.abs(seg_pred - seg_true)
+hd_loss = (dist_map * diff).sum(dim=(2,3)) / seg_true.sum(dim=(2,3)).clamp(min=1)
+Then * presence_true and normalize by presence_true
+10 epochs : 0.5D + 0.5B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+5 epochs : 0.02H + 0.49D + 0.49B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 52s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.739901     | 0.461302     | 0.386600        | 0.111112     | 0.429742          | 0.624444     0.789383     0.597079     0.981687     5.589654    | 0.497915     0.445611     0.458026     0.433196     4.095581    | 0.194176  0.069915  0.058181  | 0.375128  0.415004  0.499095 
+2     | 0.000250  | 0.577088     | 0.358503     | 0.571925        | 0.237989     | 0.205451          | 0.467657     0.623987     0.274118     0.973855     2.867632    | 0.493578     0.300613     0.185946     0.415280     1.874836    | 0.418680  0.214390  0.007257  | 0.117044  0.202345  0.296965 
+3     | 0.000375  | 0.492902     | 0.310214     | 0.634707        | 0.275045     | 0.125519          | 0.435379     0.517555     0.113642     0.921469     1.249490    | 0.512029     0.223721     0.074197     0.373246     0.572981    | 0.503446  0.246103  0.010400  | 0.099757  0.100028  0.176771 
+4     | 0.000500  | 0.403799     | 0.266098     | 0.685613        | 0.377047     | 0.108675          | 0.412044     0.400265     0.042670     0.757861     0.395964    | 0.485030     0.172270     0.034847     0.309693     0.122849    | 0.484192  0.247987  0.434740  | 0.099105  0.093923  0.132998 
+5     | 0.000483  | 0.276449     | 0.229354     | 0.726715        | 0.461486     | 0.096466          | 0.396438     0.225025     0.011580     0.438470     0.058846    | 0.449315     0.135085     0.028242     0.241929     0.032397    | 0.545508  0.348555  0.535023  | 0.099121  0.130337  0.059938 
+6     | 0.000438  | 0.199134     | 0.234033     | 0.740730        | 0.477893     | 0.084045          | 0.394284     0.115499     0.006502     0.224495     0.007436    | 0.490932     0.123933     0.028368     0.219498     0.015363    | 0.534139  0.363192  0.595154  | 0.075324  0.114720  0.062090 
+7     | 0.000375  | 0.176075     | 0.230022     | 0.748149        | 0.491785     | 0.080942          | 0.386134     0.086050     0.005555     0.166544     0.003351    | 0.473173     0.125815     0.031032     0.220597     0.011620    | 0.526075  0.351301  0.637620  | 0.087057  0.101538  0.054230 
+8     | 0.000313  | 0.165289     | 0.224700     | 0.745838        | 0.470602     | 0.070671          | 0.380231     0.073170     0.005040     0.141301     0.002004    | 0.453594     0.126603     0.032956     0.220250     0.012686    | 0.569881  0.338447  0.568874  | 0.072297  0.082057  0.057660 
+9     | 0.000267  | 0.159808     | 0.223200     | 0.750815        | 0.487117     | 0.073387          | 0.376016     0.067147     0.004977     0.129317     0.001543    | 0.444871     0.128198     0.036622     0.219775     0.013259    | 0.562285  0.342301  0.621729  | 0.079029  0.085418  0.055715 
+10    | 0.000250  | 0.152907     | 0.226209     | 0.748539        | 0.469518     | 0.065446          | 0.370191     0.059785     0.004434     0.115137     0.001238    | 0.444764     0.132542     0.037909     0.227176     0.011588    | 0.548821  0.339092  0.577166  | 0.071300  0.079949  0.045090 
+11    | 0.000250  | 0.148771     | 0.231399     | 0.750686        | 0.472283     | 0.063712          | 0.367862     0.054875     0.004236     0.107712     0.001028    | 0.478647     0.125436     0.036714     0.218856     0.010314    | 0.566482  0.360258  0.541043  | 0.069029  0.081623  0.040484 
+12    | 0.000500  | 0.152754     | 0.232709     | 0.740776        | 0.458655     | 0.071143          | 0.374077     0.057901     0.004726     0.113401     0.000937    | 0.472848     0.129793     0.041609     0.222884     0.009546    | 0.565089  0.361367  0.509169  | 0.069260  0.079619  0.064549 
+13    | 0.000438  | 0.153081     | 0.221684     | 0.748765        | 0.507187     | 0.090183          | 0.374584     0.058151     0.005003     0.113632     0.000998    | 0.452629     0.122707     0.039308     0.210671     0.010867    | 0.593729  0.337901  0.617701  | 0.088657  0.087583  0.094308 
+14    | 0.000313  | 0.146835     | 0.228993     | 0.737519        | 0.474234     | 0.086958          | 0.369244     0.051517     0.004393     0.100709     0.000858    | 0.466545     0.127185     0.040543     0.218719     0.007302    | 0.544441  0.358528  0.575115  | 0.074636  0.092805  0.093434 
+15    | 0.000250  | 0.141845     | 0.224478     | 0.746982        | 0.468371     | 0.067278          | 0.363256     0.046955     0.003956     0.091847     0.000560    | 0.440262     0.131999     0.045891     0.223124     0.009097    | 0.556834  0.337194  0.560159  | 0.074580  0.087127  0.040127 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+diff = torch.abs(seg_pred - seg_true)
+hd_loss = (dist_map * diff).sum(dim=(2,3)) / seg_true.sum(dim=(2,3)).clamp(min=1)
+Then * presence_true and normalize by presence_true
+5 epochs : 0.25D + 0.75B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.02H + 0.24D + 0.74B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 26s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.597854     | 0.364519     | 0.410156        | 0.011774     | 0.324256          | 0.593266     0.599820     0.472693     0.981202     4.573734    | 0.512698     0.301014     0.257352     0.432001     2.593790    | 0.031567  0.001301  0.001012  | 0.259083  0.396272  0.317415 
+2     | 0.000500  | 0.373891     | 0.269647     | 0.654049        | 0.313299     | 0.118785          | 0.450579     0.341025     0.133820     0.962640     1.427872    | 0.535480     0.155719     0.076044     0.394743     0.708163    | 0.363962  0.211063  0.400269  | 0.126218  0.090388  0.139748 
+3     | 0.000438  | 0.300695     | 0.221651     | 0.700962        | 0.389785     | 0.091587          | 0.416428     0.251096     0.050354     0.853320     0.527268    | 0.463991     0.117791     0.043315     0.341216     0.309320    | 0.489150  0.239697  0.486258  | 0.096447  0.095954  0.082359 
+4     | 0.000313  | 0.256449     | 0.211179     | 0.706505        | 0.399795     | 0.089022          | 0.392399     0.198186     0.024850     0.718192     0.223164    | 0.462342     0.103538     0.030544     0.322521     0.146272    | 0.421068  0.300769  0.525293  | 0.077770  0.098229  0.091066 
+5     | 0.000250  | 0.217698     | 0.200005     | 0.729528        | 0.444305     | 0.080323          | 0.381987     0.147288     0.012556     0.551483     0.095721    | 0.462337     0.087578     0.025838     0.272795     0.068893    | 0.498565  0.320255  0.581036  | 0.071857  0.097933  0.071179 
+6     | 0.000125  | 0.190156     | 0.204199     | 0.731364        | 0.423980     | 0.063714          | 0.377970     0.109664     0.008146     0.427794     0.048261    | 0.480304     0.085868     0.026788     0.271397     0.045478    | 0.448164  0.321272  0.588632  | 0.063562  0.078002  0.049577 
+7     | 0.000250  | 0.173042     | 0.188252     | 0.747715        | 0.481257     | 0.074647          | 0.377200     0.085546     0.006278     0.334915     0.026017    | 0.447369     0.077202     0.025944     0.239386     0.027529    | 0.537282  0.353112  0.612710  | 0.063451  0.083172  0.077317 
+8     | 0.000375  | 0.159648     | 0.196085     | 0.733466        | 0.444191     | 0.073684          | 0.381314     0.064648     0.005548     0.251268     0.011900    | 0.470487     0.078483     0.029077     0.236149     0.014537    | 0.503881  0.331330  0.550262  | 0.079425  0.071668  0.069961 
+9     | 0.000500  | 0.151498     | 0.193960     | 0.749742        | 0.469650     | 0.063530          | 0.384713     0.051549     0.005500     0.197327     0.006029    | 0.458033     0.080786     0.032284     0.235992     0.012893    | 0.591665  0.351458  0.517572  | 0.073750  0.068320  0.048520 
+10    | 0.000483  | 0.143644     | 0.198223     | 0.734475        | 0.445839     | 0.073101          | 0.379823     0.042425     0.004863     0.161501     0.003305    | 0.457999     0.086890     0.036422     0.247703     0.024428    | 0.513935  0.332388  0.531303  | 0.068359  0.080767  0.070177 
+11    | 0.000438  | 0.137590     | 0.200773     | 0.730103        | 0.433250     | 0.071994          | 0.374989     0.035848     0.004434     0.135494     0.002424    | 0.464400     0.087790     0.040262     0.239677     0.023701    | 0.472396  0.332665  0.571301  | 0.080412  0.078320  0.057250 
+12    | 0.000375  | 0.132513     | 0.196365     | 0.727999        | 0.436735     | 0.077826          | 0.367426     0.031836     0.003934     0.120380     0.001701    | 0.454203     0.085863     0.038182     0.239310     0.008696    | 0.487975  0.318142  0.558865  | 0.116083  0.077224  0.040171 
+13    | 0.000313  | 0.130247     | 0.193406     | 0.742431        | 0.464834     | 0.072503          | 0.363716     0.030189     0.003890     0.113679     0.001405    | 0.447801     0.084380     0.038076     0.233248     0.011186    | 0.520903  0.313389  0.602768  | 0.068984  0.077128  0.071398 
+14    | 0.000267  | 0.128772     | 0.190387     | 0.740950        | 0.479183     | 0.084539          | 0.362769     0.028488     0.003651     0.107337     0.001261    | 0.453108     0.077793     0.034092     0.218177     0.010103    | 0.552940  0.339398  0.591916  | 0.105956  0.079723  0.067937 
+15    | 0.000250  | 0.127016     | 0.192453     | 0.752557        | 0.476974     | 0.063722          | 0.360368     0.027009     0.003486     0.101699     0.001050    | 0.451357     0.081494     0.037949     0.221466     0.012998    | 0.550186  0.345268  0.576275  | 0.077125  0.073056  0.040985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+diff = torch.abs(seg_pred - seg_true)
+hd_loss = (dist_map * diff).sum(dim=(2,3)) / seg_true.sum(dim=(2,3)).clamp(min=1)
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+15 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(55m 27s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.684076     | 0.391366     | 0.479637        | 0.181742     | 0.321767          | 0.585647     0.726260     0.473257     0.979263     4.570850    | 0.497253     0.345986     0.265003     0.426968     2.629499    | 0.340690  0.141129  0.013485  | 0.261865  0.394741  0.308694 
+2     | 0.000500  | 0.507192     | 0.295031     | 0.648388        | 0.328859     | 0.138592          | 0.449111     0.532084     0.134003     0.930166     1.430834    | 0.469464     0.220274     0.067579     0.372970     0.497474    | 0.469836  0.235073  0.272284  | 0.093710  0.111428  0.210638 
+3     | 0.000438  | 0.395124     | 0.255277     | 0.709564        | 0.427928     | 0.102679          | 0.411529     0.388093     0.039065     0.737121     0.341876    | 0.461614     0.166846     0.041882     0.291810     0.155646    | 0.499257  0.258951  0.580518  | 0.104113  0.104691  0.099231 
+4     | 0.000313  | 0.310278     | 0.242213     | 0.717279        | 0.410939     | 0.078495          | 0.391828     0.275327     0.019055     0.531600     0.087207    | 0.459175     0.149230     0.029034     0.269425     0.062832    | 0.524376  0.280724  0.481299  | 0.085917  0.099645  0.049923 
+5     | 0.000250  | 0.226672     | 0.220975     | 0.745215        | 0.485178     | 0.081427          | 0.382681     0.159811     0.007354     0.312268     0.020706    | 0.449036     0.123235     0.024412     0.222058     0.019852    | 0.555872  0.358341  0.608936  | 0.082940  0.074783  0.086557 
+6     | 0.000125  | 0.186310     | 0.234703     | 0.744060        | 0.454807     | 0.063104          | 0.377214     0.104494     0.005214     0.207747     0.007120    | 0.479276     0.129886     0.028557     0.235854     0.016195    | 0.505879  0.353829  0.586485  | 0.067700  0.078873  0.042740 
+7     | 0.000250  | 0.181754     | 0.216608     | 0.763876        | 0.510931     | 0.067495          | 0.381875     0.095988     0.005507     0.190171     0.005275    | 0.441747     0.120120     0.027562     0.217037     0.013328    | 0.615813  0.356974  0.599344  | 0.084884  0.067265  0.050337 
+8     | 0.000375  | 0.173904     | 0.230956     | 0.741222        | 0.445303     | 0.061499          | 0.386314     0.082871     0.005453     0.163549     0.003008    | 0.460580     0.132546     0.035396     0.234712     0.009666    | 0.546877  0.348555  0.512424  | 0.070624  0.080084  0.033789 
+9     | 0.000500  | 0.173341     | 0.224908     | 0.745615        | 0.457919     | 0.062587          | 0.390296     0.080361     0.006247     0.157657     0.002379    | 0.437130     0.133956     0.039079     0.233872     0.010515    | 0.594730  0.351287  0.476093  | 0.073180  0.067410  0.047172 
+10    | 0.000495  | 0.162335     | 0.237347     | 0.724465        | 0.412975     | 0.067875          | 0.383867     0.067392     0.005214     0.132264     0.001412    | 0.460448     0.141732     0.042559     0.246231     0.011281    | 0.452251  0.331549  0.546802  | 0.056100  0.077799  0.069727 
+11    | 0.000480  | 0.158341     | 0.241854     | 0.725066        | 0.404989     | 0.061549          | 0.382882     0.062110     0.005129     0.121582     0.001056    | 0.469243     0.144401     0.044912     0.249403     0.009343    | 0.497294  0.346841  0.445771  | 0.069771  0.074725  0.040152 
+12    | 0.000457  | 0.151966     | 0.232940     | 0.736785        | 0.439628     | 0.065111          | 0.374467     0.056609     0.004756     0.110739     0.000817    | 0.472344     0.130338     0.043928     0.221573     0.012151    | 0.565533  0.343164  0.499601  | 0.077612  0.075731  0.041989 
+13    | 0.000427  | 0.147622     | 0.224413     | 0.748525        | 0.462314     | 0.060667          | 0.368265     0.053061     0.004573     0.103682     0.000776    | 0.449570     0.127917     0.041062     0.219666     0.007985    | 0.555970  0.312297  0.578969  | 0.070207  0.066316  0.045478 
+14    | 0.000393  | 0.144605     | 0.228535     | 0.751412        | 0.479715     | 0.067456          | 0.365990     0.049726     0.004224     0.097235     0.000562    | 0.471517     0.124399     0.040536     0.212832     0.012464    | 0.589300  0.364285  0.576736  | 0.069651  0.086694  0.046024 
+15    | 0.000357  | 0.142196     | 0.222062     | 0.748843        | 0.471259     | 0.066100          | 0.362051     0.047972     0.004039     0.093843     0.000475    | 0.434256     0.131121     0.045339     0.221933     0.007925    | 0.554696  0.361743  0.562151  | 0.068491  0.071380  0.058429 
+16    | 0.000323  | 0.141041     | 0.220112     | 0.757210        | 0.493166     | 0.066760          | 0.360597     0.046946     0.004054     0.091732     0.000531    | 0.445830     0.123376     0.040662     0.210748     0.009240    | 0.607192  0.363977  0.592159  | 0.076410  0.078132  0.045738 
+17    | 0.000293  | 0.138643     | 0.219432     | 0.756853        | 0.489547     | 0.064942          | 0.358095     0.044593     0.003802     0.087188     0.000398    | 0.439735     0.125016     0.042271     0.212507     0.008737    | 0.603059  0.352005  0.592545  | 0.073161  0.075214  0.046452 
+18    | 0.000270  | 0.139140     | 0.231360     | 0.743354        | 0.451937     | 0.062368          | 0.358807     0.044998     0.003844     0.087972     0.000392    | 0.445041     0.139782     0.047229     0.237586     0.011128    | 0.552590  0.321479  0.543570  | 0.066257  0.075865  0.044981 
+19    | 0.000255  | 0.138130     | 0.219968     | 0.749452        | 0.488178     | 0.076365          | 0.356980     0.044337     0.003816     0.086651     0.000440    | 0.436013     0.127377     0.044714     0.214828     0.010067    | 0.592405  0.362251  0.573208  | 0.076767  0.079891  0.072436 
+20    | 0.000250  | 0.136660     | 0.215931     | 0.752074        | 0.488417     | 0.072155          | 0.357354     0.042077     0.003744     0.082110     0.000431    | 0.425889     0.125950     0.044654     0.211977     0.010026    | 0.608166  0.365520  0.581358  | 0.073608  0.076094  0.066762</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on full train-valid
+diff = torch.abs(seg_pred - seg_true)
+hd_loss = (dist_map * diff).sum(dim=(2,3)) / seg_true.sum(dim=(2,3)).clamp(min=1)
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 16m 9s)
+(Max GPU mem usage : 6632.875 MB)  
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.462555     | 0.199769     | 0.799995        | 0.607594     | 0.071739          | 0.494823     0.448726     0.134807     0.762645     1.202879    | 0.462491     0.087174     0.013750     0.160598     0.016577    | 0.667809  0.516870  0.631378  | 0.081419  0.078526  0.055270 
+2     | 0.000500  | 0.210816     | 0.177897     | 0.834913        | 0.683826     | 0.064363          | 0.427906     0.117777     0.010576     0.224977     0.006418    | 0.447687     0.062273     0.014946     0.109600     0.005429    | 0.714117  0.612194  0.732509  | 0.100902  0.061696  0.030490 
+3     | 0.000438  | 0.179294     | 0.172554     | 0.844873        | 0.700723     | 0.059028          | 0.399573     0.084889     0.008900     0.160878     0.003042    | 0.430683     0.061927     0.015135     0.108720     0.004168    | 0.734216  0.623068  0.753534  | 0.068205  0.063861  0.045017 
+4     | 0.000313  | 0.167302     | 0.173744     | 0.849588        | 0.701115     | 0.051431          | 0.385079     0.073968     0.007925     0.140012     0.002229    | 0.435778     0.061444     0.015884     0.107005     0.003683    | 0.734165  0.610687  0.766654  | 0.071823  0.051215  0.031254 
+5     | 0.000250  | 0.159512     | 0.167180     | 0.856919        | 0.719844     | 0.051697          | 0.375101     0.067117     0.007186     0.127047     0.001755    | 0.421435     0.058214     0.016185     0.100243     0.004278    | 0.746362  0.642770  0.776040  | 0.067057  0.055258  0.032775 
+6     | 0.000125  | 0.151632     | 0.168660     | 0.858137        | 0.716701     | 0.047573          | 0.366200     0.059675     0.006555     0.115172     0.001425    | 0.428435     0.057328     0.016018     0.100836     0.003484    | 0.740297  0.648070  0.768098  | 0.061986  0.054994  0.025738 
+7     | 0.000250  | 0.154910     | 0.171402     | 0.855420        | 0.709406     | 0.047238          | 0.370910     0.062339     0.006901     0.120264     0.001374    | 0.434439     0.058672     0.015880     0.103721     0.003385    | 0.733604  0.642618  0.767775  | 0.059404  0.055199  0.027109 
+8     | 0.000375  | 0.155738     | 0.174070     | 0.844705        | 0.696148     | 0.056258          | 0.374775     0.061864     0.007020     0.119188     0.001114    | 0.434485     0.062464     0.017642     0.109654     0.004463    | 0.719451  0.629518  0.752014  | 0.066759  0.060328  0.041686 
+9     | 0.000500  | 0.161911     | 0.171767     | 0.840959        | 0.692785     | 0.060258          | 0.380741     0.068126     0.007862     0.131122     0.001209    | 0.434007     0.059378     0.016442     0.104556     0.004423    | 0.724798  0.618572  0.753993  | 0.071488  0.060283  0.049004 
+10    | 0.000483  | 0.155758     | 0.171512     | 0.851294        | 0.707061     | 0.052550          | 0.375483     0.061590     0.007062     0.118594     0.000912    | 0.430122     0.060679     0.017284     0.106389     0.003955    | 0.725855  0.639162  0.767306  | 0.051487  0.062384  0.043778 
+11    | 0.000438  | 0.153131     | 0.170733     | 0.848074        | 0.709486     | 0.059534          | 0.371905     0.059370     0.006793     0.114335     0.000867    | 0.433244     0.058229     0.017027     0.101619     0.004644    | 0.730698  0.639882  0.770881  | 0.066795  0.061664  0.050142 
+12    | 0.000375  | 0.148914     | 0.169085     | 0.857304        | 0.719524     | 0.050842          | 0.366366     0.055721     0.006313     0.107376     0.000644    | 0.425475     0.059203     0.016763     0.103896     0.004015    | 0.743062  0.647202  0.772068  | 0.066739  0.059853  0.025933 
+13    | 0.000313  | 0.145127     | 0.168209     | 0.859208        | 0.721924     | 0.049269          | 0.361032     0.052597     0.005884     0.101435     0.000509    | 0.429888     0.056061     0.016427     0.097832     0.003687    | 0.739802  0.647817  0.794396  | 0.062640  0.062572  0.022595 
+14    | 0.000267  | 0.143658     | 0.172125     | 0.857806        | 0.716400     | 0.047923          | 0.357823     0.051872     0.005846     0.099986     0.000722    | 0.439453     0.057556     0.017794     0.099521     0.003565    | 0.735309  0.640959  0.790207  | 0.055224  0.061500  0.027044 
+15    | 0.000250  | 0.142890     | 0.171514     | 0.854048        | 0.713713     | 0.052394          | 0.357440     0.050941     0.005691     0.098251     0.000457    | 0.438380     0.057143     0.017099     0.099340     0.004356    | 0.730797  0.638223  0.788251  | 0.064608  0.066911  0.025663</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2527  1986  1446
+FP   283   307    76
+FN    50    83    80
+TN  4436  4920  5694
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.346  0.272  0.198
+FP  0.039  0.042  0.010
+FN  0.007  0.011  0.011
+TN  0.608  0.674  0.780
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+-----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.171514     | 0.854048        | 0.713713     | 0.052394          | 0.438380     0.057143     0.017099     0.099340     0.004356    | 0.730797  0.638223  0.788251  | 0.064608  0.066911  0.025663 
+266     | 266     | 0.171858     | 0.853786        | 0.715085     | 0.053746          | 0.437783     0.057890     0.017783     0.100167     0.004740    | 0.729642  0.639586  0.793321  | 0.066481  0.069298  0.025460 
+360     | 310     | 0.160810     | 0.846926        | 0.680504     | 0.042126          | 0.430536     0.045212     0.008575     0.083655     0.000981    | 0.695721  0.601151  0.780318  | 0.051308  0.050703  0.024365 
+276     | 276     | 0.187912     | 0.868017        | 0.738752     | 0.045807          | 0.473327     0.065592     0.019099     0.114676     0.002093    | 0.798246  0.663775  0.720845  | 0.054239  0.052728  0.030454 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+diff = torch.abs(seg_pred - seg_true)
+hd_loss = (dist_map * diff).sum(dim=(2,3)) / seg_true.sum(dim=(2,3)).clamp(min=1)
+Then * presence_true and normalize by presence_true
+7 epochs : 0.5D + 0.5B  
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+8 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(43m 11s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.739456     | 0.465234     | 0.390085        | 0.119139     | 0.429285          | 0.622962     0.789382     0.597201     0.981563     5.521561    | 0.513595     0.444508     0.455718     0.433298     4.076507    | 0.205312  0.070678  0.062664  | 0.374599  0.414104  0.499151 
+2     | 0.000250  | 0.576561     | 0.356704     | 0.577136        | 0.248146     | 0.203537          | 0.465777     0.624039     0.273947     0.974132     2.865134    | 0.488980     0.300015     0.182982     0.417047     1.835055    | 0.440248  0.234320  0.008894  | 0.112648  0.197398  0.300564 
+3     | 0.000375  | 0.492569     | 0.299159     | 0.626294        | 0.266686     | 0.133968          | 0.433940     0.517696     0.113886     0.921505     1.257926    | 0.472839     0.224725     0.076623     0.372828     0.585693    | 0.497381  0.250829  0.004712  | 0.107681  0.115322  0.178900 
+4     | 0.000500  | 0.405143     | 0.264587     | 0.678050        | 0.386844     | 0.127812          | 0.416430     0.400305     0.043134     0.757477     0.402551    | 0.487156     0.169201     0.039121     0.299280     0.167663    | 0.506254  0.260551  0.415171  | 0.106008  0.107363  0.170065 
+5     | 0.000438  | 0.279109     | 0.243477     | 0.717995        | 0.392263     | 0.064851          | 0.397114     0.228535     0.011623     0.445447     0.061879    | 0.476796     0.143484     0.029868     0.257100     0.020648    | 0.438967  0.319381  0.500431  | 0.072644  0.069773  0.052137 
+6     | 0.000313  | 0.199792     | 0.226783     | 0.747741        | 0.463773     | 0.062946          | 0.387608     0.119300     0.006091     0.232508     0.008883    | 0.460627     0.126564     0.028987     0.224142     0.017730    | 0.545945  0.373478  0.550317  | 0.066537  0.075500  0.046801 
+7     | 0.000250  | 0.178778     | 0.218412     | 0.749078        | 0.491227     | 0.079021          | 0.385116     0.090348     0.005287     0.175409     0.004348    | 0.445450     0.121110     0.029059     0.213160     0.016298    | 0.584135  0.352070  0.600912  | 0.085899  0.095056  0.056108 
+8     | 0.000125  | 0.166384     | 0.224182     | 0.745594        | 0.467543     | 0.069038          | 0.377203     0.076033     0.004678     0.150378     0.002790    | 0.465030     0.120962     0.030703     0.215680     0.011698    | 0.566521  0.362891  0.552651  | 0.079261  0.072633  0.055219 
+9     | 0.000250  | 0.160779     | 0.236825     | 0.733085        | 0.425254     | 0.061694          | 0.376227     0.068444     0.004614     0.134976     0.002229    | 0.467519     0.137956     0.038885     0.242171     0.011906    | 0.485668  0.328805  0.548918  | 0.068814  0.068586  0.047681 
+10    | 0.000375  | 0.163192     | 0.234874     | 0.719353        | 0.418453     | 0.080047          | 0.380801     0.069931     0.005073     0.137564     0.001935    | 0.456854     0.139740     0.040272     0.244629     0.006922    | 0.465919  0.357056  0.496721  | 0.069863  0.075056  0.095222 
+11    | 0.000500  | 0.168142     | 0.240469     | 0.709880        | 0.422604     | 0.098602          | 0.390565     0.072818     0.005956     0.142581     0.001728    | 0.468651     0.142676     0.050839     0.239037     0.031839    | 0.502275  0.317350  0.543214  | 0.102803  0.111092  0.081912 
+12    | 0.000463  | 0.163416     | 0.249386     | 0.726755        | 0.409612     | 0.061816          | 0.384517     0.068659     0.005846     0.134197     0.001875    | 0.503635     0.140422     0.043850     0.242416     0.007585    | 0.427634  0.317674  0.548976  | 0.070205  0.067091  0.048151 
+13    | 0.000375  | 0.152643     | 0.231903     | 0.734604        | 0.439130     | 0.068414          | 0.374925     0.057379     0.004905     0.112158     0.000916    | 0.465353     0.131853     0.044067     0.224487     0.013084    | 0.529464  0.332638  0.532169  | 0.076681  0.074816  0.053743 
+14    | 0.000287  | 0.145608     | 0.224066     | 0.742311        | 0.466848     | 0.074047          | 0.367677     0.050435     0.004186     0.098715     0.000695    | 0.452725     0.126070     0.040718     0.216084     0.011834    | 0.566579  0.364903  0.549936  | 0.080123  0.070698  0.071321 
+15    | 0.000250  | 0.144108     | 0.228147     | 0.738774        | 0.450868     | 0.069288          | 0.365156     0.049374     0.004142     0.096597     0.000581    | 0.449317     0.133360     0.043988     0.227831     0.008419    | 0.534906  0.355509  0.539228  | 0.080434  0.070538  0.056894</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+7 epochs : 0.5D + 0.5B  
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+8 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 47s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.739678     | 0.462504     | 0.389762        | 0.115024     | 0.427079          | 0.623508     0.789466     0.597314     0.981617     5551.996582 | 0.499413     0.446686     0.460227     0.433146     4590.304199 | 0.192751  0.072429  0.058057  | 0.376085  0.406064  0.499089 
+2     | 0.000250  | 0.576609     | 0.363947     | 0.566088        | 0.222342     | 0.204748          | 0.466419     0.623833     0.274149     0.973517     2898.905273 | 0.511895     0.300541     0.180622     0.420461     1997.231201 | 0.396047  0.205536  0.008622  | 0.109860  0.205058  0.299326 
+3     | 0.000375  | 0.491737     | 0.299527     | 0.609425        | 0.254121     | 0.153705          | 0.432899     0.516953     0.113688     0.920218     1213.681519 | 0.468031     0.227311     0.083070     0.371551     754.067871  | 0.464873  0.234967  0.010042  | 0.122012  0.150965  0.188139 
+4     | 0.000500  | 0.405154     | 0.263768     | 0.691574        | 0.404045     | 0.116741          | 0.416080     0.400472     0.043021     0.757922     376.109619  | 0.486370     0.168367     0.040115     0.296620     194.393814  | 0.521069  0.259467  0.445312  | 0.099878  0.107973  0.142370 
+5     | 0.000438  | 0.282098     | 0.231806     | 0.726609        | 0.457098     | 0.093718          | 0.399828     0.231642     0.011855     0.451429     57.881580   | 0.456092     0.135683     0.027391     0.243976     32.425045   | 0.541899  0.338173  0.538309  | 0.072241  0.106949  0.101963 
+6     | 0.000313  | 0.201958     | 0.223725     | 0.749388        | 0.478501     | 0.070021          | 0.388284     0.122104     0.006224     0.237984     8.859145    | 0.453781     0.125129     0.027817     0.222442     17.418562   | 0.563860  0.372848  0.552545  | 0.061478  0.102698  0.045887 
+7     | 0.000250  | 0.178297     | 0.215859     | 0.762973        | 0.517616     | 0.073456          | 0.382325     0.090857     0.005314     0.176400     4.585205    | 0.442644     0.118665     0.028903     0.208427     17.794609   | 0.596007  0.361414  0.632620  | 0.070751  0.095371  0.054247 
+8     | 0.000125  | 0.196622     | 0.337324     | 0.742037        | 0.444585     | 0.059662          | 0.375854     0.119809     0.005131     0.155978     2.043277    | 0.469322     0.280753     0.033828     0.232888     7.503088    | 0.515002  0.336145  0.544734  | 0.060223  0.074448  0.044315 
+9     | 0.000250  | 0.177668     | 0.366022     | 0.738235        | 0.435556     | 0.059979          | 0.375579     0.092848     0.005330     0.142391     1.023252    | 0.455977     0.327470     0.039942     0.232854     9.689985    | 0.495412  0.364176  0.532476  | 0.057665  0.074568  0.047706 
+10    | 0.000375  | 0.178503     | 0.345098     | 0.735355        | 0.422353     | 0.055977          | 0.379620     0.092310     0.006387     0.147570     0.843560    | 0.447494     0.301214     0.044240     0.244548     7.985368    | 0.451613  0.339779  0.550968  | 0.048305  0.072999  0.046628 
+11    | 0.000500  | 0.174805     | 0.374713     | 0.748910        | 0.461664     | 0.059593          | 0.389081     0.082972     0.006597     0.138364     0.597075    | 0.466258     0.335480     0.041482     0.226320     10.212841   | 0.489244  0.339587  0.626014  | 0.059331  0.066051  0.053397 
+12    | 0.000463  | 0.165814     | 0.371617     | 0.735097        | 0.427197     | 0.059636          | 0.380607     0.073760     0.005963     0.123248     0.522355    | 0.464398     0.331855     0.048627     0.237539     9.581655    | 0.496711  0.337229  0.526880  | 0.065173  0.070601  0.043135 
+13    | 0.000375  | 0.157841     | 0.401336     | 0.749478        | 0.455005     | 0.054206          | 0.370980     0.066496     0.005475     0.112917     0.424199    | 0.453468     0.378993     0.049725     0.233467     12.011434   | 0.519980  0.344476  0.556075  | 0.060893  0.067818  0.033907 
+14    | 0.000287  | 0.154152     | 0.406405     | 0.748973        | 0.471153     | 0.065813          | 0.369409     0.061898     0.005219     0.106317     0.362294    | 0.453088     0.386397     0.044223     0.221691     12.804956   | 0.549006  0.361448  0.571126  | 0.068500  0.083076  0.045864 
+15    | 0.000250  | 0.148883     | 0.385875     | 0.751108        | 0.469433     | 0.061108          | 0.365347     0.056113     0.004719     0.097166     0.309468    | 0.444477     0.360761     0.048275     0.228549     11.255825   | 0.521501  0.343955  0.593039  | 0.066434  0.076122  0.040769</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+10 epochs : 0.5D + 0.5B  
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+10 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(55m 26s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.740509     | 0.462884     | 0.387109        | 0.111217     | 0.428963          | 0.626830     0.789228     0.596837     0.981620     5559.052734 | 0.502001     0.446120     0.459011     0.433228     4581.773438 | 0.194205  0.071662  0.056691  | 0.375284  0.412517  0.499089 
+2     | 0.000250  | 0.576488     | 0.357932     | 0.571635        | 0.252379     | 0.215527          | 0.466253     0.623731     0.273548     0.973913     2897.750488 | 0.494100     0.299574     0.182774     0.416373     2017.788574 | 0.453591  0.220437  0.015490  | 0.121175  0.225257  0.300151 
+3     | 0.000375  | 0.490896     | 0.298496     | 0.621815        | 0.258520     | 0.135987          | 0.430026     0.516982     0.113609     0.920356     1215.418213 | 0.473666     0.223423     0.073945     0.372900     699.411743  | 0.500810  0.242033  0.002550  | 0.102067  0.104808  0.201087 
+4     | 0.000500  | 0.402847     | 0.270596     | 0.708442        | 0.396076     | 0.083313          | 0.414563     0.397825     0.042541     0.753110     370.290527  | 0.507779     0.168946     0.036951     0.300940     172.377380  | 0.464519  0.249257  0.478314  | 0.085621  0.090100  0.074219 
+5     | 0.000483  | 0.279468     | 0.242824     | 0.713977        | 0.418601     | 0.089105          | 0.399451     0.228046     0.012335     0.443758     54.507206   | 0.474956     0.143340     0.030259     0.256420     30.191051   | 0.457113  0.332692  0.533071  | 0.067788  0.095637  0.103891 
+6     | 0.000438  | 0.198900     | 0.238839     | 0.737600        | 0.442463     | 0.065641          | 0.392158     0.116075     0.006579     0.225570     7.414657    | 0.496336     0.128484     0.030640     0.226327     19.776941   | 0.526901  0.346077  0.549110  | 0.081027  0.074105  0.041792 
+7     | 0.000375  | 0.175553     | 0.222685     | 0.752109        | 0.482655     | 0.068256          | 0.385456     0.085595     0.005504     0.165686     3.461946    | 0.457074     0.122233     0.031389     0.213077     13.524622   | 0.590114  0.353857  0.553776  | 0.072692  0.070083  0.061993 
+8     | 0.000313  | 0.164117     | 0.231566     | 0.737088        | 0.436503     | 0.062522          | 0.378753     0.072130     0.004844     0.139415     2.249596    | 0.465516     0.131302     0.035769     0.226835     15.673143   | 0.508368  0.324003  0.573308  | 0.075776  0.069689  0.042101 
+9     | 0.000267  | 0.154296     | 0.224427     | 0.751109        | 0.481572     | 0.069200          | 0.371135     0.061365     0.004338     0.118391     1.710815    | 0.447855     0.128672     0.037204     0.220140     17.626682   | 0.551082  0.357229  0.618315  | 0.072833  0.082276  0.052491 
+10    | 0.000250  | 0.152190     | 0.235014     | 0.735489        | 0.433799     | 0.063385          | 0.369148     0.059208     0.004291     0.114124     1.464989    | 0.449556     0.143068     0.041712     0.244424     13.347274   | 0.476946  0.328985  0.567102  | 0.064051  0.074931  0.051171 
+11    | 0.000125  | 0.162235     | 0.435935     | 0.738269        | 0.446177     | 0.067003          | 0.367406     0.074304     0.004332     0.110302     0.906661    | 0.472288     0.420356     0.037779     0.224723     14.586497   | 0.529952  0.325728  0.571245  | 0.071078  0.077492  0.052439 
+12    | 0.000250  | 0.162805     | 0.384494     | 0.741929        | 0.441402     | 0.057719          | 0.368943     0.074461     0.004960     0.115908     0.761775    | 0.456880     0.353472     0.043598     0.225954     11.069551   | 0.552057  0.337172  0.514149  | 0.063235  0.067357  0.042565 
+13    | 0.000375  | 0.166311     | 0.403436     | 0.723443        | 0.420279     | 0.074448          | 0.375086     0.076835     0.005997     0.125145     0.628798    | 0.468692     0.375470     0.047400     0.248998     11.511755   | 0.504458  0.317917  0.491109  | 0.092709  0.090237  0.040398 
+14    | 0.000500  | 0.172359     | 0.375093     | 0.720102        | 0.401374     | 0.067412          | 0.386524     0.080574     0.006574     0.130929     0.659909    | 0.494195     0.324049     0.048865     0.252020     8.830757    | 0.438452  0.349161  0.487919  | 0.071728  0.067175  0.063334 
+15    | 0.000483  | 0.165156     | 0.388510     | 0.734661        | 0.448526     | 0.074582          | 0.383684     0.071501     0.006193     0.120229     0.477715    | 0.475733     0.351128     0.047114     0.224687     10.897279   | 0.547484  0.330213  0.540571  | 0.066232  0.074002  0.083512 
+16    | 0.000438  | 0.158755     | 0.478239     | 0.719779        | 0.407575     | 0.072085          | 0.376856     0.065283     0.005786     0.111107     0.400283    | 0.503016     0.467621     0.056627     0.241751     16.070784   | 0.428577  0.362890  0.493727  | 0.062714  0.095338  0.058202 
+17    | 0.000375  | 0.157193     | 0.409541     | 0.738555        | 0.453541     | 0.071436          | 0.375189     0.063765     0.005944     0.108022     0.396112    | 0.454492     0.390276     0.051281     0.227333     12.687792   | 0.518836  0.365243  0.570732  | 0.059389  0.079311  0.075608 
+18    | 0.000313  | 0.149189     | 0.392273     | 0.745246        | 0.469607     | 0.070995          | 0.367062     0.055814     0.004893     0.096949     0.295554    | 0.448963     0.367978     0.050185     0.221902     11.732775   | 0.540667  0.359416  0.601765  | 0.075925  0.088431  0.048628 
+19    | 0.000267  | 0.146528     | 0.404479     | 0.738627        | 0.443317     | 0.064499          | 0.363772     0.053424     0.004766     0.092877     0.278941    | 0.449485     0.385191     0.052577     0.229669     12.344514   | 0.516467  0.351252  0.550142  | 0.070064  0.075249  0.048185 
+20    | 0.000250  | 0.143595     | 0.408559     | 0.743881        | 0.458478     | 0.065850          | 0.361052     0.050399     0.004569     0.088053     0.250693    | 0.436053     0.396776     0.052823     0.227528     12.970198   | 0.543265  0.360898  0.548590  | 0.064205  0.085205  0.048140</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+7 epochs : 0.5D + 0.5B  
+8 epochs : 0.02H + 0.49D + 0.49B 
+LR common – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 47s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.741613     | 0.469173     | 0.388449        | 0.115169     | 0.429364          | 0.629549     0.789640     0.597739     0.981541     5556.090820 | 0.519713     0.447513     0.461961     0.433064     4597.024414 | 0.195328  0.071178  0.060337  | 0.375497  0.413365  0.499231 
+2     | 0.000250  | 0.574979     | 0.360677     | 0.577157        | 0.251229     | 0.205557          | 0.460903     0.623869     0.274311     0.973426     2900.808838 | 0.499768     0.301066     0.186628     0.415505     2047.050903 | 0.437368  0.230938  0.007698  | 0.134184  0.182162  0.300325 
+3     | 0.000375  | 0.492438     | 0.301095     | 0.621276        | 0.251635     | 0.132296          | 0.434920     0.517088     0.113949     0.920228     1215.707275 | 0.479996     0.224422     0.077237     0.371608     715.634583  | 0.476981  0.236239  0.004897  | 0.103627  0.117851  0.175410 
+4     | 0.000500  | 0.404758     | 0.269819     | 0.675415        | 0.378377     | 0.126560          | 0.415771     0.400038     0.042868     0.757208     375.698212  | 0.500652     0.170891     0.036808     0.304975     182.262299  | 0.521479  0.262783  0.389543  | 0.090180  0.128472  0.161027 
+5     | 0.000495  | 0.275344     | 0.236233     | 0.722207        | 0.426673     | 0.080770          | 0.402213     0.220972     0.011054     0.430891     52.467171   | 0.456517     0.141825     0.029892     0.253758     32.802647   | 0.489473  0.327008  0.524247  | 0.099165  0.086840  0.056304 
+6     | 0.000480  | 0.199787     | 0.235472     | 0.729278        | 0.413692     | 0.060332          | 0.397336     0.115122     0.006733     0.223512     6.835914    | 0.462985     0.137967     0.035418     0.240517     19.501495   | 0.465398  0.350205  0.515644  | 0.054356  0.080647  0.045993 
+7     | 0.000457  | 0.177954     | 0.225922     | 0.747367        | 0.466856     | 0.065625          | 0.390532     0.086850     0.005932     0.167767     3.284976    | 0.458118     0.126410     0.034537     0.218282     14.453842   | 0.545729  0.363755  0.557675  | 0.070906  0.076089  0.049880 
+8     | 0.000427  | 0.199712     | 0.381976     | 0.699963        | 0.329481     | 0.053048          | 0.388459     0.118820     0.007483     0.175862     1.449049    | 0.491433     0.335067     0.049955     0.276663     8.751172    | 0.405201  0.239471  0.401744  | 0.059389  0.063489  0.036268 
+9     | 0.000393  | 0.176521     | 0.359242     | 0.742312        | 0.435813     | 0.053356          | 0.384277     0.087483     0.006444     0.141429     0.751239    | 0.459271     0.316372     0.046223     0.240132     8.802936    | 0.512750  0.315280  0.538709  | 0.061969  0.061673  0.036425 
+10    | 0.000357  | 0.162151     | 0.403871     | 0.753807        | 0.469307     | 0.056527          | 0.375865     0.070560     0.005351     0.118200     0.500985    | 0.443867     0.386730     0.043205     0.216156     12.982161   | 0.559380  0.339505  0.583804  | 0.060065  0.068882  0.040634 
+11    | 0.000323  | 0.156043     | 0.409997     | 0.748697        | 0.458933     | 0.058127          | 0.372168     0.063418     0.005107     0.107476     0.412599    | 0.470095     0.384241     0.044587     0.219809     12.734350   | 0.546373  0.349253  0.569895  | 0.063962  0.070509  0.039910 
+12    | 0.000293  | 0.154575     | 0.428015     | 0.751645        | 0.470160     | 0.060698          | 0.370264     0.062137     0.005073     0.106045     0.384501    | 0.451063     0.418137     0.048068     0.219831     14.343342   | 0.582713  0.344269  0.557187  | 0.066760  0.072584  0.042751 
+13    | 0.000270  | 0.149265     | 0.412816     | 0.749638        | 0.460688     | 0.057730          | 0.364134     0.057178     0.004690     0.098460     0.331717    | 0.459171     0.392950     0.047799     0.220711     13.068993   | 0.536383  0.359331  0.559566  | 0.059690  0.068802  0.044697 
+14    | 0.000255  | 0.147335     | 0.405704     | 0.750906        | 0.471227     | 0.062642          | 0.362809     0.054989     0.004504     0.094908     0.313866    | 0.467866     0.379063     0.045955     0.215533     12.546714   | 0.566041  0.343613  0.576318  | 0.064262  0.080607  0.043057 
+15    | 0.000250  | 0.145858     | 0.403184     | 0.750936        | 0.465905     | 0.059043          | 0.362607     0.052966     0.004449     0.091387     0.300291    | 0.450969     0.382704     0.049544     0.224408     12.423363   | 0.564895  0.347210  0.556043  | 0.062272  0.079532  0.035324</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on data subset
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+10 epochs : 0.5D + 0.5B
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+5 epochs :  0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, …, 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(42m 36s)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.741493     | 0.472187     | 0.387712        | 0.110573     | 0.427528          | 0.630010     0.789271     0.597043     0.981499     5554.871582 | 0.532882     0.446175     0.459065     0.433284     4583.299805 | 0.192066  0.071706  0.056098  | 0.375970  0.407506  0.499108 
+2     | 0.000250  | 0.575055     | 0.359198     | 0.572588        | 0.222824     | 0.194237          | 0.461256     0.623825     0.274173     0.973478     2899.991943 | 0.497177     0.300064     0.180879     0.419249     1999.331909 | 0.418876  0.212013  0.004181  | 0.106357  0.174491  0.301862 
+3     | 0.000375  | 0.492022     | 0.310028     | 0.610576        | 0.237939     | 0.140999          | 0.433591     0.517063     0.113733     0.920394     1216.886353 | 0.497435     0.229711     0.089290     0.370131     756.711975  | 0.419505  0.232917  0.007020  | 0.119219  0.124201  0.179578 
+4     | 0.000500  | 0.406894     | 0.268160     | 0.695154        | 0.399209     | 0.107548          | 0.416316     0.402857     0.043675     0.762038     381.576324  | 0.493712     0.171495     0.039709     0.303281     200.669113  | 0.515427  0.245062  0.444304  | 0.097600  0.098962  0.126083 
+5     | 0.000483  | 0.281877     | 0.236648     | 0.738486        | 0.458489     | 0.074849          | 0.396302     0.232838     0.012590     0.453086     60.156124   | 0.477169     0.133568     0.026057     0.241080     26.474724   | 0.548123  0.348319  0.522743  | 0.070121  0.100938  0.053489 
+6     | 0.000438  | 0.197601     | 0.234008     | 0.720066        | 0.415216     | 0.076701          | 0.392675     0.113997     0.006245     0.221750     7.430659    | 0.463966     0.135454     0.033067     0.237842     15.250703   | 0.430059  0.335354  0.575993  | 0.068102  0.080273  0.081729 
+7     | 0.000375  | 0.176842     | 0.223169     | 0.743734        | 0.480281     | 0.080631          | 0.388931     0.085947     0.005680     0.166213     3.531019    | 0.455226     0.123716     0.033383     0.214049     15.186080   | 0.530231  0.379065  0.570451  | 0.076815  0.100030  0.065047 
+8     | 0.000313  | 0.163493     | 0.231402     | 0.742086        | 0.457136     | 0.067948          | 0.378257     0.071451     0.004794     0.138108     2.246505    | 0.466649     0.130582     0.035658     0.225506     11.914804   | 0.512931  0.356063  0.554058  | 0.086643  0.074351  0.042849 
+9     | 0.000267  | 0.157735     | 0.224984     | 0.748374        | 0.470079     | 0.066096          | 0.373715     0.065172     0.004715     0.125629     1.791014    | 0.444798     0.130778     0.039056     0.222501     13.786827   | 0.577433  0.352953  0.543607  | 0.077898  0.071497  0.048894 
+10    | 0.000250  | 0.153848     | 0.224973     | 0.741743        | 0.457274     | 0.068611          | 0.370039     0.061194     0.004508     0.117881     1.482887    | 0.443785     0.131197     0.040703     0.221691     14.650076   | 0.566780  0.362944  0.510264  | 0.070322  0.087154  0.048359 
+11    | 0.000125  | 0.163437     | 0.378170     | 0.747200        | 0.468611     | 0.067074          | 0.367937     0.075794     0.004457     0.112297     0.929231    | 0.465802     0.340613     0.037420     0.214321     10.863013   | 0.565936  0.360405  0.563629  | 0.081400  0.075705  0.044118 
+12    | 0.000250  | 0.167672     | 0.367007     | 0.725908        | 0.402952     | 0.058788          | 0.368757     0.081492     0.005736     0.125764     0.852846    | 0.465015     0.325003     0.046546     0.244698     9.114689    | 0.513760  0.317604  0.428766  | 0.074050  0.065261  0.037053 
+13    | 0.000375  | 0.159623     | 0.386929     | 0.741003        | 0.444831     | 0.061549          | 0.371371     0.068874     0.005365     0.113324     0.535854    | 0.462013     0.354751     0.045899     0.223512     11.136957   | 0.557217  0.348316  0.507646  | 0.062555  0.077575  0.044518 
+14    | 0.000313  | 0.155941     | 0.417892     | 0.729570        | 0.430910     | 0.071322          | 0.370588     0.063949     0.005132     0.107403     0.440363    | 0.481851     0.390481     0.047507     0.236184     12.573644   | 0.533012  0.348013  0.470154  | 0.070735  0.100916  0.042316 
+15    | 0.000250  | 0.150067     | 0.374628     | 0.741052        | 0.444441     | 0.061207          | 0.365954     0.057544     0.004598     0.097453     0.376937    | 0.452346     0.341321     0.049548     0.230110     10.214417   | 0.514772  0.350131  0.542738  | 0.068201  0.074239  0.041179</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausdorff surrogate loss on full train-valid data
+hd_loss = (dist_map * torch.abs(seg_pred – seg_true)).sum(dim=(2,3))
+Then * presence_true and normalize by presence_true
+5 epochs : 0.5D + 0.5B  
+    LR – 2.5e-4, 5e-4, …, 2.5e-4
+10 epochs : 0.02H + 0.49D + 0.49B 
+    LR – 1.25e-4, 2.5e-4, 3.75e-4, 5e-4, …., 2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-3
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 18m 52s)
+(Max GPU mem usage : 6632.875 MB)  
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-B        TLo-D        TLo-H       | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000250  | 0.463233     | 0.195673     | 0.810646        | 0.623869     | 0.064837          | 0.493508     0.450257     0.134930     0.765585     1318.410522 | 0.455527     0.084307     0.012950     0.155665     22.165514   | 0.685044  0.531410  0.648778  | 0.073400  0.081526  0.039585 
+2     | 0.000500  | 0.209279     | 0.178484     | 0.837785        | 0.687629     | 0.062110          | 0.426821     0.116047     0.010346     0.221747     6.212606    | 0.444575     0.064445     0.014690     0.114200     7.327075    | 0.714695  0.605064  0.738984  | 0.065684  0.070358  0.050289 
+3     | 0.000438  | 0.180452     | 0.172839     | 0.844250        | 0.696815     | 0.057460          | 0.400748     0.086039     0.009051     0.163026     2.673105    | 0.435080     0.060450     0.014755     0.106145     5.543968    | 0.736334  0.617614  0.754647  | 0.063937  0.061092  0.047352 
+4     | 0.000313  | 0.167053     | 0.171905     | 0.849853        | 0.708676     | 0.056029          | 0.385056     0.073624     0.007918     0.139329     1.880181    | 0.433075     0.059975     0.015035     0.104916     5.009771    | 0.731613  0.627816  0.778448  | 0.060125  0.061574  0.046388 
+5     | 0.000250  | 0.159143     | 0.175096     | 0.840613        | 0.689571     | 0.058693          | 0.374446     0.066870     0.007173     0.126567     1.461147    | 0.440543     0.061333     0.017783     0.104882     6.765176    | 0.710854  0.610163  0.770826  | 0.078681  0.067990  0.029406 
+6     | 0.000125  | 0.165345     | 0.222071     | 0.858206        | 0.709176     | 0.042441          | 0.365956     0.079368     0.007654     0.126140     0.690444    | 0.429185     0.133308     0.017110     0.106213     3.643984    | 0.735487  0.624897  0.769922  | 0.052769  0.047509  0.027045 
+7     | 0.000250  | 0.164418     | 0.218802     | 0.857287        | 0.705953     | 0.041823          | 0.369363     0.076584     0.008088     0.124906     0.570847    | 0.425240     0.130329     0.016959     0.107284     3.472505    | 0.728925  0.630803  0.758824  | 0.054062  0.050084  0.021324 
+8     | 0.000375  | 0.176417     | 0.217759     | 0.860627        | 0.711916     | 0.040232          | 0.380440     0.088978     0.009791     0.143487     0.693595    | 0.434497     0.124871     0.017516     0.109154     3.140163    | 0.736143  0.640432  0.778200  | 0.045936  0.053447  0.021313 
+9     | 0.000500  | 0.172326     | 0.232716     | 0.840850        | 0.685000     | 0.055250          | 0.380048     0.083303     0.009140     0.136270     0.602589    | 0.434726     0.146140     0.019107     0.106446     4.230939    | 0.716109  0.598610  0.767563  | 0.060734  0.051527  0.053491 
+10    | 0.000483  | 0.164837     | 0.217805     | 0.858764        | 0.709166     | 0.041505          | 0.374748     0.074876     0.008210     0.124812     0.484768    | 0.437255     0.123755     0.017283     0.101686     3.273021    | 0.726199  0.635433  0.785103  | 0.046740  0.054562  0.023212 
+11    | 0.000438  | 0.160002     | 0.217279     | 0.858425        | 0.708153     | 0.041394          | 0.369498     0.070218     0.007676     0.117451     0.445314    | 0.436045     0.123522     0.017998     0.103156     3.207809    | 0.735710  0.625677  0.771334  | 0.050111  0.049319  0.024752 
+12    | 0.000375  | 0.156731     | 0.216649     | 0.859202        | 0.711456     | 0.042301          | 0.366573     0.066799     0.007126     0.113265     0.390387    | 0.437321     0.122076     0.017826     0.106077     3.068164    | 0.725843  0.637835  0.773729  | 0.046697  0.051361  0.028845 
+13    | 0.000313  | 0.151555     | 0.217119     | 0.857975        | 0.704551     | 0.039743          | 0.359748     0.062329     0.006658     0.105487     0.368901    | 0.433646     0.124322     0.018777     0.109444     3.074715    | 0.735207  0.604461  0.769197  | 0.052327  0.040263  0.026640 
+14    | 0.000267  | 0.151262     | 0.213822     | 0.864163        | 0.723604     | 0.042131          | 0.359579     0.061983     0.006631     0.105324     0.356245    | 0.430362     0.121019     0.017184     0.098344     3.220494    | 0.745555  0.644815  0.795001  | 0.048064  0.051341  0.026989 
+15    | 0.000250  | 0.147383     | 0.218563     | 0.862293        | 0.721732     | 0.044001          | 0.355732     0.058090     0.006195     0.099226     0.321681    | 0.429215     0.128283     0.017411     0.100540     3.524352    | 0.745810  0.636294  0.801443  | 0.054049  0.053035  0.024917</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2464  1922  1459
+FP   200   214    61
+FN   113   147    67
+TN  4519  5013  5709
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.338  0.263  0.200
+FP  0.027  0.029  0.008
+FN  0.015  0.020  0.009
+TN  0.619  0.687  0.782
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-B        VLo-D        VLo-H       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+-----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.218563     | 0.862293        | 0.721732     | 0.044001          | 0.429215     0.128283     0.017411     0.100540     3.524352    | 0.745810  0.636294  0.801443  | 0.054049  0.053035  0.024917 
+266     | 266     | 0.220775     | 0.862809        | 0.724725     | 0.045135          | 0.424742     0.133360     0.018022     0.100894     3.754561    | 0.743822  0.638651  0.815611  | 0.056616  0.053678  0.025112 
+360     | 310     | 0.190884     | 0.846883        | 0.672410     | 0.036802          | 0.470538     0.071032     0.009579     0.091203     1.082426    | 0.733163  0.576351  0.722134  | 0.040014  0.052429  0.017962 
+276     | 276     | 0.225264     | 0.875201        | 0.742867     | 0.036576          | 0.450793     0.128609     0.019719     0.113386     3.169353    | 0.795685  0.678231  0.722644  | 0.034261  0.044195  0.031273 </t>
+  </si>
 </sst>
 </file>
 
@@ -5046,7 +6564,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -5088,6 +6606,18 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF3465A4"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Courier New"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="4">
@@ -5144,7 +6674,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5261,6 +6791,18 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5318,7 +6860,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF3465A4"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -5444,7 +6986,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K429"/>
+  <dimension ref="A1:K534"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50.36"/>
@@ -9276,8 +10818,827 @@
         <v>0.84338</v>
       </c>
     </row>
-    <row r="429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A429" s="8"/>
+    <row r="428" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A428" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="B428" s="2" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="C428" s="2" t="n">
+        <v>0.85425</v>
+      </c>
+      <c r="D428" s="2" t="n">
+        <v>0.85001</v>
+      </c>
+      <c r="E428" s="12" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="429" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E429" s="12" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="430" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A430" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B430" s="2" t="n">
+        <v>0.861</v>
+      </c>
+      <c r="C430" s="2" t="n">
+        <v>0.85399</v>
+      </c>
+      <c r="D430" s="2" t="n">
+        <v>0.84944</v>
+      </c>
+    </row>
+    <row r="431" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A431" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C431" s="2" t="n">
+        <v>0.85775</v>
+      </c>
+      <c r="D431" s="2" t="n">
+        <v>0.85292</v>
+      </c>
+    </row>
+    <row r="432" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A432" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C432" s="2" t="n">
+        <v>0.85768</v>
+      </c>
+      <c r="D432" s="2" t="n">
+        <v>0.85264</v>
+      </c>
+    </row>
+    <row r="434" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A434" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="B434" s="2" t="n">
+        <v>0.861</v>
+      </c>
+      <c r="C434" s="2" t="n">
+        <v>0.85861</v>
+      </c>
+      <c r="D434" s="2" t="n">
+        <v>0.84973</v>
+      </c>
+      <c r="E434" s="12" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="435" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E435" s="12" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="436" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A436" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B436" s="2" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="C436" s="2" t="n">
+        <v>0.85176</v>
+      </c>
+      <c r="D436" s="2" t="n">
+        <v>0.84725</v>
+      </c>
+    </row>
+    <row r="437" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A437" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C437" s="2" t="n">
+        <v>0.85832</v>
+      </c>
+      <c r="D437" s="2" t="n">
+        <v>0.84905</v>
+      </c>
+    </row>
+    <row r="438" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A438" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C438" s="2" t="n">
+        <v>0.85831</v>
+      </c>
+      <c r="D438" s="2" t="n">
+        <v>0.84935</v>
+      </c>
+    </row>
+    <row r="440" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A440" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="B440" s="29" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="C440" s="29" t="n">
+        <v>0.85943</v>
+      </c>
+      <c r="D440" s="29" t="n">
+        <v>0.8508</v>
+      </c>
+      <c r="E440" s="12" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="441" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B441" s="26" t="s">
+        <v>351</v>
+      </c>
+      <c r="C441" s="29"/>
+      <c r="D441" s="29"/>
+      <c r="E441" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A442" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B442" s="29"/>
+      <c r="C442" s="29" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="D442" s="29" t="n">
+        <v>0.85336</v>
+      </c>
+    </row>
+    <row r="444" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A444" s="8" t="s">
+        <v>353</v>
+      </c>
+      <c r="B444" s="2" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="C444" s="2" t="n">
+        <v>0.85884</v>
+      </c>
+      <c r="D444" s="2" t="n">
+        <v>0.84825</v>
+      </c>
+      <c r="E444" s="12" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="445" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E445" s="12" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A446" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="B446" s="2" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="C446" s="2" t="n">
+        <v>0.85207</v>
+      </c>
+      <c r="D446" s="2" t="n">
+        <v>0.85028</v>
+      </c>
+    </row>
+    <row r="447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A447" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C447" s="2" t="n">
+        <v>0.86027</v>
+      </c>
+      <c r="D447" s="2" t="n">
+        <v>0.85205</v>
+      </c>
+    </row>
+    <row r="448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A448" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="C448" s="2" t="n">
+        <v>0.85867</v>
+      </c>
+      <c r="D448" s="2" t="n">
+        <v>0.84926</v>
+      </c>
+    </row>
+    <row r="450" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A450" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="B450" s="2" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="C450" s="2" t="n">
+        <v>0.85206</v>
+      </c>
+      <c r="D450" s="2" t="n">
+        <v>0.84125</v>
+      </c>
+      <c r="E450" s="12" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="451" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E451" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A452" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C452" s="2" t="n">
+        <v>0.85568</v>
+      </c>
+      <c r="D452" s="2" t="n">
+        <v>0.84705</v>
+      </c>
+    </row>
+    <row r="454" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A454" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="B454" s="16" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="C454" s="2" t="n">
+        <v>0.84973</v>
+      </c>
+      <c r="D454" s="2" t="n">
+        <v>0.8379</v>
+      </c>
+      <c r="E454" s="12" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="455" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E455" s="12" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A456" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B456" s="2" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="C456" s="2" t="n">
+        <v>0.84824</v>
+      </c>
+      <c r="D456" s="2" t="n">
+        <v>0.83558</v>
+      </c>
+    </row>
+    <row r="457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A457" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C457" s="2" t="n">
+        <v>0.85424</v>
+      </c>
+      <c r="D457" s="2" t="n">
+        <v>0.84337</v>
+      </c>
+    </row>
+    <row r="458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A458" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C458" s="2" t="n">
+        <v>0.85441</v>
+      </c>
+      <c r="D458" s="2" t="n">
+        <v>0.84422</v>
+      </c>
+    </row>
+    <row r="461" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A461" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="B461" s="2" t="n">
+        <v>0.853</v>
+      </c>
+      <c r="C461" s="2" t="n">
+        <v>0.85453</v>
+      </c>
+      <c r="D461" s="2" t="n">
+        <v>0.84508</v>
+      </c>
+      <c r="E461" s="12" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="462" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E462" s="12" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A463" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="C463" s="2" t="n">
+        <v>0.85711</v>
+      </c>
+      <c r="D463" s="2" t="n">
+        <v>0.84848</v>
+      </c>
+    </row>
+    <row r="465" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A465" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="B465" s="2" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="C465" s="2" t="n">
+        <v>0.85668</v>
+      </c>
+      <c r="D465" s="2" t="n">
+        <v>0.8443</v>
+      </c>
+      <c r="E465" s="12" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="466" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E466" s="12" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A467" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="B467" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="C467" s="2" t="n">
+        <v>0.84937</v>
+      </c>
+      <c r="D467" s="2" t="n">
+        <v>0.83844</v>
+      </c>
+    </row>
+    <row r="468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A468" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B468" s="3"/>
+      <c r="C468" s="2" t="n">
+        <v>0.86267</v>
+      </c>
+      <c r="D468" s="2" t="n">
+        <v>0.85311</v>
+      </c>
+    </row>
+    <row r="469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A469" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="C469" s="2" t="n">
+        <v>0.86143</v>
+      </c>
+      <c r="D469" s="2" t="n">
+        <v>0.85535</v>
+      </c>
+    </row>
+    <row r="471" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A471" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="B471" s="2" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="C471" s="2" t="n">
+        <v>0.83676</v>
+      </c>
+      <c r="D471" s="2" t="n">
+        <v>0.83205</v>
+      </c>
+      <c r="E471" s="12" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="472" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E472" s="12" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A473" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B473" s="2" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="C473" s="2" t="n">
+        <v>0.85143</v>
+      </c>
+      <c r="D473" s="2" t="n">
+        <v>0.8396</v>
+      </c>
+    </row>
+    <row r="474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A474" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="C474" s="2" t="n">
+        <v>0.86063</v>
+      </c>
+      <c r="D474" s="2" t="n">
+        <v>0.84988</v>
+      </c>
+    </row>
+    <row r="475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A475" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C475" s="2" t="n">
+        <v>0.86037</v>
+      </c>
+      <c r="D475" s="2" t="n">
+        <v>0.85035</v>
+      </c>
+    </row>
+    <row r="477" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A477" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="E477" s="12" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="479" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A479" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="E479" s="12" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="481" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A481" s="30" t="s">
+        <v>375</v>
+      </c>
+      <c r="C481" s="26" t="s">
+        <v>376</v>
+      </c>
+      <c r="E481" s="12" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="483" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A483" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="E483" s="12" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="485" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A485" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="E485" s="12" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="487" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A487" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="E487" s="12" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A488" s="3"/>
+    </row>
+    <row r="489" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A489" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="E489" s="12" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="491" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A491" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="E491" s="12" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="493" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A493" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="B493" s="2" t="n">
+        <v>0.863</v>
+      </c>
+      <c r="C493" s="2" t="n">
+        <v>0.85092</v>
+      </c>
+      <c r="D493" s="2" t="n">
+        <v>0.8412</v>
+      </c>
+      <c r="E493" s="12" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="494" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E494" s="12" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="495" customFormat="false" ht="370.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A495" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B495" s="14" t="n">
+        <v>0.868263</v>
+      </c>
+      <c r="C495" s="2" t="n">
+        <v>0.85663</v>
+      </c>
+      <c r="D495" s="2" t="n">
+        <v>0.84598</v>
+      </c>
+      <c r="E495" s="12" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A496" s="28" t="s">
+        <v>392</v>
+      </c>
+      <c r="B496" s="14" t="n">
+        <v>0.869063</v>
+      </c>
+      <c r="C496" s="2" t="n">
+        <v>0.85638</v>
+      </c>
+      <c r="D496" s="2" t="n">
+        <v>0.84504</v>
+      </c>
+    </row>
+    <row r="497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A497" s="28" t="s">
+        <v>393</v>
+      </c>
+      <c r="B497" s="14" t="n">
+        <v>0.869013</v>
+      </c>
+      <c r="C497" s="2" t="n">
+        <v>0.85638</v>
+      </c>
+      <c r="D497" s="2" t="n">
+        <v>0.84474</v>
+      </c>
+    </row>
+    <row r="498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A498" s="28" t="s">
+        <v>394</v>
+      </c>
+      <c r="B498" s="14" t="n">
+        <v>0.868889</v>
+      </c>
+      <c r="C498" s="2" t="n">
+        <v>0.85658</v>
+      </c>
+      <c r="D498" s="2" t="n">
+        <v>0.84524</v>
+      </c>
+    </row>
+    <row r="500" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A500" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="E500" s="12" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="502" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A502" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E502" s="12" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="504" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A504" s="30" t="s">
+        <v>399</v>
+      </c>
+      <c r="C504" s="26" t="s">
+        <v>400</v>
+      </c>
+      <c r="E504" s="12" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="506" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A506" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E506" s="12" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="508" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A508" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="E508" s="12" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="510" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A510" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="E510" s="12" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="512" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A512" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="E512" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="514" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A514" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="B514" s="2" t="n">
+        <v>0.854048</v>
+      </c>
+      <c r="C514" s="2" t="n">
+        <v>0.85709</v>
+      </c>
+      <c r="D514" s="2" t="n">
+        <v>0.84943</v>
+      </c>
+      <c r="E514" s="12" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="515" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A515" s="3"/>
+      <c r="B515" s="3"/>
+      <c r="E515" s="12" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="516" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A516" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B516" s="2" t="n">
+        <v>0.859208</v>
+      </c>
+      <c r="C516" s="2" t="n">
+        <v>0.85553</v>
+      </c>
+      <c r="D516" s="2" t="n">
+        <v>0.84867</v>
+      </c>
+    </row>
+    <row r="517" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A517" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C517" s="2" t="n">
+        <v>0.86139</v>
+      </c>
+      <c r="D517" s="2" t="n">
+        <v>0.85215</v>
+      </c>
+    </row>
+    <row r="518" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A518" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C518" s="2" t="n">
+        <v>0.86249</v>
+      </c>
+      <c r="D518" s="2" t="n">
+        <v>0.85222</v>
+      </c>
+    </row>
+    <row r="520" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A520" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="E520" s="12" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="522" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A522" s="8" t="s">
+        <v>415</v>
+      </c>
+      <c r="E522" s="12" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="524" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A524" s="8" t="s">
+        <v>417</v>
+      </c>
+      <c r="E524" s="12" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="526" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A526" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="E526" s="12" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="528" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A528" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="E528" s="12" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="530" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A530" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="B530" s="2" t="n">
+        <v>0.862293</v>
+      </c>
+      <c r="C530" s="2" t="n">
+        <v>0.85391</v>
+      </c>
+      <c r="D530" s="2" t="n">
+        <v>0.8439</v>
+      </c>
+      <c r="E530" s="31" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="531" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E531" s="31" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A532" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B532" s="2" t="n">
+        <v>0.864163</v>
+      </c>
+      <c r="C532" s="2" t="n">
+        <v>0.85437</v>
+      </c>
+      <c r="D532" s="2" t="n">
+        <v>0.83893</v>
+      </c>
+    </row>
+    <row r="533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A533" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C533" s="2" t="n">
+        <v>0.85716</v>
+      </c>
+      <c r="D533" s="2" t="n">
+        <v>0.84657</v>
+      </c>
+    </row>
+    <row r="534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A534" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C534" s="2" t="n">
+        <v>0.85664</v>
+      </c>
+      <c r="D534" s="2" t="n">
+        <v>0.84676</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
no presence gate in loss runs on unet, unet++, segformer
</commit_message>
<xml_diff>
--- a/Scores.xlsx
+++ b/Scores.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="496">
   <si>
     <t xml:space="preserve">Description</t>
   </si>
@@ -6690,6 +6690,992 @@
 266     | 266     | 0.174449     | 0.855559        | 0.723361     | 0.056308          | 0.441095     0.060173     0.102274     0.018072    | 0.730792  0.653108  0.790036  | 0.061968  0.070650  0.036307 
 360     | 310     | 0.177505     | 0.831065        | 0.664553     | 0.057926          | 0.473821     0.050512     0.092691     0.008333    | 0.674048  0.562805  0.768737  | 0.083158  0.055468  0.035153 
 276     | 276     | 0.201205     | 0.868722        | 0.735415     | 0.042406          | 0.491080     0.076972     0.133057     0.020888    | 0.771250  0.680121  0.709402  | 0.047864  0.053549  0.025805 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-2
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 15m 55s)
+(Max GPU mem usage : 10270.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.536556     | 0.252378     | 0.727519        | 0.491192     | 0.114929          | 0.484777     0.558747     0.913457     0.204036    | 0.471809     0.158337     0.272320     0.044353    | 0.472035  0.408636  0.600779  | 0.135580  0.132525  0.076682 
+2     | 0.000250  | 0.281710     | 0.182605     | 0.826979        | 0.665448     | 0.065333          | 0.413626     0.225174     0.430246     0.020102    | 0.435305     0.074304     0.135566     0.013043    | 0.692380  0.557296  0.749178  | 0.078651  0.074149  0.043199 
+3     | 0.000375  | 0.190397     | 0.175298     | 0.843887        | 0.694652     | 0.056623          | 0.399670     0.100708     0.192102     0.009314    | 0.434900     0.064040     0.111963     0.016116    | 0.725752  0.609203  0.754632  | 0.075813  0.067793  0.026264 
+4     | 0.000500  | 0.176602     | 0.173623     | 0.847431        | 0.701613     | 0.055356          | 0.393022     0.083851     0.158625     0.009076    | 0.434958     0.061622     0.107299     0.015944    | 0.738281  0.619398  0.761038  | 0.064914  0.058442  0.042712 
+5     | 0.000495  | 0.169604     | 0.192126     | 0.798775        | 0.660708     | 0.109179          | 0.383353     0.077998     0.147378     0.008617    | 0.490843     0.064104     0.109159     0.019050    | 0.677709  0.582409  0.754375  | 0.166650  0.125188  0.035700 
+6     | 0.000480  | 0.164322     | 0.167692     | 0.854666        | 0.715079     | 0.052275          | 0.380020     0.071880     0.135758     0.008003    | 0.418785     0.060081     0.103729     0.016434    | 0.747276  0.652876  0.750084  | 0.059880  0.069938  0.027007 
+7     | 0.000457  | 0.158393     | 0.170313     | 0.850385        | 0.721926     | 0.063975          | 0.372453     0.066653     0.125864     0.007443    | 0.428620     0.059609     0.103098     0.016120    | 0.740676  0.659901  0.764086  | 0.087796  0.079211  0.024917 
+8     | 0.000427  | 0.153869     | 0.164699     | 0.864299        | 0.735132     | 0.049589          | 0.367741     0.062209     0.117487     0.006932    | 0.418508     0.055924     0.095696     0.016152    | 0.753415  0.659862  0.805700  | 0.062011  0.059814  0.026943 
+9     | 0.000393  | 0.152455     | 0.166411     | 0.861219        | 0.729919     | 0.051248          | 0.365686     0.061070     0.115247     0.006894    | 0.420385     0.057565     0.099382     0.015748    | 0.747275  0.659058  0.786080  | 0.053769  0.066994  0.032982 
+10    | 0.000357  | 0.148359     | 0.170083     | 0.861676        | 0.727885     | 0.049130          | 0.360718     0.057348     0.108201     0.006496    | 0.428684     0.059255     0.102513     0.015996    | 0.741781  0.649699  0.798743  | 0.058789  0.058941  0.029662 
+11    | 0.000323  | 0.146229     | 0.170996     | 0.862145        | 0.726440     | 0.047385          | 0.359549     0.054807     0.103578     0.006036    | 0.431286     0.059443     0.102565     0.016322    | 0.744336  0.654203  0.790241  | 0.057461  0.058939  0.025754 
+12    | 0.000293  | 0.144009     | 0.170004     | 0.859885        | 0.720593     | 0.047254          | 0.357052     0.052705     0.099534     0.005876    | 0.432630     0.057450     0.098415     0.016485    | 0.744004  0.647770  0.776876  | 0.060206  0.058448  0.023107 
+13    | 0.000270  | 0.141846     | 0.170836     | 0.862984        | 0.727515     | 0.046703          | 0.354081     0.050889     0.096103     0.005675    | 0.431446     0.059146     0.101206     0.017087    | 0.746450  0.652521  0.791139  | 0.054662  0.064714  0.020733 
+14    | 0.000255  | 0.141074     | 0.168293     | 0.856672        | 0.723473     | 0.054529          | 0.354071     0.049790     0.094092     0.005489    | 0.428600     0.056733     0.096679     0.016787    | 0.744067  0.648638  0.796341  | 0.069668  0.061110  0.032808 
+15    | 0.000250  | 0.141101     | 0.176402     | 0.856101        | 0.718382     | 0.052087          | 0.354175     0.049784     0.094075     0.005492    | 0.442819     0.062223     0.106863     0.017583    | 0.730513  0.642588  0.792799  | 0.066461  0.068833  0.020965 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2370  1870  1418
+FP   119   140    53
+FN   207   199   108
+TN  4600  5087  5717
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.325  0.256  0.194
+FP  0.016  0.019  0.007
+FN  0.028  0.027  0.015
+TN  0.630  0.697  0.784
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.176402     | 0.856101        | 0.718382     | 0.052087          | 0.442819     0.062223     0.106863     0.017583    | 0.730513  0.642588  0.792799  | 0.066461  0.068833  0.020965 
+266     | 266     | 0.176739     | 0.855769        | 0.720269     | 0.053897          | 0.441893     0.063102     0.107756     0.018448    | 0.729426  0.641568  0.801689  | 0.069349  0.070900  0.021443 
+360     | 310     | 0.169033     | 0.848524        | 0.682333     | 0.040681          | 0.448713     0.049170     0.090447     0.007892    | 0.701398  0.627268  0.758195  | 0.052875  0.053916  0.015253 
+276     | 276     | 0.184983     | 0.870994        | 0.737680     | 0.040130          | 0.453683     0.069825     0.122151     0.017500    | 0.787102  0.680418  0.713765  | 0.041260  0.057706  0.021424 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+LLRD stage : st2-b1,b2,b3, st3-b4,b5, st4-b6
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 13m 34s)
+(Max GPU mem usage : 10278.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.540857     | 0.252635     | 0.740888        | 0.508991     | 0.104513          | 0.498261     0.559112     0.914144     0.204080    | 0.478714     0.155744     0.270882     0.040607    | 0.501118  0.413001  0.627159  | 0.121355  0.122213  0.069972 
+2     | 0.000250  | 0.279043     | 0.194743     | 0.812608        | 0.629966     | 0.065631          | 0.417987     0.219495     0.419673     0.019317    | 0.458306     0.081788     0.148269     0.015306    | 0.663767  0.521442  0.689922  | 0.068364  0.081695  0.046833 
+3     | 0.000375  | 0.189693     | 0.172215     | 0.847525        | 0.699779     | 0.053977          | 0.400590     0.099309     0.189138     0.009480    | 0.424955     0.063897     0.112872     0.014922    | 0.734806  0.625419  0.740152  | 0.059266  0.056904  0.045760 
+4     | 0.000500  | 0.179023     | 0.172605     | 0.854917        | 0.710772     | 0.048987          | 0.395192     0.086379     0.163377     0.009382    | 0.433703     0.060705     0.105951     0.015459    | 0.737837  0.631478  0.770403  | 0.058462  0.054584  0.033915 
+5     | 0.000495  | 0.167603     | 0.175383     | 0.847900        | 0.702040     | 0.054860          | 0.383482     0.075084     0.141839     0.008329    | 0.445673     0.059545     0.103149     0.015942    | 0.728417  0.639560  0.748027  | 0.068052  0.071153  0.025377 
+6     | 0.000480  | 0.163622     | 0.165659     | 0.860681        | 0.727316     | 0.050409          | 0.379527     0.071092     0.134145     0.008039    | 0.416754     0.058046     0.100459     0.015634    | 0.749518  0.653258  0.787134  | 0.054057  0.067368  0.029802 
+7     | 0.000457  | 0.157848     | 0.171571     | 0.851824        | 0.707928     | 0.052245          | 0.371797     0.066155     0.124913     0.007398    | 0.434633     0.058830     0.101431     0.016229    | 0.725894  0.633169  0.771101  | 0.058830  0.060588  0.037318 
+8     | 0.000427  | 0.152895     | 0.168482     | 0.851977        | 0.714243     | 0.056200          | 0.366130     0.061508     0.116133     0.006883    | 0.424254     0.058865     0.100337     0.017393    | 0.732032  0.636166  0.784810  | 0.064566  0.072967  0.031068 
+9     | 0.000393  | 0.150975     | 0.167575     | 0.855005        | 0.718022     | 0.053673          | 0.364354     0.059526     0.112419     0.006634    | 0.422494     0.058324     0.100327     0.016320    | 0.737820  0.655854  0.771543  | 0.059026  0.067939  0.034055 
+10    | 0.000357  | 0.147932     | 0.169635     | 0.863709        | 0.730862     | 0.047726          | 0.360843     0.056684     0.107055     0.006313    | 0.430764     0.057723     0.099009     0.016436    | 0.745516  0.656677  0.794035  | 0.057005  0.061065  0.025109 
+11    | 0.000323  | 0.147068     | 0.167753     | 0.859134        | 0.723342     | 0.050337          | 0.360694     0.055513     0.104871     0.006156    | 0.422787     0.058453     0.100570     0.016335    | 0.740604  0.650419  0.781096  | 0.054851  0.060580  0.035581 
+12    | 0.000293  | 0.142333     | 0.168051     | 0.863078        | 0.729441     | 0.047830          | 0.354572     0.051374     0.097090     0.005657    | 0.425269     0.057815     0.099627     0.016002    | 0.741945  0.664948  0.787686  | 0.055719  0.057363  0.030409 
+13    | 0.000270  | 0.140300     | 0.166529     | 0.863148        | 0.735960     | 0.052060          | 0.352739     0.049254     0.093045     0.005463    | 0.421697     0.057171     0.097860     0.016482    | 0.749376  0.662874  0.796204  | 0.056921  0.069732  0.029526 
+14    | 0.000255  | 0.140822     | 0.167056     | 0.864012        | 0.734664     | 0.049756          | 0.353470     0.049687     0.093860     0.005515    | 0.424884     0.056559     0.095945     0.017173    | 0.749005  0.667979  0.796612  | 0.058579  0.062762  0.027928 
+15    | 0.000250  | 0.139155     | 0.169969     | 0.865391        | 0.735746     | 0.048179          | 0.351472     0.048161     0.091022     0.005300    | 0.434790     0.056474     0.096680     0.016267    | 0.753935  0.663571  0.793907  | 0.060631  0.058050  0.025854 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2454  1921  1449
+FP   161   173    81
+FN   123   148    77
+TN  4558  5054  5689
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.336  0.263  0.199
+FP  0.022  0.024  0.011
+FN  0.017  0.020  0.011
+TN  0.625  0.693  0.780
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.169969     | 0.865391        | 0.735746     | 0.048179          | 0.434790     0.056474     0.096680     0.016267    | 0.753935  0.663571  0.793907  | 0.060631  0.058050  0.025854 
+266     | 266     | 0.169549     | 0.866121        | 0.739448     | 0.049431          | 0.432141     0.057009     0.097158     0.016860    | 0.752756  0.666496  0.803280  | 0.062344  0.059410  0.026539 
+360     | 310     | 0.162810     | 0.852319        | 0.692656     | 0.041238          | 0.435925     0.045761     0.083209     0.008313    | 0.748402  0.610160  0.761633  | 0.059687  0.049668  0.014360 
+276     | 276     | 0.198494     | 0.870821        | 0.735027     | 0.038650          | 0.503591     0.067738     0.116126     0.019351    | 0.779982  0.684061  0.703993  | 0.036204  0.048828  0.030917 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+LLRD stage : st2-b1,b2,b3, st3-b4,b5, st4-b6
+weight decay 1e-2
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 17m 3s)
+(Max GPU mem usage : 10278.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.542501     | 0.256716     | 0.729558        | 0.485024     | 0.107420          | 0.499411     0.560968     0.917136     0.204800    | 0.481491     0.160384     0.274693     0.046074    | 0.461199  0.403300  0.610149  | 0.125662  0.127975  0.068623 
+2     | 0.000250  | 0.289258     | 0.205106     | 0.771128        | 0.562100     | 0.089520          | 0.417485     0.234303     0.446293     0.022313    | 0.452573     0.099049     0.174444     0.023655    | 0.551117  0.425073  0.724172  | 0.104767  0.121778  0.042014 
+3     | 0.000375  | 0.205735     | 0.175674     | 0.838745        | 0.685861     | 0.059333          | 0.401064     0.122022     0.232154     0.011891    | 0.429599     0.066850     0.118191     0.015508    | 0.729470  0.573892  0.755437  | 0.089924  0.057464  0.030611 
+4     | 0.000500  | 0.177904     | 0.171378     | 0.850232        | 0.714993     | 0.059609          | 0.394086     0.085255     0.161321     0.009188    | 0.431734     0.059798     0.104016     0.015579    | 0.736779  0.637653  0.780528  | 0.070090  0.075473  0.033262 
+5     | 0.000495  | 0.167526     | 0.175586     | 0.838446        | 0.701319     | 0.070135          | 0.381924     0.075641     0.142927     0.008356    | 0.442113     0.061360     0.105857     0.016862    | 0.730993  0.627720  0.747307  | 0.072717  0.092443  0.045246 
+6     | 0.000480  | 0.162045     | 0.172764     | 0.848502        | 0.706069     | 0.056543          | 0.376110     0.070303     0.132709     0.007897    | 0.429936     0.062547     0.107558     0.017537    | 0.724285  0.638910  0.757548  | 0.068231  0.074267  0.027132 
+7     | 0.000457  | 0.158329     | 0.169513     | 0.857167        | 0.721745     | 0.052552          | 0.371897     0.066800     0.126134     0.007466    | 0.424824     0.060094     0.104096     0.016092    | 0.743303  0.646993  0.771623  | 0.056508  0.061906  0.039241 
+8     | 0.000427  | 0.153065     | 0.166851     | 0.861656        | 0.726030     | 0.047927          | 0.366620     0.061541     0.116209     0.006873    | 0.418488     0.059007     0.102151     0.015862    | 0.740703  0.647867  0.797466  | 0.055278  0.055958  0.032546 
+9     | 0.000393  | 0.149625     | 0.165454     | 0.861874        | 0.728875     | 0.049461          | 0.362241     0.058505     0.110475     0.006534    | 0.418892     0.056838     0.098226     0.015450    | 0.746629  0.657880  0.787893  | 0.058627  0.062593  0.027162 
+10    | 0.000357  | 0.146771     | 0.172137     | 0.853317        | 0.713139     | 0.053231          | 0.359335     0.055671     0.105094     0.006249    | 0.439333     0.057624     0.098688     0.016561    | 0.728098  0.643361  0.783395  | 0.066552  0.065286  0.027856 
+11    | 0.000323  | 0.148139     | 0.175029     | 0.862588        | 0.727616     | 0.047430          | 0.362063     0.056457     0.106581     0.006333    | 0.442997     0.060185     0.103584     0.016786    | 0.741472  0.658015  0.787970  | 0.058137  0.057708  0.026446 
+12    | 0.000293  | 0.142708     | 0.167127     | 0.861134        | 0.732864     | 0.053352          | 0.354829     0.051799     0.097811     0.005787    | 0.425693     0.056313     0.096618     0.016007    | 0.749980  0.660480  0.796898  | 0.072425  0.061606  0.026026 
+13    | 0.000270  | 0.142325     | 0.171203     | 0.856080        | 0.726095     | 0.057264          | 0.354843     0.051245     0.096803     0.005687    | 0.432471     0.059231     0.101301     0.017161    | 0.741614  0.651491  0.777371  | 0.086693  0.057940  0.027157 
+14    | 0.000255  | 0.139943     | 0.172693     | 0.858295        | 0.724073     | 0.052223          | 0.351500     0.049276     0.093145     0.005407    | 0.433917     0.060740     0.103170     0.018310    | 0.740806  0.642607  0.787703  | 0.061415  0.064109  0.031146 
+15    | 0.000250  | 0.138887     | 0.172409     | 0.856258        | 0.723104     | 0.054972          | 0.351574     0.047735     0.090205     0.005265    | 0.437548     0.058778     0.100585     0.016970    | 0.735335  0.652431  0.790632  | 0.070427  0.072899  0.021590</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2471  1977  1436
+FP   212   254    60
+FN   106    92    90
+TN  4507  4973  5710
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.339  0.271  0.197
+FP  0.029  0.035  0.008
+FN  0.015  0.013  0.012
+TN  0.618  0.682  0.783
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.172409     | 0.856258        | 0.723104     | 0.054972          | 0.437548     0.058778     0.100585     0.016970    | 0.735335  0.652431  0.790632  | 0.070427  0.072899  0.021590 
+266     | 266     | 0.171600     | 0.856586        | 0.725737     | 0.056182          | 0.433473     0.059369     0.101072     0.017666    | 0.735041  0.655012  0.798337  | 0.073190  0.075046  0.020311 
+360     | 310     | 0.176789     | 0.839873        | 0.679148     | 0.052977          | 0.473056     0.049817     0.090565     0.009070    | 0.700279  0.593702  0.767373  | 0.064573  0.065175  0.029182 
+276     | 276     | 0.183725     | 0.873792        | 0.743694     | 0.039476          | 0.462345     0.064316     0.111478     0.017154    | 0.789496  0.689314  0.709348  | 0.036791  0.050986  0.030652 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit-b4 with LLRD and aux weight decay 1e-5
+No presence gate in loss
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(8h 58m 53s)
+(Max GPU mem usage : 12718.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.434094     | 0.191585     | 0.817034        | 0.629981     | 0.058264          | 0.464067     0.421249     0.746863     0.095635    | 0.419099     0.094080     0.174200     0.013959    | 0.694040  0.543706  0.626553  | 0.062020  0.055447  0.057326 
+2     | 0.000250  | 0.206864     | 0.171599     | 0.851119        | 0.690335     | 0.041692          | 0.386889     0.129710     0.250653     0.008768    | 0.416103     0.066812     0.121163     0.012460    | 0.726140  0.607121  0.731538  | 0.054351  0.054161  0.016565 
+3     | 0.000375  | 0.177059     | 0.169792     | 0.848395        | 0.701064     | 0.053384          | 0.372646     0.093236     0.178251     0.008221    | 0.420215     0.062468     0.109835     0.015101    | 0.740318  0.615238  0.735847  | 0.050787  0.058510  0.050855 
+4     | 0.000500  | 0.168431     | 0.171130     | 0.849942        | 0.706537     | 0.054454          | 0.367896     0.082945     0.157890     0.008000    | 0.425320     0.062192     0.109095     0.015288    | 0.739375  0.626886  0.777917  | 0.060151  0.063202  0.040011 
+5     | 0.000495  | 0.161848     | 0.166185     | 0.857428        | 0.721128     | 0.051705          | 0.360724     0.076616     0.145627     0.007605    | 0.410458     0.061496     0.108063     0.014929    | 0.749704  0.637983  0.780856  | 0.058561  0.058645  0.037907 
+6     | 0.000480  | 0.155664     | 0.170982     | 0.851528        | 0.711308     | 0.054992          | 0.354142     0.070603     0.134012     0.007194    | 0.432983     0.058696     0.101164     0.016228    | 0.739864  0.636528  0.776144  | 0.057105  0.063046  0.044825 
+7     | 0.000457  | 0.152335     | 0.168250     | 0.852990        | 0.716565     | 0.056061          | 0.351038     0.067176     0.127523     0.006828    | 0.419967     0.060371     0.103372     0.017371    | 0.744143  0.641027  0.772446  | 0.060089  0.057658  0.050436 
+8     | 0.000427  | 0.146726     | 0.166532     | 0.860587        | 0.724509     | 0.048695          | 0.344520     0.061957     0.117657     0.006257    | 0.416684     0.059323     0.101493     0.017154    | 0.751645  0.649801  0.781632  | 0.056061  0.049719  0.040305 
+9     | 0.000393  | 0.145087     | 0.167042     | 0.858775        | 0.725473     | 0.052357          | 0.344197     0.059754     0.113347     0.006160    | 0.414443     0.061013     0.105185     0.016841    | 0.747322  0.655218  0.783431  | 0.054862  0.056684  0.045524 
+10    | 0.000357  | 0.142995     | 0.165262     | 0.866030        | 0.737116     | 0.048028          | 0.341912     0.057745     0.109577     0.005913    | 0.413557     0.058850     0.100468     0.017232    | 0.760512  0.655643  0.804268  | 0.056589  0.056992  0.030502 
+11    | 0.000323  | 0.142296     | 0.168070     | 0.855108        | 0.717628     | 0.053239          | 0.340938     0.057164     0.108426     0.005902    | 0.420177     0.060023     0.101394     0.018652    | 0.742560  0.645925  0.779033  | 0.058896  0.055549  0.045271 
+12    | 0.000293  | 0.140013     | 0.169651     | 0.864428        | 0.727709     | 0.044426          | 0.338087     0.055125     0.104569     0.005680    | 0.420351     0.062207     0.106170     0.018245    | 0.747550  0.645258  0.796149  | 0.053307  0.048798  0.031171 
+13    | 0.000270  | 0.135321     | 0.168870     | 0.865487        | 0.732073     | 0.045571          | 0.333736     0.050285     0.095395     0.005176    | 0.424594     0.059274     0.099687     0.018861    | 0.753187  0.646906  0.803322  | 0.058270  0.052060  0.026383 
+14    | 0.000255  | 0.134402     | 0.171203     | 0.864074        | 0.732922     | 0.048492          | 0.332688     0.049422     0.093771     0.005073    | 0.425146     0.062370     0.104095     0.020645    | 0.752857  0.649830  0.800912  | 0.056999  0.052714  0.035763 
+15    | 0.000250  | 0.135566     | 0.170551     | 0.866759        | 0.737515     | 0.047079          | 0.334747     0.050202     0.095112     0.005292    | 0.426173     0.060999     0.103550     0.018449    | 0.757549  0.657233  0.804335  | 0.053953  0.051496  0.035788 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2422  1858  1461
+FP   125   136    61
+FN   155   211    65
+TN  4594  5091  5709
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.332  0.255  0.200
+FP  0.017  0.019  0.008
+FN  0.021  0.029  0.009
+TN  0.630  0.698  0.782
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.170551     | 0.866759        | 0.737515     | 0.047079          | 0.426173     0.060999     0.103550     0.018449    | 0.757549  0.657233  0.804335  | 0.053953  0.051496  0.035788 
+266     | 266     | 0.171292     | 0.865870        | 0.736725     | 0.048033          | 0.425783     0.062224     0.105184     0.019264    | 0.751610  0.658172  0.812355  | 0.054554  0.052506  0.037039 
+360     | 310     | 0.156748     | 0.863655        | 0.722112     | 0.041984          | 0.416277     0.045521     0.082311     0.008731    | 0.761416  0.610166  0.797358  | 0.057807  0.046551  0.021594 
+276     | 276     | 0.183686     | 0.885661        | 0.773496     | 0.039562          | 0.460449     0.065074     0.110389     0.019758    | 0.845944  0.704793  0.687565  | 0.039802  0.042937  0.035947 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(52m 22s)
+Cutoffs(LB,SB,S) | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+---------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.163082     | 0.867084        | 0.739817     | 0.048071          | 0.413612     0.055712     0.092620     0.018803    | 0.763867  0.668276  0.803886  | 0.058453  0.051833  0.033929 
+(0.25,0.25,0.25) | 0.163082     | 0.867595        | 0.740581     | 0.047729          | 0.413612     0.055712     0.092620     0.018803    | 0.763625  0.669229  0.806364  | 0.058453  0.050909  0.033824 
+(0.50,0.50,0.50) | 0.163082     | 0.870001        | 0.746120     | 0.047412          | 0.413612     0.055712     0.092620     0.018803    | 0.768020  0.672601  0.811107  | 0.058285  0.050183  0.033767 
+(0.75,0.75,0.75) | 0.163082     | 0.871251        | 0.748560     | 0.046956          | 0.413612     0.055712     0.092620     0.018803    | 0.768646  0.675625  0.814836  | 0.056984  0.050115  0.033767 
+(0.60,0.70,0.70) | 0.163082     | 0.871302        | 0.749359     | 0.047402          | 0.413612     0.055712     0.092620     0.018803    | 0.767560  0.675383  0.814646  | 0.058285  0.050155  0.033767 
+(0.60,0.70,0.80) | 0.163082     | 0.871494        | 0.749825     | 0.047394          | 0.413612     0.055712     0.092620     0.018803    | 0.767560  0.675383  0.816364  | 0.058285  0.050155  0.033743 
+(0.50,0.75,0.75) | 0.163082     | 0.871239        | 0.749182     | 0.047389          | 0.413612     0.055712     0.092620     0.018803    | 0.768020  0.675625  0.814836  | 0.058285  0.050115  0.033767 
+(0.6, 0.7, 0.8) tensor(0.8715)
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2530  1988  1489
+FP   222   222    74
+FN    47    81    37
+TN  4497  5005  5696
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.347  0.272  0.204
+FP  0.030  0.030  0.010
+FN  0.006  0.011  0.005
+TN  0.616  0.686  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.163082     | 0.871494        | 0.749825     | 0.047394          | 0.413612     0.055712     0.092620     0.018803    | 0.767560  0.675383  0.816364  | 0.058285  0.050155  0.033743 
+266     | 266     | 0.163053     | 0.870778        | 0.749956     | 0.048674          | 0.411599     0.056534     0.093459     0.019608    | 0.763052  0.678221  0.823583  | 0.060496  0.051368  0.034159 
+360     | 310     | 0.154265     | 0.864453        | 0.724299     | 0.042111          | 0.410836     0.044306     0.079420     0.009193    | 0.761251  0.609912  0.804488  | 0.050840  0.044602  0.030890 
+276     | 276     | 0.185012     | 0.892931        | 0.785179     | 0.035235          | 0.474621     0.060895     0.101652     0.020138    | 0.849660  0.713791  0.719987  | 0.035034  0.039364  0.031308 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA with 0.75,0.75,0.75 cutoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA with 0.6,0.7,0.8 cutoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same config mitb4 with full data for training
+(9h 9m 44s)
+(Max GPU mem usage : 12718.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | TLo-Pres     TLo-Seg      TLo-D        TLo-B       
+--------------------------------------------------------------------------------------
+1     | 0.000125  | 0.395483     | 0.436627     0.377851     0.669244     0.086456    
+2     | 0.000250  | 0.193216     | 0.381991     0.112312     0.216104     0.008520    
+3     | 0.000375  | 0.172586     | 0.371703     0.087250     0.166416     0.008085    
+4     | 0.000500  | 0.167206     | 0.367053     0.081557     0.154973     0.008142    
+5     | 0.000495  | 0.160361     | 0.359737     0.074914     0.142224     0.007604    
+6     | 0.000480  | 0.155200     | 0.353607     0.070168     0.133145     0.007192    
+7     | 0.000457  | 0.151833     | 0.350934     0.066504     0.126099     0.006910    
+8     | 0.000427  | 0.146665     | 0.345013     0.061660     0.116835     0.006484    
+9     | 0.000393  | 0.145296     | 0.344820     0.059786     0.113229     0.006343    
+10    | 0.000357  | 0.142688     | 0.341811     0.057350     0.108618     0.006081    
+11    | 0.000323  | 0.139133     | 0.337842     0.053972     0.102226     0.005719    
+12    | 0.000293  | 0.138964     | 0.337916     0.053699     0.101746     0.005651    
+13    | 0.000270  | 0.136011     | 0.334799     0.050816     0.096233     0.005399    
+14    | 0.000255  | 0.136213     | 0.335457     0.050822     0.096201     0.005443    
+15    | 0.000250  | 0.134647     | 0.333949     0.049232     0.093204     0.005260    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit-b5 with LLRD and aux weight decay 1e-3
+No presence gate in loss
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(10h 19m 4s)
+(Max GPU mem usage : 15026.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.433685     | 0.192454     | 0.818533        | 0.639807     | 0.062316          | 0.452826     0.425482     0.750549     0.100414    | 0.432102     0.089748     0.166350     0.013146    | 0.683340  0.548351  0.668381  | 0.073365  0.057882  0.055701 
+2     | 0.000250  | 0.204309     | 0.177096     | 0.842102        | 0.685365     | 0.053407          | 0.385471     0.126668     0.244554     0.008783    | 0.441848     0.063631     0.113445     0.013818    | 0.713523  0.590625  0.743904  | 0.053327  0.059007  0.047887 
+3     | 0.000375  | 0.177089     | 0.168918     | 0.848791        | 0.700863     | 0.052590          | 0.374716     0.092393     0.176726     0.008060    | 0.411471     0.064967     0.116256     0.013679    | 0.730043  0.616576  0.761376  | 0.058353  0.053320  0.046098 
+4     | 0.000500  | 0.169156     | 0.178877     | 0.823524        | 0.666061     | 0.071501          | 0.367705     0.084064     0.160145     0.007983    | 0.449289     0.062986     0.107687     0.018286    | 0.695493  0.583163  0.762460  | 0.088853  0.071422  0.054227 
+5     | 0.000495  | 0.162148     | 0.167387     | 0.860060        | 0.723082     | 0.048622          | 0.361431     0.076741     0.145856     0.007626    | 0.413772     0.061794     0.108772     0.014816    | 0.743251  0.648068  0.766451  | 0.052765  0.051918  0.041183 
+6     | 0.000480  | 0.155389     | 0.164764     | 0.863444        | 0.724940     | 0.044221          | 0.354218     0.070176     0.133326     0.007026    | 0.410839     0.059303     0.102960     0.015647    | 0.756252  0.645805  0.787639  | 0.053302  0.055254  0.024106 
+7     | 0.000457  | 0.150972     | 0.166880     | 0.862776        | 0.728736     | 0.047864          | 0.348951     0.066124     0.125551     0.006696    | 0.418164     0.059188     0.102206     0.016169    | 0.747275  0.649129  0.799300  | 0.048522  0.059514  0.035556 
+8     | 0.000427  | 0.145178     | 0.167217     | 0.860685        | 0.725294     | 0.049054          | 0.343204     0.060309     0.114530     0.006089    | 0.414978     0.061034     0.104368     0.017701    | 0.755659  0.650824  0.782350  | 0.059542  0.052571  0.035048 
+9     | 0.000393  | 0.144320     | 0.169802     | 0.859824        | 0.727004     | 0.051629          | 0.343191     0.059090     0.112174     0.006006    | 0.428730     0.058833     0.100001     0.017666    | 0.755376  0.658089  0.763109  | 0.052699  0.053150  0.049039 
+10    | 0.000357  | 0.141962     | 0.166824     | 0.857427        | 0.723008     | 0.052959          | 0.340553     0.056852     0.107927     0.005776    | 0.419451     0.058556     0.098896     0.018216    | 0.747975  0.644889  0.790359  | 0.060869  0.055820  0.042188 
+11    | 0.000323  | 0.139885     | 0.171783     | 0.864598        | 0.730094     | 0.045733          | 0.338201     0.054893     0.104180     0.005605    | 0.430130     0.061062     0.104265     0.017860    | 0.752003  0.652133  0.791406  | 0.047627  0.048688  0.040883 
+12    | 0.000293  | 0.137083     | 0.170088     | 0.863667        | 0.731300     | 0.048089          | 0.335876     0.051887     0.098490     0.005283    | 0.426905     0.060023     0.101312     0.018735    | 0.741549  0.661854  0.802396  | 0.053882  0.056012  0.034372 
+13    | 0.000270  | 0.136329     | 0.166407     | 0.862193        | 0.735172     | 0.053126          | 0.335318     0.051048     0.096819     0.005278    | 0.418032     0.058567     0.097890     0.019244    | 0.757175  0.664333  0.802883  | 0.054894  0.063619  0.040866 
+14    | 0.000255  | 0.134043     | 0.168498     | 0.867682        | 0.740870     | 0.047776          | 0.333246     0.048670     0.092340     0.005000    | 0.423617     0.059162     0.098437     0.019887    | 0.763164  0.660480  0.799103  | 0.054731  0.051649  0.036949 
+15    | 0.000250  | 0.134366     | 0.165415     | 0.867395        | 0.736625     | 0.045426          | 0.333834     0.048880     0.092655     0.005104    | 0.415162     0.058380     0.097944     0.018817    | 0.759244  0.653781  0.801614  | 0.054751  0.055308  0.026219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2522  1996  1453
+FP   208   239    60
+FN    55    73    73
+TN  4511  4988  5710
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.346  0.274  0.199
+FP  0.029  0.033  0.008
+FN  0.008  0.010  0.010
+TN  0.618  0.684  0.783
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.165415     | 0.867395        | 0.736625     | 0.045426          | 0.415162     0.058380     0.097944     0.018817    | 0.759244  0.653781  0.801614  | 0.054751  0.055308  0.026219 
+266     | 266     | 0.164815     | 0.867417        | 0.738645     | 0.046736          | 0.410920     0.059341     0.099138     0.019544    | 0.758247  0.658807  0.803056  | 0.057035  0.056962  0.026211 
+360     | 310     | 0.162496     | 0.852903        | 0.688313     | 0.037370          | 0.434930     0.045738     0.081593     0.009883    | 0.708973  0.558939  0.834193  | 0.043977  0.045165  0.022967 
+276     | 276     | 0.188623     | 0.888062        | 0.774933     | 0.036519          | 0.482236     0.062789     0.104945     0.020633    | 0.846790  0.701096  0.714782  | 0.034851  0.044025  0.030682 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cutoffs(LB,SB,S) | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+---------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.163180     | 0.868247        | 0.745480     | 0.049909          | 0.415117     0.055207     0.091321     0.019094    | 0.766576  0.670553  0.809589  | 0.056124  0.053304  0.040299 
+(0.25,0.25,0.25) | 0.163180     | 0.868760        | 0.745307     | 0.048937          | 0.415117     0.055207     0.091321     0.019094    | 0.765368  0.670204  0.810969  | 0.056124  0.053304  0.037383 
+(0.50,0.50,0.50) | 0.163180     | 0.870245        | 0.748754     | 0.048761          | 0.415117     0.055207     0.091321     0.019094    | 0.768015  0.673210  0.814492  | 0.056124  0.053247  0.036913 
+(0.75,0.75,0.75) | 0.163180     | 0.872387        | 0.753779     | 0.048541          | 0.415117     0.055207     0.091321     0.019094    | 0.771531  0.679436  0.819409  | 0.055681  0.053198  0.036743 
+(0.60,0.70,0.70) | 0.163180     | 0.871850        | 0.752639     | 0.048676          | 0.415117     0.055207     0.091321     0.019094    | 0.770020  0.677535  0.817875  | 0.055895  0.053220  0.036913 
+(0.60,0.70,0.80) | 0.163180     | 0.872088        | 0.753149     | 0.048619          | 0.415117     0.055207     0.091321     0.019094    | 0.770020  0.677535  0.819670  | 0.055895  0.053220  0.036743 
+(0.50,0.75,0.75) | 0.163180     | 0.871877        | 0.752725     | 0.048688          | 0.415117     0.055207     0.091321     0.019094    | 0.768015  0.679436  0.819409  | 0.056124  0.053198  0.036743
+(0.75, 0.75, 0.75) – best cutoff
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2511  1981  1494
+FP   195   219    73
+FN    66    88    32
+TN  4524  5008  5697
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.344  0.272  0.205
+FP  0.027  0.030  0.010
+FN  0.009  0.012  0.004
+TN  0.620  0.686  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.163180     | 0.872387        | 0.753779     | 0.048541          | 0.415117     0.055207     0.091321     0.019094    | 0.771531  0.679436  0.819409  | 0.055681  0.053198  0.036743 
+266     | 266     | 0.162388     | 0.872111        | 0.755738     | 0.050307          | 0.410366     0.056112     0.092413     0.019810    | 0.770038  0.684190  0.824433  | 0.057564  0.055248  0.038110 
+360     | 310     | 0.159724     | 0.864858        | 0.717078     | 0.036622          | 0.435016     0.041742     0.073491     0.009993    | 0.738985  0.604649  0.832979  | 0.042585  0.044560  0.022721 
+276     | 276     | 0.192866     | 0.887228        | 0.774967     | 0.037932          | 0.495641     0.063106     0.104622     0.021589    | 0.840579  0.700559  0.712531  | 0.044902  0.033964  0.034932 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same config mitb5 with full data for training
+(10h 49m 18s)
+(Max GPU mem usage : 14664.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | TLo-Pres     TLo-Seg      TLo-D        TLo-B       
+--------------------------------------------------------------------------------------
+1     | 0.000125  | 0.397409     | 0.441153     0.378662     0.674419     0.082902    
+2     | 0.000250  | 0.193735     | 0.383902     0.112235     0.215630     0.008840    
+3     | 0.000375  | 0.174740     | 0.373392     0.089603     0.170778     0.008429    
+4     | 0.000500  | 0.166349     | 0.366213     0.080693     0.153233     0.008152    
+5     | 0.000495  | 0.159899     | 0.359832     0.074214     0.140821     0.007607    
+6     | 0.000480  | 0.155589     | 0.354632     0.070284     0.133327     0.007242    
+7     | 0.000457  | 0.151269     | 0.350113     0.066051     0.125225     0.006876    
+8     | 0.000427  | 0.148375     | 0.348433     0.062636     0.118722     0.006550    
+9     | 0.000393  | 0.144229     | 0.343155     0.058975     0.111800     0.006150    
+10    | 0.000357  | 0.140976     | 0.339798     0.055767     0.105735     0.005799    
+11    | 0.000323  | 0.139147     | 0.338439     0.053736     0.101829     0.005643    
+12    | 0.000293  | 0.138311     | 0.338072     0.052699     0.099833     0.005565    
+13    | 0.000270  | 0.135982     | 0.335034     0.050675     0.096002     0.005347    
+14    | 0.000255  | 0.134516     | 0.334382     0.048859     0.092543     0.005175    
+15    | 0.000250  | 0.132982     | 0.333293     0.047135     0.089273     0.004996    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA 14 with cutoff 0.75, 0.75, 0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA 14 with cutoff 0.6,0.7,0.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit-b5 with LLRD and aux weight decay 1e-3
+With presence gate in loss
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(10h 26m 54s)
+(Max GPU mem usage : 15026.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B        TLo-PmC1     TLo-PmC2     TLo-PmC3    | VLo-Pres     VLo-Seg      VLo-D        VLo-B        VLo-PmC1     VLo-PmC2     VLo-PmC3    | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.572562     | 0.289300     | 0.767334        | 0.539282     | 0.080631          | 0.547432     0.583332     0.925446     0.241217     0.549546     0.505931     0.491868    | 0.619324     0.147861     0.249265     0.046457     0.684810     0.588551     0.526792    | 0.593162  0.482569  0.544855  | 0.089559  0.078091  0.074242 
+2     | 0.000250  | 0.306401     | 0.210463     | 0.838723        | 0.681080     | 0.056182          | 0.592093     0.183962     0.355700     0.012225     0.636358     0.599329     0.593746    | 0.545959     0.066678     0.120539     0.012817     0.602175     0.556969     0.506795    | 0.712593  0.587165  0.755036  | 0.052024  0.078988  0.037534 
+3     | 0.000375  | 0.217254     | 0.194984     | 0.853834        | 0.709793     | 0.050140          | 0.472553     0.107840     0.207427     0.008253     0.553711     0.517297     0.499007    | 0.505438     0.061932     0.110106     0.013759     0.552737     0.556035     0.454943    | 0.745431  0.619852  0.768704  | 0.060516  0.057762  0.032141 
+4     | 0.000500  | 0.189756     | 0.177997     | 0.855773        | 0.717606     | 0.052117          | 0.421456     0.090455     0.172845     0.008065     0.511403     0.472402     0.444607    | 0.446898     0.062754     0.110741     0.014767     0.500758     0.460461     0.367183    | 0.752271  0.632899  0.761982  | 0.060153  0.051357  0.044839 
+5     | 0.000495  | 0.173335     | 0.171420     | 0.854706        | 0.716613     | 0.053231          | 0.391362     0.079896     0.151958     0.007833     0.485789     0.442177     0.412136    | 0.426554     0.062077     0.108870     0.015284     0.453114     0.413878     0.387642    | 0.744069  0.617351  0.787802  | 0.049903  0.066376  0.043415 
+6     | 0.000480  | 0.166988     | 0.186544     | 0.845445        | 0.685633     | 0.048014          | 0.378815     0.076204     0.144481     0.007927     0.471162     0.426029     0.392855    | 0.454526     0.071694     0.123410     0.019978     0.528559     0.392556     0.339802    | 0.714835  0.624573  0.695627  | 0.046962  0.069251  0.027828 
+7     | 0.000457  | 0.156518     | 0.173189     | 0.856754        | 0.726654     | 0.056512          | 0.363241     0.067923     0.128725     0.007121     0.459218     0.413347     0.376401    | 0.431580     0.062450     0.107194     0.017706     0.432582     0.393851     0.415654    | 0.752688  0.652611  0.777218  | 0.054286  0.067299  0.047952 
+8     | 0.000427  | 0.153441     | 0.171627     | 0.851720        | 0.716163     | 0.057909          | 0.358374     0.065613     0.124112     0.007115     0.450548     0.405715     0.366581    | 0.428395     0.061584     0.102642     0.020525     0.448136     0.395478     0.359750    | 0.747015  0.628867  0.774489  | 0.072645  0.051316  0.049765 
+9     | 0.000393  | 0.148264     | 0.170381     | 0.861485        | 0.727239     | 0.049019          | 0.352531     0.060721     0.114823     0.006618     0.444997     0.396847     0.358901    | 0.425158     0.061190     0.101704     0.020677     0.434134     0.397341     0.337323    | 0.748957  0.653510  0.783936  | 0.060330  0.053394  0.033333 
+10    | 0.000357  | 0.144199     | 0.171961     | 0.857187        | 0.723661     | 0.053796          | 0.345977     0.057723     0.109085     0.006361     0.437854     0.390671     0.352894    | 0.433043     0.060068     0.099547     0.020590     0.446895     0.394630     0.324109    | 0.744422  0.647525  0.784936  | 0.060966  0.060964  0.039457 
+11    | 0.000323  | 0.142886     | 0.168688     | 0.858897        | 0.725318     | 0.052050          | 0.344967     0.056280     0.106345     0.006215     0.433492     0.387263     0.349548    | 0.421638     0.060281     0.101172     0.019390     0.432949     0.390845     0.336313    | 0.744535  0.642406  0.799790  | 0.059722  0.055575  0.040852 
+12    | 0.000293  | 0.138508     | 0.169203     | 0.864928        | 0.733393     | 0.047381          | 0.338892     0.052629     0.099386     0.005871     0.429959     0.382401     0.344394    | 0.426025     0.059136     0.099362     0.018910     0.426598     0.376766     0.334111    | 0.755394  0.654479  0.793768  | 0.055544  0.059050  0.027548 
+13    | 0.000270  | 0.136976     | 0.166427     | 0.864110        | 0.738043     | 0.051845          | 0.337284     0.051129     0.096612     0.005646     0.427423     0.380670     0.341289    | 0.417255     0.058929     0.097657     0.020201     0.415690     0.375426     0.334393    | 0.755863  0.666165  0.805478  | 0.055278  0.058268  0.041989 
+14    | 0.000255  | 0.136240     | 0.171555     | 0.860469        | 0.730178     | 0.052670          | 0.336534     0.050399     0.095199     0.005599     0.425194     0.378489     0.339348    | 0.429990     0.060798     0.098528     0.023067     0.423105     0.374656     0.322066    | 0.750500  0.650275  0.790896  | 0.061314  0.056828  0.039868 
+15    | 0.000250  | 0.135379     | 0.168149     | 0.867126        | 0.736672     | 0.045904          | 0.336013     0.049393     0.093249     0.005536     0.423653     0.374884     0.338068    | 0.421937     0.059383     0.096959     0.021807     0.421270     0.379529     0.321932    | 0.756945  0.657131  0.808418  | 0.054746  0.053010  0.029956</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2500  1953  1473
+FP   204   233    70
+FN    77   116    53
+TN  4515  4994  5700
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.343  0.268  0.202
+FP  0.028  0.032  0.010
+FN  0.011  0.016  0.007
+TN  0.619  0.684  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B        VLo-PmC1     VLo-PmC2     VLo-PmC3    | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+-------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.168149     | 0.867126        | 0.736672     | 0.045904          | 0.421937     0.059383     0.096959     0.021807     0.421270     0.379529     0.321932    | 0.756945  0.657131  0.808418  | 0.054746  0.053010  0.029956 
+266     | 266     | 0.168180     | 0.866758        | 0.736857     | 0.046642          | 0.419323     0.060547     0.098368     0.022726     0.414327     0.377964     0.313563    | 0.753041  0.659441  0.813166  | 0.056415  0.053351  0.030159 
+360     | 310     | 0.157052     | 0.864571        | 0.721934     | 0.040338          | 0.424164     0.042575     0.075501     0.009648     0.403709     0.342189     0.371426    | 0.756953  0.609752  0.810448  | 0.045999  0.050234  0.024781 
+276     | 276     | 0.193960     | 0.876534        | 0.754724     | 0.042259          | 0.487169     0.068299     0.110411     0.026188     0.650879     0.511389     0.429102    | 0.818711  0.679914  0.727073  | 0.041376  0.051593  0.033807 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_l
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(8h 56m 56s)
+(Max GPU mem usage : 15382.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.562597     | 0.260720     | 0.768484        | 0.578422     | 0.104808          | 0.463419     0.605101     0.944487     0.265716    | 0.447180     0.180808     0.296779     0.064837    | 0.649285  0.502510  0.545084  | 0.096109  0.092496  0.125819 
+2     | 0.000250  | 0.267913     | 0.175484     | 0.846090        | 0.693242     | 0.052011          | 0.407976     0.207886     0.398835     0.016937    | 0.430531     0.066178     0.119800     0.012556    | 0.725254  0.609169  0.739112  | 0.062183  0.052522  0.041329 
+3     | 0.000375  | 0.183795     | 0.169993     | 0.848045        | 0.698409     | 0.052197          | 0.396940     0.092448     0.175743     0.009152    | 0.420669     0.062560     0.109267     0.015853    | 0.726563  0.623757  0.757640  | 0.052739  0.071266  0.032587 
+4     | 0.000500  | 0.173596     | 0.176338     | 0.841821        | 0.685858     | 0.054205          | 0.389864     0.080910     0.153011     0.008810    | 0.441005     0.062910     0.110358     0.015461    | 0.731544  0.615019  0.725255  | 0.067383  0.045896  0.049335 
+5     | 0.000495  | 0.164751     | 0.175524     | 0.854558        | 0.721820     | 0.056949          | 0.380792     0.072161     0.136298     0.008025    | 0.447017     0.059170     0.102922     0.015419    | 0.746174  0.650797  0.756056  | 0.065022  0.066711  0.039114 
+6     | 0.000480  | 0.161817     | 0.169600     | 0.849480        | 0.709138     | 0.056959          | 0.377515     0.069375     0.130975     0.007775    | 0.429517     0.058208     0.101109     0.015307    | 0.735730  0.645331  0.751837  | 0.061212  0.058733  0.050931 
+7     | 0.000457  | 0.154643     | 0.173761     | 0.853098        | 0.723567     | 0.060547          | 0.369973     0.062358     0.117711     0.007006    | 0.444111     0.057897     0.098972     0.016821    | 0.745449  0.649064  0.782245  | 0.064551  0.065928  0.051163 
+8     | 0.000427  | 0.153018     | 0.165217     | 0.858287        | 0.721490     | 0.050515          | 0.367572     0.061066     0.115288     0.006844    | 0.418754     0.056559     0.097150     0.015968    | 0.745078  0.653898  0.782020  | 0.063848  0.055836  0.031862 
+9     | 0.000393  | 0.148479     | 0.172075     | 0.858085        | 0.717400     | 0.048125          | 0.361208     0.057309     0.108296     0.006323    | 0.438992     0.057682     0.099598     0.015765    | 0.732689  0.651764  0.770968  | 0.061456  0.054914  0.028006 
+10    | 0.000357  | 0.147845     | 0.174091     | 0.853554        | 0.716129     | 0.054829          | 0.362259     0.055954     0.105578     0.006330    | 0.443345     0.058696     0.100741     0.016651    | 0.733788  0.634889  0.784524  | 0.069080  0.067120  0.028287 
+11    | 0.000323  | 0.143212     | 0.166719     | 0.859010        | 0.729556     | 0.054687          | 0.356397     0.051847     0.097922     0.005772    | 0.423674     0.056596     0.097415     0.015777    | 0.746219  0.658345  0.791035  | 0.062201  0.064731  0.037127 
+12    | 0.000293  | 0.143502     | 0.177809     | 0.856312        | 0.716519     | 0.050492          | 0.356976     0.052013     0.098264     0.005761    | 0.443818     0.063804     0.110282     0.017327    | 0.733938  0.642913  0.772413  | 0.059017  0.062542  0.029919 
+13    | 0.000270  | 0.142452     | 0.165772     | 0.862042        | 0.729971     | 0.049911          | 0.355830     0.051005     0.096422     0.005588    | 0.422133     0.055902     0.095697     0.016108    | 0.744979  0.661542  0.791394  | 0.061584  0.058370  0.029779 
+14    | 0.000255  | 0.139007     | 0.174716     | 0.857588        | 0.727865     | 0.055929          | 0.351676     0.047863     0.090526     0.005199    | 0.442154     0.060100     0.102436     0.017764    | 0.742085  0.651986  0.786880  | 0.061205  0.059147  0.047436 
+15    | 0.000250  | 0.139156     | 0.163728     | 0.860813        | 0.734429     | 0.054930          | 0.351552     0.048130     0.091010     0.005250    | 0.416685     0.055318     0.094469     0.016168    | 0.747000  0.662020  0.795732  | 0.076334  0.053568  0.034889</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2490  1965  1452
+FP   217   214    79
+FN    87   104    74
+TN  4502  5013  5691
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.341  0.269  0.199
+FP  0.030  0.029  0.011
+FN  0.012  0.014  0.010
+TN  0.617  0.687  0.780
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.163728     | 0.860813        | 0.734429     | 0.054930          | 0.416685     0.055318     0.094469     0.016168    | 0.747000  0.662020  0.795732  | 0.076334  0.053568  0.034889 
+266     | 266     | 0.163578     | 0.862019        | 0.737233     | 0.054790          | 0.413782     0.056348     0.095856     0.016840    | 0.750018  0.664001  0.799914  | 0.075699  0.054102  0.034568 
+360     | 310     | 0.151705     | 0.847863        | 0.702742     | 0.055389          | 0.412719     0.039841     0.072040     0.007643    | 0.679824  0.626080  0.818529  | 0.072101  0.054521  0.039546 
+276     | 276     | 0.196641     | 0.859185        | 0.732601     | 0.056425          | 0.504592     0.064662     0.110836     0.018489    | 0.790273  0.675794  0.684990  | 0.091498  0.044284  0.033493 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/8   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 10m 40s)
+(Max GPU mem usage : 6604.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.570434     | 0.274484     | 0.704457        | 0.465712     | 0.136380          | 0.520952     0.591641     0.940303     0.242977    | 0.479029     0.186822     0.308374     0.065271    | 0.526809  0.391173  0.473456  | 0.103548  0.110103  0.195489 
+2     | 0.000250  | 0.280812     | 0.181832     | 0.836107        | 0.668533     | 0.052176          | 0.433086     0.215552     0.413607     0.017497    | 0.446968     0.068203     0.123553     0.012853    | 0.698878  0.605446  0.710426  | 0.054207  0.061215  0.041107 
+3     | 0.000375  | 0.193721     | 0.178653     | 0.829532        | 0.687050     | 0.075480          | 0.414735     0.099001     0.188465     0.009537    | 0.445840     0.064144     0.112817     0.015471    | 0.717009  0.616452  0.728974  | 0.087248  0.098481  0.040712 
+4     | 0.000500  | 0.179904     | 0.178269     | 0.844111        | 0.691199     | 0.053948          | 0.402103     0.084676     0.160356     0.008997    | 0.451766     0.061056     0.106624     0.015487    | 0.714360  0.615638  0.758426  | 0.066645  0.064973  0.030227 
+5     | 0.000495  | 0.172267     | 0.171672     | 0.829807        | 0.685429     | 0.073941          | 0.394446     0.077048     0.145665     0.008431    | 0.428868     0.061445     0.105709     0.017181    | 0.725465  0.640442  0.711232  | 0.079741  0.067213  0.074868 
+6     | 0.000480  | 0.167043     | 0.171010     | 0.855551        | 0.714054     | 0.050117          | 0.386530     0.072977     0.137872     0.008082    | 0.428554     0.060635     0.105369     0.015901    | 0.738386  0.640482  0.783715  | 0.056902  0.052991  0.040459 
+7     | 0.000457  | 0.160487     | 0.173814     | 0.850498        | 0.709288     | 0.055362          | 0.379704     0.066537     0.125753     0.007321    | 0.442932     0.058478     0.100968     0.015988    | 0.727955  0.631574  0.783288  | 0.062328  0.073374  0.030383 
+8     | 0.000427  | 0.156623     | 0.174083     | 0.850811        | 0.710176     | 0.055433          | 0.374598     0.063205     0.119372     0.007039    | 0.441811     0.059342     0.101567     0.017116    | 0.733663  0.634061  0.774940  | 0.066965  0.061616  0.037717 
+9     | 0.000393  | 0.152889     | 0.168545     | 0.850032        | 0.714476     | 0.059597          | 0.369353     0.060119     0.113575     0.006662    | 0.428084     0.057314     0.098392     0.016236    | 0.740435  0.653853  0.761613  | 0.060540  0.064718  0.053534 
+10    | 0.000357  | 0.149960     | 0.165594     | 0.860978        | 0.730084     | 0.051758          | 0.366632     0.057100     0.107911     0.006290    | 0.417628     0.057580     0.099757     0.015402    | 0.740505  0.661623  0.797774  | 0.059298  0.061615  0.034362 
+11    | 0.000323  | 0.146055     | 0.168303     | 0.859227        | 0.724074     | 0.050671          | 0.361604     0.053677     0.101452     0.005902    | 0.428564     0.056762     0.097687     0.015836    | 0.739533  0.656945  0.787156  | 0.058347  0.060624  0.033043 
+12    | 0.000293  | 0.144455     | 0.169174     | 0.856629        | 0.721267     | 0.053130          | 0.359415     0.052330     0.098940     0.005720    | 0.431783     0.056627     0.096689     0.016566    | 0.737346  0.649121  0.784600  | 0.063427  0.062076  0.033888 
+13    | 0.000270  | 0.144324     | 0.171515     | 0.857705        | 0.719550     | 0.050191          | 0.359011     0.052315     0.098899     0.005731    | 0.435508     0.058375     0.100738     0.016012    | 0.744136  0.647970  0.770250  | 0.063254  0.061304  0.026016 
+14    | 0.000255  | 0.142099     | 0.167784     | 0.861872        | 0.725085     | 0.046937          | 0.355877     0.050479     0.095508     0.005450    | 0.421931     0.058863     0.101168     0.016560    | 0.743507  0.657594  0.772212  | 0.059773  0.052453  0.028585 
+15    | 0.000250  | 0.140155     | 0.170233     | 0.853589        | 0.717944     | 0.055981          | 0.354154     0.048441     0.091639     0.005244    | 0.435263     0.056648     0.096108     0.017188    | 0.738391  0.644320  0.787271  | 0.071172  0.064415  0.032356 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2524  1983  1446
+FP   296   301    78
+FN    53    86    80
+TN  4423  4926  5692
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.346  0.272  0.198
+FP  0.041  0.041  0.011
+FN  0.007  0.012  0.011
+TN  0.606  0.675  0.780
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.170233     | 0.853589        | 0.717944     | 0.055981          | 0.435263     0.056648     0.096108     0.017188    | 0.738391  0.644320  0.787271  | 0.071172  0.064415  0.032356 
+266     | 266     | 0.170003     | 0.853482        | 0.719811     | 0.057403          | 0.433669     0.057003     0.096207     0.017799    | 0.737436  0.648820  0.791767  | 0.073963  0.064285  0.033961 
+360     | 310     | 0.170695     | 0.840169        | 0.679265     | 0.052562          | 0.458284     0.047442     0.086035     0.008850    | 0.699411  0.582052  0.777153  | 0.053382  0.081943  0.022360 
+276     | 276     | 0.175346     | 0.873659        | 0.742960     | 0.039209          | 0.423081     0.069174     0.117631     0.020716    | 0.808485  0.648970  0.730836  | 0.053029  0.042982  0.021616 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 11m 51s)
+(Max GPU mem usage : 6604.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.482535     | 0.202516     | 0.700524        | 0.468938     | 0.145085          | 0.228790     0.591283     0.939790     0.242776    | 0.238373     0.187149     0.309298     0.065000    | 0.521750  0.386761  0.480492  | 0.103929  0.112512  0.218812 
+2     | 0.000250  | 0.188549     | 0.111764     | 0.825031        | 0.659122     | 0.064364          | 0.112438     0.221168     0.424720     0.017617    | 0.208663     0.070237     0.126312     0.014161    | 0.706522  0.582311  0.685950  | 0.072438  0.087361  0.033293 
+3     | 0.000375  | 0.096869     | 0.101206     | 0.835064        | 0.697035     | 0.072917          | 0.090058     0.099788     0.190109     0.009467    | 0.194663     0.061153     0.108086     0.014220    | 0.728013  0.628660  0.744590  | 0.083791  0.072288  0.062672 
+4     | 0.000500  | 0.083974     | 0.102410     | 0.847597        | 0.703663     | 0.056448          | 0.077900     0.086577     0.163985     0.009169    | 0.197822     0.061519     0.107589     0.015449    | 0.733711  0.624664  0.753217  | 0.070973  0.062362  0.036007 
+5     | 0.000495  | 0.073131     | 0.104744     | 0.839751        | 0.691397     | 0.061345          | 0.059459     0.078991     0.149452     0.008529    | 0.199153     0.064283     0.111522     0.017045    | 0.730713  0.595114  0.751312  | 0.065660  0.067659  0.050717 
+6     | 0.000480  | 0.063816     | 0.107248     | 0.847349        | 0.704919     | 0.057698          | 0.045407     0.071706     0.135529     0.007883    | 0.219124     0.059302     0.102873     0.015731    | 0.735732  0.630639  0.764037  | 0.073231  0.064130  0.035732 
+7     | 0.000457  | 0.058753     | 0.103841     | 0.854190        | 0.713090     | 0.051743          | 0.036921     0.068109     0.128770     0.007448    | 0.209715     0.058466     0.100786     0.016145    | 0.725500  0.648060  0.774539  | 0.050199  0.068707  0.036323 
+8     | 0.000427  | 0.052950     | 0.094352     | 0.858939        | 0.722112     | 0.049842          | 0.030544     0.062553     0.118233     0.006873    | 0.179209     0.057985     0.100762     0.015208    | 0.731903  0.661415  0.786300  | 0.052520  0.066209  0.030798 
+9     | 0.000393  | 0.050719     | 0.104325     | 0.851184        | 0.713342     | 0.056921          | 0.026956     0.060903     0.115102     0.006703    | 0.207115     0.060272     0.104220     0.016324    | 0.735475  0.645022  0.754317  | 0.070205  0.057587  0.042971 
+10    | 0.000357  | 0.047066     | 0.111284     | 0.858855        | 0.721772     | 0.049756          | 0.022896     0.057425     0.108609     0.006241    | 0.238362     0.056821     0.097693     0.015950    | 0.742587  0.654620  0.769622  | 0.055238  0.060276  0.033754 
+11    | 0.000323  | 0.043209     | 0.103231     | 0.857718        | 0.723126     | 0.052554          | 0.017137     0.054383     0.102854     0.005912    | 0.204485     0.059836     0.103320     0.016352    | 0.741372  0.656884  0.780264  | 0.052854  0.062488  0.042321 
+12    | 0.000293  | 0.039944     | 0.117523     | 0.855034        | 0.716270     | 0.052457          | 0.011464     0.052149     0.098658     0.005640    | 0.251099     0.060275     0.103952     0.016599    | 0.735256  0.650449  0.770176  | 0.054609  0.060731  0.042030 
+13    | 0.000270  | 0.039672     | 0.110174     | 0.855211        | 0.714911     | 0.051256          | 0.012260     0.051420     0.097292     0.005548    | 0.228649     0.059398     0.102071     0.016725    | 0.739706  0.639383  0.764150  | 0.058425  0.056221  0.039122 
+14    | 0.000255  | 0.039299     | 0.113193     | 0.857584        | 0.713781     | 0.046546          | 0.011750     0.051106     0.096727     0.005484    | 0.235166     0.060918     0.104715     0.017122    | 0.729034  0.640555  0.769637  | 0.057662  0.060292  0.021686 
+15    | 0.000250  | 0.037236     | 0.125735     | 0.858586        | 0.716891     | 0.046951          | 0.009151     0.049272     0.093266     0.005278    | 0.275051     0.061743     0.106019     0.017467    | 0.743785  0.642571  0.757181  | 0.056997  0.054419  0.029436</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2431  1900  1375
+FP   146   155    69
+FN   146   169   151
+TN  4573  5072  5701
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.333  0.260  0.188
+FP  0.020  0.021  0.009
+FN  0.020  0.023  0.021
+TN  0.627  0.695  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.125735     | 0.858586        | 0.716891     | 0.046951          | 0.275051     0.061743     0.106019     0.017467    | 0.743785  0.642571  0.757181  | 0.056997  0.054419  0.029436 
+266     | 266     | 0.123610     | 0.858376        | 0.718776     | 0.048558          | 0.265944     0.062609     0.106989     0.018229    | 0.742169  0.642171  0.767403  | 0.059977  0.055669  0.030027 
+360     | 310     | 0.138378     | 0.847255        | 0.674152     | 0.037342          | 0.345311     0.049693     0.090909     0.008477    | 0.725209  0.614649  0.686805  | 0.039063  0.049685  0.023278 
+276     | 276     | 0.152793     | 0.877379        | 0.746931     | 0.035656          | 0.352322     0.067280     0.116105     0.018456    | 0.795522  0.688382  0.724864  | 0.036201  0.041977  0.028789 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0 
+pres_loss_wt = 0.4, seg_loss_wt = 0.6
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 8m 56s)
+(Max GPU mem usage : 6604.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.447722     | 0.214550     | 0.699366        | 0.468486     | 0.146714          | 0.232459     0.591231     0.939506     0.242957    | 0.257076     0.186200     0.308114     0.064287    | 0.519830  0.384921  0.491091  | 0.108167  0.119055  0.212918 
+2     | 0.000250  | 0.177930     | 0.122720     | 0.828187        | 0.660649     | 0.060120          | 0.112234     0.221727     0.425796     0.017659    | 0.200688     0.070742     0.127753     0.013730    | 0.690778  0.593190  0.695526  | 0.066828  0.072427  0.041106 
+3     | 0.000375  | 0.099553     | 0.128402     | 0.833831        | 0.681181     | 0.064403          | 0.093775     0.103405     0.196912     0.009897    | 0.225842     0.063442     0.112335     0.014550    | 0.709386  0.617999  0.727509  | 0.064942  0.063805  0.064463 
+4     | 0.000500  | 0.085242     | 0.140120     | 0.838332        | 0.687680     | 0.061234          | 0.077225     0.090587     0.171550     0.009624    | 0.257391     0.061939     0.107617     0.016262    | 0.714791  0.608745  0.753852  | 0.080481  0.064438  0.038782 
+5     | 0.000495  | 0.070090     | 0.120166     | 0.845577        | 0.699806     | 0.057242          | 0.058625     0.077734     0.147064     0.008404    | 0.208535     0.061253     0.104734     0.017772    | 0.721888  0.624422  0.766575  | 0.069027  0.070025  0.032674 
+6     | 0.000480  | 0.061828     | 0.116597     | 0.843805        | 0.694809     | 0.056864          | 0.044724     0.073231     0.138387     0.008074    | 0.193154     0.065558     0.113864     0.017252    | 0.724004  0.617162  0.733911  | 0.069626  0.064527  0.036438 
+7     | 0.000457  | 0.055799     | 0.109506     | 0.853646        | 0.713760     | 0.053097          | 0.037550     0.067966     0.128503     0.007428    | 0.183571     0.060129     0.104766     0.015492    | 0.734197  0.642911  0.766873  | 0.065525  0.057082  0.036685 
+8     | 0.000427  | 0.050929     | 0.125044     | 0.854285        | 0.717440     | 0.054485          | 0.029496     0.065218     0.123279     0.007157    | 0.224628     0.058654     0.100853     0.016455    | 0.740016  0.641481  0.781891  | 0.063297  0.061996  0.038161 
+9     | 0.000393  | 0.048286     | 0.120625     | 0.849556        | 0.712751     | 0.059241          | 0.027795     0.061946     0.117110     0.006783    | 0.209371     0.061461     0.106990     0.015931    | 0.732550  0.644216  0.759335  | 0.067791  0.061001  0.048932 
+10    | 0.000357  | 0.043930     | 0.122610     | 0.848115        | 0.702132     | 0.054562          | 0.021229     0.059064     0.111660     0.006468    | 0.210306     0.064146     0.111434     0.016857    | 0.719690  0.635436  0.762760  | 0.056033  0.076153  0.031501 
+11    | 0.000323  | 0.041255     | 0.127741     | 0.852637        | 0.718018     | 0.057616          | 0.017606     0.057022     0.107828     0.006215    | 0.229152     0.060133     0.103996     0.016270    | 0.739204  0.640978  0.775563  | 0.067822  0.065304  0.039723 
+12    | 0.000293  | 0.037206     | 0.141405     | 0.853226        | 0.713674     | 0.053739          | 0.010754     0.054841     0.103800     0.005882    | 0.265212     0.058868     0.101658     0.016077    | 0.743147  0.647089  0.748107  | 0.068314  0.068314  0.024591 
+13    | 0.000270  | 0.035721     | 0.138356     | 0.848195        | 0.709237     | 0.059167          | 0.009968     0.052889     0.100089     0.005690    | 0.256355     0.059690     0.102809     0.016570    | 0.732796  0.634693  0.757038  | 0.063579  0.066631  0.047291 
+14    | 0.000255  | 0.035241     | 0.141119     | 0.856319        | 0.714060     | 0.048841          | 0.009957     0.052096     0.098637     0.005555    | 0.261336     0.060974     0.105043     0.016905    | 0.746328  0.643649  0.754308  | 0.054780  0.055932  0.035813 
+15    | 0.000250  | 0.034770     | 0.129011     | 0.858617        | 0.725055     | 0.052341          | 0.009065     0.051907     0.098216     0.005597    | 0.232643     0.059923     0.102862     0.016985    | 0.752724  0.646659  0.771948  | 0.060172  0.060656  0.036196 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2457  1906  1455
+FP   137   163   106
+FN   120   163    71
+TN  4582  5064  5664
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.337  0.261  0.199
+FP  0.019  0.022  0.015
+FN  0.016  0.022  0.010
+TN  0.628  0.694  0.776
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.129011     | 0.858617        | 0.725055     | 0.052341          | 0.232643     0.059923     0.102862     0.016985    | 0.752724  0.646659  0.771948  | 0.060172  0.060656  0.036196 
+266     | 266     | 0.125747     | 0.859383        | 0.729788     | 0.054220          | 0.224457     0.059940     0.102349     0.017531    | 0.751508  0.648798  0.787928  | 0.062704  0.063221  0.036734 
+360     | 310     | 0.116440     | 0.842524        | 0.669401     | 0.042060          | 0.210123     0.053985     0.099042     0.008929    | 0.746375  0.607811  0.686447  | 0.047699  0.043782  0.034700 
+276     | 276     | 0.247317     | 0.867106        | 0.724579     | 0.037875          | 0.507708     0.073723     0.125884     0.021563    | 0.780906  0.662160  0.674797  | 0.038828  0.044681  0.030117 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0 
+pres_loss_wt = 0.4, seg_loss_wt = 0.6
+Aux head LR : 1/8   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(4h 9m 16s)
+(Max GPU mem usage : 6604.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.446516     | 0.202630     | 0.702808        | 0.473116     | 0.144064          | 0.229406     0.591256     0.939564     0.242948    | 0.226380     0.186797     0.307908     0.065687    | 0.520987  0.388668  0.497435  | 0.102716  0.112627  0.216848 
+2     | 0.000250  | 0.177870     | 0.122429     | 0.824516        | 0.659650     | 0.065574          | 0.112133     0.221695     0.425821     0.017568    | 0.201118     0.069971     0.126079     0.013862    | 0.690969  0.587946  0.708456  | 0.072375  0.075081  0.049265 
+3     | 0.000375  | 0.097972     | 0.131992     | 0.829154        | 0.672791     | 0.066604          | 0.090304     0.103084     0.196453     0.009714    | 0.234698     0.063522     0.112379     0.014664    | 0.710639  0.605240  0.711772  | 0.079369  0.058945  0.061496 
+4     | 0.000500  | 0.083343     | 0.116442     | 0.838680        | 0.695265     | 0.065711          | 0.076170     0.088125     0.166894     0.009357    | 0.197252     0.062568     0.108828     0.016309    | 0.715461  0.618010  0.761884  | 0.073547  0.080381  0.043205 
+5     | 0.000495  | 0.072717     | 0.122424     | 0.818658        | 0.679914     | 0.088846          | 0.059844     0.081299     0.153793     0.008805    | 0.206753     0.066204     0.113002     0.019407    | 0.705017  0.597477  0.748656  | 0.131960  0.075838  0.058742 
+6     | 0.000480  | 0.062728     | 0.121463     | 0.839458        | 0.691633     | 0.061992          | 0.045169     0.074434     0.140739     0.008129    | 0.210960     0.061798     0.106803     0.016792    | 0.708964  0.631407  0.746525  | 0.074840  0.063609  0.047527 
+7     | 0.000457  | 0.055895     | 0.125200     | 0.849693        | 0.704101     | 0.053247          | 0.037303     0.068289     0.129112     0.007466    | 0.223090     0.059940     0.103899     0.015980    | 0.734342  0.637844  0.741483  | 0.068089  0.055927  0.035724 
+8     | 0.000427  | 0.048643     | 0.106803     | 0.854254        | 0.711133     | 0.050332          | 0.027246     0.062907     0.118927     0.006888    | 0.171521     0.063657     0.110546     0.016768    | 0.732955  0.632691  0.778576  | 0.059500  0.055164  0.036331 
+9     | 0.000393  | 0.045710     | 0.139910     | 0.845996        | 0.712014     | 0.064683          | 0.022523     0.061168     0.115651     0.006684    | 0.261209     0.059045     0.101217     0.016872    | 0.735960  0.644334  0.758338  | 0.077339  0.068557  0.048152 
+10    | 0.000357  | 0.045234     | 0.133651     | 0.852710        | 0.713273     | 0.054333          | 0.023563     0.059681     0.112856     0.006506    | 0.242722     0.060937     0.105012     0.016862    | 0.731354  0.647576  0.760436  | 0.057401  0.063137  0.042461 
+11    | 0.000323  | 0.041115     | 0.123533     | 0.856640        | 0.721842     | 0.053494          | 0.017222     0.057043     0.107889     0.006198    | 0.221453     0.058253     0.100512     0.015995    | 0.742153  0.658580  0.769227  | 0.062096  0.063216  0.035170 
+12    | 0.000293  | 0.038515     | 0.131325     | 0.858711        | 0.721792     | 0.050010          | 0.014659     0.054419     0.102959     0.005878    | 0.241338     0.057982     0.099692     0.016273    | 0.750483  0.657772  0.756825  | 0.063292  0.059441  0.027297 
+13    | 0.000270  | 0.034775     | 0.149084     | 0.854176        | 0.713881     | 0.052294          | 0.008705     0.052154     0.098695     0.005614    | 0.285995     0.057809     0.099502     0.016116    | 0.736649  0.642267  0.757401  | 0.061521  0.064031  0.031331 
+14    | 0.000255  | 0.035900     | 0.133066     | 0.854136        | 0.715781     | 0.053627          | 0.012151     0.051732     0.097960     0.005504    | 0.245744     0.057948     0.098763     0.017133    | 0.746578  0.646520  0.752650  | 0.071266  0.060855  0.028760 
+15    | 0.000250  | 0.035275     | 0.138936     | 0.857442        | 0.723266     | 0.053107          | 0.011325     0.051241     0.097003     0.005480    | 0.261370     0.057313     0.097842     0.016785    | 0.744779  0.653927  0.776775  | 0.060819  0.061328  0.037174 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2496  1971  1444
+FP   214   221    88
+FN    81    98    82
+TN  4505  5006  5682
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.342  0.270  0.198
+FP  0.029  0.030  0.012
+FN  0.011  0.013  0.011
+TN  0.617  0.686  0.779
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.138936     | 0.857442        | 0.723266     | 0.053107          | 0.261370     0.057313     0.097842     0.016785    | 0.744779  0.653927  0.776775  | 0.060819  0.061328  0.037174 
+266     | 266     | 0.134504     | 0.858154        | 0.727737     | 0.054902          | 0.249571     0.057793     0.098261     0.017325    | 0.746123  0.657912  0.786768  | 0.063925  0.062092  0.038689 
+360     | 310     | 0.144333     | 0.839260        | 0.661572     | 0.042282          | 0.289716     0.047411     0.085403     0.009420    | 0.699465  0.591528  0.723195  | 0.045997  0.055778  0.025072 
+276     | 276     | 0.245634     | 0.871425        | 0.739477     | 0.040610          | 0.511898     0.068125     0.116366     0.019884    | 0.787980  0.671978  0.715750  | 0.033984  0.057266  0.030579 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet++ tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(5h 10m 32s)
+(Max GPU mem usage : 7948.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.583428     | 0.272951     | 0.705917        | 0.409361     | 0.096379          | 0.518120     0.611418     0.948927     0.273908    | 0.466073     0.190184     0.315574     0.064794    | 0.633633  0.484597  0.000198  | 0.107964  0.078887  0.102287 
+2     | 0.000250  | 0.290512     | 0.184932     | 0.830594        | 0.660329     | 0.055896          | 0.434064     0.228990     0.439831     0.018149    | 0.449319     0.071623     0.128728     0.014518    | 0.696835  0.594803  0.679038  | 0.068391  0.061033  0.038264 
+3     | 0.000375  | 0.191295     | 0.174428     | 0.841552        | 0.696326     | 0.061631          | 0.413575     0.096032     0.182676     0.009388    | 0.429056     0.065302     0.115755     0.014849    | 0.731627  0.605479  0.757153  | 0.073052  0.068767  0.043073 
+4     | 0.000500  | 0.181397     | 0.179479     | 0.841765        | 0.686559     | 0.054764          | 0.405073     0.085536     0.161703     0.009370    | 0.444171     0.066040     0.115339     0.016740    | 0.704904  0.623811  0.731735  | 0.057016  0.062796  0.044481 
+5     | 0.000495  | 0.172398     | 0.171032     | 0.849734        | 0.699129     | 0.049862          | 0.393580     0.077605     0.146567     0.008644    | 0.424523     0.062393     0.109218     0.015568    | 0.708523  0.631619  0.773159  | 0.055812  0.053293  0.040479 
+6     | 0.000480  | 0.163744     | 0.179001     | 0.846403        | 0.686771     | 0.047175          | 0.384526     0.069123     0.130491     0.007755    | 0.436340     0.068712     0.119563     0.017862    | 0.703914  0.619294  0.744150  | 0.053237  0.058292  0.029998 
+7     | 0.000457  | 0.159701     | 0.175190     | 0.836269        | 0.678869     | 0.058799          | 0.377818     0.066222     0.125128     0.007315    | 0.436647     0.063137     0.108924     0.017349    | 0.710774  0.590527  0.764742  | 0.080622  0.054439  0.041335 
+8     | 0.000427  | 0.155711     | 0.169387     | 0.861725        | 0.724454     | 0.046762          | 0.373651     0.062308     0.117599     0.007016    | 0.425204     0.059751     0.103687     0.015814    | 0.744036  0.645059  0.787821  | 0.057576  0.054238  0.028471 
+9     | 0.000393  | 0.154001     | 0.171526     | 0.855514        | 0.711623     | 0.048559          | 0.371545     0.060768     0.114748     0.006787    | 0.430219     0.060657     0.104488     0.016826    | 0.728904  0.641473  0.776168  | 0.059984  0.058446  0.027248 
+10    | 0.000357  | 0.150332     | 0.171066     | 0.856689        | 0.712629     | 0.047271          | 0.366096     0.057861     0.109429     0.006293    | 0.426188     0.061728     0.106580     0.016876    | 0.732190  0.636877  0.779454  | 0.058555  0.053128  0.030131 
+11    | 0.000323  | 0.147271     | 0.173700     | 0.849343        | 0.710284     | 0.057951          | 0.362789     0.054906     0.103773     0.006039    | 0.438063     0.060401     0.103556     0.017247    | 0.731183  0.632899  0.776515  | 0.086253  0.061398  0.026202 
+12    | 0.000293  | 0.144237     | 0.169329     | 0.851249        | 0.715229     | 0.058071          | 0.358545     0.052391     0.099059     0.005723    | 0.427990     0.058475     0.098792     0.018158    | 0.738357  0.634855  0.773541  | 0.064257  0.056998  0.052958 
+13    | 0.000270  | 0.142220     | 0.169556     | 0.859165        | 0.719458     | 0.047696          | 0.355845     0.050667     0.095848     0.005486    | 0.425029     0.060067     0.103327     0.016807    | 0.743546  0.641152  0.781116  | 0.061457  0.057332  0.024301 
+14    | 0.000255  | 0.141539     | 0.166870     | 0.863802        | 0.730215     | 0.047140          | 0.355924     0.049659     0.093937     0.005381    | 0.422807     0.057183     0.097761     0.016606    | 0.744957  0.656793  0.796681  | 0.055974  0.058459  0.026988 
+15    | 0.000250  | 0.139725     | 0.169591     | 0.860324        | 0.726162     | 0.050235          | 0.354152     0.047828     0.090464     0.005192    | 0.431238     0.057456     0.098574     0.016338    | 0.748709  0.645269  0.794012  | 0.061081  0.059490  0.030135</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2523  1975  1466
+FP   241   249    80
+FN    54    94    60
+TN  4478  4978  5690
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.346  0.271  0.201
+FP  0.033  0.034  0.011
+FN  0.007  0.013  0.008
+TN  0.614  0.682  0.780
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.169591     | 0.860324        | 0.726162     | 0.050235          | 0.431238     0.057456     0.098574     0.016338    | 0.748709  0.645269  0.794012  | 0.061081  0.059490  0.030135 
+266     | 266     | 0.169421     | 0.859485        | 0.726812     | 0.052067          | 0.429236     0.058071     0.099208     0.016935    | 0.745438  0.646789  0.799692  | 0.064639  0.061375  0.030188 
+360     | 310     | 0.161836     | 0.861428        | 0.713691     | 0.040081          | 0.434383     0.045030     0.082243     0.007817    | 0.751151  0.618302  0.793972  | 0.043118  0.049525  0.027600 
+276     | 276     | 0.192792     | 0.871398        | 0.732946     | 0.036300          | 0.477746     0.070669     0.120653     0.020686    | 0.798735  0.653980  0.700754  | 0.031677  0.044498  0.032725 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet++ tu-tf_efficientnetv2_s 
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,…,1.25e-4
+with LLRD (4 stages) and decoder/seghead and aux 
+weight decay 1e-5
+pres_smooth_eps = 0.05
+Aux head LR : 1/16   dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(5h 21m 10s)
+(Max GPU mem usage : 7948.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.583799     | 0.273255     | 0.699598        | 0.403551     | 0.103037          | 0.518397     0.611829     0.949428     0.274229    | 0.465329     0.190938     0.314988     0.066888    | 0.617319  0.476680  0.000301  | 0.125283  0.083258  0.100569 
+2     | 0.000250  | 0.291849     | 0.184665     | 0.830920        | 0.660716     | 0.055611          | 0.432842     0.231424     0.444418     0.018430    | 0.446060     0.072638     0.131164     0.014112    | 0.705036  0.582648  0.684115  | 0.072191  0.060023  0.034620 
+3     | 0.000375  | 0.192123     | 0.173799     | 0.846990        | 0.695280     | 0.051869          | 0.414243     0.096928     0.184299     0.009557    | 0.429997     0.064000     0.112757     0.015242    | 0.728616  0.614413  0.755535  | 0.069236  0.049892  0.036479 
+4     | 0.000371  | 0.175515     | 0.178568     | 0.845436        | 0.692088     | 0.052331          | 0.397567     0.080349     0.152072     0.008627    | 0.454519     0.060304     0.104329     0.016278    | 0.710752  0.617410  0.761735  | 0.062795  0.063394  0.030805 
+5     | 0.000358  | 0.167806     | 0.176411     | 0.848029        | 0.690151     | 0.046719          | 0.386865     0.073923     0.139698     0.008149    | 0.431323     0.067164     0.117021     0.017307    | 0.705104  0.607518  0.767944  | 0.047839  0.052132  0.040185 
+6     | 0.000338  | 0.159920     | 0.173209     | 0.851348        | 0.707080     | 0.052474          | 0.378577     0.066210     0.125143     0.007276    | 0.434657     0.061160     0.106582     0.015738    | 0.734929  0.621948  0.770214  | 0.065191  0.064414  0.027817 
+7     | 0.000313  | 0.154755     | 0.177862     | 0.839920        | 0.674815     | 0.050010          | 0.372128     0.061595     0.116426     0.006764    | 0.434167     0.068017     0.117475     0.018559    | 0.723325  0.558729  0.750257  | 0.069782  0.043819  0.036429 
+8     | 0.000282  | 0.153004     | 0.169919     | 0.855035        | 0.715388     | 0.051866          | 0.369823     0.060082     0.113442     0.006721    | 0.431064     0.058000     0.099837     0.016163    | 0.737013  0.638241  0.783732  | 0.061681  0.063870  0.030048 
+9     | 0.000250  | 0.149787     | 0.167914     | 0.855731        | 0.717310     | 0.051988          | 0.365799     0.057210     0.108116     0.006303    | 0.426574     0.057060     0.098119     0.016000    | 0.742213  0.649964  0.780784  | 0.061577  0.065646  0.028742 
+10    | 0.000218  | 0.146112     | 0.172590     | 0.853908        | 0.715825     | 0.054037          | 0.360748     0.054125     0.102378     0.005873    | 0.435320     0.059991     0.102727     0.017255    | 0.738206  0.633677  0.785794  | 0.075901  0.056534  0.029675 
+11    | 0.000188  | 0.143527     | 0.170805     | 0.858910        | 0.721691     | 0.049610          | 0.357406     0.051865     0.098098     0.005632    | 0.428706     0.060276     0.104423     0.016131    | 0.741824  0.647339  0.779077  | 0.061667  0.063524  0.023640 
+12    | 0.000162  | 0.141393     | 0.170188     | 0.858062        | 0.722647     | 0.051662          | 0.354499     0.050061     0.094725     0.005398    | 0.430506     0.058623     0.100382     0.016863    | 0.740102  0.648183  0.792477  | 0.064258  0.057923  0.032803 
+13    | 0.000142  | 0.139830     | 0.180341     | 0.851926        | 0.699836     | 0.046681          | 0.353221     0.048377     0.091539     0.005214    | 0.443291     0.067648     0.116908     0.018389    | 0.693347  0.634616  0.787229  | 0.053120  0.058763  0.028159 
+14    | 0.000129  | 0.139366     | 0.170745     | 0.855682        | 0.716604     | 0.051599          | 0.352896     0.047853     0.090536     0.005170    | 0.434605     0.057662     0.098256     0.017067    | 0.740256  0.635338  0.786188  | 0.065664  0.056039  0.033096 
+15    | 0.000125  | 0.137940     | 0.169308     | 0.853996        | 0.717404     | 0.054943          | 0.351214     0.046536     0.088072     0.005000    | 0.427408     0.058694     0.100322     0.017066    | 0.740261  0.638037  0.789135  | 0.066826  0.071131  0.026872</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2487  1961  1477
+FP   242   243   104
+FN    90   108    49
+TN  4477  4984  5666
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.341  0.269  0.202
+FP  0.033  0.033  0.014
+FN  0.012  0.015  0.007
+TN  0.614  0.683  0.777
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.169308     | 0.853996        | 0.717404     | 0.054943          | 0.427408     0.058694     0.100322     0.017066    | 0.740261  0.638037  0.789135  | 0.066826  0.071131  0.026872 
+266     | 266     | 0.169281     | 0.855132        | 0.718986     | 0.054103          | 0.424451     0.059922     0.102080     0.017765    | 0.739083  0.639481  0.794155  | 0.069426  0.067646  0.025237 
+360     | 310     | 0.162770     | 0.838805        | 0.682247     | 0.056823          | 0.442161     0.043031     0.077791     0.008272    | 0.702310  0.605043  0.785882  | 0.056231  0.071023  0.043215 
+276     | 276     | 0.185738     | 0.858105        | 0.742811     | 0.065033          | 0.471851     0.063118     0.106933     0.019303    | 0.812462  0.657922  0.710932  | 0.041960  0.123534  0.029604 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+All layer LR same
+weight decay 1e-5
+pres_smooth_eps = 0.05
+dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 15m 27s)
+(Max GPU mem usage : 10270.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.534374     | 0.246020     | 0.754506        | 0.524822     | 0.092372          | 0.478102     0.558491     0.913489     0.203491    | 0.458983     0.154750     0.270265     0.039235    | 0.510665  0.425673  0.663709  | 0.111716  0.113040  0.052360 
+2     | 0.000250  | 0.279913     | 0.185369     | 0.819857        | 0.650401     | 0.067172          | 0.411347     0.223584     0.427178     0.019990    | 0.439893     0.076286     0.139130     0.013442    | 0.684460  0.524999  0.739984  | 0.096381  0.061142  0.043992 
+3     | 0.000375  | 0.192150     | 0.170967     | 0.834043        | 0.698622     | 0.075676          | 0.401491     0.102433     0.195272     0.009594    | 0.425650     0.061817     0.108221     0.015412    | 0.732443  0.609853  0.769821  | 0.125743  0.072653  0.028631 
+4     | 0.000500  | 0.179825     | 0.169899     | 0.855776        | 0.712161     | 0.048480          | 0.395776     0.087274     0.165011     0.009538    | 0.425022     0.060560     0.105095     0.016026    | 0.747911  0.635967  0.756263  | 0.061712  0.064508  0.019221 
+5     | 0.000495  | 0.173578     | 0.177486     | 0.849804        | 0.705368     | 0.053905          | 0.387203     0.082024     0.154937     0.009112    | 0.450919     0.060300     0.104266     0.016334    | 0.737008  0.616593  0.774585  | 0.064400  0.071827  0.025489 
+6     | 0.000480  | 0.167595     | 0.173585     | 0.855904        | 0.712249     | 0.048327          | 0.382389     0.075541     0.142589     0.008494    | 0.438770     0.059934     0.103858     0.016010    | 0.737641  0.634184  0.755611  | 0.061090  0.060682  0.023208 
+7     | 0.000457  | 0.160464     | 0.172813     | 0.851665        | 0.716903     | 0.058493          | 0.374946     0.068543     0.129398     0.007687    | 0.439278     0.058614     0.101347     0.015881    | 0.737641  0.628545  0.781929  | 0.069642  0.065249  0.040587 
+8     | 0.000427  | 0.158949     | 0.166117     | 0.855562        | 0.722857     | 0.055968          | 0.374783     0.066449     0.125309     0.007588    | 0.423028     0.056012     0.096491     0.015533    | 0.749141  0.651629  0.778915  | 0.067952  0.071266  0.028686 
+9     | 0.000393  | 0.156019     | 0.169269     | 0.855373        | 0.715726     | 0.051528          | 0.369446     0.064550     0.121816     0.007284    | 0.432744     0.056352     0.096799     0.015904    | 0.732030  0.635546  0.805292  | 0.066791  0.057187  0.030607 
+10    | 0.000357  | 0.152776     | 0.166492     | 0.862435        | 0.730191     | 0.049403          | 0.366909     0.061004     0.115095     0.006913    | 0.425744     0.055384     0.095703     0.015064    | 0.748778  0.660141  0.794903  | 0.057637  0.062212  0.028359 
+11    | 0.000323  | 0.149116     | 0.169515     | 0.861247        | 0.729717     | 0.051067          | 0.362643     0.057604     0.108796     0.006412    | 0.430151     0.057814     0.100356     0.015272    | 0.748843  0.659614  0.787141  | 0.052757  0.068562  0.031882 
+12    | 0.000293  | 0.144988     | 0.167425     | 0.861901        | 0.728886     | 0.049422          | 0.357623     0.053858     0.101656     0.006061    | 0.428334     0.055607     0.095646     0.015568    | 0.749494  0.657478  0.791044  | 0.054962  0.065350  0.027953 
+13    | 0.000270  | 0.144091     | 0.165199     | 0.860871        | 0.731485     | 0.052871          | 0.357675     0.052556     0.099265     0.005846    | 0.417878     0.056908     0.097731     0.016086    | 0.750169  0.656573  0.800612  | 0.073327  0.060100  0.025188 
+14    | 0.000255  | 0.143194     | 0.164543     | 0.859715        | 0.727828     | 0.052361          | 0.356189     0.051910     0.098014     0.005807    | 0.420209     0.054972     0.093503     0.016440    | 0.741858  0.652031  0.810087  | 0.062371  0.065021  0.029691 
+15    | 0.000250  | 0.142869     | 0.173665     | 0.860457        | 0.728599     | 0.051637          | 0.356289     0.051404     0.097049     0.005759    | 0.438802     0.060034     0.102794     0.017275    | 0.742760  0.657149  0.791959  | 0.050539  0.076029  0.028345 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2443  1895  1426
+FP   145   162    58
+FN   134   174   100
+TN  4574  5065  5712
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.335  0.260  0.195
+FP  0.020  0.022  0.008
+FN  0.018  0.024  0.014
+TN  0.627  0.694  0.783
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.173665     | 0.860457        | 0.728599     | 0.051637          | 0.438802     0.060034     0.102794     0.017275    | 0.742760  0.657149  0.791959  | 0.050539  0.076029  0.028345 
+266     | 266     | 0.173289     | 0.861235        | 0.731355     | 0.052178          | 0.436610     0.060437     0.102863     0.018012    | 0.738245  0.659716  0.805712  | 0.050886  0.077759  0.027890 
+360     | 310     | 0.167091     | 0.848190        | 0.690016     | 0.046360          | 0.436380     0.051682     0.094717     0.008647    | 0.762568  0.608663  0.707965  | 0.053998  0.064625  0.020458 
+276     | 276     | 0.199578     | 0.864314        | 0.736623     | 0.050559          | 0.503800     0.069197     0.120324     0.018070    | 0.787752  0.675912  0.728392  | 0.040707  0.065279  0.045690 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+All layer LR same
+weight decay 1e-2
+pres_smooth_eps = 0.05
+dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 14m 28s)
+(Max GPU mem usage : 10270.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.535536     | 0.246134     | 0.742552        | 0.515390     | 0.106006          | 0.478440     0.560005     0.915571     0.204440    | 0.454736     0.156732     0.271601     0.041864    | 0.495558  0.418965  0.654173  | 0.122701  0.125319  0.069998 
+2     | 0.000250  | 0.284759     | 0.199428     | 0.779590        | 0.573414     | 0.082960          | 0.410284     0.230962     0.439789     0.022136    | 0.437597     0.097355     0.172004     0.022706    | 0.572496  0.419265  0.737126  | 0.098386  0.104627  0.045865 
+3     | 0.000375  | 0.210316     | 0.174817     | 0.832089        | 0.672627     | 0.061602          | 0.402426     0.127983     0.243043     0.012925    | 0.424651     0.067745     0.119069     0.016422    | 0.698312  0.572665  0.749305  | 0.074832  0.064765  0.045210 
+4     | 0.000500  | 0.183325     | 0.170486     | 0.850540        | 0.703926     | 0.051718          | 0.398436     0.091135     0.172165     0.010105    | 0.426304     0.060850     0.105657     0.016042    | 0.729773  0.630713  0.758367  | 0.058619  0.070320  0.026216 
+5     | 0.000495  | 0.174406     | 0.175138     | 0.843113        | 0.694811     | 0.058020          | 0.388911     0.082475     0.155662     0.009288    | 0.437485     0.062704     0.107504     0.017905    | 0.720283  0.610539  0.765774  | 0.070003  0.072351  0.031705 
+6     | 0.000480  | 0.167279     | 0.165606     | 0.857724        | 0.726779     | 0.054979          | 0.383209     0.074737     0.140941     0.008533    | 0.419477     0.056805     0.098775     0.014834    | 0.749618  0.648252  0.788613  | 0.060548  0.072975  0.031413 
+7     | 0.000457  | 0.166493     | 0.173400     | 0.852683        | 0.709342     | 0.051756          | 0.381812     0.074213     0.139915     0.008511    | 0.439996     0.059145     0.102819     0.015471    | 0.735254  0.631477  0.764816  | 0.067306  0.053282  0.034681 
+8     | 0.000427  | 0.158841     | 0.166715     | 0.856538        | 0.725253     | 0.055939          | 0.373487     0.066850     0.126043     0.007657    | 0.419988     0.058169     0.100772     0.015567    | 0.745897  0.646076  0.792379  | 0.055469  0.068694  0.043655 
+9     | 0.000393  | 0.155941     | 0.172719     | 0.859462        | 0.718961     | 0.046871          | 0.369274     0.064513     0.121673     0.007353    | 0.425608     0.064338     0.111203     0.017472    | 0.739373  0.642308  0.771736  | 0.051409  0.064980  0.024225 
+10    | 0.000357  | 0.153668     | 0.170438     | 0.854285        | 0.714226     | 0.052343          | 0.367904     0.061852     0.116635     0.007069    | 0.431239     0.058666     0.102029     0.015304    | 0.738141  0.644154  0.773004  | 0.066163  0.059610  0.031256 
+11    | 0.000323  | 0.152689     | 0.164656     | 0.863003        | 0.735275     | 0.051846          | 0.366888     0.060889     0.114834     0.006944    | 0.420673     0.054934     0.095333     0.014535    | 0.756401  0.662792  0.794389  | 0.064214  0.058396  0.032928 
+12    | 0.000293  | 0.150234     | 0.168939     | 0.859122        | 0.723833     | 0.050685          | 0.363422     0.058868     0.111097     0.006638    | 0.430484     0.056848     0.098044     0.015652    | 0.742004  0.650215  0.795066  | 0.059364  0.056968  0.035724 
+13    | 0.000270  | 0.144309     | 0.168490     | 0.863014        | 0.729712     | 0.048118          | 0.356962     0.053172     0.100376     0.005969    | 0.428034     0.057257     0.098696     0.015819    | 0.748637  0.649471  0.798795  | 0.054661  0.059485  0.030207 
+14    | 0.000255  | 0.142398     | 0.167921     | 0.859087        | 0.721970     | 0.049502          | 0.353925     0.051743     0.097761     0.005726    | 0.427633     0.056616     0.096505     0.016727    | 0.735439  0.654186  0.790887  | 0.052874  0.062174  0.033458 
+15    | 0.000250  | 0.143769     | 0.170349     | 0.860371        | 0.726045     | 0.050078          | 0.356816     0.052463     0.099074     0.005852    | 0.435301     0.056798     0.097339     0.016257    | 0.743307  0.657604  0.792967  | 0.061193  0.067604  0.021438</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2458  1941  1425
+FP   212   226    55
+FN   119   128   101
+TN  4507  5001  5715
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.337  0.266  0.195
+FP  0.029  0.031  0.008
+FN  0.016  0.018  0.014
+TN  0.618  0.685  0.783
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.170349     | 0.860371        | 0.726045     | 0.050078          | 0.435301     0.056798     0.097339     0.016257    | 0.743307  0.657604  0.792967  | 0.061193  0.067604  0.021438 
+266     | 266     | 0.169420     | 0.862064        | 0.729879     | 0.049813          | 0.430690     0.057447     0.098028     0.016865    | 0.742963  0.660224  0.805730  | 0.063066  0.066789  0.019586 
+360     | 310     | 0.173585     | 0.834668        | 0.665687     | 0.052678          | 0.470922     0.046154     0.083791     0.008517    | 0.700960  0.603273  0.725142  | 0.051242  0.071742  0.035048 
+276     | 276     | 0.187670     | 0.869875        | 0.750567     | 0.050586          | 0.474326     0.064817     0.111236     0.018398    | 0.809623  0.689188  0.714936  | 0.046367  0.074320  0.031071 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+All layer LR same and aux_head LR = 1/16 LR
+weight decay 1e-2
+pres_smooth_eps = 0.05
+dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 21m 28s)
+(Max GPU mem usage : 10270.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.533918     | 0.246185     | 0.750306        | 0.519520     | 0.095836          | 0.477727     0.558000     0.912509     0.203491    | 0.459338     0.154834     0.269856     0.039811    | 0.504378  0.425524  0.633990  | 0.114454  0.113088  0.059967 
+2     | 0.000250  | 0.277913     | 0.177152     | 0.829370        | 0.685387     | 0.074642          | 0.411399     0.220704     0.421761     0.019649    | 0.429341     0.069071     0.126189     0.011953    | 0.715692  0.592219  0.764241  | 0.109534  0.075938  0.038455 
+3     | 0.000375  | 0.191433     | 0.167156     | 0.853080        | 0.711888     | 0.052792          | 0.402542     0.100957     0.192300     0.009615    | 0.419174     0.059148     0.104008     0.014287    | 0.742754  0.642422  0.760998  | 0.058475  0.066852  0.033051 
+4     | 0.000500  | 0.181396     | 0.173020     | 0.851899        | 0.707075     | 0.051552          | 0.398648     0.088288     0.166982     0.009594    | 0.434022     0.061161     0.106463     0.015860    | 0.733745  0.623049  0.780851  | 0.057696  0.071622  0.025338 
+5     | 0.000495  | 0.173710     | 0.176276     | 0.848137        | 0.702099     | 0.054503          | 0.390792     0.080674     0.152330     0.009019    | 0.443569     0.061722     0.107306     0.016137    | 0.731145  0.629541  0.747695  | 0.058960  0.082287  0.022263 
+6     | 0.000480  | 0.167961     | 0.167519     | 0.855661        | 0.722796     | 0.055763          | 0.383262     0.075689     0.142805     0.008572    | 0.417756     0.060274     0.104612     0.015936    | 0.751871  0.653306  0.760873  | 0.066763  0.072054  0.028471 
+7     | 0.000457  | 0.164476     | 0.172536     | 0.841996        | 0.701089     | 0.064066          | 0.380367     0.071950     0.135704     0.008197    | 0.436837     0.059265     0.102282     0.016247    | 0.720399  0.611810  0.787238  | 0.082847  0.076426  0.032926 
+8     | 0.000427  | 0.157508     | 0.169713     | 0.857341        | 0.722858     | 0.053004          | 0.372703     0.065282     0.123135     0.007429    | 0.422542     0.061358     0.106310     0.016406    | 0.743970  0.646564  0.785645  | 0.067857  0.062078  0.029078 
+9     | 0.000393  | 0.153645     | 0.169172     | 0.855349        | 0.716346     | 0.051982          | 0.367746     0.061887     0.116844     0.006931    | 0.428377     0.058084     0.099876     0.016293    | 0.738290  0.643541  0.780892  | 0.062952  0.063794  0.029202 
+10    | 0.000357  | 0.150917     | 0.170736     | 0.862318        | 0.725326     | 0.046355          | 0.364125     0.059542     0.112353     0.006730    | 0.429633     0.059780     0.104212     0.015348    | 0.745865  0.653371  0.780470  | 0.054890  0.060134  0.024041 
+11    | 0.000323  | 0.151494     | 0.167330     | 0.858902        | 0.728452     | 0.054132          | 0.365768     0.059662     0.112597     0.006727    | 0.422824     0.057832     0.099704     0.015960    | 0.749969  0.653480  0.784618  | 0.067041  0.061990  0.033365 
+12    | 0.000293  | 0.147624     | 0.170583     | 0.847256        | 0.712138     | 0.062666          | 0.361291     0.056052     0.105738     0.006367    | 0.430904     0.059017     0.101305     0.016729    | 0.731105  0.647268  0.773773  | 0.072969  0.081884  0.033144 
+13    | 0.000270  | 0.146768     | 0.165486     | 0.860644        | 0.728543     | 0.051288          | 0.360454     0.055189     0.104131     0.006247    | 0.420458     0.056212     0.097066     0.015358    | 0.751045  0.663819  0.772699  | 0.065612  0.059777  0.028475 
+14    | 0.000255  | 0.144065     | 0.164317     | 0.861221        | 0.734831     | 0.054518          | 0.357111     0.052760     0.099578     0.005943    | 0.421021     0.054302     0.092445     0.016158    | 0.748232  0.673347  0.800815  | 0.068446  0.062195  0.032914 
+15    | 0.000250  | 0.143531     | 0.172345     | 0.854633        | 0.717657     | 0.054051          | 0.356558     0.052234     0.098593     0.005874    | 0.439429     0.057881     0.099018     0.016744    | 0.735335  0.645440  0.791263  | 0.069831  0.065330  0.026991</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2504  1993  1427
+FP   264   271    61
+FN    73    76    99
+TN  4455  4956  5709
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.343  0.273  0.196
+FP  0.036  0.037  0.008
+FN  0.010  0.010  0.014
+TN  0.611  0.679  0.782
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.172345     | 0.854633        | 0.717657     | 0.054051          | 0.439429     0.057881     0.099018     0.016744    | 0.735335  0.645440  0.791263  | 0.069831  0.065330  0.026991 
+266     | 266     | 0.171702     | 0.855917        | 0.720451     | 0.053772          | 0.434663     0.059004     0.100548     0.017460    | 0.736965  0.644330  0.800367  | 0.069355  0.064552  0.027409 
+360     | 310     | 0.168001     | 0.837562        | 0.678820     | 0.056611          | 0.461658     0.042148     0.076571     0.007725    | 0.679721  0.648284  0.753855  | 0.093272  0.055415  0.021145 
+276     | 276     | 0.200155     | 0.857726        | 0.726546     | 0.054821          | 0.514767     0.065321     0.111587     0.019055    | 0.785758  0.661025  0.712731  | 0.045716  0.090216  0.028531 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+LLRD : 0.25, 0.5, 0.75, 1 and aux_head LR = 1/16 LR
+weight decay 1e-2
+pres_smooth_eps = 0.05
+dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 14m 35s)
+(Max GPU mem usage : 10270.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.535656     | 0.248499     | 0.733084        | 0.491627     | 0.105944          | 0.480099     0.559467     0.914670     0.204264    | 0.455994     0.159573     0.274303     0.044842    | 0.477578  0.399548  0.606541  | 0.126705  0.127886  0.063241 
+2     | 0.000250  | 0.286433     | 0.198683     | 0.772211        | 0.569152     | 0.092416          | 0.411649     0.232770     0.443314     0.022223    | 0.439469     0.095489     0.166835     0.024143    | 0.573426  0.435054  0.715981  | 0.104244  0.118303  0.054700 
+3     | 0.000375  | 0.206886     | 0.177027     | 0.832846        | 0.667560     | 0.056964          | 0.398224     0.124884     0.237429     0.012339    | 0.435138     0.066409     0.117134     0.015683    | 0.703246  0.567415  0.757745  | 0.074052  0.060700  0.036139 
+4     | 0.000500  | 0.181526     | 0.173442     | 0.853313        | 0.710091     | 0.051206          | 0.396414     0.089431     0.169114     0.009747    | 0.430805     0.063143     0.110133     0.016153    | 0.729438  0.634687  0.772159  | 0.066161  0.062692  0.024764 
+5     | 0.000495  | 0.170958     | 0.181258     | 0.823173        | 0.676800     | 0.079246          | 0.386340     0.078652     0.148564     0.008740    | 0.454003     0.064367     0.109185     0.019548    | 0.705875  0.588609  0.766324  | 0.107176  0.113817  0.016744 
+6     | 0.000480  | 0.167703     | 0.168347     | 0.851817        | 0.709712     | 0.053447          | 0.383746     0.075112     0.141722     0.008503    | 0.419798     0.060582     0.104577     0.016587    | 0.736868  0.638951  0.764446  | 0.058636  0.063234  0.038473 
+7     | 0.000457  | 0.160580     | 0.172001     | 0.854353        | 0.712144     | 0.050841          | 0.374633     0.068843     0.129881     0.007804    | 0.434466     0.059516     0.102834     0.016199    | 0.737103  0.639375  0.769024  | 0.061409  0.066279  0.024834 
+8     | 0.000427  | 0.155256     | 0.170241     | 0.856688        | 0.720056     | 0.052224          | 0.369764     0.063324     0.119485     0.007163    | 0.432562     0.057818     0.099218     0.016418    | 0.743467  0.646081  0.785071  | 0.059863  0.071177  0.025632 
+9     | 0.000393  | 0.152135     | 0.169370     | 0.853915        | 0.729396     | 0.063073          | 0.365210     0.060818     0.114794     0.006841    | 0.426317     0.059250     0.102818     0.015683    | 0.747692  0.650934  0.798515  | 0.096272  0.068403  0.024543 
+10    | 0.000357  | 0.150520     | 0.170425     | 0.862273        | 0.730098     | 0.049610          | 0.364607     0.058768     0.110847     0.006689    | 0.431008     0.058747     0.101985     0.015508    | 0.746805  0.650957  0.796676  | 0.057911  0.064039  0.026878 
+11    | 0.000323  | 0.147653     | 0.166449     | 0.865083        | 0.729953     | 0.044830          | 0.361105     0.056174     0.106047     0.006302    | 0.422066     0.056898     0.098468     0.015329    | 0.753257  0.655755  0.789876  | 0.053065  0.058260  0.023164 
+12    | 0.000293  | 0.144620     | 0.174250     | 0.859652        | 0.719603     | 0.046982          | 0.357686     0.053306     0.100655     0.005956    | 0.441471     0.059727     0.102766     0.016687    | 0.747096  0.650230  0.756063  | 0.060174  0.058138  0.022633 
+13    | 0.000270  | 0.142340     | 0.169741     | 0.862993        | 0.730650     | 0.048779          | 0.354679     0.051337     0.096925     0.005749    | 0.434300     0.056358     0.096798     0.015918    | 0.745213  0.649762  0.806874  | 0.065171  0.056893  0.024272 
+14    | 0.000255  | 0.141817     | 0.169128     | 0.860768        | 0.727395     | 0.050316          | 0.354801     0.050538     0.095476     0.005600    | 0.429687     0.057459     0.098181     0.016737    | 0.745103  0.650697  0.791315  | 0.063188  0.059403  0.028357 
+15    | 0.000250  | 0.141762     | 0.174775     | 0.850861        | 0.721540     | 0.062926          | 0.355500     0.050161     0.094754     0.005568    | 0.445711     0.058660     0.100538     0.016782    | 0.744068  0.653314  0.771949  | 0.076739  0.083759  0.028280 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2442  1940  1411
+FP   187   208    72
+FN   135   129   115
+TN  4532  5019  5698
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.335  0.266  0.193
+FP  0.026  0.029  0.010
+FN  0.019  0.018  0.016
+TN  0.621  0.688  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.174775     | 0.850861        | 0.721540     | 0.062926          | 0.445711     0.058660     0.100538     0.016782    | 0.744068  0.653314  0.771949  | 0.076739  0.083759  0.028280 
+266     | 266     | 0.171892     | 0.852554        | 0.729840     | 0.065637          | 0.436282     0.058582     0.099813     0.017351    | 0.748323  0.656776  0.793416  | 0.080612  0.088942  0.027356 
+360     | 310     | 0.196107     | 0.817591        | 0.617699     | 0.049148          | 0.523328     0.055870     0.102145     0.009596    | 0.665504  0.586843  0.650824  | 0.057746  0.053563  0.036136 
+276     | 276     | 0.201420     | 0.868857        | 0.733097     | 0.040636          | 0.514026     0.067446     0.116240     0.018651    | 0.785615  0.684663  0.658168  | 0.043974  0.046261  0.031672 </t>
   </si>
 </sst>
 </file>
@@ -7112,7 +8098,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K550"/>
+  <dimension ref="A1:K661"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50.36"/>
@@ -11893,6 +12879,12 @@
       <c r="B546" s="2" t="n">
         <v>0.854466</v>
       </c>
+      <c r="C546" s="2" t="n">
+        <v>0.85182</v>
+      </c>
+      <c r="D546" s="2" t="n">
+        <v>0.84598</v>
+      </c>
       <c r="E546" s="12" t="s">
         <v>432</v>
       </c>
@@ -11909,15 +12901,1123 @@
       <c r="B548" s="14" t="n">
         <v>0.859497</v>
       </c>
+      <c r="C548" s="2" t="n">
+        <v>0.85527</v>
+      </c>
+      <c r="D548" s="2" t="n">
+        <v>0.84407</v>
+      </c>
     </row>
     <row r="549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A549" s="28" t="s">
         <v>136</v>
       </c>
+      <c r="C549" s="2" t="n">
+        <v>0.86192</v>
+      </c>
+      <c r="D549" s="2" t="n">
+        <v>0.85166</v>
+      </c>
     </row>
     <row r="550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A550" s="28" t="s">
         <v>173</v>
+      </c>
+      <c r="C550" s="2" t="n">
+        <v>0.86062</v>
+      </c>
+      <c r="D550" s="2" t="n">
+        <v>0.85415</v>
+      </c>
+    </row>
+    <row r="552" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A552" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="B552" s="14" t="n">
+        <v>0.856101</v>
+      </c>
+      <c r="C552" s="2" t="n">
+        <v>0.84445</v>
+      </c>
+      <c r="D552" s="2" t="n">
+        <v>0.8299</v>
+      </c>
+      <c r="E552" s="12" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="553" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A553" s="3"/>
+      <c r="B553" s="3"/>
+      <c r="E553" s="12" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A554" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="B554" s="14" t="n">
+        <v>0.864299</v>
+      </c>
+      <c r="C554" s="2" t="n">
+        <v>0.85545</v>
+      </c>
+      <c r="D554" s="2" t="n">
+        <v>0.84376</v>
+      </c>
+    </row>
+    <row r="555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A555" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C555" s="2" t="n">
+        <v>0.86309</v>
+      </c>
+      <c r="D555" s="2" t="n">
+        <v>0.8526</v>
+      </c>
+    </row>
+    <row r="556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A556" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="C556" s="2" t="n">
+        <v>0.86175</v>
+      </c>
+      <c r="D556" s="2" t="n">
+        <v>0.85295</v>
+      </c>
+    </row>
+    <row r="558" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A558" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="B558" s="14" t="n">
+        <v>0.865391</v>
+      </c>
+      <c r="C558" s="2" t="n">
+        <v>0.85733</v>
+      </c>
+      <c r="D558" s="2" t="n">
+        <v>0.84428</v>
+      </c>
+      <c r="E558" s="12" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="559" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E559" s="12" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A560" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C560" s="2" t="n">
+        <v>0.86446</v>
+      </c>
+      <c r="D560" s="2" t="n">
+        <v>0.85037</v>
+      </c>
+    </row>
+    <row r="562" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A562" s="8" t="s">
+        <v>440</v>
+      </c>
+      <c r="B562" s="14" t="n">
+        <v>0.856258</v>
+      </c>
+      <c r="C562" s="2" t="n">
+        <v>0.86038</v>
+      </c>
+      <c r="D562" s="2" t="n">
+        <v>0.84394</v>
+      </c>
+      <c r="E562" s="12" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="563" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E563" s="12" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A564" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="B564" s="14" t="n">
+        <v>0.862588</v>
+      </c>
+      <c r="C564" s="2" t="n">
+        <v>0.85158</v>
+      </c>
+      <c r="D564" s="2" t="n">
+        <v>0.83718</v>
+      </c>
+    </row>
+    <row r="565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A565" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C565" s="2" t="n">
+        <v>0.86349</v>
+      </c>
+      <c r="D565" s="2" t="n">
+        <v>0.84932</v>
+      </c>
+    </row>
+    <row r="566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A566" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="C566" s="2" t="n">
+        <v>0.86258</v>
+      </c>
+      <c r="D566" s="2" t="n">
+        <v>0.85138</v>
+      </c>
+    </row>
+    <row r="568" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A568" s="8" t="s">
+        <v>443</v>
+      </c>
+      <c r="B568" s="14" t="n">
+        <v>0.866759</v>
+      </c>
+      <c r="C568" s="2" t="n">
+        <v>0.85099</v>
+      </c>
+      <c r="D568" s="2" t="n">
+        <v>0.8499</v>
+      </c>
+      <c r="E568" s="12" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="569" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E569" s="12" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="570" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A570" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B570" s="14" t="n">
+        <v>0.870001</v>
+      </c>
+      <c r="C570" s="2" t="n">
+        <v>0.86713</v>
+      </c>
+      <c r="D570" s="2" t="n">
+        <v>0.85743</v>
+      </c>
+      <c r="E570" s="12" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A571" s="28" t="s">
+        <v>447</v>
+      </c>
+      <c r="B571" s="14" t="n">
+        <v>0.871251</v>
+      </c>
+      <c r="C571" s="2" t="n">
+        <v>0.86706</v>
+      </c>
+      <c r="D571" s="2" t="n">
+        <v>0.85837</v>
+      </c>
+    </row>
+    <row r="572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A572" s="28" t="s">
+        <v>448</v>
+      </c>
+      <c r="B572" s="14" t="n">
+        <v>0.871494</v>
+      </c>
+      <c r="C572" s="2" t="n">
+        <v>0.86783</v>
+      </c>
+      <c r="D572" s="2" t="n">
+        <v>0.85838</v>
+      </c>
+    </row>
+    <row r="574" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A574" s="8" t="s">
+        <v>449</v>
+      </c>
+      <c r="C574" s="2" t="n">
+        <v>0.86276</v>
+      </c>
+      <c r="D574" s="2" t="n">
+        <v>0.85322</v>
+      </c>
+      <c r="E574" s="12" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A575" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C575" s="2" t="n">
+        <v>0.87006</v>
+      </c>
+      <c r="D575" s="2" t="n">
+        <v>0.8612</v>
+      </c>
+    </row>
+    <row r="576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A576" s="28" t="s">
+        <v>447</v>
+      </c>
+      <c r="C576" s="2" t="n">
+        <v>0.86985</v>
+      </c>
+      <c r="D576" s="2" t="n">
+        <v>0.86225</v>
+      </c>
+    </row>
+    <row r="577" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A577" s="28" t="s">
+        <v>448</v>
+      </c>
+      <c r="C577" s="2" t="n">
+        <v>0.87058</v>
+      </c>
+      <c r="D577" s="2" t="n">
+        <v>0.86199</v>
+      </c>
+    </row>
+    <row r="579" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A579" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="B579" s="2" t="n">
+        <v>0.867395</v>
+      </c>
+      <c r="C579" s="2" t="n">
+        <v>0.85389</v>
+      </c>
+      <c r="D579" s="2" t="n">
+        <v>0.85016</v>
+      </c>
+      <c r="E579" s="12" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="580" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A580" s="3"/>
+      <c r="B580" s="3"/>
+      <c r="E580" s="12" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="581" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A581" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B581" s="14" t="n">
+        <v>0.867682</v>
+      </c>
+      <c r="C581" s="2" t="n">
+        <v>0.85733</v>
+      </c>
+      <c r="D581" s="2" t="n">
+        <v>0.85199</v>
+      </c>
+    </row>
+    <row r="582" customFormat="false" ht="337.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A582" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B582" s="14" t="n">
+        <v>0.870245</v>
+      </c>
+      <c r="C582" s="2" t="n">
+        <v>0.86701</v>
+      </c>
+      <c r="D582" s="2" t="n">
+        <v>0.85993</v>
+      </c>
+      <c r="E582" s="12" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="583" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A583" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C583" s="2" t="n">
+        <v>0.86715</v>
+      </c>
+      <c r="D583" s="2" t="n">
+        <v>0.85768</v>
+      </c>
+    </row>
+    <row r="584" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A584" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="B584" s="14" t="n">
+        <v>0.872387</v>
+      </c>
+      <c r="C584" s="2" t="n">
+        <v>0.8672</v>
+      </c>
+      <c r="D584" s="2" t="n">
+        <v>0.86073</v>
+      </c>
+    </row>
+    <row r="585" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A585" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="B585" s="14" t="n">
+        <v>0.872088</v>
+      </c>
+      <c r="C585" s="2" t="n">
+        <v>0.86725</v>
+      </c>
+      <c r="D585" s="2" t="n">
+        <v>0.86098</v>
+      </c>
+    </row>
+    <row r="587" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A587" s="8" t="s">
+        <v>455</v>
+      </c>
+      <c r="C587" s="2" t="n">
+        <v>0.85939</v>
+      </c>
+      <c r="D587" s="2" t="n">
+        <v>0.84996</v>
+      </c>
+      <c r="E587" s="12" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="588" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A588" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C588" s="2" t="n">
+        <v>0.87009</v>
+      </c>
+      <c r="D588" s="2" t="n">
+        <v>0.85867</v>
+      </c>
+    </row>
+    <row r="589" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A589" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="C589" s="2" t="n">
+        <v>0.8698</v>
+      </c>
+      <c r="D589" s="2" t="n">
+        <v>0.85937</v>
+      </c>
+    </row>
+    <row r="590" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A590" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="C590" s="2" t="n">
+        <v>0.86999</v>
+      </c>
+      <c r="D590" s="2" t="n">
+        <v>0.8596</v>
+      </c>
+    </row>
+    <row r="591" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A591" s="28" t="s">
+        <v>457</v>
+      </c>
+      <c r="C591" s="2" t="n">
+        <v>0.86943</v>
+      </c>
+      <c r="D591" s="2" t="n">
+        <v>0.85874</v>
+      </c>
+    </row>
+    <row r="592" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A592" s="28" t="s">
+        <v>458</v>
+      </c>
+      <c r="C592" s="2" t="n">
+        <v>0.86989</v>
+      </c>
+      <c r="D592" s="2" t="n">
+        <v>0.85981</v>
+      </c>
+    </row>
+    <row r="593" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A593" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C593" s="2" t="n">
+        <v>0.87015</v>
+      </c>
+      <c r="D593" s="2" t="n">
+        <v>0.85991</v>
+      </c>
+    </row>
+    <row r="595" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A595" s="8" t="s">
+        <v>460</v>
+      </c>
+      <c r="B595" s="14" t="n">
+        <v>0.867126</v>
+      </c>
+      <c r="C595" s="2" t="n">
+        <v>0.85939</v>
+      </c>
+      <c r="D595" s="2" t="n">
+        <v>0.85607</v>
+      </c>
+      <c r="E595" s="12" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="596" customFormat="false" ht="281.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E596" s="12" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="597" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A597" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C597" s="2" t="n">
+        <v>0.86363</v>
+      </c>
+      <c r="D597" s="2" t="n">
+        <v>0.85773</v>
+      </c>
+    </row>
+    <row r="599" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A599" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="B599" s="14" t="n">
+        <v>0.860813</v>
+      </c>
+      <c r="C599" s="2" t="n">
+        <v>0.86276</v>
+      </c>
+      <c r="D599" s="2" t="n">
+        <v>0.84974</v>
+      </c>
+      <c r="E599" s="12" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="600" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E600" s="12" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="601" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A601" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B601" s="14" t="n">
+        <v>0.862042</v>
+      </c>
+      <c r="C601" s="2" t="n">
+        <v>0.86415</v>
+      </c>
+      <c r="D601" s="2" t="n">
+        <v>0.8486</v>
+      </c>
+    </row>
+    <row r="602" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A602" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C602" s="2" t="n">
+        <v>0.86624</v>
+      </c>
+      <c r="D602" s="2" t="n">
+        <v>0.85287</v>
+      </c>
+    </row>
+    <row r="603" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A603" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C603" s="2" t="n">
+        <v>0.86767</v>
+      </c>
+      <c r="D603" s="2" t="n">
+        <v>0.85375</v>
+      </c>
+    </row>
+    <row r="605" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A605" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="B605" s="14" t="n">
+        <v>0.853589</v>
+      </c>
+      <c r="C605" s="2" t="n">
+        <v>0.85888</v>
+      </c>
+      <c r="D605" s="2" t="n">
+        <v>0.84449</v>
+      </c>
+      <c r="E605" s="12" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="606" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E606" s="12" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="607" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A607" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B607" s="14" t="n">
+        <v>0.861872</v>
+      </c>
+      <c r="C607" s="2" t="n">
+        <v>0.85607</v>
+      </c>
+      <c r="D607" s="2" t="n">
+        <v>0.84633</v>
+      </c>
+    </row>
+    <row r="608" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A608" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C608" s="2" t="n">
+        <v>0.86151</v>
+      </c>
+      <c r="D608" s="2" t="n">
+        <v>0.8503</v>
+      </c>
+    </row>
+    <row r="609" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A609" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C609" s="2" t="n">
+        <v>0.86193</v>
+      </c>
+      <c r="D609" s="2" t="n">
+        <v>0.84971</v>
+      </c>
+    </row>
+    <row r="611" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A611" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="B611" s="14" t="n">
+        <v>0.858586</v>
+      </c>
+      <c r="C611" s="2" t="n">
+        <v>0.84384</v>
+      </c>
+      <c r="D611" s="2" t="n">
+        <v>0.83586</v>
+      </c>
+      <c r="E611" s="12" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="612" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E612" s="12" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="613" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A613" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="B613" s="14" t="n">
+        <v>0.858939</v>
+      </c>
+      <c r="C613" s="2" t="n">
+        <v>0.84882</v>
+      </c>
+      <c r="D613" s="2" t="n">
+        <v>0.84387</v>
+      </c>
+    </row>
+    <row r="614" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A614" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C614" s="2" t="n">
+        <v>0.8618</v>
+      </c>
+      <c r="D614" s="2" t="n">
+        <v>0.8556</v>
+      </c>
+    </row>
+    <row r="615" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A615" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="C615" s="2" t="n">
+        <v>0.85647</v>
+      </c>
+      <c r="D615" s="2" t="n">
+        <v>0.84867</v>
+      </c>
+    </row>
+    <row r="617" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A617" s="8" t="s">
+        <v>472</v>
+      </c>
+      <c r="B617" s="14" t="n">
+        <v>0.858617</v>
+      </c>
+      <c r="C617" s="2" t="n">
+        <v>0.85234</v>
+      </c>
+      <c r="D617" s="2" t="n">
+        <v>0.8419</v>
+      </c>
+      <c r="E617" s="12" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="618" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E618" s="12" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="619" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A619" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C619" s="2" t="n">
+        <v>0.85972</v>
+      </c>
+      <c r="D619" s="2" t="n">
+        <v>0.85352</v>
+      </c>
+    </row>
+    <row r="621" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A621" s="8" t="s">
+        <v>475</v>
+      </c>
+      <c r="B621" s="14" t="n">
+        <v>0.857442</v>
+      </c>
+      <c r="C621" s="2" t="n">
+        <v>0.85847</v>
+      </c>
+      <c r="D621" s="2" t="n">
+        <v>0.84508</v>
+      </c>
+      <c r="E621" s="12" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="622" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E622" s="12" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="623" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A623" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="B623" s="14" t="n">
+        <v>0.858711</v>
+      </c>
+      <c r="C623" s="2" t="n">
+        <v>0.85231</v>
+      </c>
+      <c r="D623" s="2" t="n">
+        <v>0.84504</v>
+      </c>
+    </row>
+    <row r="624" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A624" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C624" s="2" t="n">
+        <v>0.86027</v>
+      </c>
+      <c r="D624" s="2" t="n">
+        <v>0.8513</v>
+      </c>
+    </row>
+    <row r="625" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A625" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="C625" s="2" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="D625" s="2" t="n">
+        <v>0.84865</v>
+      </c>
+    </row>
+    <row r="627" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A627" s="8" t="s">
+        <v>478</v>
+      </c>
+      <c r="B627" s="14" t="n">
+        <v>0.860324</v>
+      </c>
+      <c r="C627" s="2" t="n">
+        <v>0.85904</v>
+      </c>
+      <c r="D627" s="2" t="n">
+        <v>0.84721</v>
+      </c>
+      <c r="E627" s="12" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="628" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E628" s="12" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="629" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A629" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B629" s="14" t="n">
+        <v>0.863802</v>
+      </c>
+      <c r="C629" s="2" t="n">
+        <v>0.85487</v>
+      </c>
+      <c r="D629" s="2" t="n">
+        <v>0.8478</v>
+      </c>
+    </row>
+    <row r="630" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A630" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C630" s="2" t="n">
+        <v>0.86115</v>
+      </c>
+      <c r="D630" s="2" t="n">
+        <v>0.85096</v>
+      </c>
+    </row>
+    <row r="631" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A631" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C631" s="2" t="n">
+        <v>0.86104</v>
+      </c>
+      <c r="D631" s="2" t="n">
+        <v>0.85109</v>
+      </c>
+    </row>
+    <row r="633" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A633" s="8" t="s">
+        <v>481</v>
+      </c>
+      <c r="B633" s="14" t="n">
+        <v>0.853996</v>
+      </c>
+      <c r="C633" s="2" t="n">
+        <v>0.85408</v>
+      </c>
+      <c r="D633" s="2" t="n">
+        <v>0.84637</v>
+      </c>
+      <c r="E633" s="12" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="634" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E634" s="12" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="635" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A635" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="B635" s="14" t="n">
+        <v>0.85891</v>
+      </c>
+      <c r="C635" s="2" t="n">
+        <v>0.84503</v>
+      </c>
+      <c r="D635" s="2" t="n">
+        <v>0.83816</v>
+      </c>
+    </row>
+    <row r="636" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A636" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C636" s="2" t="n">
+        <v>0.8581</v>
+      </c>
+      <c r="D636" s="2" t="n">
+        <v>0.84968</v>
+      </c>
+    </row>
+    <row r="637" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A637" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="C637" s="2" t="n">
+        <v>0.8591</v>
+      </c>
+      <c r="D637" s="2" t="n">
+        <v>0.84967</v>
+      </c>
+    </row>
+    <row r="639" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A639" s="8" t="s">
+        <v>484</v>
+      </c>
+      <c r="B639" s="14" t="n">
+        <v>0.860457</v>
+      </c>
+      <c r="C639" s="2" t="n">
+        <v>0.84816</v>
+      </c>
+      <c r="D639" s="2" t="n">
+        <v>0.84687</v>
+      </c>
+      <c r="E639" s="12" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="640" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E640" s="12" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="641" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A641" s="28" t="s">
+        <v>329</v>
+      </c>
+      <c r="B641" s="14" t="n">
+        <v>0.862435</v>
+      </c>
+      <c r="C641" s="2" t="n">
+        <v>0.85853</v>
+      </c>
+      <c r="D641" s="2" t="n">
+        <v>0.84765</v>
+      </c>
+    </row>
+    <row r="642" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A642" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B642" s="3"/>
+      <c r="C642" s="2" t="n">
+        <v>0.86713</v>
+      </c>
+      <c r="D642" s="2" t="n">
+        <v>0.85668</v>
+      </c>
+    </row>
+    <row r="643" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A643" s="28" t="s">
+        <v>330</v>
+      </c>
+      <c r="C643" s="2" t="n">
+        <v>0.86654</v>
+      </c>
+      <c r="D643" s="2" t="n">
+        <v>0.8581</v>
+      </c>
+    </row>
+    <row r="645" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A645" s="8" t="s">
+        <v>487</v>
+      </c>
+      <c r="B645" s="14" t="n">
+        <v>0.860371</v>
+      </c>
+      <c r="C645" s="2" t="n">
+        <v>0.85643</v>
+      </c>
+      <c r="D645" s="2" t="n">
+        <v>0.85161</v>
+      </c>
+      <c r="E645" s="12" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="646" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B646" s="3"/>
+      <c r="E646" s="12" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="647" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A647" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B647" s="14" t="n">
+        <v>0.863014</v>
+      </c>
+      <c r="C647" s="2" t="n">
+        <v>0.85733</v>
+      </c>
+      <c r="D647" s="2" t="n">
+        <v>0.84971</v>
+      </c>
+    </row>
+    <row r="648" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A648" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C648" s="2" t="n">
+        <v>0.86703</v>
+      </c>
+      <c r="D648" s="2" t="n">
+        <v>0.85855</v>
+      </c>
+    </row>
+    <row r="649" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A649" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C649" s="2" t="n">
+        <v>0.86775</v>
+      </c>
+      <c r="D649" s="2" t="n">
+        <v>0.85717</v>
+      </c>
+    </row>
+    <row r="651" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A651" s="8" t="s">
+        <v>490</v>
+      </c>
+      <c r="B651" s="14" t="n">
+        <v>0.854633</v>
+      </c>
+      <c r="C651" s="2" t="n">
+        <v>0.86175</v>
+      </c>
+      <c r="D651" s="2" t="n">
+        <v>0.84634</v>
+      </c>
+      <c r="E651" s="12" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="652" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E652" s="12" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="653" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A653" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="B653" s="14" t="n">
+        <v>0.862318</v>
+      </c>
+      <c r="C653" s="2" t="n">
+        <v>0.8493</v>
+      </c>
+      <c r="D653" s="2" t="n">
+        <v>0.84614</v>
+      </c>
+    </row>
+    <row r="654" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A654" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="B654" s="14"/>
+      <c r="C654" s="2" t="n">
+        <v>0.86523</v>
+      </c>
+      <c r="D654" s="2" t="n">
+        <v>0.85548</v>
+      </c>
+    </row>
+    <row r="655" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A655" s="21" t="s">
+        <v>330</v>
+      </c>
+      <c r="B655" s="14"/>
+      <c r="C655" s="2" t="n">
+        <v>0.86407</v>
+      </c>
+      <c r="D655" s="2" t="n">
+        <v>0.85461</v>
+      </c>
+    </row>
+    <row r="657" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A657" s="8" t="s">
+        <v>493</v>
+      </c>
+      <c r="B657" s="14" t="n">
+        <v>0.850861</v>
+      </c>
+      <c r="C657" s="2" t="n">
+        <v>0.85765</v>
+      </c>
+      <c r="D657" s="2" t="n">
+        <v>0.84015</v>
+      </c>
+      <c r="E657" s="12" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="658" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B658" s="3"/>
+      <c r="E658" s="12" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="659" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A659" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="B659" s="14" t="n">
+        <v>0.865083</v>
+      </c>
+      <c r="C659" s="2" t="n">
+        <v>0.8545</v>
+      </c>
+      <c r="D659" s="2" t="n">
+        <v>0.85111</v>
+      </c>
+    </row>
+    <row r="660" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A660" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C660" s="2" t="n">
+        <v>0.86371</v>
+      </c>
+      <c r="D660" s="2" t="n">
+        <v>0.85558</v>
+      </c>
+    </row>
+    <row r="661" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A661" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="C661" s="2" t="n">
+        <v>0.86298</v>
+      </c>
+      <c r="D661" s="2" t="n">
+        <v>0.85329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
all layer same LR, only auxhead diff LR, and others
</commit_message>
<xml_diff>
--- a/Scores.xlsx
+++ b/Scores.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="550">
   <si>
     <t xml:space="preserve">Description</t>
   </si>
@@ -7576,6 +7576,159 @@
 276     | 276     | 0.187670     | 0.869875        | 0.750567     | 0.050586          | 0.474326     0.064817     0.111236     0.018398    | 0.809623  0.689188  0.714936  | 0.046367  0.074320  0.031071 </t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">29m 43s
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Cutoffs(LB,SB,S) | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+---------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.163846     | 0.871089        | 0.746943     | 0.046147          | 0.423183     0.052702     0.090494     0.014910    | 0.763303  0.673647  0.816290  | 0.057414  0.053647  0.027380 
+(0.25,0.25,0.25) | 0.163846     | 0.871382        | 0.746921     | 0.045645          | 0.423183     0.052702     0.090494     0.014910    | 0.762571  0.674740  0.816290  | 0.056865  0.052690  0.027380 
+(0.50,0.50,0.50) | 0.163846     | 0.870889        | 0.745664     | 0.045628          | 0.423183     0.052702     0.090494     0.014910    | 0.759319  0.672277  0.817961  | 0.056814  0.052690  0.027380 
+(0.75,0.75,0.75) | 0.163846     | 0.871149        | 0.744880     | 0.044673          | 0.423183     0.052702     0.090494     0.014910    | 0.756954  0.672694  0.817514  | 0.055425  0.052462  0.026131 
+(0.60,0.70,0.70) | 0.163846     | 0.871201        | 0.745680     | 0.045118          | 0.423183     0.052702     0.090494     0.014910    | 0.757356  0.671876  0.818085  | 0.056760  0.052462  0.026131 
+(0.60,0.70,0.80) | 0.163846     | 0.871127        | 0.745494     | 0.045118          | 0.423183     0.052702     0.090494     0.014910    | 0.757356  0.671876  0.817407  | 0.056760  0.052462  0.026131 
+(0.50,0.75,0.75) | 0.163846     | 0.871362        | 0.746108     | 0.045136          | 0.423183     0.052702     0.090494     0.014910    | 0.759319  0.672694  0.817514  | 0.056814  0.052462  0.026131
+(0.25, 0.25, 0.25) tensor(0.8714)
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2516  1974  1486
+FP   234   233    84
+FN    61    95    40
+TN  4485  4994  5686
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.345  0.271  0.204
+FP  0.032  0.032  0.012
+FN  0.008  0.013  0.005
+TN  0.615  0.684  0.779
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.163846     | 0.871382        | 0.746921     | 0.045645          | 0.423183     0.052702     0.090494     0.014910    | 0.762571  0.674740  0.816290  | 0.056865  0.052690  0.027380 
+266     | 266     | 0.163544     | 0.871753        | 0.748744     | 0.046241          | 0.419642     0.053787     0.092097     0.015477    | 0.761696  0.677497  0.820229  | 0.058757  0.051972  0.027993 
+360     | 310     | 0.159083     | 0.859437        | 0.715066     | 0.044317          | 0.441606     0.038002     0.068219     0.007786    | 0.728536  0.621911  0.836394  | 0.051006  0.063559  0.018386 
+276     | 276     | 0.183451     | 0.882273        | 0.763398     | 0.038477          | 0.474577     0.058683     0.100664     0.016701    | 0.825205  0.700434  0.715203  | 0.036305  0.048961  0.030164 </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">29m 30s
+Cutoffs(LB,SB,S) | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+---------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.163149     | 0.868286        | 0.742074     | 0.047572          | 0.422088     0.052175     0.089980     0.014370    | 0.761886  0.666330  0.814600  | 0.056604  0.057852  0.028261 
+(0.25,0.25,0.25) | 0.163149     | 0.868517        | 0.742072     | 0.047187          | 0.422088     0.052175     0.089980     0.014370    | 0.760110  0.667929  0.815610  | 0.056604  0.056696  0.028261 
+(0.50,0.50,0.50) | 0.163149     | 0.868587        | 0.741791     | 0.046883          | 0.422088     0.052175     0.089980     0.014370    | 0.759784  0.666783  0.817267  | 0.056466  0.056696  0.027487 
+(0.75,0.75,0.75) | 0.163149     | 0.870620        | 0.745416     | 0.045911          | 0.422088     0.052175     0.089980     0.014370    | 0.759185  0.673771  0.818851  | 0.054839  0.056312  0.026580 
+(0.60,0.70,0.70) | 0.163149     | 0.870501        | 0.746400     | 0.046766          | 0.422088     0.052175     0.089980     0.014370    | 0.758471  0.672485  0.818575  | 0.056418  0.056616  0.027264 
+(0.60,0.70,0.80) | 0.163149     | 0.870644        | 0.746303     | 0.046463          | 0.422088     0.052175     0.089980     0.014370    | 0.758471  0.672485  0.817940  | 0.056418  0.056616  0.026355 
+(0.50,0.75,0.75) | 0.163149     | 0.870566        | 0.746094     | 0.046453          | 0.422088     0.052175     0.089980     0.014370    | 0.759784  0.673771  0.818851  | 0.056466  0.056312  0.026580 
+(0.6, 0.7, 0.8) tensor(0.8706)
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2499  1965  1475
+FP   233   238    74
+FN    78   104    51
+TN  4486  4989  5696
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.343  0.269  0.202
+FP  0.032  0.033  0.010
+FN  0.011  0.014  0.007
+TN  0.615  0.684  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.163149     | 0.870644        | 0.746303     | 0.046463          | 0.422088     0.052175     0.089980     0.014370    | 0.758471  0.672485  0.817940  | 0.056418  0.056616  0.026355 
+266     | 266     | 0.162712     | 0.871786        | 0.749390     | 0.046616          | 0.418415     0.053125     0.091344     0.014905    | 0.761063  0.675695  0.822271  | 0.058102  0.056523  0.025224 
+360     | 310     | 0.158686     | 0.853413        | 0.700410     | 0.044586          | 0.438635     0.038708     0.069758     0.007658    | 0.682367  0.617437  0.834606  | 0.052996  0.061915  0.018847 
+276     | 276     | 0.185665     | 0.876556        | 0.761386     | 0.046663          | 0.481524     0.058868     0.101687     0.016049    | 0.823417  0.692138  0.716292  | 0.035718  0.050935  0.053337 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA 0.25,0.25,0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA 0.50,0.75,0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 13 0.6,0.7,0.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 13 0.75,0.75,0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full Data
+6h 44m 40s
+Max GPU : 10270.875 MB </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | TLo-Pres     TLo-Seg      TLo-D        TLo-B       
+--------------------------------------------------------------------------------------
+1     | 0.000125  | 0.505230     | 0.471314     0.519765     0.868110     0.171421    
+2     | 0.000250  | 0.250353     | 0.411545     0.181270     0.346599     0.015942    
+3     | 0.000375  | 0.189191     | 0.402627     0.097718     0.185386     0.010050    
+4     | 0.000500  | 0.180763     | 0.397794     0.087750     0.165557     0.009942    
+5     | 0.000495  | 0.173840     | 0.390862     0.080830     0.152361     0.009300    
+6     | 0.000480  | 0.170126     | 0.386361     0.077453     0.146002     0.008904    
+7     | 0.000457  | 0.167310     | 0.382785     0.074963     0.141307     0.008620    
+8     | 0.000427  | 0.160540     | 0.374445     0.068867     0.129917     0.007817    
+9     | 0.000393  | 0.154322     | 0.368000     0.062745     0.118329     0.007162    
+10    | 0.000357  | 0.153085     | 0.366204     0.061748     0.116480     0.007015    
+11    | 0.000323  | 0.151269     | 0.364029     0.060086     0.113405     0.006766    
+12    | 0.000293  | 0.148096     | 0.360123     0.057227     0.108070     0.006385    
+13    | 0.000270  | 0.147135     | 0.359298     0.056208     0.106161     0.006255    
+14    | 0.000255  | 0.146645     | 0.359347     0.055487     0.104768     0.006207    
+15    | 0.000250  | 0.143946     | 0.355783     0.053158     0.100415     0.005902   </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">EMA Epoch 15 – cutoff </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0.25,0.25,0.25</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">EMA Epoch 13 – cutoff </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0.6,0.7,0.8</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
 No presence gate in loss
 LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
@@ -7677,6 +7830,690 @@
 360     | 310     | 0.196107     | 0.817591        | 0.617699     | 0.049148          | 0.523328     0.055870     0.102145     0.009596    | 0.665504  0.586843  0.650824  | 0.057746  0.053563  0.036136 
 276     | 276     | 0.201420     | 0.868857        | 0.733097     | 0.040636          | 0.514026     0.067446     0.116240     0.018651    | 0.785615  0.684663  0.658168  | 0.043974  0.046261  0.031672 </t>
   </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+All layer LR same and aux_head LR = 1/16 LR
+weight decay 1e-5
+pres_smooth_eps = 0.05
+dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 14m 33s)
+(Max GPU mem usage : 10270.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.536052     | 0.246243     | 0.748595        | 0.518119     | 0.097755          | 0.477391     0.561193     0.917613     0.204774    | 0.452927     0.157664     0.273123     0.042205    | 0.500940  0.422043  0.659278  | 0.113744  0.113972  0.065547 
+2     | 0.000250  | 0.285714     | 0.192119     | 0.802624        | 0.619812     | 0.075501          | 0.413090     0.231125     0.440307     0.021942    | 0.430840     0.089809     0.159689     0.019930    | 0.659339  0.443983  0.757597  | 0.081591  0.101869  0.043044 
+3     | 0.000375  | 0.197375     | 0.177898     | 0.830592        | 0.671677     | 0.063464          | 0.400389     0.110370     0.210072     0.010667    | 0.441859     0.064772     0.113361     0.016183    | 0.716478  0.579917  0.716104  | 0.073453  0.066182  0.050757 
+4     | 0.000500  | 0.184946     | 0.183155     | 0.843565        | 0.675978     | 0.044711          | 0.401976     0.091933     0.173822     0.010045    | 0.446157     0.070440     0.123372     0.017508    | 0.715663  0.586346  0.708316  | 0.068421  0.044312  0.021399 
+5     | 0.000495  | 0.176321     | 0.171706     | 0.848226        | 0.707780     | 0.058143          | 0.391617     0.084051     0.158702     0.009400    | 0.427438     0.062107     0.107477     0.016737    | 0.736053  0.626281  0.759208  | 0.063111  0.075133  0.036186 
+6     | 0.000480  | 0.166440     | 0.174257     | 0.854761        | 0.713511     | 0.051072          | 0.382334     0.073913     0.139329     0.008498    | 0.433807     0.063021     0.109811     0.016231    | 0.739106  0.641239  0.749489  | 0.056108  0.064754  0.032355 
+7     | 0.000457  | 0.163203     | 0.173683     | 0.852813        | 0.714835     | 0.055202          | 0.378289     0.071023     0.133956     0.008090    | 0.430470     0.063632     0.110864     0.016400    | 0.746597  0.632457  0.752967  | 0.066237  0.059208  0.040161 
+8     | 0.000427  | 0.158148     | 0.173971     | 0.855150        | 0.713176     | 0.050201          | 0.373610     0.065808     0.124079     0.007536    | 0.434536     0.062300     0.108021     0.016579    | 0.729973  0.632365  0.785751  | 0.061357  0.055891  0.033356 
+9     | 0.000393  | 0.155416     | 0.167303     | 0.857754        | 0.722518     | 0.052089          | 0.369715     0.063573     0.119928     0.007217    | 0.420017     0.058997     0.102804     0.015190    | 0.742610  0.648275  0.783167  | 0.054945  0.064730  0.036590 
+10    | 0.000357  | 0.151937     | 0.170397     | 0.859492        | 0.723506     | 0.049851          | 0.365650     0.060346     0.113872     0.006821    | 0.432371     0.058122     0.100564     0.015680    | 0.747203  0.659582  0.766111  | 0.056361  0.066252  0.026942 
+11    | 0.000323  | 0.150614     | 0.166819     | 0.862530        | 0.732336     | 0.050674          | 0.364682     0.058870     0.111140     0.006600    | 0.425810     0.055823     0.096686     0.014960    | 0.750571  0.659951  0.787415  | 0.058620  0.067716  0.025686 
+12    | 0.000293  | 0.148475     | 0.167548     | 0.857774        | 0.717438     | 0.048668          | 0.361996     0.056966     0.107525     0.006406    | 0.424510     0.057421     0.098569     0.016273    | 0.744813  0.649161  0.767100  | 0.057849  0.060813  0.027344 
+13    | 0.000270  | 0.144937     | 0.173958     | 0.856730        | 0.720325     | 0.052333          | 0.358016     0.053618     0.101279     0.005957    | 0.441312     0.059378     0.102563     0.016193    | 0.741627  0.645762  0.772822  | 0.059138  0.074331  0.023531 
+14    | 0.000255  | 0.143524     | 0.170128     | 0.859741        | 0.721610     | 0.048172          | 0.356290     0.052339     0.098904     0.005774    | 0.431850     0.057962     0.099327     0.016597    | 0.738021  0.653381  0.774060  | 0.057503  0.060348  0.026665 
+15    | 0.000250  | 0.142034     | 0.180749     | 0.854522        | 0.712636     | 0.050887          | 0.355111     0.050715     0.095833     0.005596    | 0.457040     0.062339     0.107160     0.017518    | 0.733249  0.641755  0.764650  | 0.067121  0.062029  0.023510 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2396  1909  1383
+FP   166   206    62
+FN   181   160   143
+TN  4553  5021  5708
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.328  0.262  0.190
+FP  0.023  0.028  0.008
+FN  0.025  0.022  0.020
+TN  0.624  0.688  0.782
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.180749     | 0.854522        | 0.712636     | 0.050887          | 0.457040     0.062339     0.107160     0.017518    | 0.733249  0.641755  0.764650  | 0.067121  0.062029  0.023510 
+266     | 266     | 0.179462     | 0.857314        | 0.717520     | 0.049489          | 0.451040     0.063072     0.107928     0.018216    | 0.734643  0.644502  0.777669  | 0.068024  0.057294  0.023149 
+360     | 310     | 0.183454     | 0.817488        | 0.643560     | 0.066559          | 0.493800     0.050449     0.092134     0.008764    | 0.683004  0.584126  0.697288  | 0.049733  0.128323  0.021622 
+276     | 276     | 0.209003     | 0.861701        | 0.730696     | 0.050962          | 0.530818     0.071083     0.122491     0.019674    | 0.779983  0.674396  0.681221  | 0.076767  0.044667  0.031451 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+LLRD : 0.25, 0.5, 0.75, 1 and aux_head LR = 1x LR
+weight decay 1e-5
+pres_smooth_eps = 0.05
+dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 15m 29s)
+(Max GPU mem usage : 10270.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.535445     | 0.247472     | 0.742268        | 0.515793     | 0.106748          | 0.481983     0.558357     0.913008     0.203707    | 0.462734     0.155217     0.270080     0.040354    | 0.503058  0.411597  0.647524  | 0.127914  0.131567  0.060764 
+2     | 0.000250  | 0.277917     | 0.182992     | 0.819717        | 0.663403     | 0.076074          | 0.410565     0.221068     0.422392     0.019743    | 0.440129     0.072790     0.132768     0.012812    | 0.691116  0.568623  0.733570  | 0.099678  0.082980  0.045563 
+3     | 0.000375  | 0.191359     | 0.175604     | 0.841318        | 0.691554     | 0.058840          | 0.400703     0.101640     0.193591     0.009688    | 0.439864     0.062351     0.109610     0.015091    | 0.720096  0.609531  0.756262  | 0.068707  0.061074  0.046739 
+4     | 0.000500  | 0.180756     | 0.170863     | 0.851982        | 0.710954     | 0.054000          | 0.397490     0.087870     0.166169     0.009571    | 0.426312     0.061385     0.106987     0.015783    | 0.731398  0.632886  0.782147  | 0.057660  0.071666  0.032676 
+5     | 0.000495  | 0.169961     | 0.178510     | 0.851399        | 0.706212     | 0.051810          | 0.385503     0.077586     0.146495     0.008677    | 0.448186     0.062935     0.109324     0.016547    | 0.735175  0.625536  0.748183  | 0.061885  0.073223  0.020321 
+6     | 0.000480  | 0.165166     | 0.171660     | 0.855106        | 0.712978     | 0.050141          | 0.380991     0.072669     0.137119     0.008220    | 0.432291     0.059961     0.102776     0.017145    | 0.733968  0.641963  0.765840  | 0.061635  0.064880  0.023908 
+7     | 0.000457  | 0.165479     | 0.169031     | 0.853141        | 0.707760     | 0.049938          | 0.381803     0.072768     0.137239     0.008297    | 0.429190     0.057534     0.100261     0.014808    | 0.732301  0.633435  0.770447  | 0.061856  0.055158  0.032801 
+8     | 0.000427  | 0.156477     | 0.165915     | 0.850416        | 0.721297     | 0.063505          | 0.371750     0.064218     0.121174     0.007262    | 0.419708     0.057146     0.098733     0.015559    | 0.751018  0.652279  0.768743  | 0.078273  0.064163  0.048078 
+9     | 0.000393  | 0.152694     | 0.167617     | 0.856754        | 0.717000     | 0.050077          | 0.365569     0.061462     0.116018     0.006907    | 0.426104     0.056836     0.097897     0.015775    | 0.738813  0.639058  0.788371  | 0.058142  0.066033  0.026055 
+10    | 0.000357  | 0.148436     | 0.167780     | 0.860567        | 0.727579     | 0.050775          | 0.360440     0.057578     0.108695     0.006460    | 0.427082     0.056651     0.097858     0.015443    | 0.743858  0.665648  0.779504  | 0.061208  0.063474  0.027643 
+11    | 0.000323  | 0.146617     | 0.170643     | 0.862560        | 0.730291     | 0.049260          | 0.359808     0.055250     0.104377     0.006123    | 0.434372     0.057617     0.098803     0.016430    | 0.756751  0.656037  0.765794  | 0.045999  0.062422  0.039359 
+12    | 0.000293  | 0.146763     | 0.165139     | 0.864511        | 0.732798     | 0.047680          | 0.360652     0.055096     0.103984     0.006208    | 0.419896     0.055957     0.096184     0.015730    | 0.752970  0.661601  0.790520  | 0.058377  0.060755  0.023909 
+13    | 0.000270  | 0.143190     | 0.167341     | 0.860111        | 0.731330     | 0.054034          | 0.355966     0.052000     0.098217     0.005784    | 0.424659     0.057062     0.097923     0.016202    | 0.747678  0.661372  0.793412  | 0.053029  0.067251  0.041823 
+14    | 0.000255  | 0.142177     | 0.166595     | 0.855913        | 0.721321     | 0.054359          | 0.355325     0.050828     0.096019     0.005636    | 0.422954     0.056728     0.096959     0.016496    | 0.733833  0.659720  0.795700  | 0.058712  0.074179  0.030187 
+15    | 0.000250  | 0.141603     | 0.173797     | 0.858275        | 0.724665     | 0.052651          | 0.354444     0.050386     0.095174     0.005598    | 0.444054     0.057972     0.099274     0.016670    | 0.743271  0.653501  0.777405  | 0.056589  0.068359  0.033005 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2502  1955  1419
+FP   238   245    79
+FN    75   114   107
+TN  4481  4982  5691
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.343  0.268  0.194
+FP  0.033  0.034  0.011
+FN  0.010  0.016  0.015
+TN  0.614  0.683  0.780
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.173797     | 0.858275        | 0.724665     | 0.052651          | 0.444054     0.057972     0.099274     0.016670    | 0.743271  0.653501  0.777405  | 0.056589  0.068359  0.033005 
+266     | 266     | 0.171924     | 0.859886        | 0.729941     | 0.053484          | 0.437335     0.058176     0.099053     0.017299    | 0.747645  0.660066  0.784611  | 0.058575  0.068043  0.033835 
+360     | 310     | 0.180906     | 0.838133        | 0.662574     | 0.044827          | 0.488449     0.049102     0.089686     0.008519    | 0.680847  0.555337  0.745940  | 0.050148  0.058764  0.025570 
+276     | 276     | 0.207305     | 0.859816        | 0.725407     | 0.050578          | 0.518920     0.073755     0.128255     0.019255    | 0.758337  0.670040  0.720737  | 0.035388  0.085889  0.030457 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,1.25e-4
+All layer LR same
+weight decay 1e-2
+pres_smooth_eps = 0.05
+dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(6h 16m 11s)
+(Max GPU mem usage : 10270.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.534438     | 0.247669     | 0.735489        | 0.496716     | 0.105329          | 0.475772     0.559581     0.914929     0.204233    | 0.453961     0.159258     0.274561     0.043954    | 0.478274  0.403531  0.614089  | 0.126133  0.126411  0.063442 
+2     | 0.000250  | 0.285233     | 0.195960     | 0.775895        | 0.573320     | 0.089056          | 0.410601     0.231504     0.440855     0.022152    | 0.429549     0.095850     0.168812     0.022889    | 0.574379  0.425410  0.729091  | 0.101263  0.113670  0.052235 
+3     | 0.000375  | 0.207905     | 0.171208     | 0.837820        | 0.685812     | 0.060842          | 0.405026     0.123424     0.234678     0.012171    | 0.424001     0.062868     0.110982     0.014754    | 0.710118  0.610871  0.748903  | 0.064721  0.073326  0.044479 
+4     | 0.000500  | 0.182512     | 0.170048     | 0.849758        | 0.710179     | 0.057190          | 0.398230     0.090061     0.170347     0.009775    | 0.426976     0.059936     0.104268     0.015604    | 0.743690  0.634714  0.768299  | 0.073121  0.067615  0.030835 
+5     | 0.000492  | 0.172749     | 0.168838     | 0.855459        | 0.718478     | 0.053220          | 0.387872     0.080553     0.152132     0.008975    | 0.425860     0.058686     0.101904     0.015468    | 0.739580  0.634399  0.790305  | 0.064762  0.068906  0.025991 
+6     | 0.000470  | 0.168302     | 0.171428     | 0.853951        | 0.715500     | 0.053749          | 0.383989     0.075865     0.143063     0.008667    | 0.424560     0.062942     0.109624     0.016261    | 0.726793  0.638243  0.791420  | 0.052343  0.072347  0.036556 
+7     | 0.000435  | 0.162350     | 0.169805     | 0.855429        | 0.713524     | 0.049967          | 0.376036     0.070770     0.133466     0.008074    | 0.424456     0.060668     0.105806     0.015531    | 0.739735  0.646924  0.751292  | 0.057160  0.063001  0.029739 
+8     | 0.000390  | 0.157355     | 0.165573     | 0.861877        | 0.729209     | 0.049678          | 0.372021     0.065355     0.123326     0.007384    | 0.418811     0.057043     0.099096     0.014990    | 0.745038  0.659907  0.788648  | 0.057732  0.064623  0.026681 
+9     | 0.000339  | 0.153581     | 0.166709     | 0.856592        | 0.724343     | 0.055242          | 0.366660     0.062261     0.117538     0.006984    | 0.422045     0.057279     0.099125     0.015433    | 0.743627  0.653054  0.783459  | 0.070005  0.065911  0.029811 
+10    | 0.000286  | 0.148840     | 0.166539     | 0.860561        | 0.722035     | 0.047089          | 0.360904     0.057955     0.109496     0.006415    | 0.422501     0.056841     0.098090     0.015591    | 0.740170  0.661752  0.781455  | 0.055362  0.060785  0.025121 
+11    | 0.000235  | 0.145739     | 0.168171     | 0.865865        | 0.737704     | 0.048694          | 0.358434     0.054584     0.103079     0.006090    | 0.427308     0.057113     0.099336     0.014890    | 0.756277  0.660782  0.800757  | 0.054936  0.065271  0.025874 
+12    | 0.000190  | 0.142937     | 0.163616     | 0.867357        | 0.739357     | 0.047310          | 0.354012     0.052476     0.099152     0.005799    | 0.417171     0.054950     0.094742     0.015157    | 0.753390  0.668044  0.810080  | 0.061069  0.057997  0.022863 
+13    | 0.000155  | 0.140173     | 0.164043     | 0.863813        | 0.737609     | 0.052051          | 0.350789     0.049910     0.094354     0.005465    | 0.418332     0.055062     0.095188     0.014937    | 0.753965  0.666208  0.799449  | 0.061900  0.066080  0.028173 
+14    | 0.000133  | 0.138892     | 0.164615     | 0.870072        | 0.742311     | 0.044754          | 0.349421     0.048665     0.092025     0.005306    | 0.417018     0.056442     0.097360     0.015525    | 0.757163  0.669758  0.803407  | 0.055373  0.056929  0.021960 
+15    | 0.000125  | 0.138154     | 0.168492     | 0.865080        | 0.735291     | 0.048393          | 0.348993     0.047794     0.090417     0.005171    | 0.432298     0.055431     0.094888     0.015975    | 0.750093  0.661385  0.804193  | 0.057884  0.065664  0.021632 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2482  1987  1446
+FP   204   247    67
+FN    95    82    80
+TN  4515  4980  5703
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.340  0.272  0.198
+FP  0.028  0.034  0.009
+FN  0.013  0.011  0.011
+TN  0.619  0.683  0.782
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.168492     | 0.865080        | 0.735291     | 0.048393          | 0.432298     0.055431     0.094888     0.015975    | 0.750093  0.661385  0.804193  | 0.057884  0.065664  0.021632 
+266     | 266     | 0.166994     | 0.867232        | 0.740947     | 0.048578          | 0.426160     0.055923     0.095332     0.016514    | 0.756088  0.667131  0.809298  | 0.058520  0.066138  0.021076 
+360     | 310     | 0.173633     | 0.839728        | 0.671555     | 0.048157          | 0.475371     0.044317     0.079737     0.008897    | 0.652874  0.593356  0.800834  | 0.054704  0.066892  0.022874 
+276     | 276     | 0.196577     | 0.866122        | 0.734205     | 0.045934          | 0.494651     0.068830     0.119257     0.018403    | 0.791482  0.658758  0.726424  | 0.052584  0.056906  0.028311 </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30m 10s
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Cutoffs(LB,SB,S) | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+---------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.163127     | 0.870653        | 0.746137     | 0.046336          | 0.418422     0.053714     0.092436     0.014992    | 0.764649  0.672358  0.808902  | 0.054174  0.061561  0.023273 
+(0.25,0.25,0.25) | 0.163127     | 0.871610        | 0.746417     | 0.044928          | 0.418422     0.053714     0.092436     0.014992    | 0.763309  0.673552  0.809404  | 0.054174  0.057338  0.023273 
+(0.50,0.50,0.50) | 0.163127     | 0.871693        | 0.746247     | 0.044676          | 0.418422     0.053714     0.092436     0.014992    | 0.759691  0.673841  0.810663  | 0.054174  0.057289  0.022566 
+(0.75,0.75,0.75) | 0.163127     | 0.872230        | 0.747347     | 0.044515          | 0.418422     0.053714     0.092436     0.014992    | 0.762146  0.675564  0.811884  | 0.053664  0.057289  0.022592 
+(0.60,0.70,0.70) | 0.163127     | 0.872073        | 0.747195     | 0.044674          | 0.418422     0.053714     0.092436     0.014992    | 0.759819  0.675165  0.810791  | 0.054165  0.057289  0.022568 
+(0.60,0.70,0.80) | 0.163127     | 0.872018        | 0.747068     | 0.044682          | 0.418422     0.053714     0.092436     0.014992    | 0.759819  0.675165  0.810843  | 0.054165  0.057289  0.022592 
+(0.50,0.75,0.75) | 0.163127     | 0.871996        | 0.747017     | 0.044685          | 0.418422     0.053714     0.092436     0.014992    | 0.759691  0.675564  0.811884  | 0.054174  0.057289  0.022592 
+(0.75, 0.75, 0.75) tensor(0.8722)
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2458  1934  1463
+FP   164   187    77
+FN   119   135    63
+TN  4555  5040  5693
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.337  0.265  0.201
+FP  0.022  0.026  0.011
+FN  0.016  0.019  0.009
+TN  0.624  0.691  0.780
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.163127     | 0.872230        | 0.747347     | 0.044515          | 0.418422     0.053714     0.092436     0.014992    | 0.762146  0.675564  0.811884  | 0.053664  0.057289  0.022592 
+266     | 266     | 0.162473     | 0.873347        | 0.751201     | 0.045222          | 0.414362     0.054521     0.093466     0.015577    | 0.766784  0.678514  0.817630  | 0.055781  0.057557  0.022328 
+360     | 310     | 0.161233     | 0.853331        | 0.694867     | 0.041027          | 0.439314     0.042055     0.076282     0.007829    | 0.666841  0.619157  0.816894  | 0.043429  0.059762  0.019890 
+276     | 276     | 0.185312     | 0.880450        | 0.758979     | 0.038569          | 0.477923     0.059908     0.103405     0.016410    | 0.820616  0.701231  0.709365  | 0.035560  0.049983  0.030164 </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Cutoffs(LB,SB,S) | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+---------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.162154     | 0.871441        | 0.747383     | 0.045853          | 0.416631     0.053093     0.091619     0.014567    | 0.766320  0.674663  0.810097  | 0.054598  0.058699  0.024261 
+(0.25,0.25,0.25) | 0.162154     | 0.872516        | 0.747915     | 0.044417          | 0.416631     0.053093     0.091619     0.014567    | 0.764732  0.676475  0.811100  | 0.054598  0.054391  0.024261 
+(0.50,0.50,0.50) | 0.162154     | 0.872540        | 0.747613     | 0.044175          | 0.416631     0.053093     0.091619     0.014567    | 0.761608  0.676588  0.811885  | 0.054598  0.054391  0.023537 
+(0.75,0.75,0.75) | 0.162154     | 0.874002        | 0.750556     | 0.043700          | 0.416631     0.053093     0.091619     0.014567    | 0.764676  0.680206  0.812510  | 0.053487  0.054029  0.023585 
+(0.60,0.70,0.70) | 0.162154     | 0.873755        | 0.750159     | 0.043848          | 0.416631     0.053093     0.091619     0.014567    | 0.764462  0.678461  0.813069  | 0.053707  0.054285  0.023551 
+(0.60,0.70,0.80) | 0.162154     | 0.873765        | 0.750188     | 0.043850          | 0.416631     0.053093     0.091619     0.014567    | 0.764462  0.678461  0.813493  | 0.053707  0.054285  0.023557 
+(0.50,0.75,0.75) | 0.162154     | 0.872916        | 0.748398     | 0.044071          | 0.416631     0.053093     0.091619     0.014567    | 0.761608  0.680206  0.812510  | 0.054598  0.054029  0.023585 
+(0.75, 0.75, 0.75) tensor(0.8740)
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2464  1933  1468
+FP   164   176    81
+FN   113   136    58
+TN  4555  5051  5689
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.338  0.265  0.201
+FP  0.022  0.024  0.011
+FN  0.015  0.019  0.008
+TN  0.624  0.692  0.780
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.162154     | 0.874002        | 0.750556     | 0.043700          | 0.416631     0.053093     0.091619     0.014567    | 0.764676  0.680206  0.812510  | 0.053487  0.054029  0.023585 
+266     | 266     | 0.161535     | 0.875459        | 0.754987     | 0.044227          | 0.412862     0.053823     0.092517     0.015129    | 0.769722  0.683800  0.818745  | 0.055713  0.053691  0.023277 
+360     | 310     | 0.159670     | 0.853128        | 0.693932     | 0.040742          | 0.433860     0.042160     0.076733     0.007588    | 0.667358  0.618056  0.813612  | 0.041066  0.059728  0.021431 
+276     | 276     | 0.184849     | 0.879428        | 0.758193     | 0.039749          | 0.477043     0.059623     0.103092     0.016154    | 0.819456  0.702151  0.709119  | 0.036654  0.051510  0.031083 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA 0.75,0.75,0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA 0.60,0.70,0.70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 14 0.75,0.75,0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 14 0.60,0.70,0.80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full Data
+6h 44m 56s
+Max GPU : 10270.875</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unet++ tu-tf_efficientnetv2_m
+No presence gate in loss
+LR : 1.25e-4,2.5e-4,3.75e-4,5e-4,…,2.5e-4
+All layer LR same
+weight decay 1e-2
+pres_smooth_eps = 0.05
+dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(7h 19m 32s)
+(Max GPU mem usage : 11936.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.573843     | 0.278671     | 0.731055        | 0.544299     | 0.144441          | 0.476153     0.615711     0.951482     0.279940    | 0.452230     0.204288     0.317588     0.090988    | 0.614874  0.526303  0.470374  | 0.191740  0.082946  0.158636 
+2     | 0.000250  | 0.278906     | 0.177828     | 0.839619        | 0.689743     | 0.060464          | 0.413373     0.221278     0.422089     0.020467    | 0.441905     0.064651     0.115738     0.013565    | 0.730601  0.600798  0.749020  | 0.087586  0.059051  0.034755 
+3     | 0.000375  | 0.188516     | 0.171914     | 0.854087        | 0.714453     | 0.052824          | 0.402474     0.096819     0.183952     0.009686    | 0.432873     0.060074     0.105414     0.014735    | 0.750292  0.641562  0.757016  | 0.058823  0.054827  0.044821 
+4     | 0.000500  | 0.180077     | 0.171371     | 0.848874        | 0.706596     | 0.056274          | 0.397385     0.086945     0.164229     0.009660    | 0.433096     0.059203     0.103360     0.015046    | 0.726070  0.632463  0.783822  | 0.066722  0.059112  0.042987 
+5     | 0.000495  | 0.170365     | 0.177812     | 0.848270        | 0.697457     | 0.051189          | 0.386821     0.077598     0.146418     0.008779    | 0.438176     0.066227     0.115400     0.017054    | 0.717907  0.622120  0.766499  | 0.060628  0.048410  0.044528 
+6     | 0.000480  | 0.164442     | 0.178004     | 0.848121        | 0.697237     | 0.051291          | 0.381311     0.071498     0.134827     0.008169    | 0.444938     0.063604     0.110153     0.017055    | 0.704727  0.634116  0.762431  | 0.051503  0.065490  0.036879 
+7     | 0.000457  | 0.162757     | 0.170116     | 0.854828        | 0.712632     | 0.050375          | 0.379314     0.069947     0.131935     0.007959    | 0.421785     0.062258     0.108048     0.016468    | 0.734190  0.629395  0.778958  | 0.050663  0.058849  0.041613 
+8     | 0.000427  | 0.161353     | 0.169056     | 0.852151        | 0.712414     | 0.054692          | 0.378418     0.068326     0.128836     0.007815    | 0.428331     0.057938     0.100785     0.015091    | 0.735830  0.637852  0.773324  | 0.060859  0.075210  0.028008 
+9     | 0.000393  | 0.158029     | 0.169053     | 0.861416        | 0.723458     | 0.046613          | 0.373742     0.065580     0.123735     0.007425    | 0.420308     0.061373     0.106920     0.015826    | 0.740697  0.648761  0.784055  | 0.048823  0.056387  0.034627 
+10    | 0.000357  | 0.151233     | 0.169844     | 0.859215        | 0.720652     | 0.048409          | 0.364878     0.059670     0.112641     0.006700    | 0.426631     0.059792     0.103301     0.016284    | 0.740855  0.649810  0.760533  | 0.062078  0.059857  0.023292 
+11    | 0.000323  | 0.149827     | 0.176940     | 0.857635        | 0.714171     | 0.046722          | 0.362095     0.058854     0.111155     0.006554    | 0.441011     0.063766     0.110654     0.016879    | 0.733892  0.639987  0.759189  | 0.055066  0.057415  0.027686 
+12    | 0.000293  | 0.146786     | 0.169590     | 0.865989        | 0.730198     | 0.043483          | 0.360286     0.055286     0.104431     0.006141    | 0.426255     0.059590     0.103233     0.015947    | 0.751019  0.664547  0.786526  | 0.052465  0.055247  0.022738 
+13    | 0.000270  | 0.143774     | 0.168238     | 0.864007        | 0.730103     | 0.046724          | 0.356092     0.052780     0.099740     0.005819    | 0.431626     0.055357     0.095911     0.014804    | 0.746757  0.657417  0.801028  | 0.055456  0.056635  0.028080 
+14    | 0.000255  | 0.143324     | 0.165599     | 0.867442        | 0.738763     | 0.046772          | 0.355986     0.052184     0.098602     0.005765    | 0.420286     0.056447     0.097692     0.015202    | 0.753854  0.667848  0.800932  | 0.056952  0.063260  0.020106 
+15    | 0.000250  | 0.142413     | 0.164036     | 0.864459        | 0.736130     | 0.049988          | 0.356285     0.050753     0.095932     0.005575    | 0.420529     0.054111     0.092424     0.015797    | 0.752204  0.666606  0.804127  | 0.060456  0.057349  0.032160 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2493  1983  1470
+FP   226   233    89
+FN    84    86    56
+TN  4493  4994  5681
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.342  0.272  0.201
+FP  0.031  0.032  0.012
+FN  0.012  0.012  0.008
+TN  0.616  0.684  0.779
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.164036     | 0.864459        | 0.736130     | 0.049988          | 0.420529     0.054111     0.092424     0.015797    | 0.752204  0.666606  0.804127  | 0.060456  0.057349  0.032160 
+266     | 266     | 0.163114     | 0.865660        | 0.741343     | 0.051462          | 0.415949     0.054756     0.093219     0.016293    | 0.756461  0.671506  0.810868  | 0.062897  0.059170  0.032320 
+360     | 310     | 0.159257     | 0.849884        | 0.682597     | 0.038591          | 0.431317     0.042660     0.076549     0.008772    | 0.674915  0.605944  0.820264  | 0.050920  0.045466  0.019387 
+276     | 276     | 0.200404     | 0.864694        | 0.726345     | 0.043073          | 0.518303     0.064162     0.109048     0.019277    | 0.791008  0.663575  0.673208  | 0.036561  0.045877  0.046782 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segformer mit-b4 
+All LR 1x
+weight_decay 1e-5
+No presence gate in loss
+pres_smooth_eps = 0.05
+Dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(9h 2m 13s)
+(Max GPU mem usage : 12718.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.427051     | 0.182992     | 0.830567        | 0.661093     | 0.056450          | 0.468656     0.409220     0.728288     0.090151    | 0.409844     0.085769     0.159072     0.012467    | 0.714305  0.578912  0.671197  | 0.065129  0.049532  0.054690 
+2     | 0.000250  | 0.205735     | 0.170226     | 0.849402        | 0.692558     | 0.046036          | 0.391905     0.125947     0.242913     0.008982    | 0.412166     0.066537     0.119828     0.013247    | 0.720924  0.600778  0.759943  | 0.047171  0.050725  0.040210 
+3     | 0.000375  | 0.181731     | 0.169864     | 0.843033        | 0.693706     | 0.057416          | 0.381511     0.096111     0.183231     0.008992    | 0.422800     0.061462     0.107955     0.014969    | 0.732584  0.611090  0.737986  | 0.062866  0.071696  0.037687 
+4     | 0.000500  | 0.178813     | 0.168376     | 0.841802        | 0.691796     | 0.058194          | 0.380415     0.092413     0.175581     0.009244    | 0.420150     0.060473     0.105871     0.015075    | 0.721794  0.615409  0.760216  | 0.066556  0.072408  0.035617 
+5     | 0.000495  | 0.168762     | 0.171229     | 0.854033        | 0.708652     | 0.049046          | 0.367797     0.083461     0.158409     0.008514    | 0.428039     0.061168     0.106578     0.015758    | 0.730171  0.628012  0.770733  | 0.057557  0.058981  0.030600 
+6     | 0.000480  | 0.162687     | 0.171316     | 0.843961        | 0.696887     | 0.057990          | 0.360645     0.077848     0.147564     0.008133    | 0.431432     0.059838     0.102643     0.017034    | 0.738212  0.621237  0.727081  | 0.060179  0.056992  0.056798 
+7     | 0.000457  | 0.158185     | 0.167825     | 0.860539        | 0.722523     | 0.047450          | 0.356529     0.073181     0.138718     0.007644    | 0.423131     0.058408     0.100807     0.016009    | 0.746703  0.636738  0.787554  | 0.059269  0.056036  0.027045 
+8     | 0.000427  | 0.158082     | 0.167621     | 0.860027        | 0.722305     | 0.048157          | 0.357354     0.072680     0.137715     0.007645    | 0.417006     0.060741     0.105652     0.015830    | 0.750952  0.650832  0.766464  | 0.054728  0.054834  0.034910 
+9     | 0.000393  | 0.150423     | 0.166826     | 0.861546        | 0.722348     | 0.045655          | 0.349108     0.065273     0.123712     0.006834    | 0.419619     0.058486     0.099778     0.017194    | 0.743904  0.645671  0.786036  | 0.063789  0.050568  0.022608 
+10    | 0.000357  | 0.149958     | 0.166301     | 0.860377        | 0.723413     | 0.048314          | 0.348117     0.065032     0.123184     0.006880    | 0.416689     0.058991     0.101246     0.016736    | 0.751665  0.644421  0.776553  | 0.059478  0.052734  0.032731 
+11    | 0.000323  | 0.146811     | 0.172097     | 0.850321        | 0.716155     | 0.060235          | 0.345451     0.061680     0.116845     0.006516    | 0.429558     0.061757     0.105153     0.018360    | 0.738733  0.628347  0.781069  | 0.061588  0.074858  0.044257 
+12    | 0.000293  | 0.144868     | 0.166957     | 0.853930        | 0.713645     | 0.052547          | 0.342538     0.060152     0.114028     0.006277    | 0.414558     0.060842     0.104511     0.017173    | 0.728495  0.638784  0.791698  | 0.066145  0.063134  0.028363 
+13    | 0.000270  | 0.142877     | 0.170625     | 0.861211        | 0.726045     | 0.048678          | 0.341334     0.057824     0.109579     0.006070    | 0.432476     0.058403     0.098441     0.018365    | 0.749937  0.648485  0.785138  | 0.058527  0.059246  0.028262 
+14    | 0.000255  | 0.139981     | 0.168317     | 0.864676        | 0.735059     | 0.048913          | 0.338173     0.055042     0.104280     0.005803    | 0.427084     0.057417     0.095552     0.019282    | 0.754412  0.662053  0.790880  | 0.064557  0.058946  0.023237 
+15    | 0.000250  | 0.139062     | 0.173318     | 0.863709        | 0.728902     | 0.046420          | 0.337508     0.054014     0.102302     0.005727    | 0.435077     0.061136     0.102996     0.019276    | 0.753721  0.654304  0.773068  | 0.056407  0.058756  0.024096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2460  1930  1420
+FP   168   181    75
+FN   117   139   106
+TN  4551  5046  5695
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.337  0.265  0.195
+FP  0.023  0.025  0.010
+FN  0.016  0.019  0.015
+TN  0.624  0.692  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.173318     | 0.863709        | 0.728902     | 0.046420          | 0.435077     0.061136     0.102996     0.019276    | 0.753721  0.654304  0.773068  | 0.056407  0.058756  0.024096 
+266     | 266     | 0.173153     | 0.863469        | 0.729372     | 0.047133          | 0.432907     0.061830     0.103537     0.020123    | 0.748023  0.657351  0.785512  | 0.057981  0.059280  0.024137 
+360     | 310     | 0.175721     | 0.849630        | 0.687585     | 0.042340          | 0.460861     0.053518     0.097029     0.010008    | 0.750207  0.582127  0.690355  | 0.053295  0.056206  0.017519 
+276     | 276     | 0.172006     | 0.887894        | 0.781476     | 0.041161          | 0.431777     0.060676     0.102700     0.018651    | 0.849305  0.698910  0.728242  | 0.036941  0.054301  0.032241 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segformer mit-b4 
+All LR 1x
+weight_decay 1e-2
+No presence gate in loss
+pres_smooth_eps = 0.05
+Dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(9h 54s)
+(Max GPU mem usage : 12718.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.427792     | 0.189531     | 0.824809        | 0.641429     | 0.052937          | 0.459722     0.414108     0.730344     0.097871    | 0.417860     0.091676     0.169577     0.013775    | 0.700515  0.549666  0.637151  | 0.065100  0.044934  0.048777 
+2     | 0.000250  | 0.205577     | 0.181840     | 0.840883        | 0.670372     | 0.045442          | 0.390591     0.126285     0.243377     0.009192    | 0.438212     0.071966     0.129539     0.014393    | 0.694375  0.565584  0.756653  | 0.044596  0.049170  0.042562 
+3     | 0.000375  | 0.182392     | 0.169331     | 0.849710        | 0.705591     | 0.054211          | 0.381353     0.097124     0.185198     0.009049    | 0.417241     0.063083     0.111140     0.015027    | 0.739522  0.622454  0.761443  | 0.046842  0.065524  0.050268 
+4     | 0.000500  | 0.179396     | 0.175649     | 0.815191        | 0.661984     | 0.082671          | 0.379972     0.093434     0.177417     0.009451    | 0.436661     0.063787     0.110569     0.017004    | 0.707093  0.568706  0.754079  | 0.089822  0.103259  0.054931 
+5     | 0.000495  | 0.170386     | 0.166823     | 0.854018        | 0.712241     | 0.051464          | 0.370202     0.084751     0.160763     0.008738    | 0.417446     0.059413     0.103115     0.015710    | 0.738333  0.628295  0.772163  | 0.064725  0.067089  0.022578 
+6     | 0.000480  | 0.166776     | 0.169351     | 0.853272        | 0.710591     | 0.051608          | 0.365467     0.081623     0.154742     0.008504    | 0.421478     0.061297     0.107028     0.015566    | 0.732662  0.637173  0.761063  | 0.059365  0.057794  0.037665 
+7     | 0.000457  | 0.162399     | 0.167760     | 0.851685        | 0.712643     | 0.055621          | 0.361681     0.076993     0.145968     0.008018    | 0.421505     0.059012     0.101498     0.016525    | 0.740654  0.635903  0.766141  | 0.071788  0.055660  0.039414 
+8     | 0.000427  | 0.157783     | 0.169293     | 0.858982        | 0.713653     | 0.044131          | 0.356911     0.072443     0.137267     0.007618    | 0.418325     0.062565     0.109341     0.015789    | 0.751922  0.624118  0.769915  | 0.047501  0.054177  0.030716 
+9     | 0.000393  | 0.154333     | 0.168777     | 0.860005        | 0.722800     | 0.048526          | 0.353559     0.068950     0.130616     0.007284    | 0.422443     0.060063     0.103293     0.016832    | 0.746363  0.645032  0.773007  | 0.049435  0.057916  0.038226 
+10    | 0.000357  | 0.149985     | 0.163680     | 0.863285        | 0.726243     | 0.045353          | 0.348807     0.064775     0.122683     0.006868    | 0.410218     0.058021     0.100943     0.015100    | 0.747673  0.640891  0.806184  | 0.055343  0.056975  0.023743 
+11    | 0.000323  | 0.149070     | 0.167082     | 0.859209        | 0.719328     | 0.047537          | 0.348490     0.063604     0.120463     0.006745    | 0.417537     0.059743     0.103031     0.016456    | 0.741452  0.638640  0.786783  | 0.057375  0.051816  0.033420 
+12    | 0.000293  | 0.146993     | 0.162364     | 0.864537        | 0.734035     | 0.048461          | 0.344566     0.062319     0.118086     0.006553    | 0.410883     0.055856     0.095244     0.016468    | 0.754487  0.657888  0.804052  | 0.059303  0.060736  0.025345 
+13    | 0.000270  | 0.141556     | 0.165996     | 0.866803        | 0.736314     | 0.046204          | 0.339704     0.056636     0.107356     0.005916    | 0.421163     0.056638     0.096479     0.016798    | 0.756638  0.660185  0.800170  | 0.053811  0.060883  0.023918 
+14    | 0.000255  | 0.140876     | 0.167348     | 0.866169        | 0.732094     | 0.044447          | 0.339470     0.055764     0.105675     0.005854    | 0.420514     0.058849     0.098606     0.019092    | 0.752894  0.656128  0.792930  | 0.050652  0.056274  0.026415 
+15    | 0.000250  | 0.139819     | 0.167226     | 0.864115        | 0.730230     | 0.046629          | 0.337965     0.054899     0.103980     0.005818    | 0.419135     0.059265     0.100714     0.017818    | 0.748390  0.650728  0.799601  | 0.049380  0.063669  0.026838</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2465  1943  1474
+FP   180   214    86
+FN   112   126    52
+TN  4539  5013  5684
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.338  0.266  0.202
+FP  0.025  0.029  0.012
+FN  0.015  0.017  0.007
+TN  0.622  0.687  0.779
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.167226     | 0.864115        | 0.730230     | 0.046629          | 0.419135     0.059265     0.100714     0.017818    | 0.748390  0.650728  0.799601  | 0.049380  0.063669  0.026838 
+266     | 266     | 0.167778     | 0.864371        | 0.731121     | 0.046795          | 0.417339     0.060823     0.103038     0.018609    | 0.745871  0.652072  0.805764  | 0.051214  0.064311  0.024859 
+360     | 310     | 0.157164     | 0.848310        | 0.691398     | 0.047083          | 0.427359     0.041366     0.073991     0.008740    | 0.713020  0.596653  0.791998  | 0.042154  0.056066  0.043028 
+276     | 276     | 0.176480     | 0.883656        | 0.774444     | 0.043536          | 0.447884     0.060164     0.102085     0.018243    | 0.838200  0.704820  0.713874  | 0.031501  0.064169  0.034937 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segformer mit-b4 
+LR : Auxhead 1/16x rest 1x
+weight_decay 1e-5
+No presence gate in loss
+pres_smooth_eps = 0.05
+Dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(8h 47m 9s)
+(Max GPU mem usage : 12718.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.434933     | 0.190488     | 0.821791        | 0.639648     | 0.056781          | 0.472288     0.418923     0.737239     0.100608    | 0.424865     0.090041     0.166449     0.013634    | 0.706653  0.560824  0.615683  | 0.063033  0.047965  0.059343 
+2     | 0.000250  | 0.204950     | 0.172670     | 0.850108        | 0.690082     | 0.043208          | 0.389598     0.125815     0.242655     0.008974    | 0.421896     0.065859     0.118869     0.012849    | 0.721594  0.586003  0.764765  | 0.048394  0.050361  0.030869 
+3     | 0.000375  | 0.181577     | 0.173111     | 0.849974        | 0.697629     | 0.048462          | 0.381018     0.096103     0.183279     0.008926    | 0.419971     0.067314     0.119814     0.014815    | 0.730511  0.610824  0.747748  | 0.054248  0.052844  0.038295 
+4     | 0.000500  | 0.178674     | 0.170016     | 0.843402        | 0.698055     | 0.059700          | 0.379368     0.092662     0.176155     0.009170    | 0.418385     0.063571     0.111572     0.015571    | 0.730467  0.600261  0.758572  | 0.066142  0.064886  0.048072 
+5     | 0.000495  | 0.170308     | 0.170743     | 0.843089        | 0.693489     | 0.057178          | 0.369223     0.085059     0.161507     0.008611    | 0.425583     0.061526     0.107959     0.015092    | 0.718630  0.615253  0.751346  | 0.055016  0.068222  0.048295 
+6     | 0.000480  | 0.163979     | 0.174432     | 0.842637        | 0.683808     | 0.051477          | 0.363523     0.078461     0.148814     0.008108    | 0.426381     0.066454     0.116290     0.016619    | 0.720075  0.581696  0.730631  | 0.061697  0.048979  0.043754 
+7     | 0.000457  | 0.159186     | 0.170234     | 0.848764        | 0.703509     | 0.054400          | 0.358617     0.073716     0.139773     0.007659    | 0.424745     0.061158     0.105774     0.016542    | 0.741355  0.629820  0.735243  | 0.054184  0.051325  0.057691 
+8     | 0.000427  | 0.156100     | 0.173583     | 0.857657        | 0.709021     | 0.043253          | 0.355018     0.070849     0.134311     0.007386    | 0.427404     0.064802     0.113091     0.016514    | 0.740356  0.617625  0.757199  | 0.056809  0.050658  0.022293 
+9     | 0.000393  | 0.155514     | 0.169395     | 0.844644        | 0.699053     | 0.058294          | 0.354663     0.070165     0.132945     0.007385    | 0.418230     0.062751     0.107737     0.017766    | 0.718564  0.629925  0.772712  | 0.061174  0.056612  0.057097 
+10    | 0.000357  | 0.150325     | 0.168544     | 0.851366        | 0.700826     | 0.048274          | 0.349121     0.065127     0.123373     0.006880    | 0.420941     0.060374     0.102737     0.018012    | 0.730822  0.617573  0.770000  | 0.063475  0.049229  0.032118 
+11    | 0.000323  | 0.147674     | 0.167128     | 0.855549        | 0.717789     | 0.052611          | 0.346461     0.062480     0.118367     0.006593    | 0.419950     0.058776     0.099981     0.017571    | 0.738514  0.642168  0.800190  | 0.068269  0.058189  0.031376 
+12    | 0.000293  | 0.144235     | 0.170153     | 0.859182        | 0.717506     | 0.046367          | 0.341850     0.059542     0.112893     0.006191    | 0.428224     0.059551     0.101266     0.017836    | 0.735934  0.642964  0.789317  | 0.053571  0.055847  0.029682 
+13    | 0.000270  | 0.142998     | 0.167524     | 0.860641        | 0.721035     | 0.046288          | 0.342074     0.057680     0.109221     0.006138    | 0.418527     0.059951     0.102804     0.017099    | 0.743957  0.638660  0.797992  | 0.055802  0.055090  0.027970 
+14    | 0.000255  | 0.140431     | 0.167197     | 0.860602        | 0.721372     | 0.046578          | 0.339199     0.055245     0.104636     0.005853    | 0.423684     0.057274     0.094960     0.019589    | 0.746612  0.647993  0.796251  | 0.054866  0.059219  0.025650 
+15    | 0.000250  | 0.138778     | 0.166788     | 0.862005        | 0.724359     | 0.046230          | 0.338025     0.053387     0.101071     0.005702    | 0.419074     0.058666     0.099496     0.017836    | 0.744748  0.653813  0.783976  | 0.052977  0.061066  0.024648 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2481  1989  1435
+FP   202   235    75
+FN    96    80    91
+TN  4517  4992  5695
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.340  0.273  0.197
+FP  0.028  0.032  0.010
+FN  0.013  0.011  0.012
+TN  0.619  0.684  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.166788     | 0.862005        | 0.724359     | 0.046230          | 0.419074     0.058666     0.099496     0.017836    | 0.744748  0.653813  0.783976  | 0.052977  0.061066  0.024648 
+266     | 266     | 0.166843     | 0.862672        | 0.725391     | 0.045808          | 0.416583     0.059811     0.100947     0.018675    | 0.743179  0.655669  0.789536  | 0.053958  0.059343  0.024123 
+360     | 310     | 0.161736     | 0.846260        | 0.688900     | 0.048833          | 0.435916     0.044231     0.080414     0.008048    | 0.705077  0.601465  0.782648  | 0.054138  0.071836  0.020524 
+276     | 276     | 0.177448     | 0.874183        | 0.759101     | 0.049097          | 0.445900     0.062397     0.106123     0.018672    | 0.824789  0.693120  0.696519  | 0.036716  0.072552  0.038021 </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">51m 17s
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">Cutoffs(LB,SB,S) | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+---------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+(0.00,0.00,0.00) | 0.164208     | 0.866245        | 0.736652     | 0.047360          | 0.419038     0.054995     0.091925     0.018066    | 0.757168  0.669904  0.792305  | 0.053947  0.052956  0.035177 
+(0.25,0.25,0.25) | 0.164208     | 0.866757        | 0.737373     | 0.046987          | 0.419038     0.054995     0.091925     0.018066    | 0.757553  0.669723  0.795031  | 0.053830  0.052956  0.034176 
+(0.50,0.50,0.50) | 0.164208     | 0.867113        | 0.737670     | 0.046592          | 0.419038     0.054995     0.091925     0.018066    | 0.758032  0.670749  0.797937  | 0.053830  0.052956  0.032988 
+(0.75,0.75,0.75) | 0.164208     | 0.868768        | 0.740796     | 0.045917          | 0.419038     0.054995     0.091925     0.018066    | 0.761943  0.674656  0.800223  | 0.051899  0.052955  0.032898 
+(0.60,0.70,0.70) | 0.164208     | 0.868573        | 0.741275     | 0.046561          | 0.419038     0.054995     0.091925     0.018066    | 0.760821  0.673499  0.799734  | 0.053830  0.052955  0.032898 
+(0.60,0.70,0.80) | 0.164208     | 0.868703        | 0.741591     | 0.046555          | 0.419038     0.054995     0.091925     0.018066    | 0.760821  0.673499  0.800669  | 0.053830  0.052955  0.032879 
+(0.50,0.75,0.75) | 0.164208     | 0.867898        | 0.739586     | 0.046561          | 0.419038     0.054995     0.091925     0.018066    | 0.758032  0.674656  0.800223  | 0.053830  0.052955  0.032898 
+(0.75, 0.75, 0.75) tensor(0.8688)
+Confusion Matrix raw counts
+      LB    SB     S
+TP  2494  1977  1489
+FP   209   230   110
+FN    83    92    37
+TN  4510  4997  5660
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.342  0.271  0.204
+FP  0.029  0.032  0.015
+FN  0.011  0.013  0.005
+TN  0.618  0.685  0.776
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.164208     | 0.868768        | 0.740796     | 0.045917          | 0.419038     0.054995     0.091925     0.018066    | 0.761943  0.674656  0.800223  | 0.051899  0.052955  0.032898 
+266     | 266     | 0.164057     | 0.868603        | 0.740989     | 0.046321          | 0.415991     0.056085     0.093309     0.018861    | 0.758115  0.677678  0.802835  | 0.053026  0.053025  0.032912 
+360     | 310     | 0.155882     | 0.861003        | 0.715078     | 0.041713          | 0.424164     0.040904     0.072962     0.008846    | 0.745020  0.611751  0.829197  | 0.052002  0.052606  0.020531 
+276     | 276     | 0.188283     | 0.882913        | 0.775484     | 0.045468          | 0.489023     0.059395     0.100054     0.018737    | 0.846371  0.708944  0.704705  | 0.034849  0.052362  0.049192 
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA cutoff 0.75,0.75,0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA cutoff 0.60,0.70,0.70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full Data
+9h 5m 27s
+Max GPU : 12718.875 MB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | TLo-Pres     TLo-Seg      TLo-D        TLo-B       
+--------------------------------------------------------------------------------------
+1     | 0.000125  | 0.389623     | 0.447056     0.365009     0.649772     0.080247    
+2     | 0.000250  | 0.197201     | 0.391336     0.114000     0.218704     0.009295    
+3     | 0.000375  | 0.184171     | 0.384876     0.098154     0.186695     0.009614    
+4     | 0.000500  | 0.177691     | 0.378160     0.091776     0.174146     0.009406    
+5     | 0.000495  | 0.173299     | 0.374259     0.087174     0.165116     0.009231    
+6     | 0.000480  | 0.166342     | 0.366222     0.080680     0.152772     0.008587    
+7     | 0.000457  | 0.162734     | 0.361930     0.077364     0.146520     0.008208    
+8     | 0.000427  | 0.160265     | 0.359044     0.075074     0.142087     0.008061    
+9     | 0.000393  | 0.155016     | 0.353997     0.069738     0.131954     0.007521    
+10    | 0.000357  | 0.150590     | 0.348647     0.065708     0.124371     0.007045    
+11    | 0.000323  | 0.150978     | 0.349902     0.065725     0.124284     0.007166    
+12    | 0.000293  | 0.147721     | 0.345639     0.062899     0.119072     0.006726    
+13    | 0.000270  | 0.142030     | 0.340755     0.056863     0.107636     0.006089    
+14    | 0.000255  | 0.142614     | 0.340941     0.057617     0.109034     0.006200    
+15    | 0.000250  | 0.142886     | 0.342112     0.057504     0.108775     0.006233    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 15 cutoff 0.75,0.75,0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMA Epoch 15 cutoff 0.60,0.70,0.70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segformer mit-b4 
+All LR 1x
+weight_decay 1e-5
+No presence gate in loss
+pres_smooth_eps = 0
+Dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(8h 47m 46s)
+(Max GPU mem usage : 12718.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.358670     | 0.112178     | 0.815607        | 0.630005     | 0.060659          | 0.195504     0.428599     0.750716     0.106482    | 0.151538     0.095309     0.175427     0.015192    | 0.691113  0.526051  0.649278  | 0.081328  0.048730  0.051919 
+2     | 0.000250  | 0.119267     | 0.094457     | 0.848905        | 0.688463     | 0.044134          | 0.093447     0.130333     0.251520     0.009147    | 0.156972     0.067665     0.123091     0.012240    | 0.712111  0.604868  0.744864  | 0.045538  0.059129  0.027734 
+3     | 0.000375  | 0.092062     | 0.090792     | 0.849866        | 0.707730     | 0.055377          | 0.080449     0.097039     0.185275     0.008802    | 0.157906     0.062029     0.110116     0.013941    | 0.744817  0.621086  0.756328  | 0.057498  0.057994  0.050639 
+4     | 0.000500  | 0.092351     | 0.092989     | 0.836175        | 0.685441     | 0.063336          | 0.081935     0.096814     0.184190     0.009439    | 0.161801     0.063498     0.112748     0.014249    | 0.713684  0.603279  0.747180  | 0.063385  0.060077  0.066548 
+5     | 0.000495  | 0.078470     | 0.083777     | 0.847050        | 0.706915     | 0.059527          | 0.062074     0.085497     0.162293     0.008702    | 0.132225     0.063014     0.110284     0.015743    | 0.726804  0.621404  0.784758  | 0.060502  0.074749  0.043329 
+6     | 0.000480  | 0.073526     | 0.092787     | 0.850950        | 0.706028     | 0.052434          | 0.054242     0.081791     0.155236     0.008345    | 0.167884     0.060602     0.105642     0.015562    | 0.739664  0.626946  0.739564  | 0.060108  0.068196  0.028999 
+7     | 0.000457  | 0.066597     | 0.095918     | 0.857457        | 0.726277     | 0.055090          | 0.046196     0.075340     0.143020     0.007660    | 0.180017     0.059875     0.103895     0.015855    | 0.744131  0.655063  0.783201  | 0.059138  0.063158  0.042974 
+8     | 0.000427  | 0.063501     | 0.088795     | 0.855783        | 0.712633     | 0.048783          | 0.041747     0.072825     0.138111     0.007538    | 0.159595     0.058451     0.099996     0.016907    | 0.732191  0.628051  0.805158  | 0.058673  0.062381  0.025296 
+9     | 0.000393  | 0.058606     | 0.094475     | 0.842377        | 0.701665     | 0.063815          | 0.035049     0.068701     0.130238     0.007164    | 0.175158     0.059896     0.102970     0.016823    | 0.725844  0.632299  0.781895  | 0.072273  0.063586  0.055585 
+10    | 0.000357  | 0.055391     | 0.103461     | 0.856162        | 0.719395     | 0.052660          | 0.031151     0.065780     0.124695     0.006865    | 0.208744     0.058340     0.101290     0.015390    | 0.737659  0.644957  0.788373  | 0.056313  0.068134  0.033532 
+11    | 0.000323  | 0.051027     | 0.104468     | 0.858563        | 0.724268     | 0.051907          | 0.025092     0.062142     0.117769     0.006515    | 0.209318     0.059532     0.101343     0.017721    | 0.746070  0.646574  0.794459  | 0.061275  0.056213  0.038234 
+12    | 0.000293  | 0.049659     | 0.097252     | 0.855788        | 0.717513     | 0.052029          | 0.022665     0.061228     0.116048     0.006407    | 0.181036     0.061344     0.105722     0.016967    | 0.737336  0.649227  0.766910  | 0.055259  0.071942  0.028886 
+13    | 0.000270  | 0.047107     | 0.099127     | 0.856074        | 0.718227     | 0.052029          | 0.020604     0.058465     0.110773     0.006156    | 0.186523     0.061672     0.106011     0.017333    | 0.744613  0.635181  0.789370  | 0.060015  0.067036  0.029036 
+14    | 0.000255  | 0.047290     | 0.107511     | 0.854521        | 0.717786     | 0.054322          | 0.020489     0.058776     0.111356     0.006196    | 0.215486     0.061237     0.102685     0.019788    | 0.736518  0.637255  0.781967  | 0.067522  0.060581  0.034864 
+15    | 0.000250  | 0.043231     | 0.100820     | 0.861426        | 0.725941     | 0.048250          | 0.016639     0.054628     0.103504     0.005752    | 0.201719     0.057578     0.097628     0.017528    | 0.742542  0.647051  0.798719  | 0.063318  0.054608  0.026825</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2494  1963  1447
+FP   241   224    59
+FN    83   106    79
+TN  4478  5003  5711
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.342  0.269  0.198
+FP  0.033  0.031  0.008
+FN  0.011  0.015  0.011
+TN  0.614  0.686  0.783
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.100820     | 0.861426        | 0.725941     | 0.048250          | 0.201719     0.057578     0.097628     0.017528    | 0.742542  0.647051  0.798719  | 0.063318  0.054608  0.026825 
+266     | 266     | 0.097857     | 0.862479        | 0.729844     | 0.049098          | 0.190256     0.058257     0.098359     0.018155    | 0.744009  0.652311  0.804342  | 0.064590  0.055273  0.027430 
+360     | 310     | 0.099105     | 0.844126        | 0.672066     | 0.041167          | 0.223471     0.045806     0.082698     0.008913    | 0.676913  0.567200  0.808025  | 0.055183  0.052206  0.016113 
+276     | 276     | 0.184955     | 0.868712        | 0.739256     | 0.044984          | 0.459022     0.067498     0.113730     0.021265    | 0.808721  0.666216  0.691323  | 0.055077  0.047838  0.032036 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segformer mit-b4 
+LR : Auxhead 1/16x rest 1x
+weight_decay 1e-5
+No presence gate in loss
+pres_smooth_eps = 0.05
+Aux head MaxPool
+Dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(8h 56m 55s)
+(Max GPU mem usage : 12718.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.453211     | 0.193345     | 0.814250        | 0.624617     | 0.059327          | 0.498270     0.433900     0.754985     0.112815    | 0.423101     0.094878     0.174180     0.015576    | 0.693044  0.538633  0.614223  | 0.067291  0.045274  0.065417 
+2     | 0.000250  | 0.209729     | 0.178303     | 0.848075        | 0.678559     | 0.038915          | 0.395556     0.130089     0.250770     0.009409    | 0.432747     0.069255     0.125774     0.012736    | 0.692802  0.598486  0.750624  | 0.036163  0.047058  0.033524 
+3     | 0.000375  | 0.183775     | 0.177581     | 0.822156        | 0.666060     | 0.073781          | 0.384953     0.097556     0.186088     0.009025    | 0.428705     0.069957     0.121182     0.018731    | 0.725909  0.578473  0.659520  | 0.066928  0.073027  0.081387 
+4     | 0.000500  | 0.179641     | 0.173477     | 0.844771        | 0.698119     | 0.057461          | 0.381414     0.093167     0.176991     0.009343    | 0.433430     0.062069     0.108160     0.015979    | 0.733432  0.625819  0.733935  | 0.063526  0.065396  0.043461 
+5     | 0.000495  | 0.167362     | 0.168687     | 0.856084        | 0.714827     | 0.049745          | 0.367808     0.081457     0.154450     0.008464    | 0.421330     0.060411     0.105021     0.015801    | 0.728021  0.636149  0.775803  | 0.047909  0.064467  0.036860 
+6     | 0.000480  | 0.162884     | 0.169166     | 0.851779        | 0.709558     | 0.053407          | 0.361532     0.077749     0.147380     0.008119    | 0.416789     0.063042     0.110137     0.015946    | 0.726275  0.638850  0.772142  | 0.048639  0.065491  0.046091 
+7     | 0.000457  | 0.159354     | 0.164872     | 0.861509        | 0.723922     | 0.046766          | 0.358855     0.073853     0.139998     0.007708    | 0.413044     0.058512     0.100141     0.016883    | 0.749319  0.650622  0.782835  | 0.056999  0.054657  0.028643 
+8     | 0.000427  | 0.158053     | 0.166323     | 0.866135        | 0.725992     | 0.040437          | 0.356686     0.072924     0.138127     0.007721    | 0.411314     0.061326     0.107072     0.015581    | 0.747323  0.646720  0.782514  | 0.044869  0.051179  0.025264 
+9     | 0.000393  | 0.153590     | 0.172053     | 0.846237        | 0.700270     | 0.056452          | 0.352396     0.068388     0.129616     0.007160    | 0.426574     0.062973     0.106749     0.019197    | 0.729183  0.621101  0.744924  | 0.063716  0.050260  0.055381 
+10    | 0.000357  | 0.149834     | 0.166867     | 0.861418        | 0.726172     | 0.048417          | 0.348712     0.064600     0.122420     0.006780    | 0.421118     0.057902     0.100140     0.015665    | 0.751966  0.652442  0.779149  | 0.061145  0.054764  0.029343 
+11    | 0.000323  | 0.145661     | 0.169132     | 0.861322        | 0.725732     | 0.048284          | 0.343838     0.060729     0.115104     0.006353    | 0.422521     0.060537     0.103392     0.017683    | 0.744668  0.646815  0.790397  | 0.046072  0.061074  0.037707 
+12    | 0.000293  | 0.142284     | 0.172562     | 0.861300        | 0.723745     | 0.046996          | 0.340468     0.057347     0.108701     0.005994    | 0.433474     0.060742     0.103394     0.018090    | 0.745384  0.651778  0.760392  | 0.067157  0.054538  0.019293 
+13    | 0.000270  | 0.143655     | 0.169987     | 0.861841        | 0.718672     | 0.042713          | 0.343515     0.058001     0.109785     0.006218    | 0.426007     0.060264     0.102587     0.017941    | 0.741823  0.646160  0.777849  | 0.048520  0.054055  0.025563 
+14    | 0.000255  | 0.141732     | 0.168458     | 0.860516        | 0.724693     | 0.048935          | 0.340536     0.056531     0.107086     0.005976    | 0.416579     0.062120     0.103970     0.020270    | 0.742642  0.637434  0.795018  | 0.076808  0.049730  0.020267 
+15    | 0.000250  | 0.138967     | 0.169214     | 0.864268        | 0.725850     | 0.043453          | 0.337677     0.053805     0.101844     0.005767    | 0.424209     0.059929     0.102448     0.017411    | 0.740429  0.651761  0.802645  | 0.050797  0.058838  0.020725</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2449  1961  1454
+FP   203   236    55
+FN   128   108    72
+TN  4516  4991  5715
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.336  0.269  0.199
+FP  0.028  0.032  0.008
+FN  0.018  0.015  0.010
+TN  0.619  0.684  0.783
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.169214     | 0.864268        | 0.725850     | 0.043453          | 0.424209     0.059929     0.102448     0.017411    | 0.740429  0.651761  0.802645  | 0.050797  0.058838  0.020725 
+266     | 266     | 0.169143     | 0.864166        | 0.726956     | 0.044360          | 0.419989     0.061637     0.105081     0.018194    | 0.740270  0.652831  0.806586  | 0.052485  0.060061  0.020534 
+360     | 310     | 0.162951     | 0.854630        | 0.690158     | 0.035722          | 0.450002     0.039929     0.071898     0.007960    | 0.676711  0.611620  0.817265  | 0.042586  0.050184  0.014395 
+276     | 276     | 0.186152     | 0.879674        | 0.759423     | 0.040159          | 0.476269     0.061817     0.104672     0.018961    | 0.830982  0.688320  0.710031  | 0.036431  0.052021  0.032023 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segformer mit-b4 
+LR : Auxhead 1/32x rest 1x
+weight_decay 1e-5
+No presence gate in loss
+pres_smooth_eps = 0.05
+Dropout = 0.3
+grad_accu=4, effBS = 16*4 = 64
+(8h 55m 59s)
+(Max GPU mem usage : 12718.875 MB)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epoch | LR        | Train Loss   | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | TLo-Pres     TLo-Seg      TLo-D        TLo-B       | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+1     | 0.000125  | 0.433426     | 0.187972     | 0.820840        | 0.643571     | 0.060981          | 0.471466     0.417123     0.734277     0.099970    | 0.416083     0.090209     0.165825     0.014594    | 0.698592  0.559307  0.651686  | 0.073504  0.051483  0.057957 
+2     | 0.000250  | 0.206636     | 0.175467     | 0.846990        | 0.679792     | 0.041546          | 0.390438     0.127864     0.246473     0.009255    | 0.421485     0.070030     0.126173     0.013888    | 0.690871  0.596496  0.761324  | 0.035433  0.062867  0.026336 
+3     | 0.000375  | 0.183400     | 0.167289     | 0.853131        | 0.710772     | 0.051963          | 0.381566     0.098471     0.187767     0.009175    | 0.415502     0.060911     0.107523     0.014299    | 0.738403  0.625375  0.780051  | 0.055913  0.066951  0.033025 
+4     | 0.000500  | 0.177559     | 0.174988     | 0.826336        | 0.670592     | 0.069835          | 0.378539     0.091424     0.173681     0.009167    | 0.434567     0.063740     0.111089     0.016392    | 0.696796  0.585428  0.758780  | 0.065171  0.090445  0.053889 
+5     | 0.000495  | 0.172160     | 0.164331     | 0.849957        | 0.716338     | 0.060964          | 0.372836     0.086155     0.163498     0.008813    | 0.408112     0.059853     0.104779     0.014927    | 0.744241  0.629163  0.770715  | 0.059274  0.060911  0.062706 
+6     | 0.000480  | 0.162092     | 0.171527     | 0.855541        | 0.713294     | 0.049628          | 0.360847     0.076911     0.145903     0.007918    | 0.439179     0.056820     0.098197     0.015442    | 0.736129  0.631037  0.783742  | 0.058307  0.061161  0.029417 
+7     | 0.000457  | 0.162161     | 0.170560     | 0.851269        | 0.702540     | 0.049579          | 0.361422     0.076764     0.145493     0.008036    | 0.422516     0.062579     0.108640     0.016517    | 0.720456  0.631357  0.763685  | 0.058694  0.053682  0.036360 
+8     | 0.000427  | 0.158006     | 0.167498     | 0.854200        | 0.710654     | 0.050103          | 0.356894     0.072768     0.137887     0.007650    | 0.415742     0.061108     0.105674     0.016541    | 0.742192  0.628163  0.765900  | 0.058224  0.059323  0.032762 
+9     | 0.000393  | 0.152873     | 0.172231     | 0.850595        | 0.711076     | 0.056393          | 0.351466     0.067761     0.128413     0.007108    | 0.437029     0.058747     0.099848     0.017646    | 0.730665  0.636467  0.774660  | 0.068413  0.059880  0.040887 
+10    | 0.000357  | 0.149131     | 0.174474     | 0.858504        | 0.715789     | 0.046353          | 0.348252     0.063794     0.120884     0.006703    | 0.437582     0.061713     0.105794     0.017632    | 0.727264  0.641543  0.780749  | 0.055671  0.054776  0.028611 
+11    | 0.000323  | 0.148918     | 0.181989     | 0.854504        | 0.699158     | 0.041931          | 0.347375     0.063865     0.120926     0.006804    | 0.445732     0.068956     0.119242     0.018671    | 0.709205  0.606088  0.789180  | 0.045954  0.052306  0.027534 
+12    | 0.000293  | 0.144584     | 0.164707     | 0.862586        | 0.727577     | 0.047408          | 0.342801     0.059634     0.112964     0.006304    | 0.411730     0.058839     0.100306     0.017373    | 0.748005  0.642908  0.795577  | 0.057612  0.051775  0.032836 
+13    | 0.000270  | 0.140907     | 0.168478     | 0.858779        | 0.722437     | 0.050326          | 0.339146     0.055947     0.105981     0.005912    | 0.424251     0.058861     0.100609     0.017113    | 0.737337  0.646691  0.798538  | 0.059686  0.060250  0.031043 
+14    | 0.000255  | 0.141491     | 0.168934     | 0.863581        | 0.728418     | 0.046311          | 0.340245     0.056311     0.106678     0.005944    | 0.422276     0.060359     0.101728     0.018991    | 0.746346  0.645703  0.804566  | 0.062885  0.054186  0.021862 
+15    | 0.000250  | 0.141446     | 0.172203     | 0.858795        | 0.719748     | 0.048508          | 0.340810     0.056004     0.105944     0.006064    | 0.434858     0.059637     0.101203     0.018070    | 0.740666  0.646640  0.772434  | 0.063253  0.056133  0.026137</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confusion Matrix raw counts
+      LB    SB     S
+TP  2473  1949  1414
+FP   218   227    69
+FN   104   120   112
+TN  4501  5000  5701
+Confusion Matrix normalized per class
+       LB     SB      S
+TP  0.339  0.267  0.194
+FP  0.030  0.031  0.009
+FN  0.014  0.016  0.015
+TN  0.617  0.685  0.781
+Slice_W | Slice_H | Valid Loss   | Combined Metric | Dice Overall | Hausdorff Overall | VLo-Pres     VLo-Seg      VLo-D        VLo-B       | D-LB      D-SB      D-S       | H-LB      H-SB      H-S      
+----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+-1      | -1      | 0.172203     | 0.858795        | 0.719748     | 0.048508          | 0.434858     0.059637     0.101203     0.018070    | 0.740666  0.646640  0.772434  | 0.063253  0.056133  0.026137 
+266     | 266     | 0.170214     | 0.858907        | 0.721851     | 0.049722          | 0.427093     0.060123     0.101481     0.018764    | 0.734258  0.648920  0.794993  | 0.065082  0.057601  0.026483 
+360     | 310     | 0.187315     | 0.846249        | 0.672817     | 0.038130          | 0.504124     0.051540     0.093887     0.009193    | 0.751240  0.589983  0.624666  | 0.051217  0.046003  0.017169 
+276     | 276     | 0.189651     | 0.874396        | 0.752183     | 0.044129          | 0.478288     0.065949     0.111257     0.020641    | 0.828743  0.684690  0.687008  | 0.051863  0.047625  0.032900 </t>
+  </si>
 </sst>
 </file>
 
@@ -7685,7 +8522,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -7734,6 +8571,16 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -7790,7 +8637,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7913,6 +8760,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -8098,7 +8949,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K661"/>
+  <dimension ref="A1:K749"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="50.36"/>
@@ -13879,145 +14730,1061 @@
         <v>0.84971</v>
       </c>
     </row>
-    <row r="648" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="648" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A648" s="28" t="s">
         <v>136</v>
       </c>
+      <c r="B648" s="2" t="n">
+        <v>0.870889</v>
+      </c>
       <c r="C648" s="2" t="n">
         <v>0.86703</v>
       </c>
       <c r="D648" s="2" t="n">
         <v>0.85855</v>
       </c>
-    </row>
-    <row r="649" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E648" s="9" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="649" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A649" s="28" t="s">
         <v>247</v>
       </c>
+      <c r="B649" s="2" t="n">
+        <v>0.868587</v>
+      </c>
       <c r="C649" s="2" t="n">
         <v>0.86775</v>
       </c>
       <c r="D649" s="2" t="n">
         <v>0.85717</v>
       </c>
-    </row>
-    <row r="651" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A651" s="8" t="s">
-        <v>490</v>
-      </c>
-      <c r="B651" s="14" t="n">
-        <v>0.854633</v>
+      <c r="E649" s="12" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="650" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A650" s="28" t="s">
+        <v>492</v>
+      </c>
+      <c r="B650" s="2" t="n">
+        <v>0.871382</v>
+      </c>
+      <c r="C650" s="2" t="n">
+        <v>0.86741</v>
+      </c>
+      <c r="D650" s="2" t="n">
+        <v>0.85876</v>
+      </c>
+    </row>
+    <row r="651" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A651" s="28" t="s">
+        <v>493</v>
+      </c>
+      <c r="B651" s="2" t="n">
+        <v>0.871362</v>
       </c>
       <c r="C651" s="2" t="n">
-        <v>0.86175</v>
+        <v>0.86688</v>
       </c>
       <c r="D651" s="2" t="n">
-        <v>0.84634</v>
-      </c>
-      <c r="E651" s="12" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="652" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E652" s="12" t="s">
-        <v>492</v>
+        <v>0.8584</v>
+      </c>
+    </row>
+    <row r="652" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A652" s="28" t="s">
+        <v>494</v>
+      </c>
+      <c r="B652" s="2" t="n">
+        <v>0.870644</v>
+      </c>
+      <c r="C652" s="2" t="n">
+        <v>0.86815</v>
+      </c>
+      <c r="D652" s="2" t="n">
+        <v>0.85718</v>
       </c>
     </row>
     <row r="653" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A653" s="21" t="s">
-        <v>329</v>
-      </c>
-      <c r="B653" s="14" t="n">
-        <v>0.862318</v>
+      <c r="A653" s="28" t="s">
+        <v>495</v>
+      </c>
+      <c r="B653" s="2" t="n">
+        <v>0.87062</v>
       </c>
       <c r="C653" s="2" t="n">
-        <v>0.8493</v>
+        <v>0.86786</v>
       </c>
       <c r="D653" s="2" t="n">
-        <v>0.84614</v>
-      </c>
-    </row>
-    <row r="654" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A654" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="B654" s="14"/>
-      <c r="C654" s="2" t="n">
-        <v>0.86523</v>
-      </c>
-      <c r="D654" s="2" t="n">
-        <v>0.85548</v>
+        <v>0.85664</v>
+      </c>
+    </row>
+    <row r="654" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A654" s="8" t="s">
+        <v>496</v>
+      </c>
+      <c r="E654" s="31" t="s">
+        <v>497</v>
       </c>
     </row>
     <row r="655" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A655" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="B655" s="14"/>
+      <c r="A655" s="28" t="s">
+        <v>318</v>
+      </c>
       <c r="C655" s="2" t="n">
-        <v>0.86407</v>
+        <v>0.86505</v>
       </c>
       <c r="D655" s="2" t="n">
-        <v>0.85461</v>
-      </c>
-    </row>
-    <row r="657" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A657" s="8" t="s">
-        <v>493</v>
-      </c>
-      <c r="B657" s="14" t="n">
-        <v>0.850861</v>
+        <v>0.85439</v>
+      </c>
+    </row>
+    <row r="656" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A656" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="C656" s="2" t="n">
+        <v>0.85852</v>
+      </c>
+      <c r="D656" s="2" t="n">
+        <v>0.8467</v>
+      </c>
+    </row>
+    <row r="657" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A657" s="28" t="s">
+        <v>319</v>
       </c>
       <c r="C657" s="2" t="n">
-        <v>0.85765</v>
+        <v>0.8676</v>
       </c>
       <c r="D657" s="2" t="n">
-        <v>0.84015</v>
-      </c>
-      <c r="E657" s="12" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="658" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B658" s="3"/>
-      <c r="E658" s="12" t="s">
-        <v>495</v>
+        <v>0.85871</v>
+      </c>
+    </row>
+    <row r="658" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A658" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C658" s="2" t="n">
+        <v>0.86626</v>
+      </c>
+      <c r="D658" s="2" t="n">
+        <v>0.85871</v>
       </c>
     </row>
     <row r="659" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A659" s="28" t="s">
-        <v>178</v>
-      </c>
-      <c r="B659" s="14" t="n">
-        <v>0.865083</v>
+        <v>498</v>
       </c>
       <c r="C659" s="2" t="n">
-        <v>0.8545</v>
+        <v>0.86749</v>
       </c>
       <c r="D659" s="2" t="n">
-        <v>0.85111</v>
+        <v>0.85872</v>
       </c>
     </row>
     <row r="660" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A660" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="C660" s="2" t="n">
+        <v>0.86615</v>
+      </c>
+      <c r="D660" s="2" t="n">
+        <v>0.86139</v>
+      </c>
+    </row>
+    <row r="663" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A663" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="B663" s="14" t="n">
+        <v>0.854633</v>
+      </c>
+      <c r="C663" s="2" t="n">
+        <v>0.86175</v>
+      </c>
+      <c r="D663" s="2" t="n">
+        <v>0.84634</v>
+      </c>
+      <c r="E663" s="12" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="664" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E664" s="12" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="665" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A665" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="B665" s="14" t="n">
+        <v>0.862318</v>
+      </c>
+      <c r="C665" s="2" t="n">
+        <v>0.8493</v>
+      </c>
+      <c r="D665" s="2" t="n">
+        <v>0.84614</v>
+      </c>
+    </row>
+    <row r="666" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A666" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="C660" s="2" t="n">
+      <c r="B666" s="14"/>
+      <c r="C666" s="2" t="n">
+        <v>0.86523</v>
+      </c>
+      <c r="D666" s="2" t="n">
+        <v>0.85548</v>
+      </c>
+    </row>
+    <row r="667" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A667" s="21" t="s">
+        <v>330</v>
+      </c>
+      <c r="B667" s="14"/>
+      <c r="C667" s="2" t="n">
+        <v>0.86407</v>
+      </c>
+      <c r="D667" s="2" t="n">
+        <v>0.85461</v>
+      </c>
+    </row>
+    <row r="669" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A669" s="8" t="s">
+        <v>503</v>
+      </c>
+      <c r="B669" s="14" t="n">
+        <v>0.850861</v>
+      </c>
+      <c r="C669" s="2" t="n">
+        <v>0.85765</v>
+      </c>
+      <c r="D669" s="2" t="n">
+        <v>0.84015</v>
+      </c>
+      <c r="E669" s="12" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="670" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B670" s="3"/>
+      <c r="E670" s="12" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="671" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A671" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="B671" s="14" t="n">
+        <v>0.865083</v>
+      </c>
+      <c r="C671" s="2" t="n">
+        <v>0.8545</v>
+      </c>
+      <c r="D671" s="2" t="n">
+        <v>0.85111</v>
+      </c>
+    </row>
+    <row r="672" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A672" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C672" s="2" t="n">
         <v>0.86371</v>
       </c>
-      <c r="D660" s="2" t="n">
+      <c r="D672" s="2" t="n">
         <v>0.85558</v>
       </c>
     </row>
-    <row r="661" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A661" s="28" t="s">
+    <row r="673" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A673" s="28" t="s">
         <v>179</v>
       </c>
-      <c r="C661" s="2" t="n">
+      <c r="C673" s="2" t="n">
         <v>0.86298</v>
       </c>
-      <c r="D661" s="2" t="n">
+      <c r="D673" s="2" t="n">
         <v>0.85329</v>
+      </c>
+    </row>
+    <row r="675" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A675" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="B675" s="14" t="n">
+        <v>0.854522</v>
+      </c>
+      <c r="C675" s="2" t="n">
+        <v>0.84718</v>
+      </c>
+      <c r="D675" s="2" t="n">
+        <v>0.84355</v>
+      </c>
+      <c r="E675" s="12" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="676" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E676" s="12" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="677" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A677" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="B677" s="14" t="n">
+        <v>0.86253</v>
+      </c>
+      <c r="C677" s="2" t="n">
+        <v>0.86004</v>
+      </c>
+      <c r="D677" s="2" t="n">
+        <v>0.85335</v>
+      </c>
+    </row>
+    <row r="678" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A678" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C678" s="2" t="n">
+        <v>0.86544</v>
+      </c>
+      <c r="D678" s="2" t="n">
+        <v>0.85462</v>
+      </c>
+    </row>
+    <row r="679" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A679" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="C679" s="2" t="n">
+        <v>0.86633</v>
+      </c>
+      <c r="D679" s="2" t="n">
+        <v>0.85734</v>
+      </c>
+    </row>
+    <row r="681" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A681" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="B681" s="2" t="n">
+        <v>0.858275</v>
+      </c>
+      <c r="C681" s="2" t="n">
+        <v>0.85739</v>
+      </c>
+      <c r="D681" s="2" t="n">
+        <v>0.8508</v>
+      </c>
+      <c r="E681" s="12" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="682" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E682" s="12" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="683" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A683" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="B683" s="2" t="n">
+        <v>0.864511</v>
+      </c>
+      <c r="C683" s="2" t="n">
+        <v>0.85621</v>
+      </c>
+      <c r="D683" s="2" t="n">
+        <v>0.84959</v>
+      </c>
+    </row>
+    <row r="684" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A684" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C684" s="2" t="n">
+        <v>0.86452</v>
+      </c>
+      <c r="D684" s="2" t="n">
+        <v>0.85619</v>
+      </c>
+    </row>
+    <row r="685" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A685" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="C685" s="2" t="n">
+        <v>0.86428</v>
+      </c>
+      <c r="D685" s="2" t="n">
+        <v>0.85551</v>
+      </c>
+    </row>
+    <row r="687" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A687" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="B687" s="2" t="n">
+        <v>0.86508</v>
+      </c>
+      <c r="C687" s="2" t="n">
+        <v>0.86081</v>
+      </c>
+      <c r="D687" s="2" t="n">
+        <v>0.85376</v>
+      </c>
+      <c r="E687" s="12" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="688" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E688" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="689" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A689" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B689" s="2" t="n">
+        <v>0.870072</v>
+      </c>
+      <c r="C689" s="2" t="n">
+        <v>0.85701</v>
+      </c>
+      <c r="D689" s="2" t="n">
+        <v>0.84528</v>
+      </c>
+    </row>
+    <row r="690" customFormat="false" ht="359.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A690" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B690" s="2" t="n">
+        <v>0.871693</v>
+      </c>
+      <c r="C690" s="2" t="n">
+        <v>0.86519</v>
+      </c>
+      <c r="D690" s="2" t="n">
+        <v>0.85813</v>
+      </c>
+      <c r="E690" s="9" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="691" customFormat="false" ht="337.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A691" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="B691" s="2" t="n">
+        <v>0.87254</v>
+      </c>
+      <c r="C691" s="2" t="n">
+        <v>0.86503</v>
+      </c>
+      <c r="D691" s="2" t="n">
+        <v>0.85795</v>
+      </c>
+      <c r="E691" s="12" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="692" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A692" s="28" t="s">
+        <v>517</v>
+      </c>
+      <c r="B692" s="2" t="n">
+        <v>0.87223</v>
+      </c>
+      <c r="C692" s="2" t="n">
+        <v>0.86389</v>
+      </c>
+      <c r="D692" s="2" t="n">
+        <v>0.86041</v>
+      </c>
+    </row>
+    <row r="693" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A693" s="28" t="s">
+        <v>518</v>
+      </c>
+      <c r="B693" s="2" t="n">
+        <v>0.872073</v>
+      </c>
+      <c r="C693" s="2" t="n">
+        <v>0.86486</v>
+      </c>
+      <c r="D693" s="2" t="n">
+        <v>0.86098</v>
+      </c>
+    </row>
+    <row r="694" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A694" s="28" t="s">
+        <v>519</v>
+      </c>
+      <c r="B694" s="2" t="n">
+        <v>0.874002</v>
+      </c>
+      <c r="C694" s="2" t="n">
+        <v>0.86418</v>
+      </c>
+      <c r="D694" s="2" t="n">
+        <v>0.86059</v>
+      </c>
+    </row>
+    <row r="695" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A695" s="28" t="s">
+        <v>520</v>
+      </c>
+      <c r="B695" s="2" t="n">
+        <v>0.873765</v>
+      </c>
+      <c r="C695" s="2" t="n">
+        <v>0.86439</v>
+      </c>
+      <c r="D695" s="2" t="n">
+        <v>0.86094</v>
+      </c>
+    </row>
+    <row r="696" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A696" s="8" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="697" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A697" s="28" t="s">
+        <v>318</v>
+      </c>
+      <c r="C697" s="2" t="n">
+        <v>0.8615</v>
+      </c>
+      <c r="D697" s="2" t="n">
+        <v>0.84813</v>
+      </c>
+    </row>
+    <row r="698" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A698" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="C698" s="2" t="n">
+        <v>0.86424</v>
+      </c>
+      <c r="D698" s="2" t="n">
+        <v>0.85186</v>
+      </c>
+    </row>
+    <row r="699" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A699" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="C699" s="2" t="n">
+        <v>0.86738</v>
+      </c>
+      <c r="D699" s="2" t="n">
+        <v>0.8567</v>
+      </c>
+    </row>
+    <row r="700" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A700" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C700" s="2" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="D700" s="2" t="n">
+        <v>0.85713</v>
+      </c>
+    </row>
+    <row r="701" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A701" s="28" t="s">
+        <v>517</v>
+      </c>
+      <c r="C701" s="2" t="n">
+        <v>0.86707</v>
+      </c>
+      <c r="D701" s="2" t="n">
+        <v>0.8585</v>
+      </c>
+    </row>
+    <row r="702" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A702" s="28" t="s">
+        <v>519</v>
+      </c>
+      <c r="C702" s="2" t="n">
+        <v>0.8666</v>
+      </c>
+      <c r="D702" s="2" t="n">
+        <v>0.85985</v>
+      </c>
+    </row>
+    <row r="704" customFormat="false" ht="382.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A704" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="B704" s="2" t="n">
+        <v>0.864459</v>
+      </c>
+      <c r="C704" s="2" t="n">
+        <v>0.85978</v>
+      </c>
+      <c r="D704" s="2" t="n">
+        <v>0.85077</v>
+      </c>
+      <c r="E704" s="12" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="705" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E705" s="12" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="706" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A706" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B706" s="2" t="n">
+        <v>0.867442</v>
+      </c>
+      <c r="C706" s="2" t="n">
+        <v>0.86194</v>
+      </c>
+      <c r="D706" s="2" t="n">
+        <v>0.84611</v>
+      </c>
+    </row>
+    <row r="707" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A707" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C707" s="2" t="n">
+        <v>0.86569</v>
+      </c>
+      <c r="D707" s="2" t="n">
+        <v>0.85634</v>
+      </c>
+    </row>
+    <row r="708" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A708" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C708" s="2" t="n">
+        <v>0.86512</v>
+      </c>
+      <c r="D708" s="2" t="n">
+        <v>0.85614</v>
+      </c>
+    </row>
+    <row r="710" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A710" s="8" t="s">
+        <v>525</v>
+      </c>
+      <c r="B710" s="2" t="n">
+        <v>0.863709</v>
+      </c>
+      <c r="C710" s="2" t="n">
+        <v>0.84933</v>
+      </c>
+      <c r="D710" s="2" t="n">
+        <v>0.85011</v>
+      </c>
+      <c r="E710" s="31" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="711" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E711" s="31" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="712" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A712" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B712" s="2" t="n">
+        <v>0.864676</v>
+      </c>
+      <c r="C712" s="2" t="n">
+        <v>0.86461</v>
+      </c>
+      <c r="D712" s="2" t="n">
+        <v>0.85517</v>
+      </c>
+    </row>
+    <row r="713" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A713" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C713" s="2" t="n">
+        <v>0.86734</v>
+      </c>
+      <c r="D713" s="2" t="n">
+        <v>0.85942</v>
+      </c>
+    </row>
+    <row r="714" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A714" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C714" s="2" t="n">
+        <v>0.86691</v>
+      </c>
+      <c r="D714" s="2" t="n">
+        <v>0.85876</v>
+      </c>
+    </row>
+    <row r="716" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A716" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="B716" s="2" t="n">
+        <v>0.864115</v>
+      </c>
+      <c r="C716" s="2" t="n">
+        <v>0.85545</v>
+      </c>
+      <c r="D716" s="2" t="n">
+        <v>0.84709</v>
+      </c>
+      <c r="E716" s="31" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="717" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E717" s="31" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="718" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A718" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B718" s="2" t="n">
+        <v>0.866803</v>
+      </c>
+      <c r="C718" s="2" t="n">
+        <v>0.85734</v>
+      </c>
+      <c r="D718" s="2" t="n">
+        <v>0.84773</v>
+      </c>
+    </row>
+    <row r="719" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A719" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C719" s="2" t="n">
+        <v>0.86575</v>
+      </c>
+      <c r="D719" s="2" t="n">
+        <v>0.85806</v>
+      </c>
+    </row>
+    <row r="720" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A720" s="28" t="s">
+        <v>247</v>
+      </c>
+      <c r="C720" s="2" t="n">
+        <v>0.86538</v>
+      </c>
+      <c r="D720" s="2" t="n">
+        <v>0.858</v>
+      </c>
+    </row>
+    <row r="722" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A722" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="B722" s="2" t="n">
+        <v>0.862005</v>
+      </c>
+      <c r="C722" s="2" t="n">
+        <v>0.85972</v>
+      </c>
+      <c r="D722" s="2" t="n">
+        <v>0.85329</v>
+      </c>
+      <c r="E722" s="31" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="723" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E723" s="31" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="724" customFormat="false" ht="370.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A724" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C724" s="2" t="n">
+        <v>0.86737</v>
+      </c>
+      <c r="D724" s="2" t="n">
+        <v>0.86271</v>
+      </c>
+      <c r="E724" s="9" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="725" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A725" s="28" t="s">
+        <v>535</v>
+      </c>
+      <c r="B725" s="2" t="n">
+        <v>0.868768</v>
+      </c>
+      <c r="C725" s="2" t="n">
+        <v>0.86808</v>
+      </c>
+      <c r="D725" s="2" t="n">
+        <v>0.86331</v>
+      </c>
+    </row>
+    <row r="726" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A726" s="28" t="s">
+        <v>536</v>
+      </c>
+      <c r="B726" s="2" t="n">
+        <v>0.868573</v>
+      </c>
+      <c r="C726" s="2" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="D726" s="2" t="n">
+        <v>0.86288</v>
+      </c>
+    </row>
+    <row r="727" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A727" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="E727" s="31" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="728" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A728" s="28" t="s">
+        <v>318</v>
+      </c>
+      <c r="C728" s="2" t="n">
+        <v>0.8644</v>
+      </c>
+      <c r="D728" s="2" t="n">
+        <v>0.85407</v>
+      </c>
+    </row>
+    <row r="729" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A729" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="C729" s="2" t="n">
+        <v>0.86884</v>
+      </c>
+      <c r="D729" s="2" t="n">
+        <v>0.85957</v>
+      </c>
+    </row>
+    <row r="730" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A730" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="C730" s="2" t="n">
+        <v>0.85935</v>
+      </c>
+      <c r="D730" s="2" t="n">
+        <v>0.84446</v>
+      </c>
+    </row>
+    <row r="731" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A731" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C731" s="2" t="n">
+        <v>0.86871</v>
+      </c>
+      <c r="D731" s="2" t="n">
+        <v>0.85875</v>
+      </c>
+    </row>
+    <row r="732" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A732" s="28" t="s">
+        <v>539</v>
+      </c>
+      <c r="C732" s="2" t="n">
+        <v>0.86897</v>
+      </c>
+      <c r="D732" s="2" t="n">
+        <v>0.8603</v>
+      </c>
+    </row>
+    <row r="733" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A733" s="28" t="s">
+        <v>540</v>
+      </c>
+      <c r="C733" s="2" t="n">
+        <v>0.86912</v>
+      </c>
+      <c r="D733" s="2" t="n">
+        <v>0.86037</v>
+      </c>
+    </row>
+    <row r="735" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A735" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="B735" s="2" t="n">
+        <v>0.861426</v>
+      </c>
+      <c r="C735" s="2" t="n">
+        <v>0.85756</v>
+      </c>
+      <c r="D735" s="2" t="n">
+        <v>0.84948</v>
+      </c>
+      <c r="E735" s="31" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="736" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E736" s="31" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="737" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A737" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C737" s="2" t="n">
+        <v>0.86642</v>
+      </c>
+      <c r="D737" s="2" t="n">
+        <v>0.85608</v>
+      </c>
+    </row>
+    <row r="739" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A739" s="8" t="s">
+        <v>544</v>
+      </c>
+      <c r="B739" s="2" t="n">
+        <v>0.864268</v>
+      </c>
+      <c r="C739" s="2" t="n">
+        <v>0.85847</v>
+      </c>
+      <c r="D739" s="2" t="n">
+        <v>0.84902</v>
+      </c>
+      <c r="E739" s="31" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="740" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E740" s="31" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="741" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A741" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="B741" s="2" t="n">
+        <v>0.866135</v>
+      </c>
+      <c r="C741" s="2" t="n">
+        <v>0.84528</v>
+      </c>
+      <c r="D741" s="2" t="n">
+        <v>0.83368</v>
+      </c>
+    </row>
+    <row r="742" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A742" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C742" s="2" t="n">
+        <v>0.86619</v>
+      </c>
+      <c r="D742" s="2" t="n">
+        <v>0.85755</v>
+      </c>
+    </row>
+    <row r="743" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A743" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="C743" s="2" t="n">
+        <v>0.86539</v>
+      </c>
+      <c r="D743" s="2" t="n">
+        <v>0.85672</v>
+      </c>
+    </row>
+    <row r="745" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A745" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="B745" s="2" t="n">
+        <v>0.858795</v>
+      </c>
+      <c r="C745" s="2" t="n">
+        <v>0.85388</v>
+      </c>
+      <c r="D745" s="2" t="n">
+        <v>0.84805</v>
+      </c>
+      <c r="E745" s="31" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="746" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E746" s="31" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="747" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A747" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B747" s="2" t="n">
+        <v>0.863581</v>
+      </c>
+      <c r="C747" s="2" t="n">
+        <v>0.85271</v>
+      </c>
+      <c r="D747" s="2" t="n">
+        <v>0.84238</v>
+      </c>
+    </row>
+    <row r="748" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A748" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C748" s="2" t="n">
+        <v>0.86574</v>
+      </c>
+      <c r="D748" s="2" t="n">
+        <v>0.85799</v>
+      </c>
+    </row>
+    <row r="749" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A749" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C749" s="2" t="n">
+        <v>0.86559</v>
+      </c>
+      <c r="D749" s="2" t="n">
+        <v>0.85841</v>
       </c>
     </row>
   </sheetData>

</xml_diff>